<commit_message>
Dados atualizados em 25/05/2026 12:25
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F308EE5C-1B3E-4571-A53B-3AD2DE684BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13522F41-E5A7-4328-B528-9DED77B67E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -448,23 +448,11 @@
   </cellStyles>
   <dxfs count="71">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -484,6 +472,297 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -507,39 +786,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -556,50 +802,15 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -626,15 +837,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -654,6 +856,18 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -670,147 +884,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -831,79 +904,6 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1009,7 +1009,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>42064.41</v>
+            <v>42064.409999999996</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
@@ -1046,7 +1046,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>5023.8099999999995</v>
+            <v>6873.1099999999988</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1080,7 +1080,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>72337.739999999976</v>
+            <v>74187.039999999979</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
@@ -1106,13 +1106,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>5565.7</v>
+            <v>7809.8</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>29</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="11">
@@ -1126,7 +1126,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>6930.15</v>
+            <v>11772.469999999996</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1186,13 +1186,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>1944.5599999999997</v>
+            <v>3513.6600000000008</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>37</v>
+            <v>38</v>
           </cell>
         </row>
         <row r="15">
@@ -1206,7 +1206,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>8841.1</v>
+            <v>10989.6</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1220,7 +1220,7 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>354515.53999999992</v>
+            <v>365838.24999999988</v>
           </cell>
           <cell r="H16" t="str">
             <v>OSASCO</v>
@@ -1240,13 +1240,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>269162.04999999993</v>
+            <v>276494.14999999997</v>
           </cell>
           <cell r="H17" t="str">
             <v>PERDIZES</v>
           </cell>
           <cell r="I17">
-            <v>2695.5</v>
+            <v>4673.7</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1260,13 +1260,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>79238.779999999984</v>
+            <v>81482.879999999961</v>
           </cell>
           <cell r="H18" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I18">
-            <v>1985.0500000000002</v>
+            <v>1985.05</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1280,13 +1280,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>113246.73999999974</v>
+            <v>118089.05999999971</v>
           </cell>
           <cell r="H19" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I19">
-            <v>8680.4700000000012</v>
+            <v>9527.3700000000008</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1306,7 +1306,7 @@
             <v>SBC</v>
           </cell>
           <cell r="I20">
-            <v>5611.2999999999993</v>
+            <v>9345.1200000000008</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1326,7 +1326,7 @@
             <v>SJC</v>
           </cell>
           <cell r="I21">
-            <v>6881.4</v>
+            <v>8404.1</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
@@ -1340,7 +1340,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>57549.270000000135</v>
+            <v>59118.370000000134</v>
           </cell>
           <cell r="H22" t="str">
             <v>SJC/VALE</v>
@@ -1360,7 +1360,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>176829.40999999963</v>
+            <v>178977.90999999963</v>
           </cell>
           <cell r="H23" t="str">
             <v>VENDEDOR INTERNO 1</v>
@@ -1380,19 +1380,19 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>240078.9549999999</v>
+            <v>240078.95500000002</v>
           </cell>
           <cell r="H24" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I24">
-            <v>112681.63500000004</v>
+            <v>133416.57500000007</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N24">
-            <v>19</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="25">
@@ -1400,7 +1400,7 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>73548.510000000038</v>
+            <v>75526.710000000036</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
@@ -1420,7 +1420,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>539</v>
+            <v>542</v>
           </cell>
         </row>
         <row r="27">
@@ -1436,7 +1436,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>127427.03999999995</v>
+            <v>128273.93999999996</v>
           </cell>
         </row>
         <row r="29">
@@ -1444,7 +1444,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>195843.32999999975</v>
+            <v>199577.14999999976</v>
           </cell>
         </row>
         <row r="30">
@@ -1452,7 +1452,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>59955.540000000066</v>
+            <v>61478.240000000063</v>
           </cell>
         </row>
         <row r="31">
@@ -1479,7 +1479,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4041783.7449999703</v>
+            <v>4081173.4949999694</v>
           </cell>
         </row>
         <row r="34">
@@ -1725,27 +1725,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C97E85A-DD10-4825-81C1-53CD3989178B}" name="Tabela1" displayName="Tabela1" ref="B4:C7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C97E85A-DD10-4825-81C1-53CD3989178B}" name="Tabela1" displayName="Tabela1" ref="B4:C7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{3308613D-E7FC-469E-B078-C5AC910E183B}" name="Coluna1" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{C994D666-6174-475E-AE71-1F12062A5225}" name="Coluna2" headerRowDxfId="7" dataDxfId="6" dataCellStyle="Moeda"/>
+    <tableColumn id="1" xr3:uid="{3308613D-E7FC-469E-B078-C5AC910E183B}" name="Coluna1" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{C994D666-6174-475E-AE71-1F12062A5225}" name="Coluna2" headerRowDxfId="67" dataDxfId="66" dataCellStyle="Moeda"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7AAFC688-3718-400A-9213-0DC213191E8B}" name="Tabela10" displayName="Tabela10" ref="T4:U7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7AAFC688-3718-400A-9213-0DC213191E8B}" name="Tabela10" displayName="Tabela10" ref="T4:U7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{870B59CA-1EA4-4CA9-BDCF-4A342A313131}" name="Coluna1" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{6FE31DF2-1DB4-4D4B-8783-48EA07B43B53}" name="Coluna2" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{870B59CA-1EA4-4CA9-BDCF-4A342A313131}" name="Coluna1" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{6FE31DF2-1DB4-4D4B-8783-48EA07B43B53}" name="Coluna2" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{8D294CDB-54E7-40E9-918D-B86BC1FA5B4D}" name="Tabela11" displayName="Tabela11" ref="S9:W27" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{8D294CDB-54E7-40E9-918D-B86BC1FA5B4D}" name="Tabela11" displayName="Tabela11" ref="S9:W27" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="S9:W27" xr:uid="{8D294CDB-54E7-40E9-918D-B86BC1FA5B4D}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1757,15 +1757,15 @@
     <sortCondition ref="T10:T27"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{6C671431-FBD2-41CB-81F2-E1D2D5C3888E}" name="REFERENCA" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{3321EAFD-68B3-45FD-82F1-B5E31F19D7D3}" name="VENDEDOR" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{AD30FAD6-BD3A-4C4F-AF4F-02A7C67B6AB2}" name="META A" dataDxfId="23">
+    <tableColumn id="1" xr3:uid="{6C671431-FBD2-41CB-81F2-E1D2D5C3888E}" name="REFERENCA" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{3321EAFD-68B3-45FD-82F1-B5E31F19D7D3}" name="VENDEDOR" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{AD30FAD6-BD3A-4C4F-AF4F-02A7C67B6AB2}" name="META A" dataDxfId="8">
       <calculatedColumnFormula>_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{35971163-4E8E-4FB4-9A55-B9150EF30EA3}" name="ATINGIDO" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{35971163-4E8E-4FB4-9A55-B9150EF30EA3}" name="ATINGIDO" dataDxfId="7">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{900877A2-EB90-4B84-84FB-93F04FC17C31}" name="FALTA" dataDxfId="22">
+    <tableColumn id="5" xr3:uid="{900877A2-EB90-4B84-84FB-93F04FC17C31}" name="FALTA" dataDxfId="6">
       <calculatedColumnFormula>U10-V10</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1774,7 +1774,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}" name="Tabela12" displayName="Tabela12" ref="T29:W33" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}" name="Tabela12" displayName="Tabela12" ref="T29:W33" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="T29:W33" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1782,14 +1782,14 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{65A441BB-28F2-4C4D-8CD8-F9F9788A0656}" name="SEMANAL" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{B849FCBC-ED0F-47D9-B4E7-149FFE3500D9}" name="META" dataDxfId="18" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{65A441BB-28F2-4C4D-8CD8-F9F9788A0656}" name="SEMANAL" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{B849FCBC-ED0F-47D9-B4E7-149FFE3500D9}" name="META" dataDxfId="2" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(T30,[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]]),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A81AB4FC-EF49-4A93-8229-1B0CBFC88744}" name="REALIZADO" dataDxfId="17">
+    <tableColumn id="3" xr3:uid="{A81AB4FC-EF49-4A93-8229-1B0CBFC88744}" name="REALIZADO" dataDxfId="1">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[PARAMETRO]","[Intervalo 2].[PARAMETRO].&amp;[DIA]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{13865A0A-FFF3-4F90-A201-753948DC8E26}" name="FALTA" dataDxfId="16">
+    <tableColumn id="4" xr3:uid="{13865A0A-FFF3-4F90-A201-753948DC8E26}" name="FALTA" dataDxfId="0">
       <calculatedColumnFormula>U30-V30</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1798,7 +1798,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AF588D8F-0EAF-4694-8155-49E9449C8646}" name="Tabela2" displayName="Tabela2" ref="A9:E36" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AF588D8F-0EAF-4694-8155-49E9449C8646}" name="Tabela2" displayName="Tabela2" ref="A9:E36" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
   <autoFilter ref="A9:E36" xr:uid="{AF588D8F-0EAF-4694-8155-49E9449C8646}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1807,15 +1807,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{DE539CA3-DD4F-4562-9255-667EB2ABB37D}" name="REFERENCIA" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{B6B5F834-D2C3-4E6B-9152-8D2305647335}" name="VENDEDOR" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{7919932F-13DB-49D5-8C5B-D7469C8E992A}" name="META A" dataDxfId="66" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{DE539CA3-DD4F-4562-9255-667EB2ABB37D}" name="REFERENCIA" dataDxfId="63"/>
+    <tableColumn id="2" xr3:uid="{B6B5F834-D2C3-4E6B-9152-8D2305647335}" name="VENDEDOR" dataDxfId="62"/>
+    <tableColumn id="3" xr3:uid="{7919932F-13DB-49D5-8C5B-D7469C8E992A}" name="META A" dataDxfId="61" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A10,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{6BCB028E-83E7-4C15-A040-683869678C23}" name="ATINGIDO" dataDxfId="65" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{6BCB028E-83E7-4C15-A040-683869678C23}" name="ATINGIDO" dataDxfId="60" dataCellStyle="Moeda">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0EA33871-188E-4A83-8657-B6F207C7245D}" name="FALTA" dataDxfId="64">
+    <tableColumn id="5" xr3:uid="{0EA33871-188E-4A83-8657-B6F207C7245D}" name="FALTA" dataDxfId="59">
       <calculatedColumnFormula>C10-D10</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1824,7 +1824,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}" name="Tabela3" displayName="Tabela3" ref="B38:E42" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}" name="Tabela3" displayName="Tabela3" ref="B38:E42" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="B38:E42" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1832,14 +1832,14 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D5CFA35F-1C13-42CF-B05C-430BF14AC2B0}" name="SEMANAL" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{06063E15-5C9E-4303-B5F6-B9D0B178DB82}" name="META" dataDxfId="60" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{D5CFA35F-1C13-42CF-B05C-430BF14AC2B0}" name="SEMANAL" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{06063E15-5C9E-4303-B5F6-B9D0B178DB82}" name="META" dataDxfId="55" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(B39,[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]]),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{425F53BB-8CBB-40E8-9773-1C7C39906AD7}" name="REALIZADO" dataDxfId="59" dataCellStyle="Moeda">
+    <tableColumn id="3" xr3:uid="{425F53BB-8CBB-40E8-9773-1C7C39906AD7}" name="REALIZADO" dataDxfId="54" dataCellStyle="Moeda">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A18F5082-185F-44C4-B163-8A3CBDDA6732}" name="FALTA" dataDxfId="58">
+    <tableColumn id="4" xr3:uid="{A18F5082-185F-44C4-B163-8A3CBDDA6732}" name="FALTA" dataDxfId="53">
       <calculatedColumnFormula>C39-D39</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1848,17 +1848,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BA69D712-8843-4CBF-AD2F-C801E56B1CFC}" name="Tabela4" displayName="Tabela4" ref="H4:I7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BA69D712-8843-4CBF-AD2F-C801E56B1CFC}" name="Tabela4" displayName="Tabela4" ref="H4:I7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C661D03F-A79A-4D24-86FD-3574B6E5537D}" name="Coluna1" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{7EF7A574-C8A3-4CB7-9C98-86948FE130EB}" name="Coluna2" headerRowDxfId="2" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{C661D03F-A79A-4D24-86FD-3574B6E5537D}" name="Coluna1" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{7EF7A574-C8A3-4CB7-9C98-86948FE130EB}" name="Coluna2" headerRowDxfId="49" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4F0EC2C2-A52E-4D47-97B3-678B19401BEF}" name="Tabela5" displayName="Tabela5" ref="G9:K28" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4F0EC2C2-A52E-4D47-97B3-678B19401BEF}" name="Tabela5" displayName="Tabela5" ref="G9:K28" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="G9:K28" xr:uid="{4F0EC2C2-A52E-4D47-97B3-678B19401BEF}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1867,15 +1867,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{0D4D84CB-5C40-4B8B-B729-ACB9E6533B94}" name="REFERENCIA" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{3E3AB0E2-F62B-4424-B617-E867D719DDB5}" name="VENDEDOR" dataDxfId="54"/>
-    <tableColumn id="3" xr3:uid="{9941E429-6355-4240-BED7-987A5372BF7E}" name="COMPROMISSO" dataDxfId="53" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{0D4D84CB-5C40-4B8B-B729-ACB9E6533B94}" name="REFERENCIA" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{3E3AB0E2-F62B-4424-B617-E867D719DDB5}" name="VENDEDOR" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{9941E429-6355-4240-BED7-987A5372BF7E}" name="COMPROMISSO" dataDxfId="43" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(G10,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{19E4A6B6-F14F-478B-9480-45017062F357}" name="ATINGIDO" dataDxfId="52" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{19E4A6B6-F14F-478B-9480-45017062F357}" name="ATINGIDO" dataDxfId="42" dataCellStyle="Moeda">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{73981291-35E4-400C-A341-764C2B1C460A}" name="FALTA" dataDxfId="51">
+    <tableColumn id="5" xr3:uid="{73981291-35E4-400C-A341-764C2B1C460A}" name="FALTA" dataDxfId="41">
       <calculatedColumnFormula>I10-J10</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1884,7 +1884,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}" name="Tabela6" displayName="Tabela6" ref="H30:K34" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}" name="Tabela6" displayName="Tabela6" ref="H30:K34" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
   <autoFilter ref="H30:K34" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1892,14 +1892,14 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{14E3BD3B-54B0-47BF-931C-064E12741C86}" name="SEMANAL" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{67CE9FE2-AA11-4BD4-9F34-EDC9123EA89F}" name="META" dataDxfId="47" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{14E3BD3B-54B0-47BF-931C-064E12741C86}" name="SEMANAL" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{67CE9FE2-AA11-4BD4-9F34-EDC9123EA89F}" name="META" dataDxfId="37" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(H31,[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]]),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{14D3AA11-9DFC-420F-8F5A-5002E14D4AAA}" name="REALIZADO" dataDxfId="46">
+    <tableColumn id="3" xr3:uid="{14D3AA11-9DFC-420F-8F5A-5002E14D4AAA}" name="REALIZADO" dataDxfId="36">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{16DC2DF3-76D8-4A80-B29C-E276BB17D8FF}" name="FALTA" dataDxfId="45">
+    <tableColumn id="4" xr3:uid="{16DC2DF3-76D8-4A80-B29C-E276BB17D8FF}" name="FALTA" dataDxfId="35">
       <calculatedColumnFormula>I31-J31</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1908,17 +1908,17 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9D5C0B8F-3138-4FD4-9A83-375E8D4AC464}" name="Tabela7" displayName="Tabela7" ref="N4:O7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9D5C0B8F-3138-4FD4-9A83-375E8D4AC464}" name="Tabela7" displayName="Tabela7" ref="N4:O7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{0139F26F-4C9F-4E96-9F64-C5C5B271DCA9}" name="Coluna1" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{1DA3E17F-38EB-4042-B2F0-3DFB7629A3F5}" name="Coluna2" headerRowDxfId="12" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{0139F26F-4C9F-4E96-9F64-C5C5B271DCA9}" name="Coluna1" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{1DA3E17F-38EB-4042-B2F0-3DFB7629A3F5}" name="Coluna2" headerRowDxfId="31" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{87A5A608-D233-46F9-8E75-B1963DE71BC6}" name="Tabela8" displayName="Tabela8" ref="M10:Q17" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43" dataCellStyle="Moeda">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{87A5A608-D233-46F9-8E75-B1963DE71BC6}" name="Tabela8" displayName="Tabela8" ref="M10:Q17" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" dataCellStyle="Moeda">
   <autoFilter ref="M10:Q17" xr:uid="{87A5A608-D233-46F9-8E75-B1963DE71BC6}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1927,15 +1927,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{EE89D966-6315-4DB4-9927-EEB09B51F44E}" name="REFERENCIA" dataDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{0B55D821-52F8-4CE2-9F16-C5BCDBCE53AC}" name="VENDEDOR" dataDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{B5D24BF0-392E-420D-BB1D-3FED1D3383B5}" name="COMPROMISSO" dataDxfId="40" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{EE89D966-6315-4DB4-9927-EEB09B51F44E}" name="REFERENCIA" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{0B55D821-52F8-4CE2-9F16-C5BCDBCE53AC}" name="VENDEDOR" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{B5D24BF0-392E-420D-BB1D-3FED1D3383B5}" name="COMPROMISSO" dataDxfId="25" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(M11,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{92C88D8B-4724-4B0F-86B9-CEB8CCE813E5}" name="ATINGIDO" dataDxfId="39" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{92C88D8B-4724-4B0F-86B9-CEB8CCE813E5}" name="ATINGIDO" dataDxfId="24" dataCellStyle="Moeda">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{CA195FA3-3822-41FA-8A93-2D86914C048E}" name="FALTA" dataDxfId="38" dataCellStyle="Moeda">
+    <tableColumn id="5" xr3:uid="{CA195FA3-3822-41FA-8A93-2D86914C048E}" name="FALTA" dataDxfId="23" dataCellStyle="Moeda">
       <calculatedColumnFormula>O11-P11</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1944,7 +1944,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{3D6BA5FD-BBE8-4A7A-9B76-3F3F6D1F10E9}" name="Tabela9" displayName="Tabela9" ref="N19:Q23" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{3D6BA5FD-BBE8-4A7A-9B76-3F3F6D1F10E9}" name="Tabela9" displayName="Tabela9" ref="N19:Q23" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="N19:Q23" xr:uid="{3D6BA5FD-BBE8-4A7A-9B76-3F3F6D1F10E9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1952,14 +1952,14 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{985251B0-0E07-4E60-9774-18D0D763437D}" name="SEMANAL" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{7B11DBA8-6FBD-4B67-BDA9-6624DF753EFD}" name="META" dataDxfId="34" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{985251B0-0E07-4E60-9774-18D0D763437D}" name="SEMANAL" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{7B11DBA8-6FBD-4B67-BDA9-6624DF753EFD}" name="META" dataDxfId="19" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(N20,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0B727490-D536-4FC5-B857-CD92C459F1FB}" name="REALIZADO" dataDxfId="33">
+    <tableColumn id="3" xr3:uid="{0B727490-D536-4FC5-B857-CD92C459F1FB}" name="REALIZADO" dataDxfId="18">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{84544AF4-5466-4CAC-A349-7B2C804BDA05}" name="FALTA" dataDxfId="32">
+    <tableColumn id="4" xr3:uid="{84544AF4-5466-4CAC-A349-7B2C804BDA05}" name="FALTA" dataDxfId="17">
       <calculatedColumnFormula>O20-P20</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4041171.8449999979</v>
+        <v>4080561.5949999979</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>112681.63499999998</v>
+        <v>133416.57500000001</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1140328.1550000021</v>
+        <v>1100938.4050000021</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>187538.36500000002</v>
+        <v>166803.42499999999</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.77992315835182824</v>
+        <v>0.78752515584290217</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.37533020784757837</v>
+        <v>0.44439602624741859</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.67374999999999996</v>
+        <v>0.67749999999999999</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2645,11 +2645,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>42064.41</v>
+        <v>42064.409999999996</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>22435.589999999997</v>
+        <v>22435.590000000004</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2738,11 +2738,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8841.1</v>
+        <v>10989.6</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>15658.9</v>
+        <v>13510.4</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1985.0500000000002</v>
+        <v>1985.05</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
@@ -2853,11 +2853,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>72337.739999999976</v>
+        <v>74187.039999999979</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>7662.2600000000239</v>
+        <v>5812.960000000021</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2892,11 +2892,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5611.2999999999993</v>
+        <v>9345.1200000000008</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>15388.7</v>
+        <v>11654.88</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3123,11 +3123,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8680.4700000000012</v>
+        <v>9527.3700000000008</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>9969.5299999999988</v>
+        <v>9122.6299999999992</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1944.5599999999997</v>
+        <v>3513.6600000000008</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>4715.4400000000005</v>
+        <v>3146.3399999999992</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3238,11 +3238,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3277,11 +3277,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5565.7</v>
+        <v>7809.8</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>6934.3</v>
+        <v>4690.2</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3341,11 +3341,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6930.15</v>
+        <v>11772.469999999996</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>10069.85</v>
+        <v>5227.5300000000043</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3394,11 +3394,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>354515.53999999992</v>
+        <v>365838.24999999988</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>145484.46000000008</v>
+        <v>134161.75000000012</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3469,11 +3469,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>269162.04999999993</v>
+        <v>276494.14999999997</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>158337.95000000007</v>
+        <v>151005.85000000003</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3488,11 +3488,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2695.5</v>
+        <v>4673.7</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>10574.5</v>
+        <v>8596.2999999999993</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3544,11 +3544,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>79238.779999999984</v>
+        <v>81482.879999999961</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>40261.220000000016</v>
+        <v>38017.120000000039</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3619,11 +3619,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>113246.73999999974</v>
+        <v>118089.05999999971</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>43753.260000000257</v>
+        <v>38910.940000000293</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3655,11 +3655,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>43994.75</v>
+        <v>62649.559999999983</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>673505.25</v>
+        <v>654850.44000000006</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3713,11 +3713,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5023.8099999999995</v>
+        <v>6873.1099999999988</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>4456.1900000000005</v>
+        <v>2606.8900000000012</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3802,11 +3802,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3822,11 +3822,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>57549.270000000135</v>
+        <v>59118.370000000134</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>32450.729999999865</v>
+        <v>30881.629999999866</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3841,11 +3841,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6881.4</v>
+        <v>8404.1</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>7308.6</v>
+        <v>5785.9</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3886,11 +3886,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>176829.40999999963</v>
+        <v>178977.90999999963</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>58170.590000000375</v>
+        <v>56022.090000000375</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>240078.9549999999</v>
+        <v>240078.95500000002</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>61921.0450000001</v>
+        <v>61921.044999999984</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -4001,11 +4001,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>73548.510000000038</v>
+        <v>75526.710000000036</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>39451.489999999962</v>
+        <v>37473.289999999964</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4121,11 +4121,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>645369.17500000284</v>
+        <v>645369.17500000272</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>54630.824999997159</v>
+        <v>54630.824999997276</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4164,11 +4164,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>127427.03999999995</v>
+        <v>128273.93999999996</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>39572.96000000005</v>
+        <v>38726.060000000041</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4224,11 +4224,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>195843.32999999975</v>
+        <v>199577.14999999976</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>59156.670000000246</v>
+        <v>55422.850000000239</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4241,11 +4241,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>685356.89500000118</v>
+        <v>685356.8950000013</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>14643.104999998817</v>
+        <v>14643.104999998701</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4264,11 +4264,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4284,11 +4284,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>59955.540000000066</v>
+        <v>61478.240000000063</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>40044.459999999934</v>
+        <v>38521.759999999937</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4301,11 +4301,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>112681.63499999995</v>
+        <v>133416.57499999995</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>587318.36499999999</v>
+        <v>566583.42500000005</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4464,11 +4464,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.5950000002</v>
+        <v>1184379.595</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.404999999795</v>
+        <v>95620.405000000028</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4536,11 +4536,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1175113.6449999928</v>
+        <v>1175113.6449999923</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>104886.3550000072</v>
+        <v>104886.35500000766</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4572,11 +4572,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>156676.38499999989</v>
+        <v>196066.13499999992</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>1123323.6150000002</v>
+        <v>1083933.865</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 25/05/2026 13:58
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13522F41-E5A7-4328-B528-9DED77B67E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35E1AF2-B5CE-4FDC-BCE7-1F541DF27D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -945,11 +945,11 @@
       <sheetName val="DIN MILHO"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
@@ -1066,7 +1066,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>10994.599999999999</v>
+            <v>12314.519999999999</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1100,7 +1100,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>178083.97999999984</v>
+            <v>179403.89999999985</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE</v>
@@ -1186,7 +1186,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>3513.6600000000008</v>
+            <v>4875.3600000000006</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1200,13 +1200,13 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>63353.700000000041</v>
+            <v>66182.300000000047</v>
           </cell>
           <cell r="H15" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>10989.6</v>
+            <v>15117.849999999995</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1220,13 +1220,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>365838.24999999988</v>
+            <v>384255.84999999992</v>
           </cell>
           <cell r="H16" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>9101.1449999999986</v>
+            <v>11646.094999999996</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1252,7 +1252,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>26</v>
+            <v>27</v>
           </cell>
         </row>
         <row r="18">
@@ -1266,13 +1266,13 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="I18">
-            <v>1985.05</v>
+            <v>1985.0500000000002</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>33</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="19">
@@ -1306,7 +1306,7 @@
             <v>SBC</v>
           </cell>
           <cell r="I20">
-            <v>9345.1200000000008</v>
+            <v>10460.219999999999</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1340,7 +1340,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>59118.370000000134</v>
+            <v>60480.070000000131</v>
           </cell>
           <cell r="H22" t="str">
             <v>SJC/VALE</v>
@@ -1360,7 +1360,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>178977.90999999963</v>
+            <v>183106.15999999963</v>
           </cell>
           <cell r="H23" t="str">
             <v>VENDEDOR INTERNO 1</v>
@@ -1380,13 +1380,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>240078.95500000002</v>
+            <v>242623.905</v>
           </cell>
           <cell r="H24" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I24">
-            <v>133416.57500000007</v>
+            <v>143886.49500000008</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
@@ -1420,7 +1420,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>542</v>
+            <v>545</v>
           </cell>
         </row>
         <row r="27">
@@ -1444,7 +1444,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>199577.14999999976</v>
+            <v>200692.24999999977</v>
           </cell>
         </row>
         <row r="30">
@@ -1479,7 +1479,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4081173.4949999694</v>
+            <v>4112889.61499997</v>
           </cell>
         </row>
         <row r="34">
@@ -1718,7 +1718,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="6"/>
+      <sheetData sheetId="6" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4080561.5949999979</v>
+        <v>4112277.7149999985</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>133416.57500000001</v>
+        <v>143886.495</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1100938.4050000021</v>
+        <v>1069222.2850000015</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>166803.42499999999</v>
+        <v>156333.505</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.78752515584290217</v>
+        <v>0.79364618643249996</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.44439602624741859</v>
+        <v>0.47927018519752179</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.67749999999999999</v>
+        <v>0.68125000000000002</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2664,11 +2664,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9101.1449999999986</v>
+        <v>11646.094999999996</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>17898.855000000003</v>
+        <v>15353.905000000004</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2738,11 +2738,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10989.6</v>
+        <v>15117.849999999995</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>13510.4</v>
+        <v>9382.1500000000051</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1985.05</v>
+        <v>1985.0500000000002</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
@@ -2892,11 +2892,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9345.1200000000008</v>
+        <v>10460.219999999999</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>11654.88</v>
+        <v>10539.78</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2950,11 +2950,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>178083.97999999984</v>
+        <v>179403.89999999985</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>36916.020000000164</v>
+        <v>35596.100000000151</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -3161,11 +3161,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3513.6600000000008</v>
+        <v>4875.3600000000006</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>3146.3399999999992</v>
+        <v>1784.6399999999994</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3302,11 +3302,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3322,11 +3322,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63353.700000000041</v>
+        <v>66182.300000000047</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>51646.299999999959</v>
+        <v>48817.699999999953</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3394,11 +3394,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>365838.24999999988</v>
+        <v>384255.84999999992</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>134161.75000000012</v>
+        <v>115744.15000000008</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3413,11 +3413,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10994.599999999999</v>
+        <v>12314.519999999999</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>11005.400000000001</v>
+        <v>9685.4800000000014</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="O20" s="2" cm="1">
         <f t="array" ref="O20">IFERROR(_xlfn.XLOOKUP(N20,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>505000</v>
+        <v>0</v>
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-15661.219999999856</v>
+        <v>-520661.21999999986</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3501,7 +3501,7 @@
       </c>
       <c r="O21" s="2" cm="1">
         <f t="array" ref="O21">IFERROR(_xlfn.XLOOKUP(N21,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>627000</v>
+        <v>0</v>
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-157238.58000000031</v>
+        <v>-784238.58000000031</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="O22" s="2" cm="1">
         <f t="array" ref="O22">IFERROR(_xlfn.XLOOKUP(N22,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>586500</v>
+        <v>0</v>
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>109246.73000000062</v>
+        <v>-477253.26999999938</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3651,15 +3651,15 @@
       </c>
       <c r="O23" s="2" cm="1">
         <f t="array" ref="O23">IFERROR(_xlfn.XLOOKUP(N23,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>717500</v>
+        <v>0</v>
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>62649.559999999983</v>
+        <v>83895.76</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>654850.44000000006</v>
+        <v>-83895.76</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3822,11 +3822,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>59118.370000000134</v>
+        <v>60480.070000000131</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>30881.629999999866</v>
+        <v>29519.929999999869</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3886,11 +3886,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>178977.90999999963</v>
+        <v>183106.15999999963</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>56022.090000000375</v>
+        <v>51893.840000000375</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>240078.95500000002</v>
+        <v>242623.905</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>61921.044999999984</v>
+        <v>59376.095000000001</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -4224,11 +4224,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>199577.14999999976</v>
+        <v>200692.24999999977</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>55422.850000000239</v>
+        <v>54307.750000000233</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4241,11 +4241,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>685356.8950000013</v>
+        <v>685356.89500000118</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>14643.104999998701</v>
+        <v>14643.104999998817</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4264,11 +4264,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4301,11 +4301,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>133416.57499999995</v>
+        <v>143886.49499999997</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>566583.42500000005</v>
+        <v>556113.505</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4536,11 +4536,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1175113.6449999923</v>
+        <v>1175113.6449999928</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>104886.35500000766</v>
+        <v>104886.3550000072</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4572,11 +4572,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>196066.13499999992</v>
+        <v>227782.25499999983</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>1083933.865</v>
+        <v>1052217.7450000001</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 25/05/2026 14:42
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35E1AF2-B5CE-4FDC-BCE7-1F541DF27D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB070F8-B543-4619-A61E-C2ED30E1DF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1009,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>42064.409999999996</v>
+            <v>44964.009999999995</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>2448.9000000000005</v>
+            <v>5348.5</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>239411.41999999952</v>
+            <v>249898.81999999957</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>11506.749999999998</v>
+            <v>21994.150000000009</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1046,7 +1046,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>6873.1099999999988</v>
+            <v>7505.1499999999987</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1066,13 +1066,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>12314.519999999999</v>
+            <v>17077.169999999998</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="N8">
-            <v>17</v>
+            <v>18</v>
           </cell>
         </row>
         <row r="9">
@@ -1080,7 +1080,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>74187.039999999979</v>
+            <v>74819.079999999987</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
@@ -1100,13 +1100,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>179403.89999999985</v>
+            <v>184166.54999999987</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>7809.8</v>
+            <v>13378.199999999999</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1126,7 +1126,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>11772.469999999996</v>
+            <v>14749.869999999997</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1146,7 +1146,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>7059.3</v>
+            <v>13846.7</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1160,19 +1160,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>146927.28999999995</v>
+            <v>160151.88999999984</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>4938.43</v>
+            <v>10806.53</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>17</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="14">
@@ -1186,7 +1186,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>4875.3600000000006</v>
+            <v>5293.26</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1206,13 +1206,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>15117.849999999995</v>
+            <v>15912.569999999994</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N15">
-            <v>12</v>
+            <v>13</v>
           </cell>
         </row>
         <row r="16">
@@ -1220,19 +1220,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>384255.84999999992</v>
+            <v>398182.64999999979</v>
           </cell>
           <cell r="H16" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>11646.094999999996</v>
+            <v>20107.494999999995</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>43</v>
+            <v>44</v>
           </cell>
         </row>
         <row r="17">
@@ -1240,13 +1240,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>276494.14999999997</v>
+            <v>280191.74999999994</v>
           </cell>
           <cell r="H17" t="str">
             <v>PERDIZES</v>
           </cell>
           <cell r="I17">
-            <v>4673.7</v>
+            <v>6312.7</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1260,19 +1260,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>81482.879999999961</v>
+            <v>87051.27999999997</v>
           </cell>
           <cell r="H18" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I18">
-            <v>1985.0500000000002</v>
+            <v>4896.75</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>35</v>
+            <v>36</v>
           </cell>
         </row>
         <row r="19">
@@ -1280,19 +1280,19 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>118089.05999999971</v>
+            <v>121066.45999999966</v>
           </cell>
           <cell r="H19" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I19">
-            <v>9527.3700000000008</v>
+            <v>12777.419999999998</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>67</v>
+            <v>69</v>
           </cell>
         </row>
         <row r="20">
@@ -1300,13 +1300,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>87592.119999999966</v>
+            <v>94379.51999999996</v>
           </cell>
           <cell r="H20" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I20">
-            <v>10460.219999999999</v>
+            <v>13866.62</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1320,19 +1320,19 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>105814.09999999941</v>
+            <v>111682.1999999994</v>
           </cell>
           <cell r="H21" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I21">
-            <v>8404.1</v>
+            <v>9381.0000000000018</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N21">
-            <v>32</v>
+            <v>33</v>
           </cell>
         </row>
         <row r="22">
@@ -1340,19 +1340,19 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>60480.070000000131</v>
+            <v>60897.970000000132</v>
           </cell>
           <cell r="H22" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I22">
-            <v>2077.7199999999998</v>
+            <v>3032.5100000000007</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N22">
-            <v>26</v>
+            <v>28</v>
           </cell>
         </row>
         <row r="23">
@@ -1360,7 +1360,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>183106.15999999963</v>
+            <v>183900.8799999996</v>
           </cell>
           <cell r="H23" t="str">
             <v>VENDEDOR INTERNO 1</v>
@@ -1380,13 +1380,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>242623.905</v>
+            <v>251085.30499999996</v>
           </cell>
           <cell r="H24" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I24">
-            <v>143886.49500000008</v>
+            <v>206682.34499999997</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
@@ -1400,7 +1400,7 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>75526.710000000036</v>
+            <v>77165.710000000021</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
@@ -1414,13 +1414,13 @@
             <v>PIRACICABA</v>
           </cell>
           <cell r="F26">
-            <v>101738.06000000006</v>
+            <v>102906.86000000004</v>
           </cell>
           <cell r="K26" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>545</v>
+            <v>556</v>
           </cell>
         </row>
         <row r="27">
@@ -1428,7 +1428,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>103040.56999999993</v>
+            <v>105952.2699999999</v>
           </cell>
         </row>
         <row r="28">
@@ -1436,7 +1436,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>128273.93999999996</v>
+            <v>131523.98999999996</v>
           </cell>
         </row>
         <row r="29">
@@ -1444,7 +1444,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>200692.24999999977</v>
+            <v>204098.64999999973</v>
           </cell>
         </row>
         <row r="30">
@@ -1452,7 +1452,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>61478.240000000063</v>
+            <v>62455.140000000007</v>
           </cell>
         </row>
         <row r="31">
@@ -1460,7 +1460,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>35939.69000000001</v>
+            <v>36894.480000000018</v>
           </cell>
         </row>
         <row r="32">
@@ -1479,7 +1479,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4112889.61499997</v>
+            <v>4207703.2649999652</v>
           </cell>
         </row>
         <row r="34">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4112277.7149999985</v>
+        <v>4207091.3649999965</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>143886.495</v>
+        <v>206682.345</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1069222.2850000015</v>
+        <v>974408.6350000035</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>156333.505</v>
+        <v>93537.654999999999</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.79364618643249996</v>
+        <v>0.81194468107690754</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.47927018519752179</v>
+        <v>0.6884362967157418</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.68125000000000002</v>
+        <v>0.69499999999999995</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2645,11 +2645,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>42064.409999999996</v>
+        <v>44964.009999999995</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>22435.590000000004</v>
+        <v>19535.990000000005</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2664,11 +2664,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11646.094999999996</v>
+        <v>20107.494999999995</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>15353.905000000004</v>
+        <v>6892.5050000000047</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2699,11 +2699,11 @@
       </c>
       <c r="V10" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W10" s="4">
         <f>U10-V10</f>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -2719,11 +2719,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>239411.41999999952</v>
+        <v>249898.81999999957</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>75588.580000000482</v>
+        <v>65101.18000000043</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2738,11 +2738,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>15117.849999999995</v>
+        <v>15912.569999999994</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>9382.1500000000051</v>
+        <v>8587.4300000000057</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2815,11 +2815,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1985.0500000000002</v>
+        <v>4896.75</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>12104.95</v>
+        <v>9193.25</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>74187.039999999979</v>
+        <v>74819.079999999987</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>5812.960000000021</v>
+        <v>5180.9200000000128</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2892,11 +2892,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10460.219999999999</v>
+        <v>13866.62</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>10539.78</v>
+        <v>7133.3799999999992</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2950,11 +2950,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>179403.89999999985</v>
+        <v>184166.54999999987</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>35596.100000000151</v>
+        <v>30833.450000000128</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2969,11 +2969,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4938.43</v>
+        <v>10806.53</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>12561.57</v>
+        <v>6693.4699999999993</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3046,11 +3046,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11506.749999999998</v>
+        <v>21994.150000000009</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>19403.25</v>
+        <v>8915.8499999999913</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3084,11 +3084,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3123,11 +3123,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9527.3700000000008</v>
+        <v>12777.419999999998</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>9122.6299999999992</v>
+        <v>5872.5800000000017</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3181,11 +3181,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>146927.28999999995</v>
+        <v>160151.88999999984</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-21927.28999999995</v>
+        <v>-35151.889999999839</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4875.3600000000006</v>
+        <v>5293.26</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>1784.6399999999994</v>
+        <v>1366.7399999999998</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3277,11 +3277,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7809.8</v>
+        <v>13378.199999999999</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>4690.2</v>
+        <v>-878.19999999999891</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3302,11 +3302,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3341,11 +3341,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11772.469999999996</v>
+        <v>14749.869999999997</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>5227.5300000000043</v>
+        <v>2250.1300000000028</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3374,11 +3374,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3394,11 +3394,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>384255.84999999992</v>
+        <v>398182.64999999979</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>115744.15000000008</v>
+        <v>101817.35000000021</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3413,11 +3413,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>12314.519999999999</v>
+        <v>17077.169999999998</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>9685.4800000000014</v>
+        <v>4922.8300000000017</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3449,11 +3449,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3469,11 +3469,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>276494.14999999997</v>
+        <v>280191.74999999994</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>151005.85000000003</v>
+        <v>147308.25000000006</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3488,11 +3488,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4673.7</v>
+        <v>6312.7</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>8596.2999999999993</v>
+        <v>6957.3</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3505,11 +3505,11 @@
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>784238.58000000031</v>
+        <v>784238.58000000019</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-784238.58000000031</v>
+        <v>-784238.58000000019</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3544,11 +3544,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>81482.879999999961</v>
+        <v>87051.27999999997</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>38017.120000000039</v>
+        <v>32448.72000000003</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3599,11 +3599,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3619,11 +3619,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>118089.05999999971</v>
+        <v>121066.45999999966</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>38910.940000000293</v>
+        <v>35933.540000000343</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3638,11 +3638,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7059.3</v>
+        <v>13846.7</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>9210.7000000000007</v>
+        <v>2423.2999999999993</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3655,11 +3655,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>83895.76</v>
+        <v>114744.76000000005</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-83895.76</v>
+        <v>-114744.76000000005</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3674,11 +3674,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3694,11 +3694,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>87592.119999999966</v>
+        <v>94379.51999999996</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>32407.880000000034</v>
+        <v>25620.48000000004</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3713,11 +3713,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6873.1099999999988</v>
+        <v>7505.1499999999987</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>2606.8900000000012</v>
+        <v>1974.8500000000013</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3758,11 +3758,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>105814.09999999941</v>
+        <v>111682.1999999994</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>29185.900000000591</v>
+        <v>23317.8000000006</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3822,11 +3822,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>60480.070000000131</v>
+        <v>60897.970000000132</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>29519.929999999869</v>
+        <v>29102.029999999868</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3841,11 +3841,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8404.1</v>
+        <v>9381.0000000000018</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>5785.9</v>
+        <v>4808.9999999999982</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3866,11 +3866,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-4</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3886,11 +3886,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>183106.15999999963</v>
+        <v>183900.8799999996</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>51893.840000000375</v>
+        <v>51099.120000000403</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2077.7199999999998</v>
+        <v>3032.5100000000007</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>4502.2800000000007</v>
+        <v>3547.4899999999993</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3950,11 +3950,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>242623.905</v>
+        <v>251085.30499999996</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>59376.095000000001</v>
+        <v>50914.695000000036</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3969,11 +3969,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2448.9000000000005</v>
+        <v>5348.5</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>5671.0999999999995</v>
+        <v>2771.5</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -4001,11 +4001,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>75526.710000000036</v>
+        <v>77165.710000000021</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>37473.289999999964</v>
+        <v>35834.289999999979</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4047,11 +4047,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>101738.06000000006</v>
+        <v>102906.86000000004</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>68261.939999999944</v>
+        <v>67093.139999999956</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4104,11 +4104,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>103040.56999999993</v>
+        <v>105952.2699999999</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>22959.430000000066</v>
+        <v>20047.730000000098</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4121,11 +4121,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>645369.17500000272</v>
+        <v>645369.17500000284</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>54630.824999997276</v>
+        <v>54630.824999997159</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4164,11 +4164,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>128273.93999999996</v>
+        <v>131523.98999999996</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>38726.060000000041</v>
+        <v>35476.010000000038</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4181,11 +4181,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000051</v>
+        <v>668938.42000000062</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.579999999492</v>
+        <v>31061.579999999376</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4224,11 +4224,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>200692.24999999977</v>
+        <v>204098.64999999973</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>54307.750000000233</v>
+        <v>50901.350000000268</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4241,11 +4241,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>685356.89500000118</v>
+        <v>685356.8950000013</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>14643.104999998817</v>
+        <v>14643.104999998701</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4264,11 +4264,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>156</v>
+        <v>132</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4284,11 +4284,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>61478.240000000063</v>
+        <v>62455.140000000007</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>38521.759999999937</v>
+        <v>37544.859999999993</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4301,11 +4301,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>143886.49499999997</v>
+        <v>206682.34499999986</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>556113.505</v>
+        <v>493317.65500000014</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4333,11 +4333,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>35939.69000000001</v>
+        <v>36894.480000000018</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>19060.30999999999</v>
+        <v>18105.519999999982</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4464,11 +4464,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.595</v>
+        <v>1184379.5950000002</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.405000000028</v>
+        <v>95620.404999999795</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4500,11 +4500,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1525614.1199999915</v>
+        <v>1525614.1199999917</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="6">C40-D40</f>
-        <v>-245614.1199999915</v>
+        <v>-245614.11999999173</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4536,11 +4536,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1175113.6449999928</v>
+        <v>1175113.644999993</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>104886.3550000072</v>
+        <v>104886.35500000697</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4572,11 +4572,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>227782.25499999983</v>
+        <v>322595.90500000055</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>1052217.7450000001</v>
+        <v>957404.09499999951</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 26/05/2026 08:13
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB070F8-B543-4619-A61E-C2ED30E1DF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A9FDA41-45DB-4F73-9262-2EAE1DC9780F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1009,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>44964.009999999995</v>
+            <v>47137.11</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>5348.5</v>
+            <v>4457.5999999999995</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>249898.81999999957</v>
+            <v>250850.96999999951</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>21994.150000000009</v>
+            <v>22946.30000000001</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1066,7 +1066,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>17077.169999999998</v>
+            <v>17556.87</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1080,7 +1080,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>74819.079999999987</v>
+            <v>74956.089999999982</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
@@ -1092,7 +1092,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>53</v>
+            <v>54</v>
           </cell>
         </row>
         <row r="10">
@@ -1100,7 +1100,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>184166.54999999987</v>
+            <v>184646.24999999991</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE</v>
@@ -1160,7 +1160,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>160151.88999999984</v>
+            <v>160151.88999999972</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE TATUAPE</v>
@@ -1180,13 +1180,13 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>745690.09999999986</v>
+            <v>754319.69999999972</v>
           </cell>
           <cell r="H14" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>5293.26</v>
+            <v>6942.11</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1220,13 +1220,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>398182.64999999979</v>
+            <v>400118.64999999979</v>
           </cell>
           <cell r="H16" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>20107.494999999995</v>
+            <v>20156.294999999998</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1260,13 +1260,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>87051.27999999997</v>
+            <v>87372.479999999967</v>
           </cell>
           <cell r="H18" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I18">
-            <v>4896.75</v>
+            <v>7342.3999999999987</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1280,7 +1280,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>121066.45999999966</v>
+            <v>125450.00999999966</v>
           </cell>
           <cell r="H19" t="str">
             <v>SANTO ANDRE</v>
@@ -1300,13 +1300,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>94379.51999999996</v>
+            <v>97424.719999999972</v>
           </cell>
           <cell r="H20" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I20">
-            <v>13866.62</v>
+            <v>19246.820000000007</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1340,7 +1340,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>60897.970000000132</v>
+            <v>62666.720000000139</v>
           </cell>
           <cell r="H22" t="str">
             <v>SJC/VALE</v>
@@ -1372,7 +1372,7 @@
             <v>SBC</v>
           </cell>
           <cell r="N23">
-            <v>38</v>
+            <v>39</v>
           </cell>
         </row>
         <row r="24">
@@ -1380,13 +1380,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>251085.30499999996</v>
+            <v>251134.10500000001</v>
           </cell>
           <cell r="H24" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I24">
-            <v>206682.34499999997</v>
+            <v>216746.79499999998</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
@@ -1400,7 +1400,7 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>77165.710000000021</v>
+            <v>79723.510000000024</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
@@ -1420,7 +1420,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>556</v>
+            <v>558</v>
           </cell>
         </row>
         <row r="27">
@@ -1428,7 +1428,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>105952.2699999999</v>
+            <v>108397.91999999988</v>
           </cell>
         </row>
         <row r="28">
@@ -1436,7 +1436,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>131523.98999999996</v>
+            <v>131523.99000000002</v>
           </cell>
         </row>
         <row r="29">
@@ -1444,7 +1444,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>204098.64999999973</v>
+            <v>209478.84999999977</v>
           </cell>
         </row>
         <row r="30">
@@ -1452,7 +1452,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>62455.140000000007</v>
+            <v>62455.140000000043</v>
           </cell>
         </row>
         <row r="31">
@@ -1468,7 +1468,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F32">
-            <v>59673.74</v>
+            <v>61714.85</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1479,7 +1479,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4207703.2649999652</v>
+            <v>4244003.0849999646</v>
           </cell>
         </row>
         <row r="34">
@@ -1495,7 +1495,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>37752.599999999962</v>
+            <v>37752.599999999984</v>
           </cell>
         </row>
         <row r="36">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I28)</f>
-        <v>300220</v>
+        <v>200030</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4207091.3649999965</v>
+        <v>4243391.1849999977</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>206682.345</v>
+        <v>216746.79500000004</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>974408.6350000035</v>
+        <v>938108.81500000227</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>93537.654999999999</v>
+        <v>-16716.795000000042</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.81194468107690754</v>
+        <v>0.81895033966997932</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.6884362967157418</v>
+        <v>1.0835714392841076</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.69499999999999995</v>
+        <v>0.69750000000000001</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2645,11 +2645,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>44964.009999999995</v>
+        <v>47137.11</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>19535.990000000005</v>
+        <v>17362.89</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2660,15 +2660,15 @@
       </c>
       <c r="I10" s="2">
         <f>_xlfn.XLOOKUP(G10,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>27000</v>
+        <v>21000</v>
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>20107.494999999995</v>
+        <v>20156.294999999998</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>6892.5050000000047</v>
+        <v>843.70500000000175</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2719,11 +2719,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>249898.81999999957</v>
+        <v>250850.96999999951</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>65101.18000000043</v>
+        <v>64149.030000000494</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="I11" s="2">
         <f>_xlfn.XLOOKUP(G11,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>24500</v>
+        <v>14000</v>
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>8587.4300000000057</v>
+        <v>-1912.5699999999943</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2776,11 +2776,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W27" si="3">U11-V11</f>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2811,15 +2811,15 @@
       </c>
       <c r="I12" s="2">
         <f>_xlfn.XLOOKUP(G12,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14090</v>
+        <v>14220</v>
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4896.75</v>
+        <v>7342.3999999999987</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>9193.25</v>
+        <v>6877.6000000000013</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>74819.079999999987</v>
+        <v>74956.089999999982</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>5180.9200000000128</v>
+        <v>5043.910000000018</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2888,15 +2888,15 @@
       </c>
       <c r="I13" s="2">
         <f>_xlfn.XLOOKUP(G13,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>21000</v>
+        <v>19000</v>
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>13866.62</v>
+        <v>19246.820000000007</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>7133.3799999999992</v>
+        <v>-246.82000000000698</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2950,11 +2950,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>184166.54999999987</v>
+        <v>184646.24999999991</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>30833.450000000128</v>
+        <v>30353.750000000087</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="I14" s="2">
         <f>_xlfn.XLOOKUP(G14,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>17500</v>
+        <v>8250</v>
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>6693.4699999999993</v>
+        <v>-2556.5300000000007</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3042,15 +3042,15 @@
       </c>
       <c r="I15" s="2">
         <f>_xlfn.XLOOKUP(G15,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>30910</v>
+        <v>25330</v>
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>21994.150000000009</v>
+        <v>22946.30000000001</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>8915.8499999999913</v>
+        <v>2383.6999999999898</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="I16" s="2">
         <f>_xlfn.XLOOKUP(G16,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>18650</v>
+        <v>9950</v>
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>5872.5800000000017</v>
+        <v>-2827.4199999999983</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3181,11 +3181,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>160151.88999999984</v>
+        <v>160151.88999999972</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-35151.889999999839</v>
+        <v>-35151.889999999723</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3196,15 +3196,15 @@
       </c>
       <c r="I17" s="2">
         <f>_xlfn.XLOOKUP(G17,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6660</v>
+        <v>3190</v>
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5293.26</v>
+        <v>6942.11</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>1366.7399999999998</v>
+        <v>-3752.1099999999997</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3219,11 +3219,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>37752.599999999962</v>
+        <v>37752.599999999984</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-37752.599999999962</v>
+        <v>-37752.599999999984</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>745690.09999999986</v>
+        <v>754319.69999999972</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>54309.90000000014</v>
+        <v>45680.300000000279</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="I18" s="2">
         <f>_xlfn.XLOOKUP(G18,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12500</v>
+        <v>5710</v>
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>-878.19999999999891</v>
+        <v>-7668.1999999999989</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="I19" s="2">
         <f>_xlfn.XLOOKUP(G19,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>17000</v>
+        <v>14000</v>
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>2250.1300000000028</v>
+        <v>-749.86999999999716</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3394,11 +3394,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>398182.64999999979</v>
+        <v>400118.64999999979</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>101817.35000000021</v>
+        <v>99881.35000000021</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3409,15 +3409,15 @@
       </c>
       <c r="I20" s="2">
         <f>_xlfn.XLOOKUP(G20,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>22000</v>
+        <v>15010</v>
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>17077.169999999998</v>
+        <v>17556.87</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>4922.8300000000017</v>
+        <v>-2546.869999999999</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="I21" s="2">
         <f>_xlfn.XLOOKUP(G21,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13270</v>
+        <v>9910</v>
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>6957.3</v>
+        <v>3597.3</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3544,11 +3544,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>87051.27999999997</v>
+        <v>87372.479999999967</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>32448.72000000003</v>
+        <v>32127.520000000033</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="I22" s="2">
         <f>_xlfn.XLOOKUP(G22,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>9500</v>
+        <v>2670</v>
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3567,7 +3567,7 @@
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>5422.22</v>
+        <v>-1407.7799999999997</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3619,11 +3619,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>121066.45999999966</v>
+        <v>125450.00999999966</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>35933.540000000343</v>
+        <v>31549.99000000034</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="I23" s="2">
         <f>_xlfn.XLOOKUP(G23,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>16270</v>
+        <v>12900</v>
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>2423.2999999999993</v>
+        <v>-946.70000000000073</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3655,11 +3655,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>114744.76000000005</v>
+        <v>125310.36000000007</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-114744.76000000005</v>
+        <v>-125310.36000000007</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3694,11 +3694,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>94379.51999999996</v>
+        <v>97424.719999999972</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>25620.48000000004</v>
+        <v>22575.280000000028</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="I24" s="2">
         <f>_xlfn.XLOOKUP(G24,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>9480</v>
+        <v>5460</v>
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>1974.8500000000013</v>
+        <v>-2045.1499999999987</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3738,11 +3738,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="I25" s="2">
         <f>_xlfn.XLOOKUP(G25,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11000</v>
+        <v>4810</v>
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>4682.0300000000007</v>
+        <v>-1507.9699999999993</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3822,11 +3822,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>60897.970000000132</v>
+        <v>62666.720000000139</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>29102.029999999868</v>
+        <v>27333.279999999861</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3837,7 +3837,7 @@
       </c>
       <c r="I26" s="2">
         <f>_xlfn.XLOOKUP(G26,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14190</v>
+        <v>6810</v>
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>4808.9999999999982</v>
+        <v>-2571.0000000000018</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="I27" s="2">
         <f>_xlfn.XLOOKUP(G27,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6580</v>
+        <v>3090</v>
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
@@ -3909,7 +3909,7 @@
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>3547.4899999999993</v>
+        <v>57.489999999999327</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3950,11 +3950,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>251085.30499999996</v>
+        <v>251134.10500000001</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>50914.695000000036</v>
+        <v>50865.89499999999</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3965,15 +3965,15 @@
       </c>
       <c r="I28" s="2">
         <f>_xlfn.XLOOKUP(G28,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>8120</v>
+        <v>4720</v>
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5348.5</v>
+        <v>4457.5999999999995</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>2771.5</v>
+        <v>262.40000000000055</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -4001,11 +4001,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>77165.710000000021</v>
+        <v>79723.510000000024</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>35834.289999999979</v>
+        <v>33276.489999999976</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4104,11 +4104,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>105952.2699999999</v>
+        <v>108397.91999999988</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>20047.730000000098</v>
+        <v>17602.080000000118</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4121,11 +4121,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>645369.17500000284</v>
+        <v>645369.17500000272</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>54630.824999997159</v>
+        <v>54630.824999997276</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4164,11 +4164,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>131523.98999999996</v>
+        <v>131523.99000000002</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>35476.010000000038</v>
+        <v>35476.00999999998</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4181,11 +4181,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000062</v>
+        <v>668938.42000000051</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.579999999376</v>
+        <v>31061.579999999492</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4224,11 +4224,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>204098.64999999973</v>
+        <v>209478.84999999977</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>50901.350000000268</v>
+        <v>45521.150000000227</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4241,11 +4241,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>685356.8950000013</v>
+        <v>685356.89500000118</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>14643.104999998701</v>
+        <v>14643.104999998817</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4264,11 +4264,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4284,11 +4284,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>62455.140000000007</v>
+        <v>62455.140000000043</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>37544.859999999993</v>
+        <v>37544.859999999957</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4301,11 +4301,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>206682.34499999986</v>
+        <v>232416.56499999994</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>493317.65500000014</v>
+        <v>467583.43500000006</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4371,11 +4371,11 @@
       </c>
       <c r="D36" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A36,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>59673.74</v>
+        <v>61714.85</v>
       </c>
       <c r="E36" s="7">
         <f t="shared" si="0"/>
-        <v>6326.260000000002</v>
+        <v>4285.1500000000015</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -4464,11 +4464,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.5950000002</v>
+        <v>1184379.5949999997</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.404999999795</v>
+        <v>95620.405000000261</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4500,11 +4500,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1525614.1199999917</v>
+        <v>1525614.1199999915</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="6">C40-D40</f>
-        <v>-245614.11999999173</v>
+        <v>-245614.1199999915</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4536,11 +4536,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1175113.644999993</v>
+        <v>1175113.6449999928</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>104886.35500000697</v>
+        <v>104886.3550000072</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4572,11 +4572,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>322595.90500000055</v>
+        <v>358895.72500000068</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>957404.09499999951</v>
+        <v>921104.27499999932</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 26/05/2026 08:29
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A9FDA41-45DB-4F73-9262-2EAE1DC9780F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C92502-AF1C-49A9-B02F-0F3867107531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-25T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-26T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -973,7 +973,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>25/05/2026</v>
+            <v>26/05/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1015,7 +1015,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>4457.5999999999995</v>
+            <v>3064</v>
           </cell>
         </row>
         <row r="6">
@@ -1026,10 +1026,10 @@
             <v>250850.96999999951</v>
           </cell>
           <cell r="H6" t="str">
-            <v>CENTRO</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I6">
-            <v>22946.30000000001</v>
+            <v>137.01</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1043,10 +1043,10 @@
             <v>939.83999999999992</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I7">
-            <v>7505.1499999999987</v>
+            <v>321.2</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1063,10 +1063,10 @@
             <v>611.9</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I8">
-            <v>17556.87</v>
+            <v>4383.5499999999993</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1083,10 +1083,10 @@
             <v>74956.089999999982</v>
           </cell>
           <cell r="H9" t="str">
-            <v>JUNDIAI</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I9">
-            <v>4077.7799999999997</v>
+            <v>3045.2000000000003</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
@@ -1103,10 +1103,10 @@
             <v>184646.24999999991</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I10">
-            <v>13378.199999999999</v>
+            <v>119.9</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1123,10 +1123,10 @@
             <v>64670.779999999977</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE MOOCA</v>
+            <v>PERDIZES</v>
           </cell>
           <cell r="I11">
-            <v>14749.869999999997</v>
+            <v>2557.8000000000002</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1143,10 +1143,10 @@
             <v>246499.13999999998</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE PENHA</v>
+            <v>SJC</v>
           </cell>
           <cell r="I12">
-            <v>13846.7</v>
+            <v>0</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1163,10 +1163,10 @@
             <v>160151.88999999972</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I13">
-            <v>10806.53</v>
+            <v>2041.11</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1183,10 +1183,10 @@
             <v>754319.69999999972</v>
           </cell>
           <cell r="H14" t="str">
-            <v>MOGI</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I14">
-            <v>6942.11</v>
+            <v>15669.77</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1202,12 +1202,6 @@
           <cell r="F15">
             <v>66182.300000000047</v>
           </cell>
-          <cell r="H15" t="str">
-            <v>NORTE</v>
-          </cell>
-          <cell r="I15">
-            <v>15912.569999999994</v>
-          </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
@@ -1222,12 +1216,6 @@
           <cell r="F16">
             <v>400118.64999999979</v>
           </cell>
-          <cell r="H16" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="I16">
-            <v>20156.294999999998</v>
-          </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
@@ -1242,12 +1230,6 @@
           <cell r="F17">
             <v>280191.74999999994</v>
           </cell>
-          <cell r="H17" t="str">
-            <v>PERDIZES</v>
-          </cell>
-          <cell r="I17">
-            <v>6312.7</v>
-          </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
@@ -1262,12 +1244,6 @@
           <cell r="F18">
             <v>87372.479999999967</v>
           </cell>
-          <cell r="H18" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I18">
-            <v>7342.3999999999987</v>
-          </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
@@ -1282,12 +1258,6 @@
           <cell r="F19">
             <v>125450.00999999966</v>
           </cell>
-          <cell r="H19" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I19">
-            <v>12777.419999999998</v>
-          </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
@@ -1302,12 +1272,6 @@
           <cell r="F20">
             <v>97424.719999999972</v>
           </cell>
-          <cell r="H20" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I20">
-            <v>19246.820000000007</v>
-          </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
           </cell>
@@ -1322,12 +1286,6 @@
           <cell r="F21">
             <v>111682.1999999994</v>
           </cell>
-          <cell r="H21" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I21">
-            <v>9381.0000000000018</v>
-          </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
           </cell>
@@ -1342,12 +1300,6 @@
           <cell r="F22">
             <v>62666.720000000139</v>
           </cell>
-          <cell r="H22" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I22">
-            <v>3032.5100000000007</v>
-          </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
           </cell>
@@ -1362,12 +1314,6 @@
           <cell r="F23">
             <v>183900.8799999996</v>
           </cell>
-          <cell r="H23" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I23">
-            <v>6317.9699999999993</v>
-          </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
           </cell>
@@ -1381,12 +1327,6 @@
           </cell>
           <cell r="F24">
             <v>251134.10500000001</v>
-          </cell>
-          <cell r="H24" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I24">
-            <v>216746.79499999998</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
@@ -2434,7 +2374,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>216746.79500000004</v>
+        <v>15669.77</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2479,7 +2419,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>-16716.795000000042</v>
+        <v>184360.23</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2524,7 +2464,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>1.0835714392841076</v>
+        <v>7.8337099435084739E-2</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2664,11 +2604,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>20156.294999999998</v>
+        <v>0</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>843.70500000000175</v>
+        <v>21000</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2738,11 +2678,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>15912.569999999994</v>
+        <v>0</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>-1912.5699999999943</v>
+        <v>14000</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2815,11 +2755,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7342.3999999999987</v>
+        <v>0</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>6877.6000000000013</v>
+        <v>14220</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2892,11 +2832,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>19246.820000000007</v>
+        <v>0</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>-246.82000000000698</v>
+        <v>19000</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2969,11 +2909,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10806.53</v>
+        <v>0</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>-2556.5300000000007</v>
+        <v>8250</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3046,11 +2986,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>22946.30000000001</v>
+        <v>0</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>2383.6999999999898</v>
+        <v>25330</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3123,11 +3063,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>12777.419999999998</v>
+        <v>0</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>-2827.4199999999983</v>
+        <v>9950</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3200,11 +3140,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6942.11</v>
+        <v>119.9</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>-3752.1099999999997</v>
+        <v>3070.1</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3277,11 +3217,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>13378.199999999999</v>
+        <v>321.2</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>-7668.1999999999989</v>
+        <v>5388.8</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3341,11 +3281,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>14749.869999999997</v>
+        <v>4383.5499999999993</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>-749.86999999999716</v>
+        <v>9616.4500000000007</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3413,11 +3353,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>17556.87</v>
+        <v>0</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>-2546.869999999999</v>
+        <v>15010</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3488,11 +3428,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6312.7</v>
+        <v>2557.8000000000002</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>3597.3</v>
+        <v>7352.2</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3563,11 +3503,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4077.7799999999997</v>
+        <v>0</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>-1407.7799999999997</v>
+        <v>2670</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3638,11 +3578,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>13846.7</v>
+        <v>3045.2000000000003</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>-946.70000000000073</v>
+        <v>9854.7999999999993</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3713,11 +3653,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7505.1499999999987</v>
+        <v>137.01</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>-2045.1499999999987</v>
+        <v>5322.99</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3777,11 +3717,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6317.9699999999993</v>
+        <v>2041.11</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>-1507.9699999999993</v>
+        <v>2768.8900000000003</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3841,11 +3781,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9381.0000000000018</v>
+        <v>0</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>-2571.0000000000018</v>
+        <v>6810</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3905,11 +3845,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3032.5100000000007</v>
+        <v>0</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>57.489999999999327</v>
+        <v>3090</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3969,11 +3909,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4457.5999999999995</v>
+        <v>3064</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>262.40000000000055</v>
+        <v>1656</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 26/05/2026 10:56
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C92502-AF1C-49A9-B02F-0F3867107531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882B39AB-953C-40EC-8D3E-0D393FFA4A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1009,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>47137.11</v>
+            <v>47906.06</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>3064</v>
+            <v>3832.95</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>250850.96999999951</v>
+            <v>254606.01999999949</v>
           </cell>
           <cell r="H6" t="str">
-            <v>INDAIATUBA</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>137.01</v>
+            <v>3755.05</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1043,10 +1043,10 @@
             <v>939.83999999999992</v>
           </cell>
           <cell r="H7" t="str">
-            <v>LESTE</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>321.2</v>
+            <v>1301.71</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1063,16 +1063,16 @@
             <v>611.9</v>
           </cell>
           <cell r="H8" t="str">
-            <v>LESTE MOOCA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>4383.5499999999993</v>
+            <v>1822.5</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="N8">
-            <v>18</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="9">
@@ -1080,13 +1080,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>74956.089999999982</v>
+            <v>76120.789999999964</v>
           </cell>
           <cell r="H9" t="str">
-            <v>LESTE PENHA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>3045.2000000000003</v>
+            <v>2121.1000000000004</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
@@ -1100,19 +1100,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>184646.24999999991</v>
+            <v>186468.74999999985</v>
           </cell>
           <cell r="H10" t="str">
-            <v>MOGI</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>119.9</v>
+            <v>1067.7</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>30</v>
+            <v>34</v>
           </cell>
         </row>
         <row r="11">
@@ -1120,13 +1120,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>64670.779999999977</v>
+            <v>66791.879999999976</v>
           </cell>
           <cell r="H11" t="str">
-            <v>PERDIZES</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>2557.8000000000002</v>
+            <v>4383.5499999999993</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1143,10 +1143,10 @@
             <v>246499.13999999998</v>
           </cell>
           <cell r="H12" t="str">
-            <v>SJC</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>0</v>
+            <v>3250.82</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1160,13 +1160,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>160151.88999999972</v>
+            <v>160151.88999999984</v>
           </cell>
           <cell r="H13" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>2041.11</v>
+            <v>2152.0500000000002</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1183,10 +1183,10 @@
             <v>754319.69999999972</v>
           </cell>
           <cell r="H14" t="str">
-            <v>Total Geral</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>15669.77</v>
+            <v>314.3</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1202,6 +1202,12 @@
           <cell r="F15">
             <v>66182.300000000047</v>
           </cell>
+          <cell r="H15" t="str">
+            <v>NORTE</v>
+          </cell>
+          <cell r="I15">
+            <v>4021.75</v>
+          </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
@@ -1214,13 +1220,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>400118.64999999979</v>
+            <v>401603.64999999979</v>
+          </cell>
+          <cell r="H16" t="str">
+            <v>OSASCO</v>
+          </cell>
+          <cell r="I16">
+            <v>7180.85</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>44</v>
+            <v>45</v>
           </cell>
         </row>
         <row r="17">
@@ -1228,7 +1240,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>280191.74999999994</v>
+            <v>290386.04999999981</v>
+          </cell>
+          <cell r="H17" t="str">
+            <v>PERDIZES</v>
+          </cell>
+          <cell r="I17">
+            <v>4347.3999999999996</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1242,7 +1260,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>87372.479999999967</v>
+            <v>88118.979999999967</v>
+          </cell>
+          <cell r="H18" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="I18">
+            <v>3090.7700000000004</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1258,11 +1282,17 @@
           <cell r="F19">
             <v>125450.00999999966</v>
           </cell>
+          <cell r="H19" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="I19">
+            <v>316.10000000000002</v>
+          </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>69</v>
+            <v>70</v>
           </cell>
         </row>
         <row r="20">
@@ -1270,13 +1300,19 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>97424.719999999972</v>
+            <v>97630.339999999982</v>
+          </cell>
+          <cell r="H20" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="I20">
+            <v>10774.330000000002</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
           </cell>
           <cell r="N20">
-            <v>18</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="21">
@@ -1284,7 +1320,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>111682.1999999994</v>
+            <v>113834.24999999939</v>
+          </cell>
+          <cell r="H21" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I21">
+            <v>1083.3600000000001</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
@@ -1298,7 +1340,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>62666.720000000139</v>
+            <v>62711.220000000132</v>
+          </cell>
+          <cell r="H22" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I22">
+            <v>813.49</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
@@ -1312,13 +1360,19 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>183900.8799999996</v>
+            <v>187922.62999999954</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I23">
+            <v>2678.31</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
           </cell>
           <cell r="N23">
-            <v>39</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="24">
@@ -1326,7 +1380,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>251134.10500000001</v>
+            <v>257945.55499999953</v>
+          </cell>
+          <cell r="H24" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I24">
+            <v>58308.090000000011</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
@@ -1340,13 +1400,13 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>79723.510000000024</v>
+            <v>81513.11000000003</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="N25">
-            <v>16</v>
+            <v>18</v>
           </cell>
         </row>
         <row r="26">
@@ -1360,7 +1420,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>558</v>
+            <v>569</v>
           </cell>
         </row>
         <row r="27">
@@ -1368,7 +1428,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>108397.91999999988</v>
+            <v>111488.68999999987</v>
           </cell>
         </row>
         <row r="28">
@@ -1376,7 +1436,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>131523.99000000002</v>
+            <v>131840.09</v>
           </cell>
         </row>
         <row r="29">
@@ -1384,7 +1444,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>209478.84999999977</v>
+            <v>220253.17999999985</v>
           </cell>
         </row>
         <row r="30">
@@ -1392,7 +1452,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>62455.140000000043</v>
+            <v>63538.499999999993</v>
           </cell>
         </row>
         <row r="31">
@@ -1400,7 +1460,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>36894.480000000018</v>
+            <v>37707.970000000016</v>
           </cell>
         </row>
         <row r="32">
@@ -1408,7 +1468,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F32">
-            <v>61714.85</v>
+            <v>62352.049999999996</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1419,7 +1479,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4244003.0849999646</v>
+            <v>4297801.4049999509</v>
           </cell>
         </row>
         <row r="34">
@@ -1435,7 +1495,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>37752.599999999984</v>
+            <v>37752.599999999962</v>
           </cell>
         </row>
         <row r="36">
@@ -2340,7 +2400,7 @@
       </c>
       <c r="O4" s="7">
         <f>SUM(O11:O17)</f>
-        <v>627000</v>
+        <v>717500</v>
       </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
@@ -2363,7 +2423,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4243391.1849999977</v>
+        <v>4297189.5049999952</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2374,7 +2434,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>15669.77</v>
+        <v>58308.089999999989</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2396,7 +2456,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2408,7 +2468,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>938108.81500000227</v>
+        <v>884310.49500000477</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2419,7 +2479,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>184360.23</v>
+        <v>141721.91</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2430,7 +2490,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-157238.57999999996</v>
+        <v>-66738.579999999958</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -2441,7 +2501,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2453,7 +2513,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.81895033966997932</v>
+        <v>0.82933310913827951</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2464,7 +2524,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>7.8337099435084739E-2</v>
+        <v>0.29149672549117628</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2475,7 +2535,7 @@
       </c>
       <c r="O7" s="3">
         <f>O5/O4</f>
-        <v>1.2507792344497608</v>
+        <v>1.0930154425087106</v>
       </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
@@ -2486,7 +2546,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.69750000000000001</v>
+        <v>0.71125000000000005</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2551,7 +2611,7 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
@@ -2585,11 +2645,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>47137.11</v>
+        <v>47906.06</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>17362.89</v>
+        <v>16593.940000000002</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2604,11 +2664,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>7180.85</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>21000</v>
+        <v>13819.15</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2639,11 +2699,11 @@
       </c>
       <c r="V10" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W10" s="4">
         <f>U10-V10</f>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -2659,11 +2719,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>250850.96999999951</v>
+        <v>254606.01999999949</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>64149.030000000494</v>
+        <v>60393.980000000505</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2678,11 +2738,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>4021.75</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>14000</v>
+        <v>9978.25</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2755,11 +2815,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>3090.7700000000004</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>14220</v>
+        <v>11129.23</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2770,7 +2830,7 @@
       </c>
       <c r="O12" s="2" cm="1">
         <f t="array" ref="O12">IFERROR(_xlfn.XLOOKUP(M12,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>73000</v>
+        <v>54000</v>
       </c>
       <c r="P12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
@@ -2778,7 +2838,7 @@
       </c>
       <c r="Q12" s="2">
         <f t="shared" si="2"/>
-        <v>73000</v>
+        <v>54000</v>
       </c>
       <c r="R12" s="2"/>
       <c r="S12" s="4" t="s">
@@ -2793,11 +2853,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2813,11 +2873,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>74956.089999999982</v>
+        <v>76120.789999999964</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>5043.910000000018</v>
+        <v>3879.2100000000355</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2832,11 +2892,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>10774.330000000002</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>19000</v>
+        <v>8225.6699999999983</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2847,7 +2907,7 @@
       </c>
       <c r="O13" s="2" cm="1">
         <f t="array" ref="O13">IFERROR(_xlfn.XLOOKUP(M13,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>220000</v>
+        <v>233000</v>
       </c>
       <c r="P13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
@@ -2855,7 +2915,7 @@
       </c>
       <c r="Q13" s="2">
         <f t="shared" si="2"/>
-        <v>130789.79000000004</v>
+        <v>143789.79000000004</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="4" t="s">
@@ -2890,11 +2950,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>184646.24999999991</v>
+        <v>186468.74999999985</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>30353.750000000087</v>
+        <v>28531.250000000146</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2909,11 +2969,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>2152.0500000000002</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>8250</v>
+        <v>6097.95</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -2924,7 +2984,7 @@
       </c>
       <c r="O14" s="2" cm="1">
         <f t="array" ref="O14">IFERROR(_xlfn.XLOOKUP(M14,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>220000</v>
+        <v>233000</v>
       </c>
       <c r="P14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
@@ -2932,7 +2992,7 @@
       </c>
       <c r="Q14" s="2">
         <f t="shared" si="2"/>
-        <v>-143074.89999999997</v>
+        <v>-130074.89999999997</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="4" t="s">
@@ -2967,11 +3027,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>64670.779999999977</v>
+        <v>66791.879999999976</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>3329.220000000023</v>
+        <v>1208.1200000000244</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2986,11 +3046,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>3755.05</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>25330</v>
+        <v>21574.95</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3001,7 +3061,7 @@
       </c>
       <c r="O15" s="2" cm="1">
         <f t="array" ref="O15">IFERROR(_xlfn.XLOOKUP(M15,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>82500</v>
+        <v>146500</v>
       </c>
       <c r="P15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
@@ -3009,7 +3069,7 @@
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="2"/>
-        <v>-40808.699999999997</v>
+        <v>23191.300000000003</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="4" t="s">
@@ -3063,11 +3123,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>316.10000000000002</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>9950</v>
+        <v>9633.9</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3078,7 +3138,7 @@
       </c>
       <c r="O16" s="2" cm="1">
         <f t="array" ref="O16">IFERROR(_xlfn.XLOOKUP(M16,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>31500</v>
+        <v>51000</v>
       </c>
       <c r="P16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
@@ -3086,7 +3146,7 @@
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="2"/>
-        <v>-2127.7999999999884</v>
+        <v>17372.200000000012</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="4" t="s">
@@ -3121,11 +3181,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>160151.88999999972</v>
+        <v>160151.88999999984</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-35151.889999999723</v>
+        <v>-35151.889999999839</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3140,11 +3200,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>119.9</v>
+        <v>314.3</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>3070.1</v>
+        <v>2875.7</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3159,11 +3219,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>37752.599999999984</v>
+        <v>37752.599999999962</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-37752.599999999984</v>
+        <v>-37752.599999999962</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3217,11 +3277,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>321.2</v>
+        <v>1067.7</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>5388.8</v>
+        <v>4642.3</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3314,11 +3374,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3334,11 +3394,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>400118.64999999979</v>
+        <v>401603.64999999979</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>99881.35000000021</v>
+        <v>98396.35000000021</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3353,11 +3413,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>1822.5</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>15010</v>
+        <v>13187.5</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3370,11 +3430,11 @@
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>520661.21999999986</v>
+        <v>520661.21999999991</v>
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-520661.21999999986</v>
+        <v>-520661.21999999991</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3409,11 +3469,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>280191.74999999994</v>
+        <v>290386.04999999981</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>147308.25000000006</v>
+        <v>137113.95000000019</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3428,11 +3488,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2557.8000000000002</v>
+        <v>4347.3999999999996</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>7352.2</v>
+        <v>5562.6</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3445,11 +3505,11 @@
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>784238.58000000019</v>
+        <v>784238.57999999914</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-784238.58000000019</v>
+        <v>-784238.57999999914</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3464,11 +3524,11 @@
       </c>
       <c r="V21" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S21,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W21" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3484,11 +3544,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>87372.479999999967</v>
+        <v>88118.979999999967</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>32127.520000000033</v>
+        <v>31381.020000000033</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3503,11 +3563,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>2121.1000000000004</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>2670</v>
+        <v>548.89999999999964</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3578,11 +3638,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3045.2000000000003</v>
+        <v>3250.82</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>9854.7999999999993</v>
+        <v>9649.18</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3595,11 +3655,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>125310.36000000007</v>
+        <v>136989.66000000003</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-125310.36000000007</v>
+        <v>-136989.66000000003</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3634,11 +3694,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>97424.719999999972</v>
+        <v>97630.339999999982</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>22575.280000000028</v>
+        <v>22369.660000000018</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3653,11 +3713,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>137.01</v>
+        <v>1301.71</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>5322.99</v>
+        <v>4158.29</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3678,11 +3738,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3698,11 +3758,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>111682.1999999994</v>
+        <v>113834.24999999939</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>23317.8000000006</v>
+        <v>21165.750000000611</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3717,11 +3777,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2041.11</v>
+        <v>2678.31</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>2768.8900000000003</v>
+        <v>2131.69</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3762,11 +3822,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>62666.720000000139</v>
+        <v>62711.220000000132</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>27333.279999999861</v>
+        <v>27288.779999999868</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3781,11 +3841,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>1083.3600000000001</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>6810</v>
+        <v>5726.6399999999994</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3806,11 +3866,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-5</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3826,11 +3886,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>183900.8799999996</v>
+        <v>187922.62999999954</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>51099.120000000403</v>
+        <v>47077.370000000461</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3845,11 +3905,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>813.49</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>3090</v>
+        <v>2276.5100000000002</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3870,11 +3930,11 @@
       </c>
       <c r="V27" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S27,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="W27" s="4">
         <f t="shared" si="3"/>
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
@@ -3890,11 +3950,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>251134.10500000001</v>
+        <v>257945.55499999953</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>50865.89499999999</v>
+        <v>44054.445000000473</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3909,11 +3969,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3064</v>
+        <v>3832.95</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>1656</v>
+        <v>887.05000000000018</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -3941,11 +4001,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>79723.510000000024</v>
+        <v>81513.11000000003</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>33276.489999999976</v>
+        <v>31486.88999999997</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4044,11 +4104,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>108397.91999999988</v>
+        <v>111488.68999999987</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>17602.080000000118</v>
+        <v>14511.310000000129</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4104,11 +4164,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>131523.99000000002</v>
+        <v>131840.09</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>35476.00999999998</v>
+        <v>35159.910000000003</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4164,11 +4224,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>209478.84999999977</v>
+        <v>220253.17999999985</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>45521.150000000227</v>
+        <v>34746.820000000153</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4181,11 +4241,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>685356.89500000118</v>
+        <v>684987.49500000116</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>14643.104999998817</v>
+        <v>15012.504999998841</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4204,11 +4264,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>126</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4224,11 +4284,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>62455.140000000043</v>
+        <v>63538.499999999993</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>37544.859999999957</v>
+        <v>36461.500000000007</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4241,11 +4301,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>232416.56499999994</v>
+        <v>274904.98500000028</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>467583.43500000006</v>
+        <v>425095.01499999972</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4273,11 +4333,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>36894.480000000018</v>
+        <v>37707.970000000016</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>18105.519999999982</v>
+        <v>17292.029999999984</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4311,11 +4371,11 @@
       </c>
       <c r="D36" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A36,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>61714.85</v>
+        <v>62352.049999999996</v>
       </c>
       <c r="E36" s="7">
         <f t="shared" si="0"/>
-        <v>4285.1500000000015</v>
+        <v>3647.9500000000044</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -4404,11 +4464,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.5949999997</v>
+        <v>1184379.5950000004</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.405000000261</v>
+        <v>95620.404999999562</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4440,11 +4500,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1525614.1199999915</v>
+        <v>1525614.1199999913</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="6">C40-D40</f>
-        <v>-245614.1199999915</v>
+        <v>-245614.11999999126</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4476,11 +4536,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1175113.6449999928</v>
+        <v>1174744.2449999934</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>104886.3550000072</v>
+        <v>105255.75500000664</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4512,11 +4572,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>358895.72500000068</v>
+        <v>413063.44500000047</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>921104.27499999932</v>
+        <v>866936.55499999947</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 26/05/2026 12:30
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882B39AB-953C-40EC-8D3E-0D393FFA4A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2315047E-30E1-4555-9735-300FC4EBC300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="2" r:id="rId1"/>
@@ -945,11 +945,11 @@
       <sheetName val="DIN MILHO"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>254606.01999999949</v>
+            <v>255853.86999999947</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>3755.05</v>
+            <v>5002.9000000000005</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1066,7 +1066,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>1822.5</v>
+            <v>3879.900000000001</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1086,13 +1086,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>2121.1000000000004</v>
+            <v>3399.1999999999994</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>54</v>
+            <v>56</v>
           </cell>
         </row>
         <row r="10">
@@ -1100,13 +1100,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>186468.74999999985</v>
+            <v>188526.14999999985</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>1067.7</v>
+            <v>2045.9</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1120,19 +1120,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>66791.879999999976</v>
+            <v>68069.979999999981</v>
           </cell>
           <cell r="H11" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>4383.5499999999993</v>
+            <v>7483.15</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>38</v>
+            <v>39</v>
           </cell>
         </row>
         <row r="12">
@@ -1140,19 +1140,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>246499.13999999998</v>
+            <v>246499.1399999999</v>
           </cell>
           <cell r="H12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>3250.82</v>
+            <v>6050.5199999999986</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N12">
-            <v>18</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="13">
@@ -1160,13 +1160,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>160151.88999999984</v>
+            <v>160151.88999999972</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>2152.0500000000002</v>
+            <v>2781.4500000000003</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1186,7 +1186,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>314.3</v>
+            <v>1068.5999999999999</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1200,19 +1200,19 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>66182.300000000047</v>
+            <v>73448.850000000035</v>
           </cell>
           <cell r="H15" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>4021.75</v>
+            <v>5105.25</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N15">
-            <v>13</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="16">
@@ -1226,13 +1226,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>7180.85</v>
+            <v>10797.129999999996</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>45</v>
+            <v>46</v>
           </cell>
         </row>
         <row r="17">
@@ -1246,7 +1246,7 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="I17">
-            <v>4347.3999999999996</v>
+            <v>5737.8000000000011</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1260,19 +1260,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>88118.979999999967</v>
+            <v>89097.179999999949</v>
           </cell>
           <cell r="H18" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I18">
-            <v>3090.7700000000004</v>
+            <v>4076.0500000000006</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>36</v>
+            <v>41</v>
           </cell>
         </row>
         <row r="19">
@@ -1280,13 +1280,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>125450.00999999966</v>
+            <v>128549.60999999967</v>
           </cell>
           <cell r="H19" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I19">
-            <v>316.10000000000002</v>
+            <v>3119.05</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1300,13 +1300,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>97630.339999999982</v>
+            <v>100430.04000000001</v>
           </cell>
           <cell r="H20" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I20">
-            <v>10774.330000000002</v>
+            <v>13809.31</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1320,13 +1320,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>113834.24999999939</v>
+            <v>114463.64999999938</v>
           </cell>
           <cell r="H21" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I21">
-            <v>1083.3600000000001</v>
+            <v>1190.3599999999999</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
@@ -1340,19 +1340,19 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>62711.220000000132</v>
+            <v>63465.520000000128</v>
           </cell>
           <cell r="H22" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I22">
-            <v>813.49</v>
+            <v>1017.3299999999999</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N22">
-            <v>28</v>
+            <v>29</v>
           </cell>
         </row>
         <row r="23">
@@ -1360,19 +1360,19 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>187922.62999999954</v>
+            <v>189006.12999999957</v>
           </cell>
           <cell r="H23" t="str">
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I23">
-            <v>2678.31</v>
+            <v>3131.67</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
           </cell>
           <cell r="N23">
-            <v>40</v>
+            <v>41</v>
           </cell>
         </row>
         <row r="24">
@@ -1380,13 +1380,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>257945.55499999953</v>
+            <v>261561.83499999988</v>
           </cell>
           <cell r="H24" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I24">
-            <v>58308.090000000011</v>
+            <v>84830.230000000054</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
@@ -1400,13 +1400,13 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>81513.11000000003</v>
+            <v>82903.510000000024</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="N25">
-            <v>18</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="26">
@@ -1420,7 +1420,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>569</v>
+            <v>583</v>
           </cell>
         </row>
         <row r="27">
@@ -1428,7 +1428,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>111488.68999999987</v>
+            <v>112473.96999999986</v>
           </cell>
         </row>
         <row r="28">
@@ -1436,7 +1436,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>131840.09</v>
+            <v>134643.04</v>
           </cell>
         </row>
         <row r="29">
@@ -1444,7 +1444,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>220253.17999999985</v>
+            <v>223288.15999999983</v>
           </cell>
         </row>
         <row r="30">
@@ -1452,7 +1452,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>63538.499999999993</v>
+            <v>63645.500000000058</v>
           </cell>
         </row>
         <row r="31">
@@ -1460,7 +1460,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>37707.970000000016</v>
+            <v>37911.810000000019</v>
           </cell>
         </row>
         <row r="32">
@@ -1468,7 +1468,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F32">
-            <v>62352.049999999996</v>
+            <v>62805.409999999989</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1479,7 +1479,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4297801.4049999509</v>
+            <v>4331590.0949999597</v>
           </cell>
         </row>
         <row r="34">
@@ -1495,7 +1495,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>37752.599999999962</v>
+            <v>37752.599999999984</v>
           </cell>
         </row>
         <row r="36">
@@ -1718,7 +1718,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="6"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4297189.5049999952</v>
+        <v>4330978.1949999966</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>58308.089999999989</v>
+        <v>84830.23000000001</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>569</v>
+        <v>583</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>884310.49500000477</v>
+        <v>850521.80500000343</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>141721.91</v>
+        <v>115199.76999999999</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.82933310913827951</v>
+        <v>0.83585413393804819</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.29149672549117628</v>
+        <v>0.42408753686946965</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.71125000000000005</v>
+        <v>0.72875000000000001</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2664,11 +2664,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7180.85</v>
+        <v>10797.129999999996</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>13819.15</v>
+        <v>10202.870000000004</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2719,11 +2719,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>254606.01999999949</v>
+        <v>255853.86999999947</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>60393.980000000505</v>
+        <v>59146.130000000529</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2738,11 +2738,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4021.75</v>
+        <v>5105.25</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>9978.25</v>
+        <v>8894.75</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2776,11 +2776,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W27" si="3">U11-V11</f>
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2815,11 +2815,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3090.7700000000004</v>
+        <v>4076.0500000000006</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>11129.23</v>
+        <v>10143.949999999999</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2892,11 +2892,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10774.330000000002</v>
+        <v>13809.31</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>8225.6699999999983</v>
+        <v>5190.6900000000005</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2930,11 +2930,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2950,11 +2950,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>186468.74999999985</v>
+        <v>188526.14999999985</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>28531.250000000146</v>
+        <v>26473.850000000151</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2969,11 +2969,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2152.0500000000002</v>
+        <v>2781.4500000000003</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>6097.95</v>
+        <v>5468.5499999999993</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3007,11 +3007,11 @@
       </c>
       <c r="V14" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W14" s="4">
         <f>U14-V14</f>
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3027,11 +3027,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>66791.879999999976</v>
+        <v>68069.979999999981</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>1208.1200000000244</v>
+        <v>-69.979999999981374</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -3046,11 +3046,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3755.05</v>
+        <v>5002.9000000000005</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>21574.95</v>
+        <v>20327.099999999999</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3104,11 +3104,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>246499.13999999998</v>
+        <v>246499.1399999999</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>13500.860000000015</v>
+        <v>13500.860000000102</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3123,11 +3123,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>316.10000000000002</v>
+        <v>3119.05</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>9633.9</v>
+        <v>6830.95</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3181,11 +3181,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>160151.88999999984</v>
+        <v>160151.88999999972</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-35151.889999999839</v>
+        <v>-35151.889999999723</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>314.3</v>
+        <v>1068.5999999999999</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>2875.7</v>
+        <v>2121.4</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3219,11 +3219,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>37752.599999999962</v>
+        <v>37752.599999999984</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-37752.599999999962</v>
+        <v>-37752.599999999984</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3277,11 +3277,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1067.7</v>
+        <v>2045.9</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>4642.3</v>
+        <v>3664.1</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3302,11 +3302,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3322,11 +3322,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>66182.300000000047</v>
+        <v>73448.850000000035</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>48817.699999999953</v>
+        <v>41551.149999999965</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3341,11 +3341,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4383.5499999999993</v>
+        <v>7483.15</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>9616.4500000000007</v>
+        <v>6516.85</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3413,11 +3413,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1822.5</v>
+        <v>3879.900000000001</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>13187.5</v>
+        <v>11130.099999999999</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="O20" s="2" cm="1">
         <f t="array" ref="O20">IFERROR(_xlfn.XLOOKUP(N20,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>0</v>
+        <v>505000</v>
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-520661.21999999991</v>
+        <v>-15661.219999999914</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3449,11 +3449,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3488,11 +3488,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4347.3999999999996</v>
+        <v>5737.8000000000011</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>5562.6</v>
+        <v>4172.1999999999989</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3501,15 +3501,15 @@
       </c>
       <c r="O21" s="2" cm="1">
         <f t="array" ref="O21">IFERROR(_xlfn.XLOOKUP(N21,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>0</v>
+        <v>627000</v>
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>784238.57999999914</v>
+        <v>784238.58000000031</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-784238.57999999914</v>
+        <v>-157238.58000000031</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3544,11 +3544,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>88118.979999999967</v>
+        <v>89097.179999999949</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>31381.020000000033</v>
+        <v>30402.820000000051</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3563,11 +3563,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2121.1000000000004</v>
+        <v>3399.1999999999994</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>548.89999999999964</v>
+        <v>-729.19999999999936</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="O22" s="2" cm="1">
         <f t="array" ref="O22">IFERROR(_xlfn.XLOOKUP(N22,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>0</v>
+        <v>586500</v>
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-477253.26999999938</v>
+        <v>109246.73000000062</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3619,11 +3619,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>125450.00999999966</v>
+        <v>128549.60999999967</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>31549.99000000034</v>
+        <v>28450.390000000334</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3638,11 +3638,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3250.82</v>
+        <v>6050.5199999999986</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>9649.18</v>
+        <v>6849.4800000000014</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3651,15 +3651,15 @@
       </c>
       <c r="O23" s="2" cm="1">
         <f t="array" ref="O23">IFERROR(_xlfn.XLOOKUP(N23,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>0</v>
+        <v>717500</v>
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>136989.66000000003</v>
+        <v>144256.21000000002</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-136989.66000000003</v>
+        <v>573243.79</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3674,11 +3674,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3694,11 +3694,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>97630.339999999982</v>
+        <v>100430.04000000001</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>22369.660000000018</v>
+        <v>19569.959999999992</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3738,11 +3738,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>113834.24999999939</v>
+        <v>114463.64999999938</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>21165.750000000611</v>
+        <v>20536.350000000617</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3777,11 +3777,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2678.31</v>
+        <v>3131.67</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>2131.69</v>
+        <v>1678.33</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3822,11 +3822,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>62711.220000000132</v>
+        <v>63465.520000000128</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>27288.779999999868</v>
+        <v>26534.479999999872</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3841,11 +3841,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1083.3600000000001</v>
+        <v>1190.3599999999999</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>5726.6399999999994</v>
+        <v>5619.64</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3866,11 +3866,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-6</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3886,11 +3886,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>187922.62999999954</v>
+        <v>189006.12999999957</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>47077.370000000461</v>
+        <v>45993.870000000432</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>813.49</v>
+        <v>1017.3299999999999</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>2276.5100000000002</v>
+        <v>2072.67</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3930,11 +3930,11 @@
       </c>
       <c r="V27" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S27,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W27" s="4">
         <f t="shared" si="3"/>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>257945.55499999953</v>
+        <v>261561.83499999988</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>44054.445000000473</v>
+        <v>40438.165000000125</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -4001,11 +4001,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>81513.11000000003</v>
+        <v>82903.510000000024</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>31486.88999999997</v>
+        <v>30096.489999999976</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4104,11 +4104,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>111488.68999999987</v>
+        <v>112473.96999999986</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>14511.310000000129</v>
+        <v>13526.030000000144</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4164,11 +4164,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>131840.09</v>
+        <v>134643.04</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>35159.910000000003</v>
+        <v>32356.959999999992</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4181,11 +4181,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000051</v>
+        <v>668938.42000000039</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.579999999492</v>
+        <v>31061.579999999609</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4224,11 +4224,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>220253.17999999985</v>
+        <v>223288.15999999983</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>34746.820000000153</v>
+        <v>31711.840000000171</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4241,11 +4241,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>684987.49500000116</v>
+        <v>684987.49500000128</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>15012.504999998841</v>
+        <v>15012.504999998724</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4264,11 +4264,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>108</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4284,11 +4284,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63538.499999999993</v>
+        <v>63645.500000000058</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>36461.500000000007</v>
+        <v>36354.499999999942</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4301,11 +4301,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>274904.98500000028</v>
+        <v>301427.12500000064</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>425095.01499999972</v>
+        <v>398572.87499999936</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4333,11 +4333,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>37707.970000000016</v>
+        <v>37911.810000000019</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>17292.029999999984</v>
+        <v>17088.189999999981</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4371,11 +4371,11 @@
       </c>
       <c r="D36" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A36,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>62352.049999999996</v>
+        <v>62805.409999999989</v>
       </c>
       <c r="E36" s="7">
         <f t="shared" si="0"/>
-        <v>3647.9500000000044</v>
+        <v>3194.5900000000111</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -4464,11 +4464,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.5950000004</v>
+        <v>1184379.5950000007</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.404999999562</v>
+        <v>95620.404999999329</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4500,11 +4500,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1525614.1199999913</v>
+        <v>1525614.1199999915</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="6">C40-D40</f>
-        <v>-245614.11999999126</v>
+        <v>-245614.1199999915</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4536,11 +4536,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1174744.2449999934</v>
+        <v>1174744.2449999929</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>105255.75500000664</v>
+        <v>105255.75500000711</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4572,11 +4572,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>413063.44500000047</v>
+        <v>446852.13500000065</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>866936.55499999947</v>
+        <v>833147.86499999929</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 26/05/2026 12:31
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2315047E-30E1-4555-9735-300FC4EBC300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150C1C69-72B8-4478-BCE3-66FDB0EA1298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="2" r:id="rId1"/>
@@ -943,6 +943,7 @@
       <sheetName val="CONVERSOR"/>
       <sheetName val="BASE PYTHON"/>
       <sheetName val="DIN MILHO"/>
+      <sheetName val="Conversor CX vs KG"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -1719,6 +1720,7 @@
         </row>
       </sheetData>
       <sheetData sheetId="6"/>
+      <sheetData sheetId="7" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>

</xml_diff>

<commit_message>
Dados atualizados em 26/05/2026 12:56
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150C1C69-72B8-4478-BCE3-66FDB0EA1298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CFBD4AD-4C9E-4B1C-9034-7166A90C322D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -943,7 +943,6 @@
       <sheetName val="CONVERSOR"/>
       <sheetName val="BASE PYTHON"/>
       <sheetName val="DIN MILHO"/>
-      <sheetName val="Conversor CX vs KG"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -1010,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>47906.06</v>
+            <v>48005.060000000005</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>3832.95</v>
+            <v>3931.95</v>
           </cell>
         </row>
         <row r="6">
@@ -1024,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>255853.86999999947</v>
+            <v>258379.61999999947</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>5002.9000000000005</v>
+            <v>7528.6500000000024</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1041,13 +1040,13 @@
             <v>ECOMMERCE</v>
           </cell>
           <cell r="F7">
-            <v>939.83999999999992</v>
+            <v>1090.08</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
+            <v>ECOMMERCE</v>
           </cell>
           <cell r="I7">
-            <v>1301.71</v>
+            <v>150.24</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1064,10 +1063,10 @@
             <v>611.9</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I8">
-            <v>3879.900000000001</v>
+            <v>1301.71</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1084,10 +1083,10 @@
             <v>76120.789999999964</v>
           </cell>
           <cell r="H9" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I9">
-            <v>3399.1999999999994</v>
+            <v>4984.55</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
@@ -1101,13 +1100,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>188526.14999999985</v>
+            <v>189630.79999999981</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I10">
-            <v>2045.9</v>
+            <v>3404.1999999999994</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1121,13 +1120,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>68069.979999999981</v>
+            <v>68074.979999999967</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I11">
-            <v>7483.15</v>
+            <v>2045.9</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1141,13 +1140,13 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>246499.1399999999</v>
+            <v>249240.74</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I12">
-            <v>6050.5199999999986</v>
+            <v>7483.15</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1161,13 +1160,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>160151.88999999972</v>
+            <v>160151.88999999984</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I13">
-            <v>2781.4500000000003</v>
+            <v>6050.5199999999986</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1184,10 +1183,10 @@
             <v>754319.69999999972</v>
           </cell>
           <cell r="H14" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I14">
-            <v>1068.5999999999999</v>
+            <v>2781.4500000000003</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1204,10 +1203,10 @@
             <v>73448.850000000035</v>
           </cell>
           <cell r="H15" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I15">
-            <v>5105.25</v>
+            <v>1074.05</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1224,10 +1223,10 @@
             <v>401603.64999999979</v>
           </cell>
           <cell r="H16" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I16">
-            <v>10797.129999999996</v>
+            <v>5105.25</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1244,10 +1243,10 @@
             <v>290386.04999999981</v>
           </cell>
           <cell r="H17" t="str">
-            <v>PERDIZES</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I17">
-            <v>5737.8000000000011</v>
+            <v>18733.109999999997</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1261,13 +1260,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>89097.179999999949</v>
+            <v>89097.179999999964</v>
           </cell>
           <cell r="H18" t="str">
-            <v>PIRITUBA</v>
+            <v>PERDIZES</v>
           </cell>
           <cell r="I18">
-            <v>4076.0500000000006</v>
+            <v>5737.8000000000011</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1281,13 +1280,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>128549.60999999967</v>
+            <v>128549.60999999965</v>
           </cell>
           <cell r="H19" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I19">
-            <v>3119.05</v>
+            <v>4076.0500000000006</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1301,13 +1300,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>100430.04000000001</v>
+            <v>100430.04</v>
           </cell>
           <cell r="H20" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I20">
-            <v>13809.31</v>
+            <v>3169.05</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1324,10 +1323,10 @@
             <v>114463.64999999938</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I21">
-            <v>1190.3599999999999</v>
+            <v>13809.310000000001</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
@@ -1341,13 +1340,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>63465.520000000128</v>
+            <v>63470.970000000125</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
           </cell>
           <cell r="I22">
-            <v>1017.3299999999999</v>
+            <v>1190.3599999999999</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
@@ -1364,10 +1363,10 @@
             <v>189006.12999999957</v>
           </cell>
           <cell r="H23" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I23">
-            <v>3131.67</v>
+            <v>1415.1300000000003</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
@@ -1381,13 +1380,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>261561.83499999988</v>
+            <v>269497.81500000006</v>
           </cell>
           <cell r="H24" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I24">
-            <v>84830.230000000054</v>
+            <v>3131.67</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
@@ -1403,6 +1402,12 @@
           <cell r="F25">
             <v>82903.510000000024</v>
           </cell>
+          <cell r="H25" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I25">
+            <v>97104.100000000035</v>
+          </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
           </cell>
@@ -1437,7 +1442,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>134643.04</v>
+            <v>134693.04</v>
           </cell>
         </row>
         <row r="29">
@@ -1453,7 +1458,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>63645.500000000058</v>
+            <v>63645.500000000065</v>
           </cell>
         </row>
         <row r="31">
@@ -1461,7 +1466,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>37911.810000000019</v>
+            <v>38309.610000000022</v>
           </cell>
         </row>
         <row r="32">
@@ -1480,7 +1485,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4331590.0949999597</v>
+            <v>4346605.5649999604</v>
           </cell>
         </row>
         <row r="34">
@@ -1496,7 +1501,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>37752.599999999984</v>
+            <v>37752.599999999962</v>
           </cell>
         </row>
         <row r="36">
@@ -1720,7 +1725,6 @@
         </row>
       </sheetData>
       <sheetData sheetId="6"/>
-      <sheetData sheetId="7" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2425,7 +2429,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4330978.1949999966</v>
+        <v>4345993.6649999982</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2436,7 +2440,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>84830.23000000001</v>
+        <v>96953.860000000015</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2470,7 +2474,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>850521.80500000343</v>
+        <v>835506.33500000183</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2481,7 +2485,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>115199.76999999999</v>
+        <v>103076.13999999998</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2515,7 +2519,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.83585413393804819</v>
+        <v>0.83875203415999189</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2526,7 +2530,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.42408753686946965</v>
+        <v>0.48469659551067346</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2647,11 +2651,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>47906.06</v>
+        <v>48005.060000000005</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>16593.940000000002</v>
+        <v>16494.939999999995</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2666,11 +2670,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10797.129999999996</v>
+        <v>18733.109999999997</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>10202.870000000004</v>
+        <v>2266.8900000000031</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2721,11 +2725,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>255853.86999999947</v>
+        <v>258379.61999999947</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>59146.130000000529</v>
+        <v>56620.380000000529</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2798,11 +2802,11 @@
       </c>
       <c r="D12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A12,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>939.83999999999992</v>
+        <v>1090.08</v>
       </c>
       <c r="E12" s="7">
         <f t="shared" si="0"/>
-        <v>60.160000000000082</v>
+        <v>-90.079999999999927</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4" t="s">
@@ -2894,11 +2898,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>13809.31</v>
+        <v>13809.310000000001</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>5190.6900000000005</v>
+        <v>5190.6899999999987</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2952,11 +2956,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>188526.14999999985</v>
+        <v>189630.79999999981</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>26473.850000000151</v>
+        <v>25369.200000000186</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -3029,11 +3033,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>68069.979999999981</v>
+        <v>68074.979999999967</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>-69.979999999981374</v>
+        <v>-74.979999999966822</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -3048,11 +3052,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5002.9000000000005</v>
+        <v>7528.6500000000024</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>20327.099999999999</v>
+        <v>17801.349999999999</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3106,11 +3110,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>246499.1399999999</v>
+        <v>249240.74</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>13500.860000000102</v>
+        <v>10759.260000000009</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3125,11 +3129,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3119.05</v>
+        <v>3169.05</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>6830.95</v>
+        <v>6780.95</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3183,11 +3187,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>160151.88999999972</v>
+        <v>160151.88999999984</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-35151.889999999723</v>
+        <v>-35151.889999999839</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3202,11 +3206,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1068.5999999999999</v>
+        <v>1074.05</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>2121.4</v>
+        <v>2115.9499999999998</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3221,11 +3225,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>37752.599999999984</v>
+        <v>37752.599999999962</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-37752.599999999984</v>
+        <v>-37752.599999999962</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3415,11 +3419,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3879.900000000001</v>
+        <v>4984.55</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>11130.099999999999</v>
+        <v>10025.450000000001</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3546,11 +3550,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>89097.179999999949</v>
+        <v>89097.179999999964</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>30402.820000000051</v>
+        <v>30402.820000000036</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3565,11 +3569,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3399.1999999999994</v>
+        <v>3404.1999999999994</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>-729.19999999999936</v>
+        <v>-734.19999999999936</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3621,11 +3625,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>128549.60999999967</v>
+        <v>128549.60999999965</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>28450.390000000334</v>
+        <v>28450.390000000349</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3657,11 +3661,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>144256.21000000002</v>
+        <v>146997.81</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>573243.79</v>
+        <v>570502.18999999994</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3696,11 +3700,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>100430.04000000001</v>
+        <v>100430.04</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>19569.959999999992</v>
+        <v>19569.960000000006</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3824,11 +3828,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63465.520000000128</v>
+        <v>63470.970000000125</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>26534.479999999872</v>
+        <v>26529.029999999875</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3907,11 +3911,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1017.3299999999999</v>
+        <v>1415.1300000000003</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>2072.67</v>
+        <v>1674.8699999999997</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3952,11 +3956,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>261561.83499999988</v>
+        <v>269497.81500000006</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>40438.165000000125</v>
+        <v>32502.184999999939</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3971,11 +3975,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3832.95</v>
+        <v>3931.95</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>887.05000000000018</v>
+        <v>788.05000000000018</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -4166,11 +4170,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>134643.04</v>
+        <v>134693.04</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>32356.959999999992</v>
+        <v>32306.959999999992</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4243,11 +4247,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>684987.49500000128</v>
+        <v>684987.49500000139</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>15012.504999998724</v>
+        <v>15012.504999998608</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4266,11 +4270,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4286,11 +4290,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63645.500000000058</v>
+        <v>63645.500000000065</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>36354.499999999942</v>
+        <v>36354.499999999935</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4303,11 +4307,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>301427.12500000064</v>
+        <v>313550.75500000105</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>398572.87499999936</v>
+        <v>386449.24499999895</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4335,11 +4339,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>37911.810000000019</v>
+        <v>38309.610000000022</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>17088.189999999981</v>
+        <v>16690.389999999978</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4466,11 +4470,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.5950000007</v>
+        <v>1184379.5950000002</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.404999999329</v>
+        <v>95620.404999999795</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4574,11 +4578,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>446852.13500000065</v>
+        <v>461867.60500000074</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>833147.86499999929</v>
+        <v>818132.39499999932</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 26/05/2026 14:20
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CFBD4AD-4C9E-4B1C-9034-7166A90C322D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9362CA-C419-4E7E-BFE5-B404C2FDF375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -945,11 +945,11 @@
       <sheetName val="DIN MILHO"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
@@ -1009,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>48005.060000000005</v>
+            <v>48699.320000000007</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>3931.95</v>
+            <v>4626.2099999999991</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>258379.61999999947</v>
+            <v>264878.11999999947</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>7528.6500000000024</v>
+            <v>14027.149999999996</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1066,7 +1066,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I8">
-            <v>1301.71</v>
+            <v>3315.2100000000005</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1080,19 +1080,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>76120.789999999964</v>
+            <v>78134.28999999995</v>
           </cell>
           <cell r="H9" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I9">
-            <v>4984.55</v>
+            <v>7262.1499999999987</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>56</v>
+            <v>57</v>
           </cell>
         </row>
         <row r="10">
@@ -1100,7 +1100,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>189630.79999999981</v>
+            <v>191430.99999999983</v>
           </cell>
           <cell r="H10" t="str">
             <v>JUNDIAI</v>
@@ -1112,7 +1112,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>34</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="11">
@@ -1126,7 +1126,7 @@
             <v>LESTE</v>
           </cell>
           <cell r="I11">
-            <v>2045.9</v>
+            <v>4738.57</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1140,13 +1140,13 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>249240.74</v>
+            <v>255920.77999999997</v>
           </cell>
           <cell r="H12" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I12">
-            <v>7483.15</v>
+            <v>8072.45</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1166,13 +1166,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I13">
-            <v>6050.5199999999986</v>
+            <v>10560.719999999998</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>19</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="14">
@@ -1186,7 +1186,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I14">
-            <v>2781.4500000000003</v>
+            <v>3011.3000000000006</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1206,7 +1206,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="I15">
-            <v>1074.05</v>
+            <v>1213.95</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1226,7 +1226,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="I16">
-            <v>5105.25</v>
+            <v>9175.15</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1240,19 +1240,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>290386.04999999981</v>
+            <v>294835.74999999977</v>
           </cell>
           <cell r="H17" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I17">
-            <v>18733.109999999997</v>
+            <v>20911.96</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>27</v>
+            <v>28</v>
           </cell>
         </row>
         <row r="18">
@@ -1260,13 +1260,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>89097.179999999964</v>
+            <v>91789.849999999933</v>
           </cell>
           <cell r="H18" t="str">
             <v>PERDIZES</v>
           </cell>
           <cell r="I18">
-            <v>5737.8000000000011</v>
+            <v>5897.7000000000007</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1280,19 +1280,19 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>128549.60999999965</v>
+            <v>129138.90999999965</v>
           </cell>
           <cell r="H19" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I19">
-            <v>4076.0500000000006</v>
+            <v>7744.2099999999991</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>70</v>
+            <v>71</v>
           </cell>
         </row>
         <row r="20">
@@ -1300,13 +1300,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>100430.04</v>
+            <v>104940.23999999999</v>
           </cell>
           <cell r="H20" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I20">
-            <v>3169.05</v>
+            <v>3373.95</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1320,7 +1320,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>114463.64999999938</v>
+            <v>114693.49999999937</v>
           </cell>
           <cell r="H21" t="str">
             <v>SBC</v>
@@ -1332,7 +1332,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="N21">
-            <v>33</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="22">
@@ -1340,13 +1340,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>63470.970000000125</v>
+            <v>63610.870000000126</v>
           </cell>
           <cell r="H22" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I22">
-            <v>1190.3599999999999</v>
+            <v>1350.36</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
@@ -1360,13 +1360,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>189006.12999999957</v>
+            <v>193076.02999999962</v>
           </cell>
           <cell r="H23" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I23">
-            <v>1415.1300000000003</v>
+            <v>1493.7300000000002</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
@@ -1380,7 +1380,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>269497.81500000006</v>
+            <v>271676.66500000039</v>
           </cell>
           <cell r="H24" t="str">
             <v>VENDEDOR INTERNO 1</v>
@@ -1400,13 +1400,13 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>82903.510000000024</v>
+            <v>83063.410000000033</v>
           </cell>
           <cell r="H25" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I25">
-            <v>97104.100000000035</v>
+            <v>127270.19</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
@@ -1426,7 +1426,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>583</v>
+            <v>590</v>
           </cell>
         </row>
         <row r="27">
@@ -1434,7 +1434,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>112473.96999999986</v>
+            <v>116142.12999999983</v>
           </cell>
         </row>
         <row r="28">
@@ -1442,7 +1442,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>134693.04</v>
+            <v>134897.94000000003</v>
           </cell>
         </row>
         <row r="29">
@@ -1458,7 +1458,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>63645.500000000065</v>
+            <v>63805.5</v>
           </cell>
         </row>
         <row r="31">
@@ -1466,7 +1466,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>38309.610000000022</v>
+            <v>38388.210000000021</v>
           </cell>
         </row>
         <row r="32">
@@ -1485,7 +1485,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4346605.5649999604</v>
+            <v>4387423.9949999517</v>
           </cell>
         </row>
         <row r="34">
@@ -1724,7 +1724,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="6"/>
+      <sheetData sheetId="6" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4345993.6649999982</v>
+        <v>4386812.0949999979</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>96953.860000000015</v>
+        <v>127119.94999999998</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>835506.33500000183</v>
+        <v>794687.90500000212</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>103076.13999999998</v>
+        <v>72910.050000000017</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.83875203415999189</v>
+        <v>0.84662975875711621</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.48469659551067346</v>
+        <v>0.63550442433634946</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.72875000000000001</v>
+        <v>0.73750000000000004</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2651,11 +2651,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>48005.060000000005</v>
+        <v>48699.320000000007</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>16494.939999999995</v>
+        <v>15800.679999999993</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2670,11 +2670,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>18733.109999999997</v>
+        <v>20911.96</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>2266.8900000000031</v>
+        <v>88.040000000000873</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2725,11 +2725,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>258379.61999999947</v>
+        <v>264878.11999999947</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>56620.380000000529</v>
+        <v>50121.880000000529</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5105.25</v>
+        <v>9175.15</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>8894.75</v>
+        <v>4824.8500000000004</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2782,11 +2782,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W27" si="3">U11-V11</f>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2821,11 +2821,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4076.0500000000006</v>
+        <v>7744.2099999999991</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>10143.949999999999</v>
+        <v>6475.7900000000009</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2859,11 +2859,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2879,11 +2879,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>76120.789999999964</v>
+        <v>78134.28999999995</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>3879.2100000000355</v>
+        <v>1865.7100000000501</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2956,11 +2956,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>189630.79999999981</v>
+        <v>191430.99999999983</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>25369.200000000186</v>
+        <v>23569.000000000175</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2975,11 +2975,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2781.4500000000003</v>
+        <v>3011.3000000000006</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>5468.5499999999993</v>
+        <v>5238.6999999999989</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3052,11 +3052,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7528.6500000000024</v>
+        <v>14027.149999999996</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>17801.349999999999</v>
+        <v>11302.850000000004</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3090,11 +3090,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>249240.74</v>
+        <v>255920.77999999997</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>10759.260000000009</v>
+        <v>4079.2200000000303</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3129,11 +3129,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3169.05</v>
+        <v>3373.95</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>6780.95</v>
+        <v>6576.05</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3167,11 +3167,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3206,11 +3206,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1074.05</v>
+        <v>1213.95</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>2115.9499999999998</v>
+        <v>1976.05</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2045.9</v>
+        <v>4738.57</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>3664.1</v>
+        <v>971.43000000000029</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3347,11 +3347,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7483.15</v>
+        <v>8072.45</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>6516.85</v>
+        <v>5927.55</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3380,11 +3380,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3419,11 +3419,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4984.55</v>
+        <v>7262.1499999999987</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>10025.450000000001</v>
+        <v>7747.8500000000013</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="O20" s="2" cm="1">
         <f t="array" ref="O20">IFERROR(_xlfn.XLOOKUP(N20,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>505000</v>
+        <v>0</v>
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-15661.219999999914</v>
+        <v>-520661.21999999991</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3475,11 +3475,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>290386.04999999981</v>
+        <v>294835.74999999977</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>137113.95000000019</v>
+        <v>132664.25000000023</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3494,11 +3494,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5737.8000000000011</v>
+        <v>5897.7000000000007</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>4172.1999999999989</v>
+        <v>4012.2999999999993</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="O21" s="2" cm="1">
         <f t="array" ref="O21">IFERROR(_xlfn.XLOOKUP(N21,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>627000</v>
+        <v>0</v>
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-157238.58000000031</v>
+        <v>-784238.58000000031</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3550,11 +3550,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>89097.179999999964</v>
+        <v>91789.849999999933</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>30402.820000000036</v>
+        <v>27710.150000000067</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3582,7 +3582,7 @@
       </c>
       <c r="O22" s="2" cm="1">
         <f t="array" ref="O22">IFERROR(_xlfn.XLOOKUP(N22,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>586500</v>
+        <v>0</v>
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>109246.73000000062</v>
+        <v>-477253.26999999938</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3605,11 +3605,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3625,11 +3625,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>128549.60999999965</v>
+        <v>129138.90999999965</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>28450.390000000349</v>
+        <v>27861.090000000346</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3644,11 +3644,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6050.5199999999986</v>
+        <v>10560.719999999998</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>6849.4800000000014</v>
+        <v>2339.2800000000025</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3657,15 +3657,15 @@
       </c>
       <c r="O23" s="2" cm="1">
         <f t="array" ref="O23">IFERROR(_xlfn.XLOOKUP(N23,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
-        <v>717500</v>
+        <v>0</v>
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>146997.81</v>
+        <v>158127.54999999999</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>570502.18999999994</v>
+        <v>-158127.54999999999</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3700,11 +3700,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>100430.04</v>
+        <v>104940.23999999999</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>19569.960000000006</v>
+        <v>15059.760000000009</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3719,11 +3719,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1301.71</v>
+        <v>3315.2100000000005</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>4158.29</v>
+        <v>2144.7899999999995</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3764,11 +3764,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>114463.64999999938</v>
+        <v>114693.49999999937</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>20536.350000000617</v>
+        <v>20306.500000000626</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3828,11 +3828,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63470.970000000125</v>
+        <v>63610.870000000126</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>26529.029999999875</v>
+        <v>26389.129999999874</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3847,11 +3847,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1190.3599999999999</v>
+        <v>1350.36</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>5619.64</v>
+        <v>5459.64</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3892,11 +3892,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>189006.12999999957</v>
+        <v>193076.02999999962</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>45993.870000000432</v>
+        <v>41923.97000000038</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3911,11 +3911,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1415.1300000000003</v>
+        <v>1493.7300000000002</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>1674.8699999999997</v>
+        <v>1596.2699999999998</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3956,11 +3956,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>269497.81500000006</v>
+        <v>271676.66500000039</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>32502.184999999939</v>
+        <v>30323.334999999614</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3975,11 +3975,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3931.95</v>
+        <v>4626.2099999999991</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>788.05000000000018</v>
+        <v>93.790000000000873</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -4007,11 +4007,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>82903.510000000024</v>
+        <v>83063.410000000033</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>30096.489999999976</v>
+        <v>29936.589999999967</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4110,11 +4110,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>112473.96999999986</v>
+        <v>116142.12999999983</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>13526.030000000144</v>
+        <v>9857.87000000017</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4170,11 +4170,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>134693.04</v>
+        <v>134897.94000000003</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>32306.959999999992</v>
+        <v>32102.059999999969</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4187,11 +4187,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000039</v>
+        <v>668938.42000000074</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.579999999609</v>
+        <v>31061.57999999926</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4247,11 +4247,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>684987.49500000139</v>
+        <v>684510.09500000125</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>15012.504999998608</v>
+        <v>15489.904999998747</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4270,11 +4270,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>91</v>
+        <v>79</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4290,11 +4290,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63645.500000000065</v>
+        <v>63805.5</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>36354.499999999935</v>
+        <v>36194.5</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4307,11 +4307,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>313550.75500000105</v>
+        <v>343716.84500000125</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>386449.24499999895</v>
+        <v>356283.15499999875</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4339,11 +4339,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>38309.610000000022</v>
+        <v>38388.210000000021</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>16690.389999999978</v>
+        <v>16611.789999999979</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4542,11 +4542,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1174744.2449999929</v>
+        <v>1174266.844999993</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>105255.75500000711</v>
+        <v>105733.15500000701</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4578,11 +4578,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>461867.60500000074</v>
+        <v>503163.43500000087</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>818132.39499999932</v>
+        <v>776836.56499999913</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 27/05/2026 08:47
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9362CA-C419-4E7E-BFE5-B404C2FDF375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D83CD124-54C7-489F-B458-979974F95C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-26T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-27T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -973,7 +973,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>26/05/2026</v>
+            <v>27/05/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1012,10 +1012,10 @@
             <v>48699.320000000007</v>
           </cell>
           <cell r="H5" t="str">
-            <v>CAMPINAS</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I5">
-            <v>4626.2099999999991</v>
+            <v>4174.6000000000004</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>264878.11999999947</v>
+            <v>270054.51999999949</v>
           </cell>
           <cell r="H6" t="str">
-            <v>CENTRO</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I6">
-            <v>14027.149999999996</v>
+            <v>872.3</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1043,10 +1043,10 @@
             <v>1090.08</v>
           </cell>
           <cell r="H7" t="str">
-            <v>ECOMMERCE</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I7">
-            <v>150.24</v>
+            <v>259.8</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1063,10 +1063,10 @@
             <v>611.9</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INDAIATUBA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I8">
-            <v>3315.2100000000005</v>
+            <v>455.4</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1080,13 +1080,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>78134.28999999995</v>
+            <v>79006.589999999953</v>
           </cell>
           <cell r="H9" t="str">
-            <v>INTERLAGOS</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I9">
-            <v>7262.1499999999987</v>
+            <v>2692.6</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
@@ -1100,19 +1100,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>191430.99999999983</v>
+            <v>192792.94999999981</v>
           </cell>
           <cell r="H10" t="str">
-            <v>JUNDIAI</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I10">
-            <v>3404.1999999999994</v>
+            <v>608.6</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>35</v>
+            <v>37</v>
           </cell>
         </row>
         <row r="11">
@@ -1120,13 +1120,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>68074.979999999967</v>
+            <v>69590.679999999978</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE</v>
+            <v>PERDIZES</v>
           </cell>
           <cell r="I11">
-            <v>4738.57</v>
+            <v>753.9</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1143,16 +1143,16 @@
             <v>255920.77999999997</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE MOOCA</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I12">
-            <v>8072.45</v>
+            <v>748.9</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N12">
-            <v>19</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="13">
@@ -1163,16 +1163,16 @@
             <v>160151.88999999984</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE PENHA</v>
+            <v>SBC</v>
           </cell>
           <cell r="I13">
-            <v>10560.719999999998</v>
+            <v>0</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>20</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="14">
@@ -1180,13 +1180,13 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>754319.69999999972</v>
+            <v>892316.99999999965</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>SJC</v>
           </cell>
           <cell r="I14">
-            <v>3011.3000000000006</v>
+            <v>280</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1200,13 +1200,13 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>73448.850000000035</v>
+            <v>78883.050000000061</v>
           </cell>
           <cell r="H15" t="str">
-            <v>MOGI</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I15">
-            <v>1213.95</v>
+            <v>10846.1</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1220,13 +1220,7 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>401603.64999999979</v>
-          </cell>
-          <cell r="H16" t="str">
-            <v>NORTE</v>
-          </cell>
-          <cell r="I16">
-            <v>9175.15</v>
+            <v>447350.14999999979</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1240,13 +1234,7 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>294835.74999999977</v>
-          </cell>
-          <cell r="H17" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="I17">
-            <v>20911.96</v>
+            <v>298614.14999999979</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1260,19 +1248,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>91789.849999999933</v>
-          </cell>
-          <cell r="H18" t="str">
-            <v>PERDIZES</v>
-          </cell>
-          <cell r="I18">
-            <v>5897.7000000000007</v>
+            <v>92517.149999999921</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>41</v>
+            <v>42</v>
           </cell>
         </row>
         <row r="19">
@@ -1280,19 +1262,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>129138.90999999965</v>
-          </cell>
-          <cell r="H19" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I19">
-            <v>7744.2099999999991</v>
+            <v>131986.50999999966</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>71</v>
+            <v>72</v>
           </cell>
         </row>
         <row r="20">
@@ -1300,13 +1276,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>104940.23999999999</v>
-          </cell>
-          <cell r="H20" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I20">
-            <v>3373.95</v>
+            <v>104940.24</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1322,17 +1292,11 @@
           <cell r="F21">
             <v>114693.49999999937</v>
           </cell>
-          <cell r="H21" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I21">
-            <v>13809.310000000001</v>
-          </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N21">
-            <v>35</v>
+            <v>37</v>
           </cell>
         </row>
         <row r="22">
@@ -1340,13 +1304,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>63610.870000000126</v>
-          </cell>
-          <cell r="H22" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I22">
-            <v>1350.36</v>
+            <v>64189.970000000125</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
@@ -1360,13 +1318,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>193076.02999999962</v>
-          </cell>
-          <cell r="H23" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I23">
-            <v>1493.7300000000002</v>
+            <v>193684.6299999996</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
@@ -1380,13 +1332,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>271676.66500000039</v>
-          </cell>
-          <cell r="H24" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I24">
-            <v>3131.67</v>
+            <v>272880.62500000012</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
@@ -1400,13 +1346,7 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>83063.410000000033</v>
-          </cell>
-          <cell r="H25" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I25">
-            <v>127270.19</v>
+            <v>83817.310000000027</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
@@ -1420,13 +1360,13 @@
             <v>PIRACICABA</v>
           </cell>
           <cell r="F26">
-            <v>102906.86000000004</v>
+            <v>129513.65999999999</v>
           </cell>
           <cell r="K26" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>590</v>
+            <v>598</v>
           </cell>
         </row>
         <row r="27">
@@ -1434,7 +1374,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>116142.12999999983</v>
+            <v>117603.32999999983</v>
           </cell>
         </row>
         <row r="28">
@@ -1442,7 +1382,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>134897.94000000003</v>
+            <v>135219.54</v>
           </cell>
         </row>
         <row r="29">
@@ -1450,7 +1390,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>223288.15999999983</v>
+            <v>223288.1599999998</v>
           </cell>
         </row>
         <row r="30">
@@ -1458,7 +1398,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>63805.5</v>
+            <v>64663.800000000061</v>
           </cell>
         </row>
         <row r="31">
@@ -1466,7 +1406,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>38388.210000000021</v>
+            <v>38604.060000000019</v>
           </cell>
         </row>
         <row r="32">
@@ -1485,7 +1425,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4387423.9949999517</v>
+            <v>4625490.9549999479</v>
           </cell>
         </row>
         <row r="34">
@@ -2429,7 +2369,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4386812.0949999979</v>
+        <v>4624879.0549999969</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2440,7 +2380,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>127119.94999999998</v>
+        <v>10846.099999999999</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2462,7 +2402,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>590</v>
+        <v>598</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2474,7 +2414,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>794687.90500000212</v>
+        <v>556620.94500000309</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2485,7 +2425,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>72910.050000000017</v>
+        <v>189183.9</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2507,7 +2447,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2519,7 +2459,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.84662975875711621</v>
+        <v>0.89257532664286343</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2530,7 +2470,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.63550442433634946</v>
+        <v>5.4222366645003239E-2</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2552,7 +2492,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.73750000000000004</v>
+        <v>0.74750000000000005</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2670,11 +2610,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>20911.96</v>
+        <v>0</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>88.040000000000873</v>
+        <v>21000</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2725,11 +2665,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>264878.11999999947</v>
+        <v>270054.51999999949</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>50121.880000000529</v>
+        <v>44945.480000000505</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2744,11 +2684,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9175.15</v>
+        <v>608.6</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>4824.8500000000004</v>
+        <v>13391.4</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2821,11 +2761,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7744.2099999999991</v>
+        <v>748.9</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>6475.7900000000009</v>
+        <v>13471.1</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2859,11 +2799,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2879,11 +2819,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>78134.28999999995</v>
+        <v>79006.589999999953</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>1865.7100000000501</v>
+        <v>993.41000000004715</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2898,11 +2838,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>13809.310000000001</v>
+        <v>0</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>5190.6899999999987</v>
+        <v>19000</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2956,11 +2896,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>191430.99999999983</v>
+        <v>192792.94999999981</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>23569.000000000175</v>
+        <v>22207.050000000192</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2975,11 +2915,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3011.3000000000006</v>
+        <v>0</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>5238.6999999999989</v>
+        <v>8250</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3013,11 +2953,11 @@
       </c>
       <c r="V14" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W14" s="4">
         <f>U14-V14</f>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3033,11 +2973,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>68074.979999999967</v>
+        <v>69590.679999999978</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>-74.979999999966822</v>
+        <v>-1590.6799999999785</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -3052,11 +2992,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>14027.149999999996</v>
+        <v>4174.6000000000004</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>11302.850000000004</v>
+        <v>21155.4</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3090,11 +3030,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3129,11 +3069,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3373.95</v>
+        <v>0</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>6576.05</v>
+        <v>9950</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3206,11 +3146,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1213.95</v>
+        <v>0</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>1976.05</v>
+        <v>3190</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3264,11 +3204,11 @@
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>754319.69999999972</v>
+        <v>892316.99999999965</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>45680.300000000279</v>
+        <v>-92316.999999999651</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3283,11 +3223,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4738.57</v>
+        <v>455.4</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>971.43000000000029</v>
+        <v>5254.6</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3308,11 +3248,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3328,11 +3268,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>73448.850000000035</v>
+        <v>78883.050000000061</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>41551.149999999965</v>
+        <v>36116.949999999939</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3347,11 +3287,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8072.45</v>
+        <v>2692.6</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>5927.55</v>
+        <v>11307.4</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3380,11 +3320,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3400,11 +3340,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>401603.64999999979</v>
+        <v>447350.14999999979</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>98396.35000000021</v>
+        <v>52649.85000000021</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3419,11 +3359,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7262.1499999999987</v>
+        <v>0</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>7747.8500000000013</v>
+        <v>15010</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3475,11 +3415,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>294835.74999999977</v>
+        <v>298614.14999999979</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>132664.25000000023</v>
+        <v>128885.85000000021</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3494,11 +3434,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5897.7000000000007</v>
+        <v>753.9</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>4012.2999999999993</v>
+        <v>9156.1</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3550,11 +3490,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>91789.849999999933</v>
+        <v>92517.149999999921</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>27710.150000000067</v>
+        <v>26982.850000000079</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3569,11 +3509,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3404.1999999999994</v>
+        <v>259.8</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>-734.19999999999936</v>
+        <v>2410.1999999999998</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3605,11 +3545,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3625,11 +3565,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>129138.90999999965</v>
+        <v>131986.50999999966</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>27861.090000000346</v>
+        <v>25013.49000000034</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3644,11 +3584,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10560.719999999998</v>
+        <v>0</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>2339.2800000000025</v>
+        <v>12900</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3661,11 +3601,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>158127.54999999999</v>
+        <v>351083.95000000013</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-158127.54999999999</v>
+        <v>-351083.95000000013</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3700,11 +3640,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>104940.23999999999</v>
+        <v>104940.24</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>15059.760000000009</v>
+        <v>15059.759999999995</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3719,11 +3659,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3315.2100000000005</v>
+        <v>872.3</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>2144.7899999999995</v>
+        <v>4587.7</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3783,11 +3723,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3131.67</v>
+        <v>0</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>1678.33</v>
+        <v>4810</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3828,11 +3768,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63610.870000000126</v>
+        <v>64189.970000000125</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>26389.129999999874</v>
+        <v>25810.029999999875</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3847,11 +3787,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1350.36</v>
+        <v>280</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>5459.64</v>
+        <v>6530</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3892,11 +3832,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>193076.02999999962</v>
+        <v>193684.6299999996</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>41923.97000000038</v>
+        <v>41315.370000000403</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3911,11 +3851,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1493.7300000000002</v>
+        <v>0</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>1596.2699999999998</v>
+        <v>3090</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3956,11 +3896,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>271676.66500000039</v>
+        <v>272880.62500000012</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>30323.334999999614</v>
+        <v>29119.374999999884</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3975,11 +3915,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4626.2099999999991</v>
+        <v>0</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>93.790000000000873</v>
+        <v>4720</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -4007,11 +3947,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>83063.410000000033</v>
+        <v>83817.310000000027</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>29936.589999999967</v>
+        <v>29182.689999999973</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4053,11 +3993,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>102906.86000000004</v>
+        <v>129513.65999999999</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>67093.139999999956</v>
+        <v>40486.340000000011</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4110,11 +4050,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>116142.12999999983</v>
+        <v>117603.32999999983</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>9857.87000000017</v>
+        <v>8396.6700000001729</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4170,11 +4110,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>134897.94000000003</v>
+        <v>135219.54</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>32102.059999999969</v>
+        <v>31780.459999999992</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4187,11 +4127,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000074</v>
+        <v>668938.42000000051</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.57999999926</v>
+        <v>31061.579999999492</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4230,11 +4170,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>223288.15999999983</v>
+        <v>223288.1599999998</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>31711.840000000171</v>
+        <v>31711.8400000002</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4247,11 +4187,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>684510.09500000125</v>
+        <v>684366.59500000149</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>15489.904999998747</v>
+        <v>15633.404999998515</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4270,11 +4210,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>79</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4290,11 +4230,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63805.5</v>
+        <v>64663.800000000061</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>36194.5</v>
+        <v>35336.199999999939</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4307,11 +4247,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>343716.84500000125</v>
+        <v>362364.10500000085</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>356283.15499999875</v>
+        <v>337635.89499999915</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4339,11 +4279,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>38388.210000000021</v>
+        <v>38604.060000000019</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>16611.789999999979</v>
+        <v>16395.939999999981</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4470,11 +4410,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.5950000002</v>
+        <v>1184379.595</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.404999999795</v>
+        <v>95620.405000000028</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4542,11 +4482,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1174266.844999993</v>
+        <v>1174123.3449999928</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>105733.15500000701</v>
+        <v>105876.65500000725</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4578,11 +4518,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>503163.43500000087</v>
+        <v>741373.89500000095</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>776836.56499999913</v>
+        <v>538626.10499999905</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 27/05/2026 14:29
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8E5CD9-A91E-44AC-9E43-C5AF3B3BFC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D1CF02-9827-4DF1-BC6F-8595431235FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1009,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>48699.320000000007</v>
+            <v>49432.270000000004</v>
           </cell>
           <cell r="H5" t="str">
-            <v>CENTRO</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>4174.6000000000004</v>
+            <v>732.95</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>270054.51999999949</v>
+            <v>275447.5099999996</v>
           </cell>
           <cell r="H6" t="str">
-            <v>INDAIATUBA</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>872.3</v>
+            <v>9567.59</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1043,10 +1043,10 @@
             <v>1090.08</v>
           </cell>
           <cell r="H7" t="str">
-            <v>JUNDIAI</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>259.8</v>
+            <v>6169.4000000000005</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1060,13 +1060,13 @@
             <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F8">
-            <v>611.9</v>
+            <v>1136.3</v>
           </cell>
           <cell r="H8" t="str">
-            <v>LESTE</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>455.4</v>
+            <v>10790.949999999999</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1080,19 +1080,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>79006.589999999953</v>
+            <v>84343.489999999976</v>
           </cell>
           <cell r="H9" t="str">
-            <v>LESTE MOOCA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>2692.6</v>
+            <v>2322.1000000000004</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>57</v>
+            <v>59</v>
           </cell>
         </row>
         <row r="10">
@@ -1100,19 +1100,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>192792.94999999981</v>
+            <v>203583.8999999997</v>
           </cell>
           <cell r="H10" t="str">
-            <v>NORTE</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>608.6</v>
+            <v>2212.35</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>37</v>
+            <v>39</v>
           </cell>
         </row>
         <row r="11">
@@ -1120,19 +1120,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>69590.679999999978</v>
+            <v>71652.979999999967</v>
           </cell>
           <cell r="H11" t="str">
-            <v>PERDIZES</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>753.9</v>
+            <v>6418.9999999999982</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>39</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="12">
@@ -1140,13 +1140,13 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>255920.77999999997</v>
+            <v>257638.77999999997</v>
           </cell>
           <cell r="H12" t="str">
-            <v>PIRITUBA</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>748.9</v>
+            <v>2360.7500000000005</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1163,16 +1163,16 @@
             <v>160151.88999999984</v>
           </cell>
           <cell r="H13" t="str">
-            <v>SBC</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>0</v>
+            <v>2594.0500000000002</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>21</v>
+            <v>22</v>
           </cell>
         </row>
         <row r="14">
@@ -1180,19 +1180,19 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>892316.99999999965</v>
+            <v>910576.39999999967</v>
           </cell>
           <cell r="H14" t="str">
-            <v>SJC</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>280</v>
+            <v>745.25</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>38</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="15">
@@ -1200,19 +1200,19 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>78883.050000000061</v>
+            <v>84084.20000000007</v>
           </cell>
           <cell r="H15" t="str">
-            <v>Total Geral</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>10846.1</v>
+            <v>8743.4199999999983</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N15">
-            <v>14</v>
+            <v>16</v>
           </cell>
         </row>
         <row r="16">
@@ -1222,11 +1222,17 @@
           <cell r="F16">
             <v>447350.14999999979</v>
           </cell>
+          <cell r="H16" t="str">
+            <v>OSASCO</v>
+          </cell>
+          <cell r="I16">
+            <v>15584.940000000002</v>
+          </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>46</v>
+            <v>48</v>
           </cell>
         </row>
         <row r="17">
@@ -1234,13 +1240,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>298614.14999999979</v>
+            <v>320215.64999999967</v>
+          </cell>
+          <cell r="H17" t="str">
+            <v>PERDIZES</v>
+          </cell>
+          <cell r="I17">
+            <v>5354.02</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>28</v>
+            <v>29</v>
           </cell>
         </row>
         <row r="18">
@@ -1248,13 +1260,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>92517.149999999921</v>
+            <v>94274.099999999919</v>
+          </cell>
+          <cell r="H18" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="I18">
+            <v>3668.11</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>42</v>
+            <v>47</v>
           </cell>
         </row>
         <row r="19">
@@ -1262,13 +1280,19 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>131986.50999999966</v>
+            <v>135712.90999999965</v>
+          </cell>
+          <cell r="H19" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="I19">
+            <v>10133.829999999998</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>72</v>
+            <v>74</v>
           </cell>
         </row>
         <row r="20">
@@ -1276,13 +1300,19 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>104940.24</v>
+            <v>107300.98999999999</v>
+          </cell>
+          <cell r="H20" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="I20">
+            <v>6267.4000000000005</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
           </cell>
           <cell r="N20">
-            <v>19</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="21">
@@ -1290,13 +1320,19 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>114693.49999999937</v>
+            <v>117287.54999999938</v>
+          </cell>
+          <cell r="H21" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I21">
+            <v>5180.329999999999</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N21">
-            <v>37</v>
+            <v>39</v>
           </cell>
         </row>
         <row r="22">
@@ -1304,7 +1340,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>64189.970000000125</v>
+            <v>64945.220000000125</v>
+          </cell>
+          <cell r="H22" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I22">
+            <v>329.25</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
@@ -1318,13 +1360,19 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>193684.6299999996</v>
+            <v>201819.44999999955</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I23">
+            <v>99175.689999999988</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
           </cell>
           <cell r="N23">
-            <v>41</v>
+            <v>42</v>
           </cell>
         </row>
         <row r="24">
@@ -1332,13 +1380,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>272880.62500000012</v>
+            <v>288465.56499999971</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N24">
-            <v>20</v>
+            <v>22</v>
           </cell>
         </row>
         <row r="25">
@@ -1346,7 +1394,7 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>83817.310000000027</v>
+            <v>88417.430000000022</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
@@ -1366,7 +1414,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>598</v>
+            <v>625</v>
           </cell>
         </row>
         <row r="27">
@@ -1374,7 +1422,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>117603.32999999983</v>
+            <v>120522.53999999979</v>
           </cell>
         </row>
         <row r="28">
@@ -1382,7 +1430,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>135219.54</v>
+            <v>145353.36999999997</v>
           </cell>
         </row>
         <row r="29">
@@ -1390,7 +1438,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>223288.1599999998</v>
+            <v>229555.55999999976</v>
           </cell>
         </row>
         <row r="30">
@@ -1398,7 +1446,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>64663.800000000061</v>
+            <v>69564.130000000092</v>
           </cell>
         </row>
         <row r="31">
@@ -1406,7 +1454,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>38604.060000000019</v>
+            <v>38933.310000000019</v>
           </cell>
         </row>
         <row r="32">
@@ -1425,7 +1473,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4625490.9549999479</v>
+            <v>4761174.7949999413</v>
           </cell>
         </row>
         <row r="34">
@@ -2369,7 +2417,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4624879.0549999969</v>
+        <v>4760038.4949999973</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2380,7 +2428,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>10846.099999999999</v>
+        <v>99175.69</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2402,7 +2450,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>598</v>
+        <v>625</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2414,7 +2462,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>556620.94500000309</v>
+        <v>421461.50500000268</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2425,7 +2473,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>189183.9</v>
+        <v>100854.31</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2447,7 +2495,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>202</v>
+        <v>175</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2459,7 +2507,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.89257532664286343</v>
+        <v>0.91866032905529238</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2470,7 +2518,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>5.4222366645003239E-2</v>
+        <v>0.49580407938809179</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2492,7 +2540,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.74750000000000005</v>
+        <v>0.78125</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2591,11 +2639,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>48699.320000000007</v>
+        <v>49432.270000000004</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>15800.679999999993</v>
+        <v>15067.729999999996</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2610,11 +2658,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>15584.940000000002</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>21000</v>
+        <v>5415.0599999999977</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2665,11 +2713,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>270054.51999999949</v>
+        <v>275447.5099999996</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>44945.480000000505</v>
+        <v>39552.490000000398</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2684,11 +2732,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>608.6</v>
+        <v>8743.4199999999983</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>13391.4</v>
+        <v>5256.5800000000017</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2722,11 +2770,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W27" si="3">U11-V11</f>
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2761,11 +2809,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>748.9</v>
+        <v>3668.11</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>13471.1</v>
+        <v>10551.89</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2799,11 +2847,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2819,11 +2867,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>79006.589999999953</v>
+        <v>84343.489999999976</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>993.41000000004715</v>
+        <v>-4343.4899999999761</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2838,11 +2886,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>6267.4000000000005</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>19000</v>
+        <v>12732.599999999999</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2876,11 +2924,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2896,11 +2944,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>192792.94999999981</v>
+        <v>203583.8999999997</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>22207.050000000192</v>
+        <v>11416.100000000297</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2915,11 +2963,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>2594.0500000000002</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>8250</v>
+        <v>5655.95</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -2973,11 +3021,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>69590.679999999978</v>
+        <v>71652.979999999967</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>-1590.6799999999785</v>
+        <v>-3652.9799999999668</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2992,11 +3040,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4174.6000000000004</v>
+        <v>9567.59</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>21155.4</v>
+        <v>15762.41</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3030,11 +3078,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3050,11 +3098,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>255920.77999999997</v>
+        <v>257638.77999999997</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>4079.2200000000303</v>
+        <v>2361.2200000000303</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3069,11 +3117,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>10133.829999999998</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>9950</v>
+        <v>-183.82999999999811</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3107,11 +3155,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3146,11 +3194,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>745.25</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>3190</v>
+        <v>2444.75</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3184,11 +3232,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3204,11 +3252,11 @@
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>892316.99999999965</v>
+        <v>910576.39999999967</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>-92316.999999999651</v>
+        <v>-110576.39999999967</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3223,11 +3271,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>455.4</v>
+        <v>2212.35</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>5254.6</v>
+        <v>3497.65</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3248,11 +3296,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3268,11 +3316,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>78883.050000000061</v>
+        <v>84084.20000000007</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>36116.949999999939</v>
+        <v>30915.79999999993</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3287,11 +3335,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2692.6</v>
+        <v>6418.9999999999982</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>11307.4</v>
+        <v>7581.0000000000018</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3320,11 +3368,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3359,11 +3407,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>10790.949999999999</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>15010</v>
+        <v>4219.0500000000011</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3395,11 +3443,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3415,11 +3463,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>298614.14999999979</v>
+        <v>320215.64999999967</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>128885.85000000021</v>
+        <v>107284.35000000033</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3434,11 +3482,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>753.9</v>
+        <v>5354.02</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>9156.1</v>
+        <v>4555.9799999999996</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3470,11 +3518,11 @@
       </c>
       <c r="V21" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S21,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="W21" s="4">
         <f t="shared" si="3"/>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3490,11 +3538,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>92517.149999999921</v>
+        <v>94274.099999999919</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>26982.850000000079</v>
+        <v>25225.900000000081</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3509,11 +3557,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>259.8</v>
+        <v>2322.1000000000004</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>2410.1999999999998</v>
+        <v>347.89999999999964</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3545,11 +3593,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3565,11 +3613,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>131986.50999999966</v>
+        <v>135712.90999999965</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>25013.49000000034</v>
+        <v>21287.090000000346</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3584,11 +3632,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>2360.7500000000005</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>12900</v>
+        <v>10539.25</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3601,11 +3649,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>351083.95000000013</v>
+        <v>397864</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-351083.95000000013</v>
+        <v>-397864</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3640,11 +3688,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>104940.24</v>
+        <v>107300.98999999999</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>15059.759999999995</v>
+        <v>12699.010000000009</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3659,11 +3707,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>872.3</v>
+        <v>6169.4000000000005</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>4587.7</v>
+        <v>-709.40000000000055</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3684,11 +3732,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3704,11 +3752,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>114693.49999999937</v>
+        <v>117287.54999999938</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>20306.500000000626</v>
+        <v>17712.450000000623</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3748,11 +3796,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3768,11 +3816,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>64189.970000000125</v>
+        <v>64945.220000000125</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>25810.029999999875</v>
+        <v>25054.779999999875</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3787,11 +3835,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>280</v>
+        <v>5180.329999999999</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>6530</v>
+        <v>1629.670000000001</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3812,11 +3860,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-7</v>
+        <v>-9</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3832,11 +3880,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>193684.6299999996</v>
+        <v>201819.44999999955</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>41315.370000000403</v>
+        <v>33180.550000000454</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3851,11 +3899,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>329.25</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>3090</v>
+        <v>2760.75</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3896,11 +3944,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>272880.62500000012</v>
+        <v>288465.56499999971</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>29119.374999999884</v>
+        <v>13534.435000000289</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3915,11 +3963,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>732.95</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>4720</v>
+        <v>3987.05</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -3947,11 +3995,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>83817.310000000027</v>
+        <v>88417.430000000022</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>29182.689999999973</v>
+        <v>24582.569999999978</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4050,11 +4098,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>117603.32999999983</v>
+        <v>120522.53999999979</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>8396.6700000001729</v>
+        <v>5477.4600000002101</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4067,11 +4115,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>645369.17500000272</v>
+        <v>645369.17500000249</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>54630.824999997276</v>
+        <v>54630.824999997509</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4110,11 +4158,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>135219.54</v>
+        <v>145353.36999999997</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>31780.459999999992</v>
+        <v>21646.630000000034</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4170,11 +4218,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>223288.1599999998</v>
+        <v>229555.55999999976</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>31711.8400000002</v>
+        <v>25444.440000000235</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4187,11 +4235,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>684366.59500000149</v>
+        <v>684366.59500000125</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>15633.404999998515</v>
+        <v>15633.404999998747</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4210,11 +4258,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>134</v>
+        <v>177</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>66</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4230,11 +4278,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>64663.800000000061</v>
+        <v>69564.130000000092</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>35336.199999999939</v>
+        <v>30435.869999999908</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4247,11 +4295,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>362364.10500000085</v>
+        <v>450743.49500000151</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>337635.89499999915</v>
+        <v>249256.50499999849</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4279,11 +4327,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>38604.060000000019</v>
+        <v>38933.310000000019</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>16395.939999999981</v>
+        <v>16066.689999999981</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4410,11 +4458,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.595</v>
+        <v>1184379.5949999997</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.405000000028</v>
+        <v>95620.405000000261</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4482,11 +4530,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1174123.3449999928</v>
+        <v>1174123.3449999935</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>105876.65500000725</v>
+        <v>105876.65500000655</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4518,11 +4566,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>741373.89500000095</v>
+        <v>877057.73500000034</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>538626.10499999905</v>
+        <v>402942.26499999966</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 28/05/2026 10:55
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D1CF02-9827-4DF1-BC6F-8595431235FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A197B90E-9CE2-4DE1-B4D3-FD07C9C29605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-27T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-28T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -973,7 +973,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>27/05/2026</v>
+            <v>28/05/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1009,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>49432.270000000004</v>
+            <v>51296.62000000001</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>732.95</v>
+            <v>1864.35</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>275447.5099999996</v>
+            <v>281742.71999999962</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>9567.59</v>
+            <v>6295.2099999999991</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1046,7 +1046,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>6169.4000000000005</v>
+            <v>150</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1066,7 +1066,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>10790.949999999999</v>
+            <v>5234</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1080,19 +1080,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>84343.489999999976</v>
+            <v>84353.489999999976</v>
           </cell>
           <cell r="H9" t="str">
-            <v>JUNDIAI</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I9">
-            <v>2322.1000000000004</v>
+            <v>3513.69</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>59</v>
+            <v>62</v>
           </cell>
         </row>
         <row r="10">
@@ -1100,13 +1100,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>203583.8999999997</v>
+            <v>208221.09999999969</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I10">
-            <v>2212.35</v>
+            <v>2938.8000000000006</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1120,19 +1120,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>71652.979999999967</v>
+            <v>71652.98</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I11">
-            <v>6418.9999999999982</v>
+            <v>1987.6500000000003</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>40</v>
+            <v>42</v>
           </cell>
         </row>
         <row r="12">
@@ -1140,13 +1140,13 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>257638.77999999997</v>
+            <v>264436.77999999997</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I12">
-            <v>2360.7500000000005</v>
+            <v>953.93</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1160,19 +1160,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>160151.88999999984</v>
+            <v>160151.88999999996</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I13">
-            <v>2594.0500000000002</v>
+            <v>1432.2200000000003</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>22</v>
+            <v>25</v>
           </cell>
         </row>
         <row r="14">
@@ -1180,19 +1180,19 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>910576.39999999967</v>
+            <v>982675.7999999997</v>
           </cell>
           <cell r="H14" t="str">
-            <v>MOGI</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I14">
-            <v>745.25</v>
+            <v>829.19999999999993</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>40</v>
+            <v>43</v>
           </cell>
         </row>
         <row r="15">
@@ -1200,19 +1200,19 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>84084.20000000007</v>
+            <v>88567.600000000064</v>
           </cell>
           <cell r="H15" t="str">
-            <v>NORTE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I15">
-            <v>8743.4199999999983</v>
+            <v>4060.4600000000005</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N15">
-            <v>16</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="16">
@@ -1220,19 +1220,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>447350.14999999979</v>
+            <v>454485.34999999992</v>
           </cell>
           <cell r="H16" t="str">
-            <v>OSASCO</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I16">
-            <v>15584.940000000002</v>
+            <v>674.75</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>48</v>
+            <v>51</v>
           </cell>
         </row>
         <row r="17">
@@ -1240,19 +1240,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>320215.64999999967</v>
+            <v>320616.14999999967</v>
           </cell>
           <cell r="H17" t="str">
-            <v>PERDIZES</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I17">
-            <v>5354.02</v>
+            <v>259.8</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>29</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="18">
@@ -1260,19 +1260,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>94274.099999999919</v>
+            <v>98434.389999999883</v>
           </cell>
           <cell r="H18" t="str">
-            <v>PIRITUBA</v>
+            <v>SBC</v>
           </cell>
           <cell r="I18">
-            <v>3668.11</v>
+            <v>5909.01</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>47</v>
+            <v>49</v>
           </cell>
         </row>
         <row r="19">
@@ -1280,13 +1280,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>135712.90999999965</v>
+            <v>138560.34999999966</v>
           </cell>
           <cell r="H19" t="str">
-            <v>SANTO ANDRE</v>
+            <v>SJC</v>
           </cell>
           <cell r="I19">
-            <v>10133.829999999998</v>
+            <v>1310.0999999999999</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1300,13 +1300,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>107300.98999999999</v>
+            <v>108789.73999999999</v>
           </cell>
           <cell r="H20" t="str">
-            <v>SBC</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I20">
-            <v>6267.4000000000005</v>
+            <v>553.16999999999996</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1320,19 +1320,19 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>117287.54999999938</v>
+            <v>118241.47999999934</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SJC</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I21">
-            <v>5180.329999999999</v>
+            <v>1159.99</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N21">
-            <v>39</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="22">
@@ -1340,19 +1340,19 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>64945.220000000125</v>
+            <v>69424.940000000075</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SJC/VALE</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I22">
-            <v>329.25</v>
+            <v>39126.330000000009</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N22">
-            <v>29</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="23">
@@ -1360,13 +1360,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>201819.44999999955</v>
-          </cell>
-          <cell r="H23" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I23">
-            <v>99175.689999999988</v>
+            <v>202648.6499999995</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
@@ -1380,13 +1374,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>288465.56499999971</v>
+            <v>292526.02499999985</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N24">
-            <v>22</v>
+            <v>26</v>
           </cell>
         </row>
         <row r="25">
@@ -1394,13 +1388,13 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>88417.430000000022</v>
+            <v>89968.829999999973</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="N25">
-            <v>19</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="26">
@@ -1414,7 +1408,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>625</v>
+            <v>652</v>
           </cell>
         </row>
         <row r="27">
@@ -1422,7 +1416,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>120522.53999999979</v>
+            <v>122636.4899999998</v>
           </cell>
         </row>
         <row r="28">
@@ -1430,7 +1424,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>145353.36999999997</v>
+            <v>149500.07</v>
           </cell>
         </row>
         <row r="29">
@@ -1438,7 +1432,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>229555.55999999976</v>
+            <v>235464.56999999969</v>
           </cell>
         </row>
         <row r="30">
@@ -1446,7 +1440,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>69564.130000000092</v>
+            <v>70874.230000000098</v>
           </cell>
         </row>
         <row r="31">
@@ -1454,7 +1448,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>38933.310000000019</v>
+            <v>39486.480000000025</v>
           </cell>
         </row>
         <row r="32">
@@ -1462,7 +1456,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F32">
-            <v>62805.409999999989</v>
+            <v>63965.399999999987</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1473,7 +1467,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4761174.7949999413</v>
+            <v>4900462.1649999404</v>
           </cell>
         </row>
         <row r="34">
@@ -2417,7 +2411,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4760038.4949999973</v>
+        <v>4899325.8649999984</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2428,7 +2422,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>99175.69</v>
+        <v>39126.329999999994</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2450,7 +2444,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>625</v>
+        <v>652</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2462,7 +2456,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>421461.50500000268</v>
+        <v>282174.13500000164</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2473,7 +2467,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>100854.31</v>
+        <v>160903.67000000001</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2495,7 +2489,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>175</v>
+        <v>148</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2507,7 +2501,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.91866032905529238</v>
+        <v>0.94554199845604525</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2518,7 +2512,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.49580407938809179</v>
+        <v>0.19560230965355194</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2540,7 +2534,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.78125</v>
+        <v>0.81499999999999995</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2639,11 +2633,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>49432.270000000004</v>
+        <v>51296.62000000001</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>15067.729999999996</v>
+        <v>13203.37999999999</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2658,11 +2652,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>15584.940000000002</v>
+        <v>4060.4600000000005</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>5415.0599999999977</v>
+        <v>16939.54</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2713,11 +2707,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>275447.5099999996</v>
+        <v>281742.71999999962</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>39552.490000000398</v>
+        <v>33257.280000000377</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2732,11 +2726,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8743.4199999999983</v>
+        <v>829.19999999999993</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>5256.5800000000017</v>
+        <v>13170.8</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2770,11 +2764,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W27" si="3">U11-V11</f>
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2809,11 +2803,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3668.11</v>
+        <v>674.75</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>10551.89</v>
+        <v>13545.25</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2867,11 +2861,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>84343.489999999976</v>
+        <v>84353.489999999976</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>-4343.4899999999761</v>
+        <v>-4353.4899999999761</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2886,11 +2880,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6267.4000000000005</v>
+        <v>5909.01</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>12732.599999999999</v>
+        <v>13090.99</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2924,11 +2918,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2944,11 +2938,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>203583.8999999997</v>
+        <v>208221.09999999969</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>11416.100000000297</v>
+        <v>6778.9000000003143</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2963,11 +2957,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2594.0500000000002</v>
+        <v>953.93</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>5655.95</v>
+        <v>7296.07</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3021,11 +3015,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>71652.979999999967</v>
+        <v>71652.98</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>-3652.9799999999668</v>
+        <v>-3652.9799999999959</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -3040,11 +3034,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9567.59</v>
+        <v>6295.2099999999991</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>15762.41</v>
+        <v>19034.79</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3078,11 +3072,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3098,11 +3092,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>257638.77999999997</v>
+        <v>264436.77999999997</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>2361.2200000000303</v>
+        <v>-4436.7799999999697</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3117,11 +3111,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10133.829999999998</v>
+        <v>259.8</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>-183.82999999999811</v>
+        <v>9690.2000000000007</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3155,11 +3149,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3175,11 +3169,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>160151.88999999984</v>
+        <v>160151.88999999996</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-35151.889999999839</v>
+        <v>-35151.889999999956</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3194,11 +3188,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>745.25</v>
+        <v>1432.2200000000003</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>2444.75</v>
+        <v>1757.7799999999997</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3232,11 +3226,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3252,11 +3246,11 @@
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>910576.39999999967</v>
+        <v>982675.7999999997</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>-110576.39999999967</v>
+        <v>-182675.7999999997</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3271,11 +3265,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2212.35</v>
+        <v>3513.69</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>3497.65</v>
+        <v>2196.31</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3296,11 +3290,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3316,11 +3310,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>84084.20000000007</v>
+        <v>88567.600000000064</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>30915.79999999993</v>
+        <v>26432.399999999936</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3335,11 +3329,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6418.9999999999982</v>
+        <v>2938.8000000000006</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>7581.0000000000018</v>
+        <v>11061.199999999999</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3388,11 +3382,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>447350.14999999979</v>
+        <v>454485.34999999992</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>52649.85000000021</v>
+        <v>45514.650000000081</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3407,11 +3401,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10790.949999999999</v>
+        <v>5234</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>4219.0500000000011</v>
+        <v>9776</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3443,11 +3437,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3463,11 +3457,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>320215.64999999967</v>
+        <v>320616.14999999967</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>107284.35000000033</v>
+        <v>106883.85000000033</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3482,11 +3476,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5354.02</v>
+        <v>0</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>4555.9799999999996</v>
+        <v>9910</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3538,11 +3532,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>94274.099999999919</v>
+        <v>98434.389999999883</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>25225.900000000081</v>
+        <v>21065.610000000117</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3557,11 +3551,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2322.1000000000004</v>
+        <v>0</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>347.89999999999964</v>
+        <v>2670</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3574,11 +3568,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>477253.26999999938</v>
+        <v>476897.76999999938</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-477253.26999999938</v>
+        <v>-476897.76999999938</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3593,11 +3587,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3613,11 +3607,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>135712.90999999965</v>
+        <v>138560.34999999966</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>21287.090000000346</v>
+        <v>18439.650000000343</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3632,11 +3626,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2360.7500000000005</v>
+        <v>1987.6500000000003</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>10539.25</v>
+        <v>10912.35</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3649,11 +3643,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>397864</v>
+        <v>489136.00000000012</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-397864</v>
+        <v>-489136.00000000012</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3668,11 +3662,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3688,11 +3682,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>107300.98999999999</v>
+        <v>108789.73999999999</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>12699.010000000009</v>
+        <v>11210.260000000009</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3707,11 +3701,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6169.4000000000005</v>
+        <v>150</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>-709.40000000000055</v>
+        <v>5310</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3752,11 +3746,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>117287.54999999938</v>
+        <v>118241.47999999934</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>17712.450000000623</v>
+        <v>16758.520000000659</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3771,11 +3765,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>1159.99</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>4810</v>
+        <v>3650.01</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3796,11 +3790,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3816,11 +3810,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>64945.220000000125</v>
+        <v>69424.940000000075</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>25054.779999999875</v>
+        <v>20575.059999999925</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3835,11 +3829,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5180.329999999999</v>
+        <v>1310.0999999999999</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>1629.670000000001</v>
+        <v>5499.9</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3860,11 +3854,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-9</v>
+        <v>-12</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3880,11 +3874,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>201819.44999999955</v>
+        <v>202648.6499999995</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>33180.550000000454</v>
+        <v>32351.350000000501</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3899,11 +3893,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>329.25</v>
+        <v>553.16999999999996</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>2760.75</v>
+        <v>2536.83</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3924,11 +3918,11 @@
       </c>
       <c r="V27" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S27,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W27" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
@@ -3944,11 +3938,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>288465.56499999971</v>
+        <v>292526.02499999985</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>13534.435000000289</v>
+        <v>9473.9750000001513</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3963,11 +3957,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>732.95</v>
+        <v>1864.35</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>3987.05</v>
+        <v>2855.65</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -3995,11 +3989,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>88417.430000000022</v>
+        <v>89968.829999999973</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>24582.569999999978</v>
+        <v>23031.170000000027</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4098,11 +4092,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>120522.53999999979</v>
+        <v>122636.4899999998</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>5477.4600000002101</v>
+        <v>3363.5100000001985</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4115,11 +4109,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>645369.17500000249</v>
+        <v>645369.17500000272</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>54630.824999997509</v>
+        <v>54630.824999997276</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4158,11 +4152,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>145353.36999999997</v>
+        <v>149500.07</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>21646.630000000034</v>
+        <v>17499.929999999993</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4175,11 +4169,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000051</v>
+        <v>668938.42000000039</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.579999999492</v>
+        <v>31061.579999999609</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4218,11 +4212,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>229555.55999999976</v>
+        <v>235464.56999999969</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>25444.440000000235</v>
+        <v>19535.430000000313</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4235,11 +4229,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>684366.59500000125</v>
+        <v>683867.69500000135</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>15633.404999998747</v>
+        <v>16132.304999998654</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4258,11 +4252,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>177</v>
+        <v>212</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>23</v>
+        <v>-12</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4278,11 +4272,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>69564.130000000092</v>
+        <v>70874.230000000098</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>30435.869999999908</v>
+        <v>29125.769999999902</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4295,11 +4289,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>450743.49500000151</v>
+        <v>499613.26500000223</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>249256.50499999849</v>
+        <v>200386.73499999777</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4327,11 +4321,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>38933.310000000019</v>
+        <v>39486.480000000025</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>16066.689999999981</v>
+        <v>15513.519999999975</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4365,11 +4359,11 @@
       </c>
       <c r="D36" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A36,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>62805.409999999989</v>
+        <v>63965.399999999987</v>
       </c>
       <c r="E36" s="7">
         <f t="shared" si="0"/>
-        <v>3194.5900000000111</v>
+        <v>2034.6000000000131</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -4530,11 +4524,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1174123.3449999935</v>
+        <v>1173268.9449999928</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>105876.65500000655</v>
+        <v>106731.05500000715</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4566,11 +4560,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>877057.73500000034</v>
+        <v>1017199.5050000011</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>402942.26499999966</v>
+        <v>262800.49499999895</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 28/05/2026 12:24
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A197B90E-9CE2-4DE1-B4D3-FD07C9C29605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25683927-4277-437A-9307-C932A7104E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1009,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>51296.62000000001</v>
+            <v>51895.320000000007</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>1864.35</v>
+            <v>2463.0499999999997</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>281742.71999999962</v>
+            <v>283599.41999999963</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>6295.2099999999991</v>
+            <v>8151.909999999998</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1046,7 +1046,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>150</v>
+            <v>687.8</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1066,7 +1066,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>5234</v>
+            <v>9061.4</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1080,13 +1080,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>84353.489999999976</v>
+            <v>84891.289999999964</v>
           </cell>
           <cell r="H9" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="I9">
-            <v>3513.69</v>
+            <v>4955.1899999999996</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
@@ -1100,19 +1100,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>208221.09999999969</v>
+            <v>212048.49999999965</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I10">
-            <v>2938.8000000000006</v>
+            <v>4160.1000000000004</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>39</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="11">
@@ -1120,7 +1120,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>71652.98</v>
+            <v>71652.979999999967</v>
           </cell>
           <cell r="H11" t="str">
             <v>LESTE PENHA</v>
@@ -1132,7 +1132,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>42</v>
+            <v>43</v>
           </cell>
         </row>
         <row r="12">
@@ -1140,13 +1140,13 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>264436.77999999997</v>
+            <v>279342.77999999997</v>
           </cell>
           <cell r="H12" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I12">
-            <v>953.93</v>
+            <v>1503.5300000000004</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1160,19 +1160,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>160151.88999999996</v>
+            <v>160151.8899999999</v>
           </cell>
           <cell r="H13" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="I13">
-            <v>1432.2200000000003</v>
+            <v>3386.9200000000005</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>25</v>
+            <v>26</v>
           </cell>
         </row>
         <row r="14">
@@ -1186,13 +1186,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="I14">
-            <v>829.19999999999993</v>
+            <v>11677.25</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>43</v>
+            <v>44</v>
           </cell>
         </row>
         <row r="15">
@@ -1206,7 +1206,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="I15">
-            <v>4060.4600000000005</v>
+            <v>10443.859999999999</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1223,16 +1223,16 @@
             <v>454485.34999999992</v>
           </cell>
           <cell r="H16" t="str">
-            <v>PIRITUBA</v>
+            <v>PERDIZES</v>
           </cell>
           <cell r="I16">
-            <v>674.75</v>
+            <v>1129.3</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>51</v>
+            <v>53</v>
           </cell>
         </row>
         <row r="17">
@@ -1243,16 +1243,16 @@
             <v>320616.14999999967</v>
           </cell>
           <cell r="H17" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I17">
-            <v>259.8</v>
+            <v>1640.55</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>30</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="18">
@@ -1260,13 +1260,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>98434.389999999883</v>
+            <v>99875.889999999883</v>
           </cell>
           <cell r="H18" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I18">
-            <v>5909.01</v>
+            <v>3724.23</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1280,19 +1280,19 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>138560.34999999966</v>
+            <v>139781.64999999964</v>
           </cell>
           <cell r="H19" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I19">
-            <v>1310.0999999999999</v>
+            <v>7318.01</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>74</v>
+            <v>75</v>
           </cell>
         </row>
         <row r="20">
@@ -1303,10 +1303,10 @@
             <v>108789.73999999999</v>
           </cell>
           <cell r="H20" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
           </cell>
           <cell r="I20">
-            <v>553.16999999999996</v>
+            <v>2405.6000000000004</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1320,13 +1320,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>118241.47999999934</v>
+            <v>118791.0799999993</v>
           </cell>
           <cell r="H21" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I21">
-            <v>1159.99</v>
+            <v>553.16999999999996</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
@@ -1340,19 +1340,19 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>69424.940000000075</v>
+            <v>71379.640000000058</v>
           </cell>
           <cell r="H22" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I22">
-            <v>39126.330000000009</v>
+            <v>1159.99</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N22">
-            <v>30</v>
+            <v>31</v>
           </cell>
         </row>
         <row r="23">
@@ -1360,7 +1360,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>202648.6499999995</v>
+            <v>213496.69999999949</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I23">
+            <v>76409.510000000009</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
@@ -1374,13 +1380,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>292526.02499999985</v>
+            <v>298909.42500000005</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N24">
-            <v>26</v>
+            <v>27</v>
           </cell>
         </row>
         <row r="25">
@@ -1388,7 +1394,7 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>89968.829999999973</v>
+            <v>91098.129999999976</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
@@ -1408,7 +1414,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>652</v>
+            <v>663</v>
           </cell>
         </row>
         <row r="27">
@@ -1416,7 +1422,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>122636.4899999998</v>
+            <v>123602.2899999998</v>
           </cell>
         </row>
         <row r="28">
@@ -1424,7 +1430,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>149500.07</v>
+            <v>152964.5</v>
           </cell>
         </row>
         <row r="29">
@@ -1432,7 +1438,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>235464.56999999969</v>
+            <v>236873.56999999972</v>
           </cell>
         </row>
         <row r="30">
@@ -1440,7 +1446,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>70874.230000000098</v>
+            <v>71969.730000000112</v>
           </cell>
         </row>
         <row r="31">
@@ -1456,7 +1462,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F32">
-            <v>63965.399999999987</v>
+            <v>63965.4</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1467,7 +1473,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4900462.1649999404</v>
+            <v>4952651.3449999383</v>
           </cell>
         </row>
         <row r="34">
@@ -1483,7 +1489,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>37752.599999999962</v>
+            <v>37752.599999999977</v>
           </cell>
         </row>
         <row r="36">
@@ -2411,7 +2417,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4899325.8649999984</v>
+        <v>4951515.0449999971</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2422,7 +2428,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>39126.329999999994</v>
+        <v>76409.510000000009</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2444,7 +2450,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>652</v>
+        <v>663</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2456,7 +2462,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>282174.13500000164</v>
+        <v>229984.95500000287</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2467,7 +2473,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>160903.67000000001</v>
+        <v>123620.48999999999</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2489,7 +2495,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2501,7 +2507,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.94554199845604525</v>
+        <v>0.95561421306571404</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2512,7 +2518,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.19560230965355194</v>
+        <v>0.38199025146228072</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2534,7 +2540,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.81499999999999995</v>
+        <v>0.82874999999999999</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2633,11 +2639,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>51296.62000000001</v>
+        <v>51895.320000000007</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>13203.37999999999</v>
+        <v>12604.679999999993</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2652,11 +2658,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4060.4600000000005</v>
+        <v>10443.859999999999</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>16939.54</v>
+        <v>10556.140000000001</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2707,11 +2713,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>281742.71999999962</v>
+        <v>283599.41999999963</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>33257.280000000377</v>
+        <v>31400.580000000366</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2726,11 +2732,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>829.19999999999993</v>
+        <v>11677.25</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>13170.8</v>
+        <v>2322.75</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2803,11 +2809,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>674.75</v>
+        <v>1640.55</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>13545.25</v>
+        <v>12579.45</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2841,11 +2847,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2861,11 +2867,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>84353.489999999976</v>
+        <v>84891.289999999964</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>-4353.4899999999761</v>
+        <v>-4891.2899999999645</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2880,11 +2886,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5909.01</v>
+        <v>7318.01</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>13090.99</v>
+        <v>11681.99</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2918,11 +2924,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2938,11 +2944,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>208221.09999999969</v>
+        <v>212048.49999999965</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>6778.9000000003143</v>
+        <v>2951.5000000003492</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2957,11 +2963,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>953.93</v>
+        <v>1503.5300000000004</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>7296.07</v>
+        <v>6746.4699999999993</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3015,11 +3021,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>71652.98</v>
+        <v>71652.979999999967</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>-3652.9799999999959</v>
+        <v>-3652.9799999999668</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -3034,11 +3040,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6295.2099999999991</v>
+        <v>8151.909999999998</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>19034.79</v>
+        <v>17178.090000000004</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3072,11 +3078,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3092,11 +3098,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>264436.77999999997</v>
+        <v>279342.77999999997</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>-4436.7799999999697</v>
+        <v>-19342.77999999997</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3111,11 +3117,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>259.8</v>
+        <v>3724.23</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>9690.2000000000007</v>
+        <v>6225.77</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3149,11 +3155,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3169,11 +3175,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>160151.88999999996</v>
+        <v>160151.8899999999</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-35151.889999999956</v>
+        <v>-35151.889999999898</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3188,11 +3194,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1432.2200000000003</v>
+        <v>3386.9200000000005</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>1757.7799999999997</v>
+        <v>-196.92000000000053</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3207,11 +3213,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>37752.599999999962</v>
+        <v>37752.599999999977</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-37752.599999999962</v>
+        <v>-37752.599999999977</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3226,11 +3232,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3265,11 +3271,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3513.69</v>
+        <v>4955.1899999999996</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>2196.31</v>
+        <v>754.8100000000004</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3329,11 +3335,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2938.8000000000006</v>
+        <v>4160.1000000000004</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>11061.199999999999</v>
+        <v>9839.9</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3362,11 +3368,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3401,11 +3407,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5234</v>
+        <v>9061.4</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>9776</v>
+        <v>5948.6</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3418,11 +3424,11 @@
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>520661.21999999991</v>
+        <v>520661.21999999986</v>
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-520661.21999999991</v>
+        <v>-520661.21999999986</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3476,11 +3482,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>1129.3</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>9910</v>
+        <v>8780.7000000000007</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3532,11 +3538,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>98434.389999999883</v>
+        <v>99875.889999999883</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>21065.610000000117</v>
+        <v>19624.110000000117</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3607,11 +3613,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>138560.34999999966</v>
+        <v>139781.64999999964</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>18439.650000000343</v>
+        <v>17218.350000000355</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3643,11 +3649,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>489136.00000000012</v>
+        <v>504042.00000000017</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-489136.00000000012</v>
+        <v>-504042.00000000017</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3662,11 +3668,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3701,11 +3707,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>150</v>
+        <v>687.8</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>5310</v>
+        <v>4772.2</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3746,11 +3752,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>118241.47999999934</v>
+        <v>118791.0799999993</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>16758.520000000659</v>
+        <v>16208.920000000697</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3790,11 +3796,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3810,11 +3816,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>69424.940000000075</v>
+        <v>71379.640000000058</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>20575.059999999925</v>
+        <v>18620.359999999942</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3829,11 +3835,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1310.0999999999999</v>
+        <v>2405.6000000000004</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>5499.9</v>
+        <v>4404.3999999999996</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3854,11 +3860,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-12</v>
+        <v>-14</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3874,11 +3880,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>202648.6499999995</v>
+        <v>213496.69999999949</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>32351.350000000501</v>
+        <v>21503.300000000512</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3938,11 +3944,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>292526.02499999985</v>
+        <v>298909.42500000005</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>9473.9750000001513</v>
+        <v>3090.5749999999534</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3957,11 +3963,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1864.35</v>
+        <v>2463.0499999999997</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>2855.65</v>
+        <v>2256.9500000000003</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -3989,11 +3995,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>89968.829999999973</v>
+        <v>91098.129999999976</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>23031.170000000027</v>
+        <v>21901.870000000024</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4092,11 +4098,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>122636.4899999998</v>
+        <v>123602.2899999998</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>3363.5100000001985</v>
+        <v>2397.7100000001956</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4109,11 +4115,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>645369.17500000272</v>
+        <v>645369.17500000296</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>54630.824999997276</v>
+        <v>54630.824999997043</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4152,11 +4158,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>149500.07</v>
+        <v>152964.5</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>17499.929999999993</v>
+        <v>14035.5</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4169,11 +4175,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000039</v>
+        <v>668938.42000000051</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.579999999609</v>
+        <v>31061.579999999492</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4212,11 +4218,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>235464.56999999969</v>
+        <v>236873.56999999972</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>19535.430000000313</v>
+        <v>18126.430000000284</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4229,11 +4235,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>683867.69500000135</v>
+        <v>683867.69500000123</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>16132.304999998654</v>
+        <v>16132.304999998771</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4252,11 +4258,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>-12</v>
+        <v>-29</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4272,11 +4278,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>70874.230000000098</v>
+        <v>71969.730000000112</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>29125.769999999902</v>
+        <v>28030.269999999888</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4289,11 +4295,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>499613.26500000223</v>
+        <v>536896.44500000239</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>200386.73499999777</v>
+        <v>163103.55499999761</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4359,11 +4365,11 @@
       </c>
       <c r="D36" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A36,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63965.399999999987</v>
+        <v>63965.4</v>
       </c>
       <c r="E36" s="7">
         <f t="shared" si="0"/>
-        <v>2034.6000000000131</v>
+        <v>2034.5999999999985</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -4560,11 +4566,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>1017199.5050000011</v>
+        <v>1069388.6849999991</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>262800.49499999895</v>
+        <v>210611.31500000088</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 29/05/2026 07:45
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25683927-4277-437A-9307-C932A7104E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{556F587A-74FC-47E3-8672-0DA21B5BDEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1009,13 +1009,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>51895.320000000007</v>
+            <v>52503.62000000001</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>2463.0499999999997</v>
+            <v>3071.35</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>283599.41999999963</v>
+            <v>291417.46999999968</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>8151.909999999998</v>
+            <v>15969.959999999992</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1046,7 +1046,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>687.8</v>
+            <v>1578.95</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1066,7 +1066,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>9061.4</v>
+            <v>11870.599999999999</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1080,19 +1080,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>84891.289999999964</v>
+            <v>85782.439999999959</v>
           </cell>
           <cell r="H9" t="str">
-            <v>LESTE</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>4955.1899999999996</v>
+            <v>359.25</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>62</v>
+            <v>64</v>
           </cell>
         </row>
         <row r="10">
@@ -1100,19 +1100,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>212048.49999999965</v>
+            <v>214857.69999999969</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>4160.1000000000004</v>
+            <v>6677.4399999999978</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>40</v>
+            <v>41</v>
           </cell>
         </row>
         <row r="11">
@@ -1120,19 +1120,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>71652.979999999967</v>
+            <v>72012.23</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>1987.6500000000003</v>
+            <v>6530.2199999999993</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>43</v>
+            <v>44</v>
           </cell>
         </row>
         <row r="12">
@@ -1140,19 +1140,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>279342.77999999997</v>
+            <v>283103.17</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>1503.5300000000004</v>
+            <v>2437.7000000000003</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N12">
-            <v>20</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="13">
@@ -1160,19 +1160,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>160151.8899999999</v>
+            <v>218866.28999999998</v>
           </cell>
           <cell r="H13" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>3386.9200000000005</v>
+            <v>2068.130000000001</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>26</v>
+            <v>29</v>
           </cell>
         </row>
         <row r="14">
@@ -1183,10 +1183,10 @@
             <v>982675.7999999997</v>
           </cell>
           <cell r="H14" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>11677.25</v>
+            <v>4427.6200000000008</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1200,13 +1200,13 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>88567.600000000064</v>
+            <v>88567.600000000079</v>
           </cell>
           <cell r="H15" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>10443.859999999999</v>
+            <v>18165.399999999998</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1220,19 +1220,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>454485.34999999992</v>
+            <v>460645.54999999993</v>
           </cell>
           <cell r="H16" t="str">
-            <v>PERDIZES</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>1129.3</v>
+            <v>12530.8</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>53</v>
+            <v>55</v>
           </cell>
         </row>
         <row r="17">
@@ -1240,19 +1240,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>320616.14999999967</v>
+            <v>326587.44999999972</v>
           </cell>
           <cell r="H17" t="str">
-            <v>PIRITUBA</v>
+            <v>PERDIZES</v>
           </cell>
           <cell r="I17">
-            <v>1640.55</v>
+            <v>1645.2</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>32</v>
+            <v>33</v>
           </cell>
         </row>
         <row r="18">
@@ -1260,13 +1260,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>99875.889999999883</v>
+            <v>101598.13999999987</v>
           </cell>
           <cell r="H18" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I18">
-            <v>3724.23</v>
+            <v>2280.0500000000002</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1280,13 +1280,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>139781.64999999964</v>
+            <v>142151.76999999958</v>
           </cell>
           <cell r="H19" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I19">
-            <v>7318.01</v>
+            <v>3899.03</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1300,13 +1300,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>108789.73999999999</v>
+            <v>109239.79000000001</v>
           </cell>
           <cell r="H20" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I20">
-            <v>2405.6000000000004</v>
+            <v>11745.509999999997</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1320,13 +1320,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>118791.0799999993</v>
+            <v>119355.67999999928</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
           </cell>
           <cell r="I21">
-            <v>553.16999999999996</v>
+            <v>2845.3000000000006</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
@@ -1340,19 +1340,19 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>71379.640000000058</v>
+            <v>72614.340000000055</v>
           </cell>
           <cell r="H22" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I22">
-            <v>1159.99</v>
+            <v>1376.6700000000003</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N22">
-            <v>31</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="23">
@@ -1360,13 +1360,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>213496.69999999949</v>
+            <v>219984.84999999954</v>
           </cell>
           <cell r="H23" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I23">
-            <v>76409.510000000009</v>
+            <v>1159.99</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
@@ -1380,13 +1380,19 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>298909.42500000005</v>
+            <v>300996.36499999999</v>
+          </cell>
+          <cell r="H24" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I24">
+            <v>110639.17000000004</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N24">
-            <v>27</v>
+            <v>28</v>
           </cell>
         </row>
         <row r="25">
@@ -1394,7 +1400,7 @@
             <v>PERDIZES</v>
           </cell>
           <cell r="F25">
-            <v>91098.129999999976</v>
+            <v>91614.02999999997</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
@@ -1414,7 +1420,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>663</v>
+            <v>676</v>
           </cell>
         </row>
         <row r="27">
@@ -1422,7 +1428,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F27">
-            <v>123602.2899999998</v>
+            <v>124241.7899999998</v>
           </cell>
         </row>
         <row r="28">
@@ -1430,7 +1436,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F28">
-            <v>152964.5</v>
+            <v>153139.29999999999</v>
           </cell>
         </row>
         <row r="29">
@@ -1438,7 +1444,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F29">
-            <v>236873.56999999972</v>
+            <v>241301.06999999972</v>
           </cell>
         </row>
         <row r="30">
@@ -1446,7 +1452,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F30">
-            <v>71969.730000000112</v>
+            <v>72409.43000000008</v>
           </cell>
         </row>
         <row r="31">
@@ -1454,7 +1460,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F31">
-            <v>39486.480000000025</v>
+            <v>40309.980000000018</v>
           </cell>
         </row>
         <row r="32">
@@ -1473,7 +1479,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F33">
-            <v>4952651.3449999383</v>
+            <v>5061681.2949999329</v>
           </cell>
         </row>
         <row r="34">
@@ -1489,7 +1495,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>37752.599999999977</v>
+            <v>37752.599999999962</v>
           </cell>
         </row>
         <row r="36">
@@ -2417,7 +2423,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4951515.0449999971</v>
+        <v>5060544.9949999964</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2428,7 +2434,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>76409.510000000009</v>
+        <v>110639.16999999998</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2450,7 +2456,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>663</v>
+        <v>676</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2462,7 +2468,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>229984.95500000287</v>
+        <v>120955.00500000361</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2473,7 +2479,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>123620.48999999999</v>
+        <v>89390.830000000016</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2495,7 +2501,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2507,7 +2513,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.95561421306571404</v>
+        <v>0.97665637267200545</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2518,7 +2524,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.38199025146228072</v>
+        <v>0.55311288306753981</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2540,7 +2546,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.82874999999999999</v>
+        <v>0.84499999999999997</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2639,11 +2645,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>51895.320000000007</v>
+        <v>52503.62000000001</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>12604.679999999993</v>
+        <v>11996.37999999999</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2658,11 +2664,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>10443.859999999999</v>
+        <v>12530.8</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>10556.140000000001</v>
+        <v>8469.2000000000007</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2713,11 +2719,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>283599.41999999963</v>
+        <v>291417.46999999968</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>31400.580000000366</v>
+        <v>23582.530000000319</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2732,11 +2738,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11677.25</v>
+        <v>18165.399999999998</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>2322.75</v>
+        <v>-4165.3999999999978</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2770,11 +2776,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W27" si="3">U11-V11</f>
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2809,11 +2815,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1640.55</v>
+        <v>2280.0500000000002</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>12579.45</v>
+        <v>11939.95</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2847,11 +2853,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2867,11 +2873,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>84891.289999999964</v>
+        <v>85782.439999999959</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>-4891.2899999999645</v>
+        <v>-5782.4399999999587</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2886,11 +2892,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7318.01</v>
+        <v>11745.509999999997</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>11681.99</v>
+        <v>7254.4900000000034</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2924,11 +2930,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2944,11 +2950,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>212048.49999999965</v>
+        <v>214857.69999999969</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>2951.5000000003492</v>
+        <v>142.3000000003085</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2963,11 +2969,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1503.5300000000004</v>
+        <v>2068.130000000001</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>6746.4699999999993</v>
+        <v>6181.869999999999</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3001,11 +3007,11 @@
       </c>
       <c r="V14" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W14" s="4">
         <f>U14-V14</f>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3021,11 +3027,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>71652.979999999967</v>
+        <v>72012.23</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>-3652.9799999999668</v>
+        <v>-4012.2299999999959</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -3040,11 +3046,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8151.909999999998</v>
+        <v>15969.959999999992</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>17178.090000000004</v>
+        <v>9360.0400000000081</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3078,11 +3084,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3098,11 +3104,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>279342.77999999997</v>
+        <v>283103.17</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>-19342.77999999997</v>
+        <v>-23103.169999999984</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3117,11 +3123,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3724.23</v>
+        <v>3899.03</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>6225.77</v>
+        <v>6050.9699999999993</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3155,11 +3161,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3175,11 +3181,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>160151.8899999999</v>
+        <v>218866.28999999998</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-35151.889999999898</v>
+        <v>-93866.289999999979</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3194,11 +3200,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3386.9200000000005</v>
+        <v>4427.6200000000008</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>-196.92000000000053</v>
+        <v>-1237.6200000000008</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3213,11 +3219,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>37752.599999999977</v>
+        <v>37752.599999999962</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-37752.599999999977</v>
+        <v>-37752.599999999962</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3271,11 +3277,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4955.1899999999996</v>
+        <v>6677.4399999999978</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>754.8100000000004</v>
+        <v>-967.43999999999778</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3316,11 +3322,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>88567.600000000064</v>
+        <v>88567.600000000079</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>26432.399999999936</v>
+        <v>26432.399999999921</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3335,11 +3341,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4160.1000000000004</v>
+        <v>6530.2199999999993</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>9839.9</v>
+        <v>7469.7800000000007</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3388,11 +3394,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>454485.34999999992</v>
+        <v>460645.54999999993</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>45514.650000000081</v>
+        <v>39354.45000000007</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3407,11 +3413,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9061.4</v>
+        <v>11870.599999999999</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>5948.6</v>
+        <v>3139.4000000000015</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3424,11 +3430,11 @@
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>520661.21999999986</v>
+        <v>520661.2199999998</v>
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-520661.21999999986</v>
+        <v>-520661.2199999998</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3463,11 +3469,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>320616.14999999967</v>
+        <v>326587.44999999972</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>106883.85000000033</v>
+        <v>100912.55000000028</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3482,11 +3488,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1129.3</v>
+        <v>1645.2</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>8780.7000000000007</v>
+        <v>8264.7999999999993</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3538,11 +3544,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>99875.889999999883</v>
+        <v>101598.13999999987</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>19624.110000000117</v>
+        <v>17901.860000000132</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3557,11 +3563,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>359.25</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>2670</v>
+        <v>2310.75</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3613,11 +3619,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>139781.64999999964</v>
+        <v>142151.76999999958</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>17218.350000000355</v>
+        <v>14848.230000000418</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3632,11 +3638,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1987.6500000000003</v>
+        <v>2437.7000000000003</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>10912.35</v>
+        <v>10462.299999999999</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3649,11 +3655,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>504042.00000000017</v>
+        <v>578648.2899999998</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-504042.00000000017</v>
+        <v>-578648.2899999998</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3668,11 +3674,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3688,11 +3694,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>108789.73999999999</v>
+        <v>109239.79000000001</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>11210.260000000009</v>
+        <v>10760.209999999992</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3707,11 +3713,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>687.8</v>
+        <v>1578.95</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>4772.2</v>
+        <v>3881.05</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3752,11 +3758,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>118791.0799999993</v>
+        <v>119355.67999999928</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>16208.920000000697</v>
+        <v>15644.32000000072</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3796,11 +3802,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3816,11 +3822,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>71379.640000000058</v>
+        <v>72614.340000000055</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>18620.359999999942</v>
+        <v>17385.659999999945</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3835,11 +3841,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2405.6000000000004</v>
+        <v>2845.3000000000006</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>4404.3999999999996</v>
+        <v>3964.6999999999994</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3860,11 +3866,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-14</v>
+        <v>-16</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3880,11 +3886,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>213496.69999999949</v>
+        <v>219984.84999999954</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>21503.300000000512</v>
+        <v>15015.15000000046</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3899,11 +3905,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>553.16999999999996</v>
+        <v>1376.6700000000003</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>2536.83</v>
+        <v>1713.3299999999997</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3944,11 +3950,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>298909.42500000005</v>
+        <v>300996.36499999999</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>3090.5749999999534</v>
+        <v>1003.6350000000093</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3963,11 +3969,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2463.0499999999997</v>
+        <v>3071.35</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>2256.9500000000003</v>
+        <v>1648.65</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -3995,11 +4001,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>91098.129999999976</v>
+        <v>91614.02999999997</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>21901.870000000024</v>
+        <v>21385.97000000003</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4098,11 +4104,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>123602.2899999998</v>
+        <v>124241.7899999998</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>2397.7100000001956</v>
+        <v>1758.2100000001956</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4158,11 +4164,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>152964.5</v>
+        <v>153139.29999999999</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>14035.5</v>
+        <v>13860.700000000012</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4218,11 +4224,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>236873.56999999972</v>
+        <v>241301.06999999972</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>18126.430000000284</v>
+        <v>13698.930000000284</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4258,11 +4264,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>229</v>
+        <v>249</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>-29</v>
+        <v>-49</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4278,11 +4284,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>71969.730000000112</v>
+        <v>72409.43000000008</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>28030.269999999888</v>
+        <v>27590.56999999992</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4295,11 +4301,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>536896.44500000239</v>
+        <v>571320.10500000336</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>163103.55499999761</v>
+        <v>128679.89499999664</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4327,11 +4333,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>39486.480000000025</v>
+        <v>40309.980000000018</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>15513.519999999975</v>
+        <v>14690.019999999982</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4566,11 +4572,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>1069388.6849999991</v>
+        <v>1178418.6349999933</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>210611.31500000088</v>
+        <v>101581.36500000674</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 29/05/2026 17:15
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{556F587A-74FC-47E3-8672-0DA21B5BDEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A96CA9B-396F-4723-BCCF-0C65A9364D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-28T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-29T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -973,7 +973,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>28/05/2026</v>
+            <v>29/05/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1006,30 +1006,30 @@
         </row>
         <row r="5">
           <cell r="E5" t="str">
-            <v>CAMPINAS</v>
+            <v>(vazio)</v>
           </cell>
           <cell r="F5">
-            <v>52503.62000000001</v>
+            <v>164.7</v>
           </cell>
           <cell r="H5" t="str">
-            <v>CAMPINAS</v>
+            <v>(vazio)</v>
           </cell>
           <cell r="I5">
-            <v>3071.35</v>
+            <v>164.7</v>
           </cell>
         </row>
         <row r="6">
           <cell r="E6" t="str">
-            <v>CENTRO</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="F6">
-            <v>291417.46999999968</v>
+            <v>55240.320000000014</v>
           </cell>
           <cell r="H6" t="str">
-            <v>CENTRO</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="I6">
-            <v>15969.959999999992</v>
+            <v>2736.7000000000003</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1037,16 +1037,16 @@
         </row>
         <row r="7">
           <cell r="E7" t="str">
-            <v>ECOMMERCE</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>1090.08</v>
+            <v>308099.26999999955</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I7">
-            <v>1578.95</v>
+            <v>16681.8</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1057,56 +1057,56 @@
         </row>
         <row r="8">
           <cell r="E8" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>ECOMMERCE</v>
           </cell>
           <cell r="F8">
-            <v>1136.3</v>
+            <v>1090.08</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I8">
-            <v>11870.599999999999</v>
+            <v>1479.8100000000002</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="N8">
-            <v>19</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="9">
           <cell r="E9" t="str">
-            <v>INDAIATUBA</v>
+            <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F9">
-            <v>85782.439999999959</v>
+            <v>1136.3</v>
           </cell>
           <cell r="H9" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I9">
-            <v>359.25</v>
+            <v>3267.0500000000006</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>64</v>
+            <v>72</v>
           </cell>
         </row>
         <row r="10">
           <cell r="E10" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="F10">
-            <v>214857.69999999969</v>
+            <v>87262.249999999927</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I10">
-            <v>6677.4399999999978</v>
+            <v>3128.5</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1117,36 +1117,36 @@
         </row>
         <row r="11">
           <cell r="E11" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="F11">
-            <v>72012.23</v>
+            <v>219514.74999999965</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I11">
-            <v>6530.2199999999993</v>
+            <v>2315.1</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>44</v>
+            <v>52</v>
           </cell>
         </row>
         <row r="12">
           <cell r="E12" t="str">
-            <v>KEY ABC</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="F12">
-            <v>283103.17</v>
+            <v>75140.73</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I12">
-            <v>2437.7000000000003</v>
+            <v>7158.6699999999964</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1157,156 +1157,156 @@
         </row>
         <row r="13">
           <cell r="E13" t="str">
-            <v>KEY CASA</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="F13">
-            <v>218866.28999999998</v>
+            <v>314498.23</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I13">
-            <v>2068.130000000001</v>
+            <v>12748.4</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>29</v>
+            <v>34</v>
           </cell>
         </row>
         <row r="14">
           <cell r="E14" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="F14">
-            <v>982675.7999999997</v>
+            <v>218866.29000000007</v>
           </cell>
           <cell r="H14" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I14">
-            <v>4427.6200000000008</v>
+            <v>17754.000000000004</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>44</v>
+            <v>50</v>
           </cell>
         </row>
         <row r="15">
           <cell r="E15" t="str">
-            <v>KEY SJC</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="F15">
-            <v>88567.600000000079</v>
+            <v>1005438.5999999996</v>
           </cell>
           <cell r="H15" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I15">
-            <v>18165.399999999998</v>
+            <v>4064.7000000000012</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N15">
-            <v>19</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="16">
           <cell r="E16" t="str">
-            <v>KEY SP</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>460645.54999999993</v>
+            <v>119722.00000000012</v>
           </cell>
           <cell r="H16" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I16">
-            <v>12530.8</v>
+            <v>3974.4300000000012</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>55</v>
+            <v>60</v>
           </cell>
         </row>
         <row r="17">
           <cell r="E17" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>326587.44999999972</v>
+            <v>515980.64999999997</v>
           </cell>
           <cell r="H17" t="str">
-            <v>PERDIZES</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I17">
-            <v>1645.2</v>
+            <v>4612.8700000000008</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>33</v>
+            <v>44</v>
           </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
-            <v>LESTE</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>101598.13999999987</v>
+            <v>369533.82999999996</v>
           </cell>
           <cell r="H18" t="str">
-            <v>PIRITUBA</v>
+            <v>PERDIZES</v>
           </cell>
           <cell r="I18">
-            <v>2280.0500000000002</v>
+            <v>810.5</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>49</v>
+            <v>51</v>
           </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>142151.76999999958</v>
+            <v>103913.23999999987</v>
           </cell>
           <cell r="H19" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I19">
-            <v>3899.03</v>
+            <v>4450.9000000000015</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>75</v>
+            <v>79</v>
           </cell>
         </row>
         <row r="20">
           <cell r="E20" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>109239.79000000001</v>
+            <v>149310.43999999954</v>
           </cell>
           <cell r="H20" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I20">
-            <v>11745.509999999997</v>
+            <v>4737.6000000000004</v>
           </cell>
           <cell r="K20" t="str">
             <v>PERDIZES</v>
@@ -1317,36 +1317,36 @@
         </row>
         <row r="21">
           <cell r="E21" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>119355.67999999928</v>
+            <v>121988.18999999994</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I21">
-            <v>2845.3000000000006</v>
+            <v>7403.2799999999988</v>
           </cell>
           <cell r="K21" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N21">
-            <v>40</v>
+            <v>51</v>
           </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>72614.340000000055</v>
+            <v>137109.67999999927</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
           </cell>
           <cell r="I22">
-            <v>1376.6700000000003</v>
+            <v>760.62</v>
           </cell>
           <cell r="K22" t="str">
             <v>SANTO ANDRE</v>
@@ -1357,118 +1357,124 @@
         </row>
         <row r="23">
           <cell r="E23" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>219984.84999999954</v>
+            <v>76579.040000000052</v>
           </cell>
           <cell r="H23" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I23">
-            <v>1159.99</v>
+            <v>739.5</v>
           </cell>
           <cell r="K23" t="str">
             <v>SBC</v>
           </cell>
           <cell r="N23">
-            <v>42</v>
+            <v>43</v>
           </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>300996.36499999999</v>
+            <v>223959.27999999945</v>
           </cell>
           <cell r="H24" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I24">
-            <v>110639.17000000004</v>
+            <v>941.57999999999993</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N24">
-            <v>28</v>
+            <v>29</v>
           </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
-            <v>PERDIZES</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>91614.02999999997</v>
+            <v>305609.23500000063</v>
+          </cell>
+          <cell r="H25" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I25">
+            <v>99930.710000000094</v>
           </cell>
           <cell r="K25" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="N25">
-            <v>20</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
-            <v>PIRACICABA</v>
+            <v>PERDIZES</v>
           </cell>
           <cell r="F26">
-            <v>129513.65999999999</v>
+            <v>92424.52999999997</v>
           </cell>
           <cell r="K26" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N26">
-            <v>676</v>
+            <v>742</v>
           </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
-            <v>PIRITUBA</v>
+            <v>PIRACICABA</v>
           </cell>
           <cell r="F27">
-            <v>124241.7899999998</v>
+            <v>138033.66</v>
           </cell>
         </row>
         <row r="28">
           <cell r="E28" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="F28">
-            <v>153139.29999999999</v>
+            <v>128732.68999999971</v>
           </cell>
         </row>
         <row r="29">
           <cell r="E29" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="F29">
-            <v>241301.06999999972</v>
+            <v>157876.89999999997</v>
           </cell>
         </row>
         <row r="30">
           <cell r="E30" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="F30">
-            <v>72409.43000000008</v>
+            <v>248704.34999999971</v>
           </cell>
         </row>
         <row r="31">
           <cell r="E31" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
           </cell>
           <cell r="F31">
-            <v>40309.980000000018</v>
+            <v>73170.05000000009</v>
           </cell>
         </row>
         <row r="32">
           <cell r="E32" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="F32">
-            <v>63965.4</v>
+            <v>41049.48000000001</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1476,13 +1482,19 @@
         </row>
         <row r="33">
           <cell r="E33" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="F33">
+            <v>64809.780000000006</v>
+          </cell>
+        </row>
+        <row r="34">
+          <cell r="E34" t="str">
             <v>Total Geral</v>
           </cell>
-          <cell r="F33">
-            <v>5061681.2949999329</v>
-          </cell>
-        </row>
-        <row r="34">
+          <cell r="F34">
+            <v>5354958.5449999254</v>
+          </cell>
           <cell r="P34" t="str">
             <v>KEY ABC</v>
           </cell>
@@ -1495,7 +1507,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>37752.599999999962</v>
+            <v>37752.599999999991</v>
           </cell>
         </row>
         <row r="36">
@@ -2423,7 +2435,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>5060544.9949999964</v>
+        <v>5353657.5449999971</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2434,7 +2446,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J28)</f>
-        <v>110639.16999999998</v>
+        <v>99766.010000000009</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2456,7 +2468,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>676</v>
+        <v>742</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2468,7 +2480,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>120955.00500000361</v>
+        <v>-172157.54499999713</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2479,7 +2491,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>89390.830000000016</v>
+        <v>100263.98999999999</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2501,7 +2513,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>124</v>
+        <v>58</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2513,7 +2525,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.97665637267200545</v>
+        <v>1.0332254260349314</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2524,7 +2536,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.55311288306753981</v>
+        <v>0.4987552367144929</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2546,7 +2558,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.84499999999999997</v>
+        <v>0.92749999999999999</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2645,11 +2657,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>52503.62000000001</v>
+        <v>55240.320000000014</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>11996.37999999999</v>
+        <v>9259.6799999999857</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2664,11 +2676,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>12530.8</v>
+        <v>4612.8700000000008</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>8469.2000000000007</v>
+        <v>16387.129999999997</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2699,11 +2711,11 @@
       </c>
       <c r="V10" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W10" s="4">
         <f>U10-V10</f>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -2719,11 +2731,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>291417.46999999968</v>
+        <v>308099.26999999955</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>23582.530000000319</v>
+        <v>6900.730000000447</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2738,11 +2750,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>18165.399999999998</v>
+        <v>3974.4300000000012</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>-4165.3999999999978</v>
+        <v>10025.57</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2776,11 +2788,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W27" si="3">U11-V11</f>
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2815,11 +2827,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2280.0500000000002</v>
+        <v>4450.9000000000015</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>11939.95</v>
+        <v>9769.0999999999985</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2873,11 +2885,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>85782.439999999959</v>
+        <v>87262.249999999927</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>-5782.4399999999587</v>
+        <v>-7262.2499999999272</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2892,11 +2904,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11745.509999999997</v>
+        <v>7403.2799999999988</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>7254.4900000000034</v>
+        <v>11596.720000000001</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2930,11 +2942,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2950,11 +2962,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>214857.69999999969</v>
+        <v>219514.74999999965</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>142.3000000003085</v>
+        <v>-4514.7499999996508</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2969,11 +2981,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2068.130000000001</v>
+        <v>17754.000000000004</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>6181.869999999999</v>
+        <v>-9504.0000000000036</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3027,11 +3039,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>72012.23</v>
+        <v>75140.73</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>-4012.2299999999959</v>
+        <v>-7140.7299999999959</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -3046,11 +3058,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>15969.959999999992</v>
+        <v>16681.8</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>9360.0400000000081</v>
+        <v>8648.2000000000007</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3084,11 +3096,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3104,11 +3116,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>283103.17</v>
+        <v>314498.23</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>-23103.169999999984</v>
+        <v>-54498.229999999981</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3123,11 +3135,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3899.03</v>
+        <v>4737.6000000000004</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>6050.9699999999993</v>
+        <v>5212.3999999999996</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3161,11 +3173,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3181,11 +3193,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>218866.28999999998</v>
+        <v>218866.29000000007</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-93866.289999999979</v>
+        <v>-93866.290000000066</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3200,11 +3212,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4427.6200000000008</v>
+        <v>4064.7000000000012</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>-1237.6200000000008</v>
+        <v>-874.70000000000118</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3219,11 +3231,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>37752.599999999962</v>
+        <v>37752.599999999991</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-37752.599999999962</v>
+        <v>-37752.599999999991</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3238,11 +3250,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3258,11 +3270,11 @@
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>982675.7999999997</v>
+        <v>1005438.5999999996</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>-182675.7999999997</v>
+        <v>-205438.59999999963</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3277,11 +3289,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6677.4399999999978</v>
+        <v>2315.1</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>-967.43999999999778</v>
+        <v>3394.9</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3302,11 +3314,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3322,11 +3334,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>88567.600000000079</v>
+        <v>119722.00000000012</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>26432.399999999921</v>
+        <v>-4722.0000000001164</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3341,11 +3353,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6530.2199999999993</v>
+        <v>7158.6699999999964</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>7469.7800000000007</v>
+        <v>6841.3300000000036</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3374,11 +3386,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>-2</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3394,11 +3406,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>460645.54999999993</v>
+        <v>515980.64999999997</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>39354.45000000007</v>
+        <v>-15980.649999999965</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3413,11 +3425,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11870.599999999999</v>
+        <v>3267.0500000000006</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>3139.4000000000015</v>
+        <v>11742.949999999999</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3430,11 +3442,11 @@
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>520661.2199999998</v>
+        <v>520661.21999999974</v>
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-520661.2199999998</v>
+        <v>-520661.21999999974</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3449,11 +3461,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3469,11 +3481,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>326587.44999999972</v>
+        <v>369533.82999999996</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>100912.55000000028</v>
+        <v>57966.170000000042</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3488,11 +3500,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1645.2</v>
+        <v>810.5</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>8264.7999999999993</v>
+        <v>9099.5</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3544,11 +3556,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>101598.13999999987</v>
+        <v>103913.23999999987</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>17901.860000000132</v>
+        <v>15586.760000000126</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3563,11 +3575,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>359.25</v>
+        <v>3128.5</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>2310.75</v>
+        <v>-458.5</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3599,11 +3611,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3619,11 +3631,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>142151.76999999958</v>
+        <v>149310.43999999954</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>14848.230000000418</v>
+        <v>7689.5600000004633</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3638,11 +3650,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2437.7000000000003</v>
+        <v>12748.4</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>10462.299999999999</v>
+        <v>151.60000000000036</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3655,11 +3667,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>578648.2899999998</v>
+        <v>762242.0299999998</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-578648.2899999998</v>
+        <v>-762242.0299999998</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3694,11 +3706,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>109239.79000000001</v>
+        <v>121988.18999999994</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>10760.209999999992</v>
+        <v>-1988.1899999999441</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3713,11 +3725,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1578.95</v>
+        <v>1479.8100000000002</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>3881.05</v>
+        <v>3980.1899999999996</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3738,11 +3750,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3758,11 +3770,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>119355.67999999928</v>
+        <v>137109.67999999927</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>15644.32000000072</v>
+        <v>-2109.6799999992654</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3777,11 +3789,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1159.99</v>
+        <v>941.57999999999993</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>3650.01</v>
+        <v>3868.42</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3802,11 +3814,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3822,11 +3834,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>72614.340000000055</v>
+        <v>76579.040000000052</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>17385.659999999945</v>
+        <v>13420.959999999948</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3841,11 +3853,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2845.3000000000006</v>
+        <v>760.62</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>3964.6999999999994</v>
+        <v>6049.38</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3866,11 +3878,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-16</v>
+        <v>-21</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3886,11 +3898,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>219984.84999999954</v>
+        <v>223959.27999999945</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>15015.15000000046</v>
+        <v>11040.720000000554</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3905,11 +3917,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1376.6700000000003</v>
+        <v>739.5</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>1713.3299999999997</v>
+        <v>2350.5</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3930,11 +3942,11 @@
       </c>
       <c r="V27" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S27,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W27" s="4">
         <f t="shared" si="3"/>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
@@ -3950,11 +3962,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>300996.36499999999</v>
+        <v>305609.23500000063</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>1003.6350000000093</v>
+        <v>-3609.2350000006263</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
@@ -3969,11 +3981,11 @@
       </c>
       <c r="J28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3071.35</v>
+        <v>2736.7000000000003</v>
       </c>
       <c r="K28" s="7">
         <f t="shared" si="1"/>
-        <v>1648.65</v>
+        <v>1983.2999999999997</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -4001,11 +4013,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>91614.02999999997</v>
+        <v>92424.52999999997</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>21385.97000000003</v>
+        <v>20575.47000000003</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4047,11 +4059,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>129513.65999999999</v>
+        <v>138033.66</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>40486.340000000011</v>
+        <v>31966.339999999997</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4104,11 +4116,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>124241.7899999998</v>
+        <v>128732.68999999971</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>1758.2100000001956</v>
+        <v>-2732.6899999997113</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4121,11 +4133,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>645369.17500000296</v>
+        <v>645369.17500000284</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>54630.824999997043</v>
+        <v>54630.824999997159</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4164,11 +4176,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>153139.29999999999</v>
+        <v>157876.89999999997</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>13860.700000000012</v>
+        <v>9123.1000000000349</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4181,11 +4193,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000051</v>
+        <v>668938.42000000074</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.579999999492</v>
+        <v>31061.57999999926</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4224,11 +4236,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>241301.06999999972</v>
+        <v>248704.34999999971</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>13698.930000000284</v>
+        <v>6295.6500000002852</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4241,11 +4253,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>683867.69500000123</v>
+        <v>683867.69500000111</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>16132.304999998771</v>
+        <v>16132.304999998887</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4264,11 +4276,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>249</v>
+        <v>327</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>-49</v>
+        <v>-127</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4284,11 +4296,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>72409.43000000008</v>
+        <v>73170.05000000009</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>27590.56999999992</v>
+        <v>26829.94999999991</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4301,11 +4313,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>571320.10500000336</v>
+        <v>672318.91500000155</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>128679.89499999664</v>
+        <v>27681.084999998449</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4333,11 +4345,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>40309.980000000018</v>
+        <v>41049.48000000001</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>14690.019999999982</v>
+        <v>13950.51999999999</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4371,11 +4383,11 @@
       </c>
       <c r="D36" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A36,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>63965.4</v>
+        <v>64809.780000000006</v>
       </c>
       <c r="E36" s="7">
         <f t="shared" si="0"/>
-        <v>2034.5999999999985</v>
+        <v>1190.2199999999939</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -4464,11 +4476,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.5949999997</v>
+        <v>1184379.5950000002</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>95620.405000000261</v>
+        <v>95620.404999999795</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4536,11 +4548,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1173268.9449999928</v>
+        <v>1173268.9449999931</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>106731.05500000715</v>
+        <v>106731.05500000692</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4572,11 +4584,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>1178418.6349999933</v>
+        <v>1471695.8849999926</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="6"/>
-        <v>101581.36500000674</v>
+        <v>-191695.88499999256</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 25/06/2026 08:33
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A96CA9B-396F-4723-BCCF-0C65A9364D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEEAE799-3E71-4ACB-8552-AB9C9C65B370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-05-29T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-06-11T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="53">
   <si>
     <t>META DIA</t>
   </si>
@@ -138,9 +138,6 @@
   </si>
   <si>
     <t>OSASCO</t>
-  </si>
-  <si>
-    <t>PERDIZES</t>
   </si>
   <si>
     <t>PIRITUBA</t>
@@ -939,10 +936,11 @@
       <sheetName val="14H"/>
       <sheetName val="TOTAL"/>
       <sheetName val="VENDA DIA"/>
+      <sheetName val="CONVERSOR"/>
       <sheetName val="SENSUM"/>
-      <sheetName val="CONVERSOR"/>
+      <sheetName val="Planilha5"/>
+      <sheetName val="Planilha4"/>
       <sheetName val="BASE PYTHON"/>
-      <sheetName val="DIN MILHO"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0" refreshError="1"/>
@@ -950,7 +948,9 @@
       <sheetData sheetId="2" refreshError="1"/>
       <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5">
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7">
         <row r="1">
           <cell r="E1" t="str">
             <v>GERAL</v>
@@ -959,7 +959,7 @@
             <v>VAREJO</v>
           </cell>
           <cell r="K1" t="str">
-            <v>POSITIVACAO MILHO</v>
+            <v>POSITIVACAO BRIOCHE</v>
           </cell>
         </row>
         <row r="2">
@@ -973,7 +973,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>29/05/2026</v>
+            <v>11/06/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1009,13 +1009,13 @@
             <v>(vazio)</v>
           </cell>
           <cell r="F5">
-            <v>164.7</v>
+            <v>0</v>
           </cell>
           <cell r="H5" t="str">
-            <v>(vazio)</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>164.7</v>
+            <v>1818.01</v>
           </cell>
         </row>
         <row r="6">
@@ -1023,13 +1023,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F6">
-            <v>55240.320000000014</v>
+            <v>48598.409999999989</v>
           </cell>
           <cell r="H6" t="str">
-            <v>CAMPINAS</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>2736.7000000000003</v>
+            <v>12476.879999999996</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1040,19 +1040,16 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>308099.26999999955</v>
+            <v>281771.82999999961</v>
           </cell>
           <cell r="H7" t="str">
-            <v>CENTRO</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>16681.8</v>
+            <v>2976.94</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
-          </cell>
-          <cell r="N7" t="str">
-            <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
@@ -1060,446 +1057,351 @@
             <v>ECOMMERCE</v>
           </cell>
           <cell r="F8">
-            <v>1090.08</v>
+            <v>1237.53</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INDAIATUBA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>1479.8100000000002</v>
+            <v>17091.899999999994</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
-          <cell r="N8">
-            <v>20</v>
-          </cell>
         </row>
         <row r="9">
           <cell r="E9" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>1136.3</v>
+            <v>72959.349999999948</v>
           </cell>
           <cell r="H9" t="str">
-            <v>INTERLAGOS</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>3267.0500000000006</v>
+            <v>2180.9</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
-          <cell r="N9">
-            <v>72</v>
-          </cell>
         </row>
         <row r="10">
           <cell r="E10" t="str">
-            <v>INDAIATUBA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>87262.249999999927</v>
+            <v>210952.18999999962</v>
           </cell>
           <cell r="H10" t="str">
-            <v>JUNDIAI</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>3128.5</v>
+            <v>2559.6299999999997</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
-          <cell r="N10">
-            <v>41</v>
-          </cell>
         </row>
         <row r="11">
           <cell r="E11" t="str">
-            <v>INTERLAGOS</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>219514.74999999965</v>
+            <v>57163.810000000041</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I11">
-            <v>2315.1</v>
+            <v>4461.5000000000009</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
-          <cell r="N11">
-            <v>52</v>
-          </cell>
         </row>
         <row r="12">
           <cell r="E12" t="str">
-            <v>JUNDIAI</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>75140.73</v>
+            <v>237391.93</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I12">
-            <v>7158.6699999999964</v>
+            <v>1327.45</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
-          <cell r="N12">
-            <v>21</v>
-          </cell>
         </row>
         <row r="13">
           <cell r="E13" t="str">
-            <v>KEY ABC</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>314498.23</v>
+            <v>165508.78999999998</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE PENHA</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I13">
-            <v>12748.4</v>
+            <v>3852.0000000000005</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
-          <cell r="N13">
-            <v>34</v>
-          </cell>
         </row>
         <row r="14">
           <cell r="E14" t="str">
-            <v>KEY CASA</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>218866.29000000007</v>
+            <v>769210.07999999984</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I14">
-            <v>17754.000000000004</v>
+            <v>6939.45</v>
           </cell>
           <cell r="K14" t="str">
-            <v>LESTE MOOCA</v>
-          </cell>
-          <cell r="N14">
-            <v>50</v>
+            <v>LESTE PENHA</v>
           </cell>
         </row>
         <row r="15">
           <cell r="E15" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>1005438.5999999996</v>
+            <v>85412.150000000009</v>
           </cell>
           <cell r="H15" t="str">
-            <v>MOGI</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I15">
-            <v>4064.7000000000012</v>
+            <v>9250.9849999999988</v>
           </cell>
           <cell r="K15" t="str">
-            <v>LESTE PENHA</v>
-          </cell>
-          <cell r="N15">
-            <v>21</v>
+            <v>LESTE TATUAPE</v>
           </cell>
         </row>
         <row r="16">
           <cell r="E16" t="str">
-            <v>KEY SJC</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>119722.00000000012</v>
+            <v>508154.89000000036</v>
           </cell>
           <cell r="H16" t="str">
-            <v>NORTE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I16">
-            <v>3974.4300000000012</v>
+            <v>3926.98</v>
           </cell>
           <cell r="K16" t="str">
-            <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="N16">
-            <v>60</v>
+            <v>MOGI</v>
           </cell>
         </row>
         <row r="17">
           <cell r="E17" t="str">
-            <v>KEY SP</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>515980.64999999997</v>
+            <v>382790.12000000029</v>
           </cell>
           <cell r="H17" t="str">
-            <v>OSASCO</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I17">
-            <v>4612.8700000000008</v>
+            <v>4458.46</v>
           </cell>
           <cell r="K17" t="str">
-            <v>MOGI</v>
-          </cell>
-          <cell r="N17">
-            <v>44</v>
+            <v>NORTE</v>
           </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
-            <v>KEY ZL</v>
+            <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>369533.82999999996</v>
+            <v>106392.33999999989</v>
           </cell>
           <cell r="H18" t="str">
-            <v>PERDIZES</v>
+            <v>SBC</v>
           </cell>
           <cell r="I18">
-            <v>810.5</v>
+            <v>9471.1200000000008</v>
           </cell>
           <cell r="K18" t="str">
-            <v>NORTE</v>
-          </cell>
-          <cell r="N18">
-            <v>51</v>
+            <v>OSASCO</v>
           </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
-            <v>LESTE</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>103913.23999999987</v>
+            <v>169427.9999999998</v>
           </cell>
           <cell r="H19" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I19">
+            <v>2871.75</v>
+          </cell>
+          <cell r="K19" t="str">
             <v>PIRITUBA</v>
-          </cell>
-          <cell r="I19">
-            <v>4450.9000000000015</v>
-          </cell>
-          <cell r="K19" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="N19">
-            <v>79</v>
           </cell>
         </row>
         <row r="20">
           <cell r="E20" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>149310.43999999954</v>
+            <v>110771.99999999993</v>
           </cell>
           <cell r="H20" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I20">
+            <v>2480.1100000000006</v>
+          </cell>
+          <cell r="K20" t="str">
             <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I20">
-            <v>4737.6000000000004</v>
-          </cell>
-          <cell r="K20" t="str">
-            <v>PERDIZES</v>
-          </cell>
-          <cell r="N20">
-            <v>21</v>
           </cell>
         </row>
         <row r="21">
           <cell r="E21" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>121988.18999999994</v>
+            <v>105123.02999999966</v>
           </cell>
           <cell r="H21" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I21">
+            <v>2745.8</v>
+          </cell>
+          <cell r="K21" t="str">
             <v>SBC</v>
-          </cell>
-          <cell r="I21">
-            <v>7403.2799999999988</v>
-          </cell>
-          <cell r="K21" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="N21">
-            <v>51</v>
           </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>137109.67999999927</v>
+            <v>51925.380000000077</v>
           </cell>
           <cell r="H22" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I22">
+            <v>90889.865000000034</v>
+          </cell>
+          <cell r="K22" t="str">
             <v>SJC</v>
-          </cell>
-          <cell r="I22">
-            <v>760.62</v>
-          </cell>
-          <cell r="K22" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="N22">
-            <v>32</v>
           </cell>
         </row>
         <row r="23">
           <cell r="E23" t="str">
-            <v>MOGI</v>
+            <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>76579.040000000052</v>
-          </cell>
-          <cell r="H23" t="str">
+            <v>194895.83999999933</v>
+          </cell>
+          <cell r="K23" t="str">
             <v>SJC/VALE</v>
-          </cell>
-          <cell r="I23">
-            <v>739.5</v>
-          </cell>
-          <cell r="K23" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="N23">
-            <v>43</v>
           </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
-            <v>NORTE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>223959.27999999945</v>
-          </cell>
-          <cell r="H24" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I24">
-            <v>941.57999999999993</v>
+            <v>276074.34999999992</v>
           </cell>
           <cell r="K24" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="N24">
-            <v>29</v>
+            <v>Total Geral</v>
           </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
-            <v>OSASCO</v>
+            <v>PIRACICABA</v>
           </cell>
           <cell r="F25">
-            <v>305609.23500000063</v>
-          </cell>
-          <cell r="H25" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I25">
-            <v>99930.710000000094</v>
-          </cell>
-          <cell r="K25" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="N25">
-            <v>21</v>
+            <v>155370.25999999998</v>
           </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
-            <v>PERDIZES</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>92424.52999999997</v>
-          </cell>
-          <cell r="K26" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="N26">
-            <v>742</v>
+            <v>114539.58999999982</v>
           </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
-            <v>PIRACICABA</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>138033.66</v>
+            <v>137860.06999999989</v>
           </cell>
         </row>
         <row r="28">
           <cell r="E28" t="str">
-            <v>PIRITUBA</v>
+            <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>128732.68999999971</v>
+            <v>238192.00999999966</v>
           </cell>
         </row>
         <row r="29">
           <cell r="E29" t="str">
-            <v>SANTO ANDRE</v>
+            <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>157876.89999999997</v>
+            <v>67721.850000000064</v>
           </cell>
         </row>
         <row r="30">
           <cell r="E30" t="str">
-            <v>SBC</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>248704.34999999971</v>
+            <v>42026.570000000058</v>
           </cell>
         </row>
         <row r="31">
           <cell r="E31" t="str">
-            <v>SJC</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>73170.05000000009</v>
+            <v>64480.80999999999</v>
           </cell>
         </row>
         <row r="32">
           <cell r="E32" t="str">
-            <v>SJC/VALE</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>41049.48000000001</v>
+            <v>4655953.1799999475</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
           </cell>
         </row>
-        <row r="33">
-          <cell r="E33" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="F33">
-            <v>64809.780000000006</v>
-          </cell>
-        </row>
         <row r="34">
-          <cell r="E34" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="F34">
-            <v>5354958.5449999254</v>
-          </cell>
           <cell r="P34" t="str">
             <v>KEY ABC</v>
           </cell>
           <cell r="R34">
-            <v>137264.37</v>
+            <v>72929.350000000006</v>
           </cell>
         </row>
         <row r="35">
@@ -1507,7 +1409,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>37752.599999999991</v>
+            <v>49116.749999999964</v>
           </cell>
         </row>
         <row r="36">
@@ -1515,7 +1417,7 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="R36">
-            <v>363074.89999999997</v>
+            <v>216157.5</v>
           </cell>
         </row>
         <row r="37">
@@ -1523,7 +1425,7 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="R37">
-            <v>33627.799999999988</v>
+            <v>25347.399999999994</v>
           </cell>
         </row>
         <row r="38">
@@ -1531,7 +1433,7 @@
             <v>KEY SP</v>
           </cell>
           <cell r="R38">
-            <v>123308.7</v>
+            <v>113281.61999999997</v>
           </cell>
         </row>
         <row r="39">
@@ -1539,7 +1441,7 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="R39">
-            <v>89210.209999999963</v>
+            <v>154624.23999999996</v>
           </cell>
         </row>
         <row r="47">
@@ -1552,7 +1454,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="B63">
-            <v>73</v>
+            <v>57</v>
           </cell>
         </row>
         <row r="64">
@@ -1560,7 +1462,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="B64">
-            <v>49</v>
+            <v>41</v>
           </cell>
         </row>
         <row r="65">
@@ -1568,7 +1470,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="B65">
-            <v>47</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="66">
@@ -1576,7 +1478,7 @@
             <v>SBC</v>
           </cell>
           <cell r="B66">
-            <v>53</v>
+            <v>55</v>
           </cell>
         </row>
         <row r="67">
@@ -1584,7 +1486,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="B67">
-            <v>39</v>
+            <v>47</v>
           </cell>
         </row>
         <row r="68">
@@ -1592,7 +1494,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="B68">
-            <v>72</v>
+            <v>52</v>
           </cell>
         </row>
         <row r="69">
@@ -1600,7 +1502,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="B69">
-            <v>46</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="70">
@@ -1608,7 +1510,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="B70">
-            <v>44</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="71">
@@ -1616,7 +1518,7 @@
             <v>LESTE</v>
           </cell>
           <cell r="B71">
-            <v>39</v>
+            <v>44</v>
           </cell>
         </row>
         <row r="72">
@@ -1624,7 +1526,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="B72">
-            <v>47</v>
+            <v>45</v>
           </cell>
         </row>
         <row r="73">
@@ -1632,63 +1534,55 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="B73">
-            <v>58</v>
+            <v>55</v>
           </cell>
         </row>
         <row r="74">
           <cell r="A74" t="str">
-            <v>PERDIZES</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="B74">
-            <v>32</v>
+            <v>23</v>
           </cell>
         </row>
         <row r="75">
           <cell r="A75" t="str">
-            <v>JUNDIAI</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="B75">
-            <v>29</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="76">
           <cell r="A76" t="str">
-            <v>LESTE PENHA</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="B76">
-            <v>39</v>
+            <v>37</v>
           </cell>
         </row>
         <row r="77">
           <cell r="A77" t="str">
-            <v>INDAIATUBA</v>
+            <v>SJC</v>
           </cell>
           <cell r="B77">
-            <v>40</v>
+            <v>33</v>
           </cell>
         </row>
         <row r="78">
           <cell r="A78" t="str">
-            <v>SJC</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="B78">
-            <v>27</v>
+            <v>31</v>
           </cell>
         </row>
         <row r="79">
           <cell r="A79" t="str">
-            <v>SJC/VALE</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="B79">
-            <v>33</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="A80" t="str">
-            <v>CAMPINAS</v>
-          </cell>
-          <cell r="B80">
-            <v>33</v>
+            <v>36</v>
           </cell>
         </row>
         <row r="85">
@@ -1704,33 +1598,7 @@
             <v>SEMANA 5</v>
           </cell>
         </row>
-        <row r="88">
-          <cell r="E88">
-            <v>54000</v>
-          </cell>
-        </row>
-        <row r="89">
-          <cell r="E89">
-            <v>233000</v>
-          </cell>
-        </row>
-        <row r="90">
-          <cell r="E90">
-            <v>233000</v>
-          </cell>
-        </row>
-        <row r="91">
-          <cell r="E91">
-            <v>146500</v>
-          </cell>
-        </row>
-        <row r="92">
-          <cell r="E92">
-            <v>51000</v>
-          </cell>
-        </row>
       </sheetData>
-      <sheetData sheetId="6" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1757,16 +1625,16 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{8D294CDB-54E7-40E9-918D-B86BC1FA5B4D}" name="Tabela11" displayName="Tabela11" ref="S9:W27" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="S9:W27" xr:uid="{8D294CDB-54E7-40E9-918D-B86BC1FA5B4D}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{8D294CDB-54E7-40E9-918D-B86BC1FA5B4D}" name="Tabela11" displayName="Tabela11" ref="S9:W26" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="S9:W26" xr:uid="{8D294CDB-54E7-40E9-918D-B86BC1FA5B4D}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
     <filterColumn colId="3" hiddenButton="1"/>
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="S10:W27">
-    <sortCondition ref="T10:T27"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="S10:W26">
+    <sortCondition ref="T10:T26"/>
   </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{6C671431-FBD2-41CB-81F2-E1D2D5C3888E}" name="REFERENCA" dataDxfId="10"/>
@@ -1786,8 +1654,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}" name="Tabela12" displayName="Tabela12" ref="T29:W33" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="T29:W33" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}" name="Tabela12" displayName="Tabela12" ref="T28:W32" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="T28:W32" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1796,13 +1664,13 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{65A441BB-28F2-4C4D-8CD8-F9F9788A0656}" name="SEMANAL" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{B849FCBC-ED0F-47D9-B4E7-149FFE3500D9}" name="META" dataDxfId="2" dataCellStyle="Moeda">
-      <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(T30,[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]]),0)</calculatedColumnFormula>
+      <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(T29,[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]]),0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{A81AB4FC-EF49-4A93-8229-1B0CBFC88744}" name="REALIZADO" dataDxfId="1">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[PARAMETRO]","[Intervalo 2].[PARAMETRO].&amp;[DIA]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{13865A0A-FFF3-4F90-A201-753948DC8E26}" name="FALTA" dataDxfId="0">
-      <calculatedColumnFormula>U30-V30</calculatedColumnFormula>
+      <calculatedColumnFormula>U29-V29</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1810,8 +1678,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AF588D8F-0EAF-4694-8155-49E9449C8646}" name="Tabela2" displayName="Tabela2" ref="A9:E36" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
-  <autoFilter ref="A9:E36" xr:uid="{AF588D8F-0EAF-4694-8155-49E9449C8646}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AF588D8F-0EAF-4694-8155-49E9449C8646}" name="Tabela2" displayName="Tabela2" ref="A9:E35" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
+  <autoFilter ref="A9:E35" xr:uid="{AF588D8F-0EAF-4694-8155-49E9449C8646}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1836,8 +1704,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}" name="Tabela3" displayName="Tabela3" ref="B38:E42" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
-  <autoFilter ref="B38:E42" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}" name="Tabela3" displayName="Tabela3" ref="B37:E41" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
+  <autoFilter ref="B37:E41" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1846,13 +1714,13 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{D5CFA35F-1C13-42CF-B05C-430BF14AC2B0}" name="SEMANAL" dataDxfId="56"/>
     <tableColumn id="2" xr3:uid="{06063E15-5C9E-4303-B5F6-B9D0B178DB82}" name="META" dataDxfId="55" dataCellStyle="Moeda">
-      <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(B39,[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]]),0)</calculatedColumnFormula>
+      <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(B38,[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]]),0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{425F53BB-8CBB-40E8-9773-1C7C39906AD7}" name="REALIZADO" dataDxfId="54" dataCellStyle="Moeda">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{A18F5082-185F-44C4-B163-8A3CBDDA6732}" name="FALTA" dataDxfId="53">
-      <calculatedColumnFormula>C39-D39</calculatedColumnFormula>
+      <calculatedColumnFormula>C38-D38</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1870,8 +1738,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4F0EC2C2-A52E-4D47-97B3-678B19401BEF}" name="Tabela5" displayName="Tabela5" ref="G9:K28" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
-  <autoFilter ref="G9:K28" xr:uid="{4F0EC2C2-A52E-4D47-97B3-678B19401BEF}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4F0EC2C2-A52E-4D47-97B3-678B19401BEF}" name="Tabela5" displayName="Tabela5" ref="G9:K27" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
+  <autoFilter ref="G9:K27" xr:uid="{4F0EC2C2-A52E-4D47-97B3-678B19401BEF}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1896,8 +1764,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}" name="Tabela6" displayName="Tabela6" ref="H30:K34" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
-  <autoFilter ref="H30:K34" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}" name="Tabela6" displayName="Tabela6" ref="H29:K33" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+  <autoFilter ref="H29:K33" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1906,13 +1774,13 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{14E3BD3B-54B0-47BF-931C-064E12741C86}" name="SEMANAL" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{67CE9FE2-AA11-4BD4-9F34-EDC9123EA89F}" name="META" dataDxfId="37" dataCellStyle="Moeda">
-      <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(H31,[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]]),0)</calculatedColumnFormula>
+      <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(H30,[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]]),0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{14D3AA11-9DFC-420F-8F5A-5002E14D4AAA}" name="REALIZADO" dataDxfId="36">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{16DC2DF3-76D8-4A80-B29C-E276BB17D8FF}" name="FALTA" dataDxfId="35">
-      <calculatedColumnFormula>I31-J31</calculatedColumnFormula>
+      <calculatedColumnFormula>I30-J30</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2304,7 +2172,7 @@
     <row r="1" spans="1:23" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4"/>
       <c r="B1" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
@@ -2312,7 +2180,7 @@
       <c r="F1" s="14"/>
       <c r="G1" s="14"/>
       <c r="H1" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I1" s="14"/>
       <c r="J1" s="14"/>
@@ -2320,7 +2188,7 @@
       <c r="L1" s="14"/>
       <c r="M1" s="14"/>
       <c r="N1" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O1" s="14"/>
       <c r="P1" s="14"/>
@@ -2328,7 +2196,7 @@
       <c r="R1" s="14"/>
       <c r="S1" s="14"/>
       <c r="T1" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="U1" s="14"/>
       <c r="V1" s="4"/>
@@ -2386,11 +2254,11 @@
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C4" s="2">
-        <f>SUM(C10:C36)</f>
-        <v>5181500</v>
+        <f>SUM(C10:C35)</f>
+        <v>5507000</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="4"/>
@@ -2400,30 +2268,30 @@
         <v>0</v>
       </c>
       <c r="I4" s="7">
-        <f>SUM(I10:I28)</f>
-        <v>200030</v>
+        <f>SUM(I10:I27)</f>
+        <v>135000</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O4" s="7">
         <f>SUM(O11:O17)</f>
-        <v>717500</v>
+        <v>0</v>
       </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="U4" s="4">
-        <f>SUM(U10:U27)</f>
-        <v>800</v>
+        <f>SUM(U10:U26)</f>
+        <v>706</v>
       </c>
       <c r="V4" s="4"/>
       <c r="W4" s="4"/>
@@ -2434,8 +2302,8 @@
         <v>1</v>
       </c>
       <c r="C5" s="2">
-        <f>SUM(D10:D36)</f>
-        <v>5353657.5449999971</v>
+        <f>SUM(D10:D35)</f>
+        <v>4655953.1799999969</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2445,8 +2313,8 @@
         <v>1</v>
       </c>
       <c r="I5" s="7">
-        <f>SUM(J10:J28)</f>
-        <v>99766.010000000009</v>
+        <f>SUM(J10:J27)</f>
+        <v>90889.864999999976</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2457,7 +2325,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>784238.58</v>
+        <v>631456.86</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -2468,7 +2336,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>742</v>
+        <v>0</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2480,7 +2348,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>-172157.54499999713</v>
+        <v>851046.82000000309</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2491,7 +2359,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>100263.98999999999</v>
+        <v>44110.135000000024</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2502,7 +2370,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-66738.579999999958</v>
+        <v>-631456.86</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -2513,7 +2381,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>58</v>
+        <v>706</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2525,7 +2393,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>1.0332254260349314</v>
+        <v>0.84546090067187163</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2536,7 +2404,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.4987552367144929</v>
+        <v>0.67325825925925908</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2545,9 +2413,9 @@
       <c r="N7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="O7" s="3">
+      <c r="O7" s="3" t="e">
         <f>O5/O4</f>
-        <v>1.0930154425087106</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
@@ -2558,7 +2426,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.92749999999999999</v>
+        <v>0</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2589,13 +2457,13 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>1</v>
@@ -2605,7 +2473,7 @@
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>5</v>
@@ -2623,19 +2491,19 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="T9" s="4" t="s">
         <v>5</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="V9" s="4" t="s">
         <v>1</v>
@@ -2657,11 +2525,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>55240.320000000014</v>
+        <v>48598.409999999989</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>9259.6799999999857</v>
+        <v>15901.590000000011</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2672,19 +2540,19 @@
       </c>
       <c r="I10" s="2">
         <f>_xlfn.XLOOKUP(G10,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>21000</v>
+        <v>12430</v>
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4612.8700000000008</v>
+        <v>9250.9849999999988</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>16387.129999999997</v>
+        <v>3179.0150000000012</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N10" s="4" t="s">
         <v>5</v>
@@ -2707,15 +2575,15 @@
       </c>
       <c r="U10" s="4">
         <f>_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="V10" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="W10" s="4">
         <f>U10-V10</f>
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -2727,15 +2595,15 @@
       </c>
       <c r="C11" s="2">
         <f>_xlfn.XLOOKUP(A11,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>315000</v>
+        <v>320000</v>
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>308099.26999999955</v>
+        <v>281771.82999999961</v>
       </c>
       <c r="E11" s="7">
-        <f t="shared" ref="E11:E36" si="0">C11-D11</f>
-        <v>6900.730000000447</v>
+        <f t="shared" ref="E11:E35" si="0">C11-D11</f>
+        <v>38228.170000000391</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2746,22 +2614,22 @@
       </c>
       <c r="I11" s="2">
         <f>_xlfn.XLOOKUP(G11,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14000</v>
+        <v>17550</v>
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3974.4300000000012</v>
+        <v>6939.45</v>
       </c>
       <c r="K11" s="7">
-        <f t="shared" ref="K11:K28" si="1">I11-J11</f>
-        <v>10025.57</v>
+        <f t="shared" ref="K11:K27" si="1">I11-J11</f>
+        <v>10610.55</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O11" s="2" cm="1">
         <f t="array" ref="O11">IFERROR(_xlfn.XLOOKUP(M11,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
@@ -2769,11 +2637,11 @@
       </c>
       <c r="P11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>137264.37</v>
+        <v>72929.350000000006</v>
       </c>
       <c r="Q11" s="2">
         <f t="shared" ref="Q11:Q17" si="2">O11-P11</f>
-        <v>-137264.37</v>
+        <v>-72929.350000000006</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="4" t="s">
@@ -2784,23 +2652,23 @@
       </c>
       <c r="U11" s="4">
         <f>_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="W11" s="4">
-        <f t="shared" ref="W11:W27" si="3">U11-V11</f>
-        <v>0</v>
+        <f t="shared" ref="W11:W26" si="3">U11-V11</f>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="2">
         <f>_xlfn.XLOOKUP(A12,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
@@ -2808,41 +2676,41 @@
       </c>
       <c r="D12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A12,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>1090.08</v>
+        <v>1237.53</v>
       </c>
       <c r="E12" s="7">
         <f t="shared" si="0"/>
-        <v>-90.079999999999927</v>
+        <v>-237.52999999999997</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I12" s="2">
         <f>_xlfn.XLOOKUP(G12,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14220</v>
+        <v>4930</v>
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4450.9000000000015</v>
+        <v>3926.98</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>9769.0999999999985</v>
+        <v>1003.02</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O12" s="2" cm="1">
         <f t="array" ref="O12">IFERROR(_xlfn.XLOOKUP(M12,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>54000</v>
+        <v>0</v>
       </c>
       <c r="P12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
@@ -2850,7 +2718,7 @@
       </c>
       <c r="Q12" s="2">
         <f t="shared" si="2"/>
-        <v>54000</v>
+        <v>0</v>
       </c>
       <c r="R12" s="2"/>
       <c r="S12" s="4" t="s">
@@ -2861,15 +2729,15 @@
       </c>
       <c r="U12" s="4">
         <f>_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>-1</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2881,53 +2749,53 @@
       </c>
       <c r="C13" s="2">
         <f>_xlfn.XLOOKUP(A13,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>80000</v>
+        <v>89000</v>
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>87262.249999999927</v>
+        <v>72959.349999999948</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>-7262.2499999999272</v>
+        <v>16040.650000000052</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I13" s="2">
         <f>_xlfn.XLOOKUP(G13,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>19000</v>
+        <v>11780</v>
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7403.2799999999988</v>
+        <v>9471.1200000000008</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>11596.720000000001</v>
+        <v>2308.8799999999992</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O13" s="2" cm="1">
         <f t="array" ref="O13">IFERROR(_xlfn.XLOOKUP(M13,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>233000</v>
+        <v>0</v>
       </c>
       <c r="P13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>89210.209999999963</v>
+        <v>154624.23999999996</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" si="2"/>
-        <v>143789.79000000004</v>
+        <v>-154624.23999999996</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="4" t="s">
@@ -2938,15 +2806,15 @@
       </c>
       <c r="U13" s="4">
         <f>_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2958,53 +2826,53 @@
       </c>
       <c r="C14" s="2">
         <f>_xlfn.XLOOKUP(A14,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>215000</v>
+        <v>270000</v>
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>219514.74999999965</v>
+        <v>210952.18999999962</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>-4514.7499999996508</v>
+        <v>59047.810000000376</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I14" s="2">
         <f>_xlfn.XLOOKUP(G14,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>8250</v>
+        <v>6540</v>
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>17754.000000000004</v>
+        <v>1327.45</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>-9504.0000000000036</v>
+        <v>5212.55</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O14" s="2" cm="1">
         <f t="array" ref="O14">IFERROR(_xlfn.XLOOKUP(M14,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>233000</v>
+        <v>0</v>
       </c>
       <c r="P14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>363074.89999999997</v>
+        <v>216157.5</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" si="2"/>
-        <v>-130074.89999999997</v>
+        <v>-216157.5</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="4" t="s">
@@ -3015,15 +2883,15 @@
       </c>
       <c r="U14" s="4">
         <f>_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="V14" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="W14" s="4">
         <f>U14-V14</f>
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3035,15 +2903,15 @@
       </c>
       <c r="C15" s="2">
         <f>_xlfn.XLOOKUP(A15,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>68000</v>
+        <v>77000</v>
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>75140.73</v>
+        <v>57163.810000000041</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>-7140.7299999999959</v>
+        <v>19836.189999999959</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -3054,34 +2922,34 @@
       </c>
       <c r="I15" s="2">
         <f>_xlfn.XLOOKUP(G15,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>25330</v>
+        <v>18190</v>
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>16681.8</v>
+        <v>12476.879999999996</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>8648.2000000000007</v>
+        <v>5713.1200000000044</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O15" s="2" cm="1">
         <f t="array" ref="O15">IFERROR(_xlfn.XLOOKUP(M15,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>146500</v>
+        <v>0</v>
       </c>
       <c r="P15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>123308.7</v>
+        <v>113281.61999999997</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="2"/>
-        <v>23191.300000000003</v>
+        <v>-113281.61999999997</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="4" t="s">
@@ -3092,73 +2960,73 @@
       </c>
       <c r="U15" s="4">
         <f>_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="2">
         <f>_xlfn.XLOOKUP(A16,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>260000</v>
+        <v>325000</v>
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>314498.23</v>
+        <v>237391.93</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>-54498.229999999981</v>
+        <v>87608.07</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I16" s="2">
         <f>_xlfn.XLOOKUP(G16,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>9950</v>
+        <v>6200</v>
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4737.6000000000004</v>
+        <v>4458.46</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>5212.3999999999996</v>
+        <v>1741.54</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O16" s="2" cm="1">
         <f t="array" ref="O16">IFERROR(_xlfn.XLOOKUP(M16,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>51000</v>
+        <v>0</v>
       </c>
       <c r="P16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>33627.799999999988</v>
+        <v>25347.399999999994</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="2"/>
-        <v>17372.200000000012</v>
+        <v>-25347.399999999994</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="4" t="s">
@@ -3169,35 +3037,35 @@
       </c>
       <c r="U16" s="4">
         <f>_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C17" s="2">
         <f>_xlfn.XLOOKUP(A17,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>125000</v>
+        <v>160000</v>
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>218866.29000000007</v>
+        <v>165508.78999999998</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-93866.290000000066</v>
+        <v>-5508.789999999979</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3208,22 +3076,22 @@
       </c>
       <c r="I17" s="2">
         <f>_xlfn.XLOOKUP(G17,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3190</v>
+        <v>5000</v>
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4064.7000000000012</v>
+        <v>3852.0000000000005</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>-874.70000000000118</v>
+        <v>1147.9999999999995</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O17" s="2" cm="1">
         <f t="array" ref="O17">IFERROR(_xlfn.XLOOKUP(M17,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
@@ -3231,50 +3099,50 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>37752.599999999991</v>
+        <v>49116.749999999964</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-37752.599999999991</v>
+        <v>-49116.749999999964</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
         <v>13</v>
       </c>
       <c r="T17" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="U17" s="4">
         <f>_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>-3</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C18" s="2">
         <f>_xlfn.XLOOKUP(A18,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>800000</v>
+        <v>950000</v>
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>1005438.5999999996</v>
+        <v>769210.07999999984</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>-205438.59999999963</v>
+        <v>180789.92000000016</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3285,15 +3153,15 @@
       </c>
       <c r="I18" s="2">
         <f>_xlfn.XLOOKUP(G18,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5710</v>
+        <v>5690</v>
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2315.1</v>
+        <v>2559.6299999999997</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>3394.9</v>
+        <v>3130.3700000000003</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3310,62 +3178,62 @@
       </c>
       <c r="U18" s="4">
         <f>_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>-2</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" s="2">
         <f>_xlfn.XLOOKUP(A19,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>115000</v>
+        <v>125000</v>
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>119722.00000000012</v>
+        <v>85412.150000000009</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>-4722.0000000001164</v>
+        <v>39587.849999999991</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
         <v>13</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I19" s="2">
         <f>_xlfn.XLOOKUP(G19,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14000</v>
+        <v>10190</v>
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7158.6699999999964</v>
+        <v>0</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>6841.3300000000036</v>
+        <v>10190</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
       <c r="N19" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="P19" s="4" t="s">
         <v>3</v>
@@ -3382,35 +3250,35 @@
       </c>
       <c r="U19" s="4">
         <f>_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>-6</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" s="2">
         <f>_xlfn.XLOOKUP(A20,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>500000</v>
+        <v>540000</v>
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>515980.64999999997</v>
+        <v>508154.89000000036</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>-15980.649999999965</v>
+        <v>31845.109999999637</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3421,15 +3289,15 @@
       </c>
       <c r="I20" s="2">
         <f>_xlfn.XLOOKUP(G20,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15010</v>
+        <v>14980</v>
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3267.0500000000006</v>
+        <v>17091.899999999994</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>11742.949999999999</v>
+        <v>-2111.8999999999942</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3442,74 +3310,74 @@
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>520661.21999999974</v>
+        <v>631456.86000000034</v>
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-520661.21999999974</v>
+        <v>-631456.86000000034</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
         <v>14</v>
       </c>
       <c r="T20" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U20" s="4">
         <f>_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C21" s="2">
         <f>_xlfn.XLOOKUP(A21,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>427500</v>
+        <v>410000</v>
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>369533.82999999996</v>
+        <v>382790.12000000029</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>57966.170000000042</v>
+        <v>27209.879999999714</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I21" s="2">
         <f>_xlfn.XLOOKUP(G21,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>9910</v>
+        <v>3030</v>
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>810.5</v>
+        <v>2180.9</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>9099.5</v>
+        <v>849.09999999999991</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
       <c r="N21" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O21" s="2" cm="1">
         <f t="array" ref="O21">IFERROR(_xlfn.XLOOKUP(N21,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
@@ -3517,11 +3385,11 @@
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>784238.58000000031</v>
+        <v>578275.1599999998</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-784238.58000000031</v>
+        <v>-578275.1599999998</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3532,15 +3400,15 @@
       </c>
       <c r="U21" s="4">
         <f>_xlfn.XLOOKUP(S21,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="V21" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S21,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="W21" s="4">
         <f t="shared" si="3"/>
-        <v>11</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3556,35 +3424,35 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>103913.23999999987</v>
+        <v>106392.33999999989</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>15586.760000000126</v>
+        <v>13107.660000000105</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I22" s="2">
         <f>_xlfn.XLOOKUP(G22,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2670</v>
+        <v>4160</v>
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3128.5</v>
+        <v>4461.5000000000009</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>-458.5</v>
+        <v>-301.50000000000091</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O22" s="2" cm="1">
         <f t="array" ref="O22">IFERROR(_xlfn.XLOOKUP(N22,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
@@ -3592,11 +3460,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>476897.76999999938</v>
+        <v>479800.33999999973</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-476897.76999999938</v>
+        <v>-479800.33999999973</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3607,15 +3475,15 @@
       </c>
       <c r="U22" s="4">
         <f>_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>-4</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3623,43 +3491,43 @@
         <v>13</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" s="2">
         <f>_xlfn.XLOOKUP(A23,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>157000</v>
+        <v>190000</v>
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>149310.43999999954</v>
+        <v>169427.9999999998</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>7689.5600000004633</v>
+        <v>20572.000000000204</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="I23" s="2">
         <f>_xlfn.XLOOKUP(G23,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12900</v>
+        <v>4040</v>
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>12748.4</v>
+        <v>2976.94</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>151.60000000000036</v>
+        <v>1063.06</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
       <c r="N23" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O23" s="2" cm="1">
         <f t="array" ref="O23">IFERROR(_xlfn.XLOOKUP(N23,[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]]),0)</f>
@@ -3667,11 +3535,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>762242.0299999998</v>
+        <v>0</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-762242.0299999998</v>
+        <v>0</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3682,15 +3550,15 @@
       </c>
       <c r="U23" s="4">
         <f>_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3698,38 +3566,38 @@
         <v>14</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C24" s="2">
         <f>_xlfn.XLOOKUP(A24,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>120000</v>
+        <v>140000</v>
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>121988.18999999994</v>
+        <v>110771.99999999993</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>-1988.1899999999441</v>
+        <v>29228.000000000073</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="I24" s="2">
         <f>_xlfn.XLOOKUP(G24,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5460</v>
+        <v>3500</v>
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1479.8100000000002</v>
+        <v>2745.8</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>3980.1899999999996</v>
+        <v>754.19999999999982</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3746,15 +3614,15 @@
       </c>
       <c r="U24" s="4">
         <f>_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3762,38 +3630,38 @@
         <v>15</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C25" s="2">
         <f>_xlfn.XLOOKUP(A25,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>135000</v>
+        <v>140000</v>
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>137109.67999999927</v>
+        <v>105123.02999999966</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>-2109.6799999992654</v>
+        <v>34876.970000000336</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I25" s="2">
         <f>_xlfn.XLOOKUP(G25,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4810</v>
+        <v>1780</v>
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>941.57999999999993</v>
+        <v>2871.75</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>3868.42</v>
+        <v>-1091.75</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3803,22 +3671,22 @@
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="T25" s="4" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="U25" s="4">
         <f>_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>-2</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3834,30 +3702,30 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>76579.040000000052</v>
+        <v>51925.380000000077</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>13420.959999999948</v>
+        <v>38074.619999999923</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
         <v>23</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="I26" s="2">
         <f>_xlfn.XLOOKUP(G26,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6810</v>
+        <v>2890</v>
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>760.62</v>
+        <v>2480.1100000000006</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>6049.38</v>
+        <v>409.88999999999942</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3867,22 +3735,22 @@
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
       <c r="S26" s="4" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="T26" s="4" t="s">
         <v>44</v>
       </c>
       <c r="U26" s="4">
         <f>_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3898,30 +3766,30 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>223959.27999999945</v>
+        <v>194895.83999999933</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>11040.720000000554</v>
+        <v>40104.160000000673</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="I27" s="2">
         <f>_xlfn.XLOOKUP(G27,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3090</v>
+        <v>2120</v>
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>739.5</v>
+        <v>1818.01</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>2350.5</v>
+        <v>301.99</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3930,24 +3798,11 @@
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
-      <c r="S27" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="T27" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="U27" s="4">
-        <f>_xlfn.XLOOKUP(S27,'[1]BASE PYTHON'!$A$63:$A$80,'[1]BASE PYTHON'!$B$63:$B$80)</f>
-        <v>33</v>
-      </c>
-      <c r="V27" s="4">
-        <f>IFERROR(_xlfn.XLOOKUP(S27,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>21</v>
-      </c>
-      <c r="W27" s="4">
-        <f t="shared" si="3"/>
-        <v>12</v>
-      </c>
+      <c r="S27" s="4"/>
+      <c r="T27" s="4"/>
+      <c r="U27" s="4"/>
+      <c r="V27" s="4"/>
+      <c r="W27" s="4"/>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
@@ -3958,35 +3813,22 @@
       </c>
       <c r="C28" s="2">
         <f>_xlfn.XLOOKUP(A28,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>302000</v>
+        <v>315000</v>
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>305609.23500000063</v>
+        <v>276074.34999999992</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>-3609.2350000006263</v>
+        <v>38925.650000000081</v>
       </c>
       <c r="F28" s="4"/>
-      <c r="G28" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I28" s="2">
-        <f>_xlfn.XLOOKUP(G28,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4720</v>
-      </c>
-      <c r="J28" s="2">
-        <f>IFERROR(_xlfn.XLOOKUP(G28,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2736.7000000000003</v>
-      </c>
-      <c r="K28" s="7">
-        <f t="shared" si="1"/>
-        <v>1983.2999999999997</v>
-      </c>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
@@ -3995,36 +3837,52 @@
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
-      <c r="T28" s="4"/>
-      <c r="U28" s="4"/>
-      <c r="V28" s="4"/>
-      <c r="W28" s="4"/>
+      <c r="T28" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="U28" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="V28" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="W28" s="4" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C29" s="2">
         <f>_xlfn.XLOOKUP(A29,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>113000</v>
+        <v>167000</v>
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>92424.52999999997</v>
+        <v>155370.25999999998</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>20575.47000000003</v>
+        <v>11629.74000000002</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
+      <c r="H29" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>2</v>
+      </c>
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
       <c r="N29" s="4"/>
@@ -4034,50 +3892,56 @@
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
       <c r="T29" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="U29" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="V29" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="W29" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="U29" s="5" cm="1">
+        <f t="array" ref="U29">IFERROR(_xlfn.XLOOKUP(T29,[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]]),0)</f>
+        <v>185</v>
+      </c>
+      <c r="V29" s="5">
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
+        <v>287</v>
+      </c>
+      <c r="W29" s="6">
+        <f>U29-V29</f>
+        <v>-102</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C30" s="2">
         <f>_xlfn.XLOOKUP(A30,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>170000</v>
+        <v>132000</v>
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>138033.66</v>
+        <v>114539.58999999982</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>31966.339999999997</v>
+        <v>17460.410000000178</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="I30" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J30" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="K30" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="I30" s="2" cm="1">
+        <f t="array" ref="I30">IFERROR(_xlfn.XLOOKUP(H30,[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]]),0)</f>
+        <v>700000</v>
+      </c>
+      <c r="J30" s="2">
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
+        <v>621289.19500000437</v>
+      </c>
+      <c r="K30" s="7">
+        <f>I30-J30</f>
+        <v>78710.804999995627</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -4088,19 +3952,19 @@
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
       <c r="T30" s="4" t="s">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="U30" s="5" cm="1">
         <f t="array" ref="U30">IFERROR(_xlfn.XLOOKUP(T30,[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]]),0)</f>
-        <v>200</v>
-      </c>
-      <c r="V30" s="5">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>178</v>
+        <v>185</v>
+      </c>
+      <c r="V30" s="6">
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
+        <v>244</v>
       </c>
       <c r="W30" s="6">
         <f>U30-V30</f>
-        <v>22</v>
+        <v>-59</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
@@ -4112,32 +3976,32 @@
       </c>
       <c r="C31" s="2">
         <f>_xlfn.XLOOKUP(A31,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>126000</v>
+        <v>167000</v>
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>128732.68999999971</v>
+        <v>137860.06999999989</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>-2732.6899999997113</v>
+        <v>29139.930000000109</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4" t="s">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="I31" s="2" cm="1">
         <f t="array" ref="I31">IFERROR(_xlfn.XLOOKUP(H31,[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]]),0)</f>
         <v>700000</v>
       </c>
-      <c r="J31" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>645369.17500000284</v>
+      <c r="J31" s="7">
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
+        <v>606385.88500000478</v>
       </c>
       <c r="K31" s="7">
-        <f>I31-J31</f>
-        <v>54630.824999997159</v>
+        <f t="shared" ref="K31:K33" si="4">I31-J31</f>
+        <v>93614.114999995218</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4148,19 +4012,19 @@
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
       <c r="T31" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="U31" s="5" cm="1">
         <f t="array" ref="U31">IFERROR(_xlfn.XLOOKUP(T31,[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]]),0)</f>
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="V31" s="6">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>254</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
+        <v>188</v>
       </c>
       <c r="W31" s="6">
         <f>U31-V31</f>
-        <v>-54</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4172,32 +4036,32 @@
       </c>
       <c r="C32" s="2">
         <f>_xlfn.XLOOKUP(A32,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>167000</v>
+        <v>255000</v>
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>157876.89999999997</v>
+        <v>238192.00999999966</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>9123.1000000000349</v>
+        <v>16807.99000000034</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I32" s="2" cm="1">
         <f t="array" ref="I32">IFERROR(_xlfn.XLOOKUP(H32,[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]]),0)</f>
         <v>700000</v>
       </c>
       <c r="J32" s="7">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>668938.42000000074</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
+        <v>427196.10000000207</v>
       </c>
       <c r="K32" s="7">
-        <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>31061.57999999926</v>
+        <f t="shared" si="4"/>
+        <v>272803.89999999793</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4212,15 +4076,15 @@
       </c>
       <c r="U32" s="5" cm="1">
         <f t="array" ref="U32">IFERROR(_xlfn.XLOOKUP(T32,[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]]),0)</f>
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="V32" s="6">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>257</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
+        <v>0</v>
       </c>
       <c r="W32" s="6">
-        <f>U32-V32</f>
-        <v>-57</v>
+        <f t="shared" ref="W32" si="5">U32-V32</f>
+        <v>185</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4232,15 +4096,15 @@
       </c>
       <c r="C33" s="2">
         <f>_xlfn.XLOOKUP(A33,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>255000</v>
+        <v>100000</v>
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>248704.34999999971</v>
+        <v>67721.850000000064</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>6295.6500000002852</v>
+        <v>32278.149999999936</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4252,12 +4116,12 @@
         <v>700000</v>
       </c>
       <c r="J33" s="7">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>683867.69500000111</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
+        <v>0</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>16132.304999998887</v>
+        <v>700000</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4267,58 +4131,36 @@
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
-      <c r="T33" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="U33" s="5" cm="1">
-        <f t="array" ref="U33">IFERROR(_xlfn.XLOOKUP(T33,[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]]),0)</f>
-        <v>200</v>
-      </c>
-      <c r="V33" s="6">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>327</v>
-      </c>
-      <c r="W33" s="6">
-        <f t="shared" ref="W33" si="5">U33-V33</f>
-        <v>-127</v>
-      </c>
+      <c r="T33" s="4"/>
+      <c r="U33" s="2"/>
+      <c r="V33" s="4"/>
+      <c r="W33" s="4"/>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="C34" s="2">
         <f>_xlfn.XLOOKUP(A34,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>100000</v>
+        <v>55000</v>
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>73170.05000000009</v>
+        <v>42026.570000000058</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>26829.94999999991</v>
+        <v>12973.429999999942</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
-      <c r="H34" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I34" s="2" cm="1">
-        <f t="array" ref="I34">IFERROR(_xlfn.XLOOKUP(H34,[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]]),0)</f>
-        <v>700000</v>
-      </c>
-      <c r="J34" s="7">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>672318.91500000155</v>
-      </c>
-      <c r="K34" s="7">
-        <f t="shared" si="4"/>
-        <v>27681.084999998449</v>
-      </c>
+      <c r="H34" s="4"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
@@ -4341,15 +4183,15 @@
       </c>
       <c r="C35" s="2">
         <f>_xlfn.XLOOKUP(A35,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>55000</v>
+        <v>70000</v>
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>41049.48000000001</v>
+        <v>64480.80999999999</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>13950.51999999999</v>
+        <v>5519.1900000000096</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4371,28 +4213,14 @@
       <c r="W35" s="4"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C36" s="2">
-        <f>_xlfn.XLOOKUP(A36,[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</f>
-        <v>66000</v>
-      </c>
-      <c r="D36" s="2">
-        <f>IFERROR(_xlfn.XLOOKUP(A36,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>64809.780000000006</v>
-      </c>
-      <c r="E36" s="7">
-        <f t="shared" si="0"/>
-        <v>1190.2199999999939</v>
-      </c>
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
-      <c r="I36" s="2"/>
+      <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
@@ -4404,15 +4232,24 @@
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
       <c r="T36" s="4"/>
-      <c r="U36" s="2"/>
+      <c r="U36" s="4"/>
       <c r="V36" s="4"/>
       <c r="W36" s="4"/>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="4"/>
+      <c r="B37" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>2</v>
+      </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -4435,16 +4272,19 @@
     <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="C38" s="2" cm="1">
+        <f t="array" ref="C38">IFERROR(_xlfn.XLOOKUP(B38,[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]]),0)</f>
+        <v>1377500</v>
+      </c>
+      <c r="D38" s="2">
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
+        <v>1321237.5949999932</v>
+      </c>
+      <c r="E38" s="7">
+        <f>C38-D38</f>
+        <v>56262.40500000678</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -4468,19 +4308,19 @@
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="C39" s="2" cm="1">
         <f t="array" ref="C39">IFERROR(_xlfn.XLOOKUP(B39,[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]]),0)</f>
-        <v>1280000</v>
+        <v>1377500</v>
       </c>
       <c r="D39" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1184379.5950000002</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
+        <v>1290113.2949999932</v>
       </c>
       <c r="E39" s="7">
-        <f>C39-D39</f>
-        <v>95620.404999999795</v>
+        <f t="shared" ref="E39:E41" si="6">C39-D39</f>
+        <v>87386.705000006827</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4504,19 +4344,19 @@
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C40" s="2" cm="1">
         <f t="array" ref="C40">IFERROR(_xlfn.XLOOKUP(B40,[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]]),0)</f>
-        <v>1280000</v>
+        <v>1377500</v>
       </c>
       <c r="D40" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1525614.1199999915</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
+        <v>980298.82000000076</v>
       </c>
       <c r="E40" s="7">
-        <f t="shared" ref="E40:E42" si="6">C40-D40</f>
-        <v>-245614.1199999915</v>
+        <f t="shared" si="6"/>
+        <v>397201.17999999924</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4544,15 +4384,15 @@
       </c>
       <c r="C41" s="2" cm="1">
         <f t="array" ref="C41">IFERROR(_xlfn.XLOOKUP(B41,[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]]),0)</f>
-        <v>1280000</v>
+        <v>1377500</v>
       </c>
       <c r="D41" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1173268.9449999931</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
+        <v>0</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>106731.05500000692</v>
+        <v>1377500</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4574,28 +4414,7 @@
       <c r="W41" s="4"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C42" s="2" cm="1">
-        <f t="array" ref="C42">IFERROR(_xlfn.XLOOKUP(B42,[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]]),0)</f>
-        <v>1280000</v>
-      </c>
-      <c r="D42" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>1471695.8849999926</v>
-      </c>
-      <c r="E42" s="7">
-        <f t="shared" si="6"/>
-        <v>-191695.88499999256</v>
-      </c>
       <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-      <c r="I42" s="4"/>
-      <c r="J42" s="4"/>
-      <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4"/>
       <c r="N42" s="4"/>
@@ -4603,11 +4422,6 @@
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
-      <c r="S42" s="4"/>
-      <c r="T42" s="4"/>
-      <c r="U42" s="4"/>
-      <c r="V42" s="4"/>
-      <c r="W42" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Dados atualizados em 25/06/2026 08:40
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEEAE799-3E71-4ACB-8552-AB9C9C65B370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A152F5-7082-4A98-A05F-14BA76E90D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-06-11T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-06-25T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -973,7 +973,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>11/06/2026</v>
+            <v>25/06/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1012,10 +1012,10 @@
             <v>0</v>
           </cell>
           <cell r="H5" t="str">
-            <v>CAMPINAS</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I5">
-            <v>1818.01</v>
+            <v>752.55</v>
           </cell>
         </row>
         <row r="6">
@@ -1026,10 +1026,10 @@
             <v>48598.409999999989</v>
           </cell>
           <cell r="H6" t="str">
-            <v>CENTRO</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I6">
-            <v>12476.879999999996</v>
+            <v>240</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1040,16 +1040,19 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>281771.82999999961</v>
+            <v>282524.3799999996</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I7">
-            <v>2976.94</v>
+            <v>2645.5</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
+          </cell>
+          <cell r="N7" t="str">
+            <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
@@ -1060,13 +1063,16 @@
             <v>1237.53</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I8">
-            <v>17091.899999999994</v>
+            <v>1548.7300000000005</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
+          </cell>
+          <cell r="N8">
+            <v>30</v>
           </cell>
         </row>
         <row r="9">
@@ -1074,16 +1080,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>72959.349999999948</v>
+            <v>73199.349999999933</v>
           </cell>
           <cell r="H9" t="str">
-            <v>JUNDIAI</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I9">
-            <v>2180.9</v>
+            <v>1183.5999999999999</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
+          </cell>
+          <cell r="N9">
+            <v>40</v>
           </cell>
         </row>
         <row r="10">
@@ -1091,16 +1100,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>210952.18999999962</v>
+            <v>213597.68999999962</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I10">
-            <v>2559.6299999999997</v>
+            <v>1717.2</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
+          </cell>
+          <cell r="N10">
+            <v>40</v>
           </cell>
         </row>
         <row r="11">
@@ -1108,16 +1120,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>57163.810000000041</v>
+            <v>58712.540000000045</v>
           </cell>
           <cell r="H11" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I11">
-            <v>4461.5000000000009</v>
+            <v>307.35000000000002</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
+          </cell>
+          <cell r="N11">
+            <v>54</v>
           </cell>
         </row>
         <row r="12">
@@ -1128,13 +1143,16 @@
             <v>237391.93</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I12">
-            <v>1327.45</v>
+            <v>334.09999999999997</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
+          </cell>
+          <cell r="N12">
+            <v>29</v>
           </cell>
         </row>
         <row r="13">
@@ -1145,13 +1163,16 @@
             <v>165508.78999999998</v>
           </cell>
           <cell r="H13" t="str">
-            <v>MOGI</v>
+            <v>SJC</v>
           </cell>
           <cell r="I13">
-            <v>3852.0000000000005</v>
+            <v>292.39999999999998</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
+          </cell>
+          <cell r="N13">
+            <v>37</v>
           </cell>
         </row>
         <row r="14">
@@ -1162,13 +1183,16 @@
             <v>769210.07999999984</v>
           </cell>
           <cell r="H14" t="str">
-            <v>NORTE</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I14">
-            <v>6939.45</v>
+            <v>9021.4300000000021</v>
           </cell>
           <cell r="K14" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
+          </cell>
+          <cell r="N14">
+            <v>42</v>
           </cell>
         </row>
         <row r="15">
@@ -1178,14 +1202,11 @@
           <cell r="F15">
             <v>85412.150000000009</v>
           </cell>
-          <cell r="H15" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="I15">
-            <v>9250.9849999999988</v>
-          </cell>
           <cell r="K15" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
+          </cell>
+          <cell r="N15">
+            <v>37</v>
           </cell>
         </row>
         <row r="16">
@@ -1193,16 +1214,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>508154.89000000036</v>
-          </cell>
-          <cell r="H16" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I16">
-            <v>3926.98</v>
+            <v>508154.89000000031</v>
           </cell>
           <cell r="K16" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
+          </cell>
+          <cell r="N16">
+            <v>44</v>
           </cell>
         </row>
         <row r="17">
@@ -1210,16 +1228,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>382790.12000000029</v>
-          </cell>
-          <cell r="H17" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I17">
-            <v>4458.46</v>
+            <v>382790.12000000034</v>
           </cell>
           <cell r="K17" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
+          </cell>
+          <cell r="N17">
+            <v>34</v>
           </cell>
         </row>
         <row r="18">
@@ -1227,16 +1242,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>106392.33999999989</v>
-          </cell>
-          <cell r="H18" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I18">
-            <v>9471.1200000000008</v>
+            <v>107575.9399999999</v>
           </cell>
           <cell r="K18" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
+          </cell>
+          <cell r="N18">
+            <v>44</v>
           </cell>
         </row>
         <row r="19">
@@ -1244,16 +1256,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>169427.9999999998</v>
-          </cell>
-          <cell r="H19" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I19">
-            <v>2871.75</v>
+            <v>171145.19999999978</v>
           </cell>
           <cell r="K19" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
+          </cell>
+          <cell r="N19">
+            <v>71</v>
           </cell>
         </row>
         <row r="20">
@@ -1261,16 +1270,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>110771.99999999993</v>
-          </cell>
-          <cell r="H20" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I20">
-            <v>2480.1100000000006</v>
+            <v>111079.34999999993</v>
           </cell>
           <cell r="K20" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="N20">
+            <v>35</v>
           </cell>
         </row>
         <row r="21">
@@ -1280,14 +1286,11 @@
           <cell r="F21">
             <v>105123.02999999966</v>
           </cell>
-          <cell r="H21" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I21">
-            <v>2745.8</v>
-          </cell>
           <cell r="K21" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="N21">
+            <v>31</v>
           </cell>
         </row>
         <row r="22">
@@ -1295,16 +1298,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>51925.380000000077</v>
-          </cell>
-          <cell r="H22" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I22">
-            <v>90889.865000000034</v>
+            <v>52259.480000000083</v>
           </cell>
           <cell r="K22" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
+          </cell>
+          <cell r="N22">
+            <v>43</v>
           </cell>
         </row>
         <row r="23">
@@ -1315,7 +1315,10 @@
             <v>194895.83999999933</v>
           </cell>
           <cell r="K23" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
+          </cell>
+          <cell r="N23">
+            <v>30</v>
           </cell>
         </row>
         <row r="24">
@@ -1323,10 +1326,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>276074.34999999992</v>
+            <v>276074.34999999998</v>
           </cell>
           <cell r="K24" t="str">
-            <v>Total Geral</v>
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="N24">
+            <v>34</v>
           </cell>
         </row>
         <row r="25">
@@ -1336,6 +1342,12 @@
           <cell r="F25">
             <v>155370.25999999998</v>
           </cell>
+          <cell r="K25" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="N25">
+            <v>675</v>
+          </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
@@ -1366,7 +1378,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>67721.850000000064</v>
+            <v>68014.250000000044</v>
           </cell>
         </row>
         <row r="30">
@@ -1374,7 +1386,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>42026.570000000058</v>
+            <v>42026.570000000065</v>
           </cell>
         </row>
         <row r="31">
@@ -1390,7 +1402,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4655953.1799999475</v>
+            <v>4664974.6099999472</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1441,7 +1453,7 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="R39">
-            <v>154624.23999999996</v>
+            <v>154624.23999999993</v>
           </cell>
         </row>
         <row r="47">
@@ -2269,7 +2281,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>135000</v>
+        <v>150020</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -2303,7 +2315,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>4655953.1799999969</v>
+        <v>4664974.6099999975</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2314,7 +2326,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>90889.864999999976</v>
+        <v>9021.43</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2336,7 +2348,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>0</v>
+        <v>675</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2348,7 +2360,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>851046.82000000309</v>
+        <v>842025.39000000246</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2359,7 +2371,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>44110.135000000024</v>
+        <v>140998.57</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2381,7 +2393,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>706</v>
+        <v>31</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2393,7 +2405,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.84546090067187163</v>
+        <v>0.8470990757218082</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2404,7 +2416,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.67325825925925908</v>
+        <v>6.0134848686841755E-2</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2426,7 +2438,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0</v>
+        <v>0.9560906515580736</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2540,15 +2552,15 @@
       </c>
       <c r="I10" s="2">
         <f>_xlfn.XLOOKUP(G10,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12430</v>
+        <v>14620</v>
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9250.9849999999988</v>
+        <v>0</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>3179.0150000000012</v>
+        <v>14620</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2579,11 +2591,11 @@
       </c>
       <c r="V10" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W10" s="4">
         <f>U10-V10</f>
-        <v>36</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -2599,11 +2611,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>281771.82999999961</v>
+        <v>282524.3799999996</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E35" si="0">C11-D11</f>
-        <v>38228.170000000391</v>
+        <v>37475.620000000403</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2614,15 +2626,15 @@
       </c>
       <c r="I11" s="2">
         <f>_xlfn.XLOOKUP(G11,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>17550</v>
+        <v>17000</v>
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6939.45</v>
+        <v>0</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K27" si="1">I11-J11</f>
-        <v>10610.55</v>
+        <v>17000</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2656,11 +2668,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W26" si="3">U11-V11</f>
-        <v>52</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2691,15 +2703,15 @@
       </c>
       <c r="I12" s="2">
         <f>_xlfn.XLOOKUP(G12,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4930</v>
+        <v>5790</v>
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3926.98</v>
+        <v>0</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>1003.02</v>
+        <v>5790</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2733,11 +2745,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>37</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2753,11 +2765,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>72959.349999999948</v>
+        <v>73199.349999999933</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>16040.650000000052</v>
+        <v>15800.650000000067</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2768,15 +2780,15 @@
       </c>
       <c r="I13" s="2">
         <f>_xlfn.XLOOKUP(G13,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11780</v>
+        <v>13850</v>
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9471.1200000000008</v>
+        <v>0</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>2308.8799999999992</v>
+        <v>13850</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2791,11 +2803,11 @@
       </c>
       <c r="P13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>154624.23999999996</v>
+        <v>154624.23999999993</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" si="2"/>
-        <v>-154624.23999999996</v>
+        <v>-154624.23999999993</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="4" t="s">
@@ -2810,11 +2822,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>55</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2830,11 +2842,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>210952.18999999962</v>
+        <v>213597.68999999962</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>59047.810000000376</v>
+        <v>56402.310000000376</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2845,15 +2857,15 @@
       </c>
       <c r="I14" s="2">
         <f>_xlfn.XLOOKUP(G14,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6540</v>
+        <v>7690</v>
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1327.45</v>
+        <v>0</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>5212.55</v>
+        <v>7690</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -2887,11 +2899,11 @@
       </c>
       <c r="V14" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="W14" s="4">
         <f>U14-V14</f>
-        <v>23</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -2907,11 +2919,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>57163.810000000041</v>
+        <v>58712.540000000045</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>19836.189999999959</v>
+        <v>18287.459999999955</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2922,15 +2934,15 @@
       </c>
       <c r="I15" s="2">
         <f>_xlfn.XLOOKUP(G15,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>18190</v>
+        <v>18000</v>
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>12476.879999999996</v>
+        <v>752.55</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>5713.1200000000044</v>
+        <v>17247.45</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -2964,11 +2976,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>44</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -2999,15 +3011,15 @@
       </c>
       <c r="I16" s="2">
         <f>_xlfn.XLOOKUP(G16,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6200</v>
+        <v>7290</v>
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4458.46</v>
+        <v>0</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>1741.54</v>
+        <v>7290</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3041,11 +3053,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>35</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3076,15 +3088,15 @@
       </c>
       <c r="I17" s="2">
         <f>_xlfn.XLOOKUP(G17,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5000</v>
+        <v>5920</v>
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3852.0000000000005</v>
+        <v>334.09999999999997</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>1147.9999999999995</v>
+        <v>5585.9</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3118,11 +3130,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>45</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3153,15 +3165,15 @@
       </c>
       <c r="I18" s="2">
         <f>_xlfn.XLOOKUP(G18,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5690</v>
+        <v>6690</v>
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2559.6299999999997</v>
+        <v>1183.5999999999999</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>3130.3700000000003</v>
+        <v>5506.4</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3182,11 +3194,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>41</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3217,15 +3229,15 @@
       </c>
       <c r="I19" s="2">
         <f>_xlfn.XLOOKUP(G19,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>10190</v>
+        <v>11000</v>
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>1717.2</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>10190</v>
+        <v>9282.7999999999993</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3254,11 +3266,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>57</v>
+        <v>-14</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3274,11 +3286,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>508154.89000000036</v>
+        <v>508154.89000000031</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>31845.109999999637</v>
+        <v>31845.109999999695</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3289,15 +3301,15 @@
       </c>
       <c r="I20" s="2">
         <f>_xlfn.XLOOKUP(G20,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14980</v>
+        <v>14860</v>
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>17091.899999999994</v>
+        <v>2645.5</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>-2111.8999999999942</v>
+        <v>12214.5</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3310,11 +3322,11 @@
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>631456.86000000034</v>
+        <v>656771.87000000034</v>
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-631456.86000000034</v>
+        <v>-656771.87000000034</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3329,11 +3341,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>35</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3349,11 +3361,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>382790.12000000029</v>
+        <v>382790.12000000034</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>27209.879999999714</v>
+        <v>27209.879999999655</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3364,15 +3376,15 @@
       </c>
       <c r="I21" s="2">
         <f>_xlfn.XLOOKUP(G21,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3030</v>
+        <v>3710</v>
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2180.9</v>
+        <v>1548.7300000000005</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>849.09999999999991</v>
+        <v>2161.2699999999995</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3385,11 +3397,11 @@
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>578275.1599999998</v>
+        <v>632364.50999999989</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-578275.1599999998</v>
+        <v>-632364.50999999989</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3404,11 +3416,11 @@
       </c>
       <c r="V21" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S21,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W21" s="4">
         <f t="shared" si="3"/>
-        <v>40</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3424,11 +3436,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>106392.33999999989</v>
+        <v>107575.9399999999</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>13107.660000000105</v>
+        <v>11924.0600000001</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3439,15 +3451,15 @@
       </c>
       <c r="I22" s="2">
         <f>_xlfn.XLOOKUP(G22,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4160</v>
+        <v>5520</v>
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4461.5000000000009</v>
+        <v>307.35000000000002</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>-301.50000000000091</v>
+        <v>5212.6499999999996</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3460,11 +3472,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>479800.33999999973</v>
+        <v>519190.63999999978</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-479800.33999999973</v>
+        <v>-519190.63999999978</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3479,11 +3491,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>40</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3499,11 +3511,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>169427.9999999998</v>
+        <v>171145.19999999978</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>20572.000000000204</v>
+        <v>18854.800000000221</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3514,15 +3526,15 @@
       </c>
       <c r="I23" s="2">
         <f>_xlfn.XLOOKUP(G23,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4040</v>
+        <v>4990</v>
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2976.94</v>
+        <v>240</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>1063.06</v>
+        <v>4750</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3554,11 +3566,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>55</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3574,11 +3586,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>110771.99999999993</v>
+        <v>111079.34999999993</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>29228.000000000073</v>
+        <v>28920.650000000067</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3589,15 +3601,15 @@
       </c>
       <c r="I24" s="2">
         <f>_xlfn.XLOOKUP(G24,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3500</v>
+        <v>3800</v>
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2745.8</v>
+        <v>0</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>754.19999999999982</v>
+        <v>3800</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3618,11 +3630,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>33</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3653,15 +3665,15 @@
       </c>
       <c r="I25" s="2">
         <f>_xlfn.XLOOKUP(G25,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>1780</v>
+        <v>2900</v>
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2871.75</v>
+        <v>292.39999999999998</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>-1091.75</v>
+        <v>2607.6</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3682,11 +3694,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>47</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3702,11 +3714,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>51925.380000000077</v>
+        <v>52259.480000000083</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>38074.619999999923</v>
+        <v>37740.519999999917</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3717,15 +3729,15 @@
       </c>
       <c r="I26" s="2">
         <f>_xlfn.XLOOKUP(G26,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2890</v>
+        <v>3530</v>
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2480.1100000000006</v>
+        <v>0</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>409.88999999999942</v>
+        <v>3530</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3746,11 +3758,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>31</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3781,15 +3793,15 @@
       </c>
       <c r="I27" s="2">
         <f>_xlfn.XLOOKUP(G27,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2120</v>
+        <v>2860</v>
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1818.01</v>
+        <v>0</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>301.99</v>
+        <v>2860</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3817,11 +3829,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>276074.34999999992</v>
+        <v>276074.34999999998</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>38925.650000000081</v>
+        <v>38925.650000000023</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -3937,11 +3949,11 @@
       </c>
       <c r="J30" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>621289.19500000437</v>
+        <v>664009.24500000395</v>
       </c>
       <c r="K30" s="7">
         <f>I30-J30</f>
-        <v>78710.804999995627</v>
+        <v>35990.754999996047</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -3997,11 +4009,11 @@
       </c>
       <c r="J31" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>606385.88500000478</v>
+        <v>657515.23500000301</v>
       </c>
       <c r="K31" s="7">
         <f t="shared" ref="K31:K33" si="4">I31-J31</f>
-        <v>93614.114999995218</v>
+        <v>42484.764999996987</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4020,11 +4032,11 @@
       </c>
       <c r="V31" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="W31" s="6">
         <f>U31-V31</f>
-        <v>-3</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4057,11 +4069,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>427196.10000000207</v>
+        <v>469732.35000000277</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" si="4"/>
-        <v>272803.89999999793</v>
+        <v>230267.64999999723</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4100,11 +4112,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>67721.850000000064</v>
+        <v>68014.250000000044</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>32278.149999999936</v>
+        <v>31985.749999999956</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4149,11 +4161,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>42026.570000000058</v>
+        <v>42026.570000000065</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>12973.429999999942</v>
+        <v>12973.429999999935</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4280,11 +4292,11 @@
       </c>
       <c r="D38" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1321237.5949999932</v>
+        <v>1321237.5949999935</v>
       </c>
       <c r="E38" s="7">
         <f>C38-D38</f>
-        <v>56262.40500000678</v>
+        <v>56262.405000006547</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -4352,11 +4364,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>980298.82000000076</v>
+        <v>989320.25000000081</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" si="6"/>
-        <v>397201.17999999924</v>
+        <v>388179.74999999919</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 25/06/2026 09:35
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A152F5-7082-4A98-A05F-14BA76E90D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2343D331-8BCC-4EB0-A06C-18C7A16AB364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -938,19 +938,15 @@
       <sheetName val="VENDA DIA"/>
       <sheetName val="CONVERSOR"/>
       <sheetName val="SENSUM"/>
-      <sheetName val="Planilha5"/>
-      <sheetName val="Planilha4"/>
       <sheetName val="BASE PYTHON"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7">
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
             <v>GERAL</v>
@@ -1015,7 +1011,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="I5">
-            <v>752.55</v>
+            <v>1024.2</v>
           </cell>
         </row>
         <row r="6">
@@ -1029,7 +1025,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I6">
-            <v>240</v>
+            <v>443</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1040,13 +1036,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>282524.3799999996</v>
+            <v>282796.02999999962</v>
           </cell>
           <cell r="H7" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I7">
-            <v>2645.5</v>
+            <v>8906.1</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1066,7 +1062,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="I8">
-            <v>1548.7300000000005</v>
+            <v>4072.09</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1080,13 +1076,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>73199.349999999933</v>
+            <v>73402.349999999933</v>
           </cell>
           <cell r="H9" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="I9">
-            <v>1183.5999999999999</v>
+            <v>1933.55</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
@@ -1100,19 +1096,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>213597.68999999962</v>
+            <v>219858.2899999996</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I10">
-            <v>1717.2</v>
+            <v>2542.3000000000002</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>40</v>
+            <v>41</v>
           </cell>
         </row>
         <row r="11">
@@ -1120,7 +1116,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>58712.540000000045</v>
+            <v>61238.560000000056</v>
           </cell>
           <cell r="H11" t="str">
             <v>LESTE PENHA</v>
@@ -1160,13 +1156,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>165508.78999999998</v>
+            <v>166045.78999999998</v>
           </cell>
           <cell r="H13" t="str">
-            <v>SJC</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I13">
-            <v>292.39999999999998</v>
+            <v>2386.2000000000003</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1183,16 +1179,16 @@
             <v>769210.07999999984</v>
           </cell>
           <cell r="H14" t="str">
-            <v>Total Geral</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I14">
-            <v>9021.4300000000021</v>
+            <v>693.1</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>42</v>
+            <v>43</v>
           </cell>
         </row>
         <row r="15">
@@ -1202,6 +1198,12 @@
           <cell r="F15">
             <v>85412.150000000009</v>
           </cell>
+          <cell r="H15" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="I15">
+            <v>674.84999999999991</v>
+          </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
@@ -1214,7 +1216,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>508154.89000000031</v>
+            <v>508154.89000000036</v>
+          </cell>
+          <cell r="H16" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I16">
+            <v>502.4</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1228,7 +1236,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>382790.12000000034</v>
+            <v>382790.12000000029</v>
+          </cell>
+          <cell r="H17" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I17">
+            <v>897.05</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1242,7 +1256,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>107575.9399999999</v>
+            <v>108325.8899999999</v>
+          </cell>
+          <cell r="H18" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I18">
+            <v>24716.29</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1256,7 +1276,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>171145.19999999978</v>
+            <v>171970.29999999976</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1290,7 +1310,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N21">
-            <v>31</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="22">
@@ -1312,7 +1332,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>194895.83999999933</v>
+            <v>197282.03999999934</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
@@ -1326,7 +1346,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>276074.34999999998</v>
+            <v>276074.34999999992</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
@@ -1346,7 +1366,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>675</v>
+            <v>678</v>
           </cell>
         </row>
         <row r="26">
@@ -1354,7 +1374,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>114539.58999999982</v>
+            <v>115239.38999999982</v>
           </cell>
         </row>
         <row r="27">
@@ -1362,7 +1382,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>137860.06999999989</v>
+            <v>138534.91999999987</v>
           </cell>
         </row>
         <row r="28">
@@ -1378,7 +1398,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>68014.250000000044</v>
+            <v>68224.250000000029</v>
           </cell>
         </row>
         <row r="30">
@@ -1386,7 +1406,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>42026.570000000065</v>
+            <v>42923.620000000061</v>
           </cell>
         </row>
         <row r="31">
@@ -1394,7 +1414,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>64480.80999999999</v>
+            <v>64480.809999999983</v>
           </cell>
         </row>
         <row r="32">
@@ -1402,7 +1422,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4664974.6099999472</v>
+            <v>4681215.8299999479</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2315,7 +2335,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>4664974.6099999975</v>
+        <v>4681215.8299999973</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2326,7 +2346,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>9021.43</v>
+        <v>24716.29</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2348,7 +2368,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2360,7 +2380,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>842025.39000000246</v>
+        <v>825784.17000000272</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2371,7 +2391,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>140998.57</v>
+        <v>125303.70999999999</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2393,7 +2413,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2405,7 +2425,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.8470990757218082</v>
+        <v>0.85004827129108362</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2416,7 +2436,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>6.0134848686841755E-2</v>
+        <v>0.16475329956005866</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2438,7 +2458,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.9560906515580736</v>
+        <v>0.96033994334277617</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2611,11 +2631,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>282524.3799999996</v>
+        <v>282796.02999999962</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E35" si="0">C11-D11</f>
-        <v>37475.620000000403</v>
+        <v>37203.97000000038</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2630,11 +2650,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>2386.2000000000003</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K27" si="1">I11-J11</f>
-        <v>17000</v>
+        <v>14613.8</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2707,11 +2727,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>693.1</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>5790</v>
+        <v>5096.8999999999996</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2745,11 +2765,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>-3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2765,11 +2785,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>73199.349999999933</v>
+        <v>73402.349999999933</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>15800.650000000067</v>
+        <v>15597.650000000067</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2842,11 +2862,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>213597.68999999962</v>
+        <v>219858.2899999996</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>56402.310000000376</v>
+        <v>50141.710000000399</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2919,11 +2939,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>58712.540000000045</v>
+        <v>61238.560000000056</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>18287.459999999955</v>
+        <v>15761.439999999944</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2938,11 +2958,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>752.55</v>
+        <v>1024.2</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>17247.45</v>
+        <v>16975.8</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3015,11 +3035,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>674.84999999999991</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>7290</v>
+        <v>6615.15</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3073,11 +3093,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>165508.78999999998</v>
+        <v>166045.78999999998</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-5508.789999999979</v>
+        <v>-6045.789999999979</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3130,11 +3150,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3169,11 +3189,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1183.5999999999999</v>
+        <v>1933.55</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>5506.4</v>
+        <v>4756.45</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3233,11 +3253,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1717.2</v>
+        <v>2542.3000000000002</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>9282.7999999999993</v>
+        <v>8457.7000000000007</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3286,11 +3306,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>508154.89000000031</v>
+        <v>508154.89000000036</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>31845.109999999695</v>
+        <v>31845.109999999637</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3305,11 +3325,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2645.5</v>
+        <v>8906.1</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>12214.5</v>
+        <v>5953.9</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3361,11 +3381,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>382790.12000000034</v>
+        <v>382790.12000000029</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>27209.879999999655</v>
+        <v>27209.879999999714</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3380,11 +3400,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1548.7300000000005</v>
+        <v>4072.09</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>2161.2699999999995</v>
+        <v>-362.09000000000015</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3436,11 +3456,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>107575.9399999999</v>
+        <v>108325.8899999999</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>11924.0600000001</v>
+        <v>11174.110000000102</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3472,11 +3492,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>519190.63999999978</v>
+        <v>519727.63999999978</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-519190.63999999978</v>
+        <v>-519727.63999999978</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3491,11 +3511,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3511,11 +3531,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>171145.19999999978</v>
+        <v>171970.29999999976</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>18854.800000000221</v>
+        <v>18029.700000000244</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3530,11 +3550,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>240</v>
+        <v>443</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>4750</v>
+        <v>4547</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3669,11 +3689,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>292.39999999999998</v>
+        <v>502.4</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>2607.6</v>
+        <v>2397.6</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3733,11 +3753,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>897.05</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>3530</v>
+        <v>2632.95</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3778,11 +3798,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>194895.83999999933</v>
+        <v>197282.03999999934</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>40104.160000000673</v>
+        <v>37717.960000000661</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3829,11 +3849,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>276074.34999999998</v>
+        <v>276074.34999999992</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>38925.650000000023</v>
+        <v>38925.650000000081</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -3932,11 +3952,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>114539.58999999982</v>
+        <v>115239.38999999982</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>17460.410000000178</v>
+        <v>16760.610000000175</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -3949,11 +3969,11 @@
       </c>
       <c r="J30" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>664009.24500000395</v>
+        <v>664009.24500000407</v>
       </c>
       <c r="K30" s="7">
         <f>I30-J30</f>
-        <v>35990.754999996047</v>
+        <v>35990.75499999593</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -3992,11 +4012,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>137860.06999999989</v>
+        <v>138534.91999999987</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>29139.930000000109</v>
+        <v>28465.080000000133</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4032,11 +4052,11 @@
       </c>
       <c r="V31" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="W31" s="6">
         <f>U31-V31</f>
-        <v>-6</v>
+        <v>-11</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4069,11 +4089,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>469732.35000000277</v>
+        <v>485436.57000000292</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" si="4"/>
-        <v>230267.64999999723</v>
+        <v>214563.42999999708</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4112,11 +4132,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>68014.250000000044</v>
+        <v>68224.250000000029</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>31985.749999999956</v>
+        <v>31775.749999999971</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4161,11 +4181,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>42026.570000000065</v>
+        <v>42923.620000000061</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>12973.429999999935</v>
+        <v>12076.379999999939</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4199,11 +4219,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>64480.80999999999</v>
+        <v>64480.809999999983</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>5519.1900000000096</v>
+        <v>5519.1900000000169</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4292,11 +4312,11 @@
       </c>
       <c r="D38" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1321237.5949999935</v>
+        <v>1321237.5949999932</v>
       </c>
       <c r="E38" s="7">
         <f>C38-D38</f>
-        <v>56262.405000006547</v>
+        <v>56262.40500000678</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -4364,11 +4384,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>989320.25000000081</v>
+        <v>1005561.4700000008</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" si="6"/>
-        <v>388179.74999999919</v>
+        <v>371938.52999999921</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 25/06/2026 11:45
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2343D331-8BCC-4EB0-A06C-18C7A16AB364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3CF5C0-9D33-4C25-8912-95E63043A2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -941,11 +941,11 @@
       <sheetName val="BASE PYTHON"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
@@ -1008,10 +1008,10 @@
             <v>0</v>
           </cell>
           <cell r="H5" t="str">
-            <v>CENTRO</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>1024.2</v>
+            <v>332.2</v>
           </cell>
         </row>
         <row r="6">
@@ -1019,13 +1019,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F6">
-            <v>48598.409999999989</v>
+            <v>48930.609999999993</v>
           </cell>
           <cell r="H6" t="str">
-            <v>INDAIATUBA</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>443</v>
+            <v>2330.96</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1036,13 +1036,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>282796.02999999962</v>
+            <v>284102.78999999963</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>8906.1</v>
+            <v>1615.65</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1059,10 +1059,10 @@
             <v>1237.53</v>
           </cell>
           <cell r="H8" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>4072.09</v>
+            <v>11526.649999999998</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1076,13 +1076,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>73402.349999999933</v>
+            <v>74574.999999999854</v>
           </cell>
           <cell r="H9" t="str">
-            <v>LESTE</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>1933.55</v>
+            <v>4099</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
@@ -1096,13 +1096,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>219858.2899999996</v>
+            <v>222478.83999999959</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>2542.3000000000002</v>
+            <v>2768.88</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1116,19 +1116,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>61238.560000000056</v>
+            <v>61265.470000000059</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>307.35000000000002</v>
+            <v>4945.4500000000007</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>54</v>
+            <v>55</v>
           </cell>
         </row>
         <row r="12">
@@ -1139,10 +1139,10 @@
             <v>237391.93</v>
           </cell>
           <cell r="H12" t="str">
-            <v>MOGI</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>334.09999999999997</v>
+            <v>1610.95</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1156,13 +1156,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>166045.78999999998</v>
+            <v>166045.78999999995</v>
           </cell>
           <cell r="H13" t="str">
-            <v>NORTE</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>2386.2000000000003</v>
+            <v>1243.9000000000001</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1179,16 +1179,16 @@
             <v>769210.07999999984</v>
           </cell>
           <cell r="H14" t="str">
-            <v>PIRITUBA</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>693.1</v>
+            <v>700.38000000000011</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>43</v>
+            <v>45</v>
           </cell>
         </row>
         <row r="15">
@@ -1199,16 +1199,16 @@
             <v>85412.150000000009</v>
           </cell>
           <cell r="H15" t="str">
-            <v>SANTO ANDRE</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>674.84999999999991</v>
+            <v>4982</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N15">
-            <v>37</v>
+            <v>36</v>
           </cell>
         </row>
         <row r="16">
@@ -1216,13 +1216,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>508154.89000000036</v>
+            <v>519423.29000000039</v>
           </cell>
           <cell r="H16" t="str">
-            <v>SJC</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>502.4</v>
+            <v>4962.12</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1236,13 +1236,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>382790.12000000029</v>
+            <v>393898.52000000031</v>
           </cell>
           <cell r="H17" t="str">
-            <v>SJC/VALE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I17">
-            <v>897.05</v>
+            <v>2058.6999999999998</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1256,13 +1256,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>108325.8899999999</v>
+            <v>109163.06999999988</v>
           </cell>
           <cell r="H18" t="str">
-            <v>Total Geral</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I18">
-            <v>24716.29</v>
+            <v>1210.45</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1276,7 +1276,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>171970.29999999976</v>
+            <v>174389.32999999975</v>
+          </cell>
+          <cell r="H19" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="I19">
+            <v>8156.6399999999994</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1290,7 +1296,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>111079.34999999993</v>
+            <v>111977.59999999992</v>
+          </cell>
+          <cell r="H20" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I20">
+            <v>1172.0600000000002</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
@@ -1304,7 +1316,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>105123.02999999966</v>
+            <v>106366.92999999967</v>
+          </cell>
+          <cell r="H21" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I21">
+            <v>956.36</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
@@ -1318,7 +1336,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>52259.480000000083</v>
+            <v>52625.760000000082</v>
+          </cell>
+          <cell r="H22" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I22">
+            <v>4295.34</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
@@ -1332,7 +1356,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>197282.03999999934</v>
+            <v>199877.83999999936</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I23">
+            <v>58967.69</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
@@ -1346,7 +1376,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>276074.34999999992</v>
+            <v>281036.46999999968</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
@@ -1366,7 +1396,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>678</v>
+            <v>680</v>
           </cell>
         </row>
         <row r="26">
@@ -1374,7 +1404,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>115239.38999999982</v>
+            <v>116604.9899999998</v>
           </cell>
         </row>
         <row r="27">
@@ -1382,7 +1412,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>138534.91999999987</v>
+            <v>139070.5199999999</v>
           </cell>
         </row>
         <row r="28">
@@ -1390,7 +1420,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>238192.00999999966</v>
+            <v>246348.64999999967</v>
           </cell>
         </row>
         <row r="29">
@@ -1398,7 +1428,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>68224.250000000029</v>
+            <v>68893.910000000047</v>
           </cell>
         </row>
         <row r="30">
@@ -1406,7 +1436,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>42923.620000000061</v>
+            <v>42982.930000000066</v>
           </cell>
         </row>
         <row r="31">
@@ -1414,7 +1444,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>64480.809999999983</v>
+            <v>68776.149999999951</v>
           </cell>
         </row>
         <row r="32">
@@ -1422,7 +1452,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4681215.8299999479</v>
+            <v>4737456.4099999443</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1441,7 +1471,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>49116.749999999964</v>
+            <v>49116.749999999993</v>
           </cell>
         </row>
         <row r="36">
@@ -2335,7 +2365,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>4681215.8299999973</v>
+        <v>4737456.4099999974</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2346,7 +2376,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>24716.29</v>
+        <v>58967.69</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2368,7 +2398,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2380,7 +2410,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>825784.17000000272</v>
+        <v>769543.59000000264</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2391,7 +2421,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>125303.70999999999</v>
+        <v>91052.31</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2413,7 +2443,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2425,7 +2455,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.85004827129108362</v>
+        <v>0.86026083348465543</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2436,7 +2466,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.16475329956005866</v>
+        <v>0.39306552459672045</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2458,7 +2488,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.96033994334277617</v>
+        <v>0.96317280453257792</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2557,11 +2587,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>48598.409999999989</v>
+        <v>48930.609999999993</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>15901.590000000011</v>
+        <v>15569.390000000007</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2576,11 +2606,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>4962.12</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>14620</v>
+        <v>9657.880000000001</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2631,11 +2661,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>282796.02999999962</v>
+        <v>284102.78999999963</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E35" si="0">C11-D11</f>
-        <v>37203.97000000038</v>
+        <v>35897.21000000037</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2650,11 +2680,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2386.2000000000003</v>
+        <v>4982</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K27" si="1">I11-J11</f>
-        <v>14613.8</v>
+        <v>12018</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2727,11 +2757,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>693.1</v>
+        <v>2058.6999999999998</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>5096.8999999999996</v>
+        <v>3731.3</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2785,11 +2815,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>73402.349999999933</v>
+        <v>74574.999999999854</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>15597.650000000067</v>
+        <v>14425.000000000146</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2804,11 +2834,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>8156.6399999999994</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>13850</v>
+        <v>5693.3600000000006</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2842,11 +2872,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2862,11 +2892,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>219858.2899999996</v>
+        <v>222478.83999999959</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>50141.710000000399</v>
+        <v>47521.160000000411</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2881,11 +2911,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>1243.9000000000001</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>7690</v>
+        <v>6446.1</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -2939,11 +2969,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>61238.560000000056</v>
+        <v>61265.470000000059</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>15761.439999999944</v>
+        <v>15734.529999999941</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2958,11 +2988,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1024.2</v>
+        <v>2330.96</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>16975.8</v>
+        <v>15669.04</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3035,11 +3065,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>674.84999999999991</v>
+        <v>1210.45</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>6615.15</v>
+        <v>6079.55</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3093,11 +3123,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>166045.78999999998</v>
+        <v>166045.78999999995</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-6045.789999999979</v>
+        <v>-6045.7899999999499</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3112,11 +3142,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>334.09999999999997</v>
+        <v>700.38000000000011</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>5585.9</v>
+        <v>5219.62</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3131,11 +3161,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>49116.749999999964</v>
+        <v>49116.749999999993</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-49116.749999999964</v>
+        <v>-49116.749999999993</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3150,11 +3180,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3189,11 +3219,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1933.55</v>
+        <v>2768.88</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>4756.45</v>
+        <v>3921.12</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3253,11 +3283,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2542.3000000000002</v>
+        <v>4945.4500000000007</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>8457.7000000000007</v>
+        <v>6054.5499999999993</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3306,11 +3336,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>508154.89000000036</v>
+        <v>519423.29000000039</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>31845.109999999637</v>
+        <v>20576.709999999614</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3325,11 +3355,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8906.1</v>
+        <v>11526.649999999998</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>5953.9</v>
+        <v>3333.3500000000022</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3361,11 +3391,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3381,11 +3411,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>382790.12000000029</v>
+        <v>393898.52000000031</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>27209.879999999714</v>
+        <v>16101.47999999969</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3400,11 +3430,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4072.09</v>
+        <v>4099</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>-362.09000000000015</v>
+        <v>-389</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3456,11 +3486,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>108325.8899999999</v>
+        <v>109163.06999999988</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>11174.110000000102</v>
+        <v>10336.930000000124</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3475,11 +3505,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>307.35000000000002</v>
+        <v>1610.95</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>5212.6499999999996</v>
+        <v>3909.05</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3492,11 +3522,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>519727.63999999978</v>
+        <v>542104.43999999983</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-519727.63999999978</v>
+        <v>-542104.43999999983</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3531,11 +3561,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>171970.29999999976</v>
+        <v>174389.32999999975</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>18029.700000000244</v>
+        <v>15610.670000000246</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3550,11 +3580,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>443</v>
+        <v>1615.65</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>4547</v>
+        <v>3374.35</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3606,11 +3636,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>111079.34999999993</v>
+        <v>111977.59999999992</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>28920.650000000067</v>
+        <v>28022.400000000081</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3625,11 +3655,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>4295.34</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>3800</v>
+        <v>-495.34000000000015</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3670,11 +3700,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>105123.02999999966</v>
+        <v>106366.92999999967</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>34876.970000000336</v>
+        <v>33633.070000000327</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3689,11 +3719,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>502.4</v>
+        <v>1172.0600000000002</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>2397.6</v>
+        <v>1727.9399999999998</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3734,11 +3764,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>52259.480000000083</v>
+        <v>52625.760000000082</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>37740.519999999917</v>
+        <v>37374.239999999918</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3753,11 +3783,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>897.05</v>
+        <v>956.36</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>2632.95</v>
+        <v>2573.64</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3798,11 +3828,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>197282.03999999934</v>
+        <v>199877.83999999936</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>37717.960000000661</v>
+        <v>35122.160000000644</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3817,11 +3847,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>332.2</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>2860</v>
+        <v>2527.8000000000002</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3849,11 +3879,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>276074.34999999992</v>
+        <v>281036.46999999968</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>38925.650000000081</v>
+        <v>33963.530000000319</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -3932,11 +3962,11 @@
       </c>
       <c r="V29" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="W29" s="6">
         <f>U29-V29</f>
-        <v>-102</v>
+        <v>-101</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
@@ -3952,11 +3982,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>115239.38999999982</v>
+        <v>116604.9899999998</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>16760.610000000175</v>
+        <v>15395.010000000198</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -3969,11 +3999,11 @@
       </c>
       <c r="J30" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>664009.24500000407</v>
+        <v>663603.89500000398</v>
       </c>
       <c r="K30" s="7">
         <f>I30-J30</f>
-        <v>35990.75499999593</v>
+        <v>36396.104999996023</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -4012,11 +4042,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>138534.91999999987</v>
+        <v>139070.5199999999</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>28465.080000000133</v>
+        <v>27929.480000000098</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4052,11 +4082,11 @@
       </c>
       <c r="V31" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="W31" s="6">
         <f>U31-V31</f>
-        <v>-11</v>
+        <v>-17</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4072,11 +4102,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>238192.00999999966</v>
+        <v>246348.64999999967</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>16807.99000000034</v>
+        <v>8651.350000000326</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4089,11 +4119,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>485436.57000000292</v>
+        <v>519705.70000000304</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" si="4"/>
-        <v>214563.42999999708</v>
+        <v>180294.29999999696</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4132,11 +4162,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>68224.250000000029</v>
+        <v>68893.910000000047</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>31775.749999999971</v>
+        <v>31106.089999999953</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4181,11 +4211,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>42923.620000000061</v>
+        <v>42982.930000000066</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>12076.379999999939</v>
+        <v>12017.069999999934</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4219,11 +4249,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>64480.809999999983</v>
+        <v>68776.149999999951</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>5519.1900000000169</v>
+        <v>1223.8500000000495</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4312,11 +4342,11 @@
       </c>
       <c r="D38" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1321237.5949999932</v>
+        <v>1320832.2449999931</v>
       </c>
       <c r="E38" s="7">
         <f>C38-D38</f>
-        <v>56262.40500000678</v>
+        <v>56667.755000006873</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -4384,11 +4414,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1005561.4700000008</v>
+        <v>1062207.3999999992</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" si="6"/>
-        <v>371938.52999999921</v>
+        <v>315292.60000000079</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 29/06/2026 07:39
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3CF5C0-9D33-4C25-8912-95E63043A2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2308E18-A2B8-471F-BBB6-97D6EC8FD7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1011,7 +1011,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>332.2</v>
+            <v>510.9</v>
           </cell>
         </row>
         <row r="6">
@@ -1019,13 +1019,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F6">
-            <v>48930.609999999993</v>
+            <v>52841.079999999987</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>2330.96</v>
+            <v>7483.76</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1036,19 +1036,16 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>284102.78999999963</v>
+            <v>297627.2399999997</v>
           </cell>
           <cell r="H7" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>1615.65</v>
+            <v>2872.65</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
-          </cell>
-          <cell r="N7" t="str">
-            <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
@@ -1062,13 +1059,10 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>11526.649999999998</v>
+            <v>17938.599999999995</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
-          </cell>
-          <cell r="N8">
-            <v>30</v>
           </cell>
         </row>
         <row r="9">
@@ -1076,7 +1070,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>74574.999999999854</v>
+            <v>77213.75999999982</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
@@ -1086,9 +1080,6 @@
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
-          </cell>
-          <cell r="N9">
-            <v>40</v>
           </cell>
         </row>
         <row r="10">
@@ -1096,19 +1087,16 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>222478.83999999959</v>
+            <v>236353.43999999954</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>2768.88</v>
+            <v>2848.92</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
-          </cell>
-          <cell r="N10">
-            <v>41</v>
           </cell>
         </row>
         <row r="11">
@@ -1116,19 +1104,16 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>61265.470000000059</v>
+            <v>66356.810000000027</v>
           </cell>
           <cell r="H11" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>4945.4500000000007</v>
+            <v>5896.35</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
-          </cell>
-          <cell r="N11">
-            <v>55</v>
           </cell>
         </row>
         <row r="12">
@@ -1136,7 +1121,7 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>237391.93</v>
+            <v>258678.93</v>
           </cell>
           <cell r="H12" t="str">
             <v>LESTE PENHA</v>
@@ -1146,9 +1131,6 @@
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
-          </cell>
-          <cell r="N12">
-            <v>29</v>
           </cell>
         </row>
         <row r="13">
@@ -1156,19 +1138,16 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>166045.78999999995</v>
+            <v>239000.78999999995</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>1243.9000000000001</v>
+            <v>4573.8999999999996</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
-          </cell>
-          <cell r="N13">
-            <v>37</v>
           </cell>
         </row>
         <row r="14">
@@ -1176,19 +1155,16 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>769210.07999999984</v>
+            <v>779822.08000000007</v>
           </cell>
           <cell r="H14" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>700.38000000000011</v>
+            <v>2509.0800000000004</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
-          </cell>
-          <cell r="N14">
-            <v>45</v>
           </cell>
         </row>
         <row r="15">
@@ -1196,19 +1172,16 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>85412.150000000009</v>
+            <v>111572.95000000007</v>
           </cell>
           <cell r="H15" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>4982</v>
+            <v>13421.870000000006</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
-          </cell>
-          <cell r="N15">
-            <v>36</v>
           </cell>
         </row>
         <row r="16">
@@ -1216,19 +1189,16 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>519423.29000000039</v>
+            <v>531685.79000000039</v>
           </cell>
           <cell r="H16" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>4962.12</v>
+            <v>8801.0499999999993</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="N16">
-            <v>44</v>
           </cell>
         </row>
         <row r="17">
@@ -1236,19 +1206,16 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>393898.52000000031</v>
+            <v>389719.22000000038</v>
           </cell>
           <cell r="H17" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I17">
-            <v>2058.6999999999998</v>
+            <v>4171.75</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
-          </cell>
-          <cell r="N17">
-            <v>34</v>
           </cell>
         </row>
         <row r="18">
@@ -1256,19 +1223,16 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>109163.06999999988</v>
+            <v>115679.6399999998</v>
           </cell>
           <cell r="H18" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I18">
-            <v>1210.45</v>
+            <v>3062.47</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
-          </cell>
-          <cell r="N18">
-            <v>44</v>
           </cell>
         </row>
         <row r="19">
@@ -1276,19 +1240,16 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>174389.32999999975</v>
+            <v>179836.22999999972</v>
           </cell>
           <cell r="H19" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I19">
-            <v>8156.6399999999994</v>
+            <v>11167.14</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
-          </cell>
-          <cell r="N19">
-            <v>71</v>
           </cell>
         </row>
         <row r="20">
@@ -1296,7 +1257,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>111977.59999999992</v>
+            <v>113177.64999999991</v>
           </cell>
           <cell r="H20" t="str">
             <v>SJC</v>
@@ -1306,9 +1267,6 @@
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
-          </cell>
-          <cell r="N20">
-            <v>35</v>
           </cell>
         </row>
         <row r="21">
@@ -1316,19 +1274,16 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>106366.92999999967</v>
+            <v>111494.7899999996</v>
           </cell>
           <cell r="H21" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I21">
-            <v>956.36</v>
+            <v>2387.7000000000007</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="N21">
-            <v>32</v>
           </cell>
         </row>
         <row r="22">
@@ -1336,19 +1291,16 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>52625.760000000082</v>
+            <v>58166.910000000113</v>
           </cell>
           <cell r="H22" t="str">
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I22">
-            <v>4295.34</v>
+            <v>5396.91</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
-          </cell>
-          <cell r="N22">
-            <v>43</v>
           </cell>
         </row>
         <row r="23">
@@ -1356,19 +1308,16 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>199877.83999999936</v>
+            <v>210407.45999999944</v>
           </cell>
           <cell r="H23" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I23">
-            <v>58967.69</v>
+            <v>99925.060000000012</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
-          </cell>
-          <cell r="N23">
-            <v>30</v>
           </cell>
         </row>
         <row r="24">
@@ -1376,13 +1325,10 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>281036.46999999968</v>
+            <v>297412.17000000016</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
-          </cell>
-          <cell r="N24">
-            <v>34</v>
           </cell>
         </row>
         <row r="25">
@@ -1395,16 +1341,13 @@
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
-          <cell r="N25">
-            <v>680</v>
-          </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>116604.9899999998</v>
+            <v>122958.22999999979</v>
           </cell>
         </row>
         <row r="27">
@@ -1412,7 +1355,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>139070.5199999999</v>
+            <v>142794.87999999989</v>
           </cell>
         </row>
         <row r="28">
@@ -1420,7 +1363,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>246348.64999999967</v>
+            <v>255366.7399999997</v>
           </cell>
         </row>
         <row r="29">
@@ -1428,7 +1371,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>68893.910000000047</v>
+            <v>69502.410000000033</v>
           </cell>
         </row>
         <row r="30">
@@ -1436,7 +1379,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>42982.930000000066</v>
+            <v>47169.730000000069</v>
           </cell>
         </row>
         <row r="31">
@@ -1444,7 +1387,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>68776.149999999951</v>
+            <v>72817.384999999951</v>
           </cell>
         </row>
         <row r="32">
@@ -1452,7 +1395,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4737456.4099999443</v>
+            <v>4994264.1049999278</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2365,7 +2308,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>4737456.4099999974</v>
+        <v>4994264.1049999977</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2376,7 +2319,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>58967.69</v>
+        <v>99925.059999999983</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2398,7 +2341,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>680</v>
+        <v>0</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2410,7 +2353,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>769543.59000000264</v>
+        <v>512735.89500000235</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2421,7 +2364,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>91052.31</v>
+        <v>50094.940000000017</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2443,7 +2386,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>26</v>
+        <v>706</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2455,7 +2398,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.86026083348465543</v>
+        <v>0.90689379063010667</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2466,7 +2409,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.39306552459672045</v>
+        <v>0.66607825623250227</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2488,7 +2431,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0.96317280453257792</v>
+        <v>0</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2587,11 +2530,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>48930.609999999993</v>
+        <v>52841.079999999987</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>15569.390000000007</v>
+        <v>11658.920000000013</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2606,11 +2549,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4962.12</v>
+        <v>8801.0499999999993</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>9657.880000000001</v>
+        <v>5818.9500000000007</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2641,11 +2584,11 @@
       </c>
       <c r="V10" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="W10" s="4">
         <f>U10-V10</f>
-        <v>6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -2661,11 +2604,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>284102.78999999963</v>
+        <v>297627.2399999997</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E35" si="0">C11-D11</f>
-        <v>35897.21000000037</v>
+        <v>22372.7600000003</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2680,11 +2623,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4982</v>
+        <v>13421.870000000006</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K27" si="1">I11-J11</f>
-        <v>12018</v>
+        <v>3578.1299999999937</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2718,11 +2661,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W26" si="3">U11-V11</f>
-        <v>12</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2757,11 +2700,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2058.6999999999998</v>
+        <v>4171.75</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>3731.3</v>
+        <v>1618.25</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2795,11 +2738,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>-4</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2815,11 +2758,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>74574.999999999854</v>
+        <v>77213.75999999982</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>14425.000000000146</v>
+        <v>11786.24000000018</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2834,11 +2777,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8156.6399999999994</v>
+        <v>11167.14</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>5693.3600000000006</v>
+        <v>2682.8600000000006</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2872,11 +2815,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2892,11 +2835,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>222478.83999999959</v>
+        <v>236353.43999999954</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>47521.160000000411</v>
+        <v>33646.560000000463</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2911,11 +2854,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1243.9000000000001</v>
+        <v>4573.8999999999996</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>6446.1</v>
+        <v>3116.1000000000004</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -2949,11 +2892,11 @@
       </c>
       <c r="V14" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="W14" s="4">
         <f>U14-V14</f>
-        <v>-6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -2969,11 +2912,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>61265.470000000059</v>
+        <v>66356.810000000027</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>15734.529999999941</v>
+        <v>10643.189999999973</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2988,11 +2931,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2330.96</v>
+        <v>7483.76</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>15669.04</v>
+        <v>10516.24</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3026,11 +2969,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3046,11 +2989,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>237391.93</v>
+        <v>258678.93</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>87608.07</v>
+        <v>66321.070000000007</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3065,11 +3008,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1210.45</v>
+        <v>3062.47</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>6079.55</v>
+        <v>4227.5300000000007</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3103,11 +3046,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3123,11 +3066,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>166045.78999999995</v>
+        <v>239000.78999999995</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-6045.7899999999499</v>
+        <v>-79000.78999999995</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3142,11 +3085,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>700.38000000000011</v>
+        <v>2509.0800000000004</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>5219.62</v>
+        <v>3410.9199999999996</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3180,11 +3123,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3200,11 +3143,11 @@
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>769210.07999999984</v>
+        <v>779822.08000000007</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>180789.92000000016</v>
+        <v>170177.91999999993</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3219,11 +3162,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2768.88</v>
+        <v>2848.92</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>3921.12</v>
+        <v>3841.08</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3244,11 +3187,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>-3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3264,11 +3207,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>85412.150000000009</v>
+        <v>111572.95000000007</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>39587.849999999991</v>
+        <v>13427.04999999993</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3283,11 +3226,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4945.4500000000007</v>
+        <v>5896.35</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>6054.5499999999993</v>
+        <v>5103.6499999999996</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3316,11 +3259,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>-14</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3336,11 +3279,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>519423.29000000039</v>
+        <v>531685.79000000039</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>20576.709999999614</v>
+        <v>8314.2099999996135</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3355,11 +3298,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11526.649999999998</v>
+        <v>17938.599999999995</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>3333.3500000000022</v>
+        <v>-3078.5999999999949</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3372,11 +3315,11 @@
       </c>
       <c r="P20" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>656771.87000000034</v>
+        <v>656771.87000000046</v>
       </c>
       <c r="Q20" s="7">
         <f>O20-P20</f>
-        <v>-656771.87000000034</v>
+        <v>-656771.87000000046</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
@@ -3391,11 +3334,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>-1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3411,11 +3354,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>393898.52000000031</v>
+        <v>389719.22000000038</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>16101.47999999969</v>
+        <v>20280.77999999962</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3447,11 +3390,11 @@
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>632364.50999999989</v>
+        <v>623685.80999999982</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-632364.50999999989</v>
+        <v>-623685.80999999982</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3466,11 +3409,11 @@
       </c>
       <c r="V21" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S21,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="W21" s="4">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3486,11 +3429,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>109163.06999999988</v>
+        <v>115679.6399999998</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>10336.930000000124</v>
+        <v>3820.3600000002043</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3522,11 +3465,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>542104.43999999983</v>
+        <v>689881.14000000013</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-542104.43999999983</v>
+        <v>-689881.14000000013</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
@@ -3541,11 +3484,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3561,11 +3504,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>174389.32999999975</v>
+        <v>179836.22999999972</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>15610.670000000246</v>
+        <v>10163.770000000281</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3580,11 +3523,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1615.65</v>
+        <v>2872.65</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>3374.35</v>
+        <v>2117.35</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3616,11 +3559,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3636,11 +3579,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>111977.59999999992</v>
+        <v>113177.64999999991</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>28022.400000000081</v>
+        <v>26822.350000000093</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3655,11 +3598,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4295.34</v>
+        <v>5396.91</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>-495.34000000000015</v>
+        <v>-1596.9099999999999</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3680,11 +3623,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3700,11 +3643,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>106366.92999999967</v>
+        <v>111494.7899999996</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>33633.070000000327</v>
+        <v>28505.210000000399</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3744,11 +3687,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3764,11 +3707,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>52625.760000000082</v>
+        <v>58166.910000000113</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>37374.239999999918</v>
+        <v>31833.089999999887</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3783,11 +3726,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>956.36</v>
+        <v>2387.7000000000007</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>2573.64</v>
+        <v>1142.2999999999993</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3808,11 +3751,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>-3</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3828,11 +3771,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>199877.83999999936</v>
+        <v>210407.45999999944</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>35122.160000000644</v>
+        <v>24592.540000000561</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3847,11 +3790,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>332.2</v>
+        <v>510.9</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>2527.8000000000002</v>
+        <v>2349.1</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3879,11 +3822,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>281036.46999999968</v>
+        <v>297412.17000000016</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>33963.530000000319</v>
+        <v>17587.829999999842</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -3962,11 +3905,11 @@
       </c>
       <c r="V29" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="W29" s="6">
         <f>U29-V29</f>
-        <v>-101</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
@@ -3982,11 +3925,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>116604.9899999998</v>
+        <v>122958.22999999979</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>15395.010000000198</v>
+        <v>9041.7700000002078</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -3999,11 +3942,11 @@
       </c>
       <c r="J30" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>663603.89500000398</v>
+        <v>663421.19500000414</v>
       </c>
       <c r="K30" s="7">
         <f>I30-J30</f>
-        <v>36396.104999996023</v>
+        <v>36578.80499999586</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -4042,11 +3985,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>139070.5199999999</v>
+        <v>142794.87999999989</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>27929.480000000098</v>
+        <v>24205.120000000112</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4059,11 +4002,11 @@
       </c>
       <c r="J31" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>657515.23500000301</v>
+        <v>656169.61500000302</v>
       </c>
       <c r="K31" s="7">
         <f t="shared" ref="K31:K33" si="4">I31-J31</f>
-        <v>42484.764999996987</v>
+        <v>43830.384999996983</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4082,11 +4025,11 @@
       </c>
       <c r="V31" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>202</v>
+        <v>264</v>
       </c>
       <c r="W31" s="6">
         <f>U31-V31</f>
-        <v>-17</v>
+        <v>-79</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4102,11 +4045,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>246348.64999999967</v>
+        <v>255366.7399999997</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>8651.350000000326</v>
+        <v>-366.73999999969965</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4119,11 +4062,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>519705.70000000304</v>
+        <v>638943.71500000253</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" si="4"/>
-        <v>180294.29999999696</v>
+        <v>61056.284999997471</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4162,11 +4105,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>68893.910000000047</v>
+        <v>69502.410000000033</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>31106.089999999953</v>
+        <v>30497.589999999967</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4211,11 +4154,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>42982.930000000066</v>
+        <v>47169.730000000069</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>12017.069999999934</v>
+        <v>7830.2699999999313</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4249,11 +4192,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>68776.149999999951</v>
+        <v>72817.384999999951</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>1223.8500000000495</v>
+        <v>-2817.3849999999511</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4342,11 +4285,11 @@
       </c>
       <c r="D38" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1320832.2449999931</v>
+        <v>1320649.5449999932</v>
       </c>
       <c r="E38" s="7">
         <f>C38-D38</f>
-        <v>56667.755000006873</v>
+        <v>56850.455000006827</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -4378,11 +4321,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1290113.2949999932</v>
+        <v>1280088.9749999936</v>
       </c>
       <c r="E39" s="7">
         <f t="shared" ref="E39:E41" si="6">C39-D39</f>
-        <v>87386.705000006827</v>
+        <v>97411.025000006426</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4414,11 +4357,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1062207.3999999992</v>
+        <v>1329222.1149999904</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" si="6"/>
-        <v>315292.60000000079</v>
+        <v>48277.885000009555</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 29/06/2026 09:33
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2308E18-A2B8-471F-BBB6-97D6EC8FD7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176EDCF5-9247-4B3E-865F-9EA65D383C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-06-25T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-06-29T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -969,7 +969,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>25/06/2026</v>
+            <v>29/06/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1011,7 +1011,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>510.9</v>
+            <v>905.05</v>
           </cell>
         </row>
         <row r="6">
@@ -1019,13 +1019,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F6">
-            <v>52841.079999999987</v>
+            <v>53806.12999999999</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>7483.76</v>
+            <v>5445.0999999999995</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1036,16 +1036,19 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>297627.2399999997</v>
+            <v>303072.33999999979</v>
           </cell>
           <cell r="H7" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>2872.65</v>
+            <v>2246</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
+          </cell>
+          <cell r="N7" t="str">
+            <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
@@ -1059,10 +1062,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>17938.599999999995</v>
+            <v>9428.2999999999993</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
+          </cell>
+          <cell r="N8">
+            <v>31</v>
           </cell>
         </row>
         <row r="9">
@@ -1070,16 +1076,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>77213.75999999982</v>
+            <v>79459.759999999835</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>4099</v>
+            <v>2886.37</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
+          </cell>
+          <cell r="N9">
+            <v>42</v>
           </cell>
         </row>
         <row r="10">
@@ -1087,16 +1096,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>236353.43999999954</v>
+            <v>245781.73999999953</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>2848.92</v>
+            <v>1967.66</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
+          </cell>
+          <cell r="N10">
+            <v>43</v>
           </cell>
         </row>
         <row r="11">
@@ -1104,16 +1116,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>66356.810000000027</v>
+            <v>69283.180000000022</v>
           </cell>
           <cell r="H11" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>5896.35</v>
+            <v>9866.0999999999985</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
+          </cell>
+          <cell r="N11">
+            <v>57</v>
           </cell>
         </row>
         <row r="12">
@@ -1121,16 +1136,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>258678.93</v>
+            <v>268215.93</v>
           </cell>
           <cell r="H12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>1610.95</v>
+            <v>6149.3000000000011</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
+          </cell>
+          <cell r="N12">
+            <v>30</v>
           </cell>
         </row>
         <row r="13">
@@ -1138,16 +1156,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>239000.78999999995</v>
+            <v>242195.78999999995</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>4573.8999999999996</v>
+            <v>439.70000000000005</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
+          </cell>
+          <cell r="N13">
+            <v>40</v>
           </cell>
         </row>
         <row r="14">
@@ -1158,13 +1179,16 @@
             <v>779822.08000000007</v>
           </cell>
           <cell r="H14" t="str">
-            <v>MOGI</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I14">
-            <v>2509.0800000000004</v>
+            <v>1797.8999999999999</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
+          </cell>
+          <cell r="N14">
+            <v>47</v>
           </cell>
         </row>
         <row r="15">
@@ -1175,13 +1199,16 @@
             <v>111572.95000000007</v>
           </cell>
           <cell r="H15" t="str">
-            <v>NORTE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I15">
-            <v>13421.870000000006</v>
+            <v>2394.44</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
+          </cell>
+          <cell r="N15">
+            <v>36</v>
           </cell>
         </row>
         <row r="16">
@@ -1192,13 +1219,16 @@
             <v>531685.79000000039</v>
           </cell>
           <cell r="H16" t="str">
-            <v>OSASCO</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I16">
-            <v>8801.0499999999993</v>
+            <v>2628.95</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
+          </cell>
+          <cell r="N16">
+            <v>50</v>
           </cell>
         </row>
         <row r="17">
@@ -1209,13 +1239,16 @@
             <v>389719.22000000038</v>
           </cell>
           <cell r="H17" t="str">
-            <v>PIRITUBA</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I17">
-            <v>4171.75</v>
+            <v>1123.7</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
+          </cell>
+          <cell r="N17">
+            <v>35</v>
           </cell>
         </row>
         <row r="18">
@@ -1223,16 +1256,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>115679.6399999998</v>
+            <v>117647.29999999981</v>
           </cell>
           <cell r="H18" t="str">
-            <v>SANTO ANDRE</v>
+            <v>SBC</v>
           </cell>
           <cell r="I18">
-            <v>3062.47</v>
+            <v>13243.519999999997</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
+          </cell>
+          <cell r="N18">
+            <v>47</v>
           </cell>
         </row>
         <row r="19">
@@ -1240,16 +1276,19 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>179836.22999999972</v>
+            <v>189702.3299999997</v>
           </cell>
           <cell r="H19" t="str">
-            <v>SBC</v>
+            <v>SJC</v>
           </cell>
           <cell r="I19">
-            <v>11167.14</v>
+            <v>127.96</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
+          </cell>
+          <cell r="N19">
+            <v>76</v>
           </cell>
         </row>
         <row r="20">
@@ -1257,16 +1296,19 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>113177.64999999991</v>
+            <v>119326.94999999985</v>
           </cell>
           <cell r="H20" t="str">
-            <v>SJC</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I20">
-            <v>1172.0600000000002</v>
+            <v>1255.0500000000002</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
+          </cell>
+          <cell r="N20">
+            <v>36</v>
           </cell>
         </row>
         <row r="21">
@@ -1274,16 +1316,19 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>111494.7899999996</v>
+            <v>111934.48999999958</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SJC/VALE</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I21">
-            <v>2387.7000000000007</v>
+            <v>61905.099999999984</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="N21">
+            <v>35</v>
           </cell>
         </row>
         <row r="22">
@@ -1291,16 +1336,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>58166.910000000113</v>
-          </cell>
-          <cell r="H22" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I22">
-            <v>5396.91</v>
+            <v>58216.910000000113</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
+          </cell>
+          <cell r="N22">
+            <v>43</v>
           </cell>
         </row>
         <row r="23">
@@ -1308,16 +1350,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>210407.45999999944</v>
-          </cell>
-          <cell r="H23" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I23">
-            <v>99925.060000000012</v>
+            <v>212205.35999999943</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
+          </cell>
+          <cell r="N23">
+            <v>30</v>
           </cell>
         </row>
         <row r="24">
@@ -1325,10 +1364,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>297412.17000000016</v>
+            <v>299954.80999999912</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
+          </cell>
+          <cell r="N24">
+            <v>35</v>
           </cell>
         </row>
         <row r="25">
@@ -1336,10 +1378,13 @@
             <v>PIRACICABA</v>
           </cell>
           <cell r="F25">
-            <v>155370.25999999998</v>
+            <v>156397.05999999997</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
+          </cell>
+          <cell r="N25">
+            <v>713</v>
           </cell>
         </row>
         <row r="26">
@@ -1347,7 +1392,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>122958.22999999979</v>
+            <v>125752.37999999979</v>
           </cell>
         </row>
         <row r="27">
@@ -1355,7 +1400,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>142794.87999999989</v>
+            <v>143918.5799999999</v>
           </cell>
         </row>
         <row r="28">
@@ -1363,7 +1408,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>255366.7399999997</v>
+            <v>268610.25999999978</v>
           </cell>
         </row>
         <row r="29">
@@ -1371,7 +1416,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>69502.410000000033</v>
+            <v>69637.45000000007</v>
           </cell>
         </row>
         <row r="30">
@@ -1379,7 +1424,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>47169.730000000069</v>
+            <v>47176.690000000068</v>
           </cell>
         </row>
         <row r="31">
@@ -1387,7 +1432,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>72817.384999999951</v>
+            <v>74072.434999999925</v>
           </cell>
         </row>
         <row r="32">
@@ -1395,7 +1440,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4994264.1049999278</v>
+            <v>5070405.4449999304</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2308,7 +2353,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>4994264.1049999977</v>
+        <v>5070405.4449999975</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2319,7 +2364,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>99925.059999999983</v>
+        <v>61905.100000000006</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2341,7 +2386,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>0</v>
+        <v>713</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2353,7 +2398,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>512735.89500000235</v>
+        <v>436594.5550000025</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2364,7 +2409,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>50094.940000000017</v>
+        <v>88114.9</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2386,7 +2431,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>706</v>
+        <v>-7</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2398,7 +2443,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.90689379063010667</v>
+        <v>0.92072007354276331</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2409,7 +2454,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.66607825623250227</v>
+        <v>0.41264564724703379</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2431,7 +2476,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>0</v>
+        <v>1.0099150141643058</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2530,11 +2575,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>52841.079999999987</v>
+        <v>53806.12999999999</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>11658.920000000013</v>
+        <v>10693.87000000001</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2549,11 +2594,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>8801.0499999999993</v>
+        <v>2394.44</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>5818.9500000000007</v>
+        <v>12225.56</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2584,11 +2629,11 @@
       </c>
       <c r="V10" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="W10" s="4">
         <f>U10-V10</f>
-        <v>36</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -2604,11 +2649,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>297627.2399999997</v>
+        <v>303072.33999999979</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E35" si="0">C11-D11</f>
-        <v>22372.7600000003</v>
+        <v>16927.660000000207</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2623,11 +2668,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>13421.870000000006</v>
+        <v>1797.8999999999999</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K27" si="1">I11-J11</f>
-        <v>3578.1299999999937</v>
+        <v>15202.1</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2661,11 +2706,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W26" si="3">U11-V11</f>
-        <v>52</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2700,11 +2745,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4171.75</v>
+        <v>2628.95</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>1618.25</v>
+        <v>3161.05</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2738,11 +2783,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>37</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2758,11 +2803,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>77213.75999999982</v>
+        <v>79459.759999999835</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>11786.24000000018</v>
+        <v>9540.2400000001653</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2777,11 +2822,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11167.14</v>
+        <v>13243.519999999997</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>2682.8600000000006</v>
+        <v>606.4800000000032</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2815,11 +2860,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>55</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2835,11 +2880,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>236353.43999999954</v>
+        <v>245781.73999999953</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>33646.560000000463</v>
+        <v>24218.260000000475</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2854,11 +2899,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4573.8999999999996</v>
+        <v>439.70000000000005</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>3116.1000000000004</v>
+        <v>7250.3</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -2892,11 +2937,11 @@
       </c>
       <c r="V14" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W14" s="4">
         <f>U14-V14</f>
-        <v>23</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -2912,11 +2957,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>66356.810000000027</v>
+        <v>69283.180000000022</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>10643.189999999973</v>
+        <v>7716.8199999999779</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2931,11 +2976,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7483.76</v>
+        <v>5445.0999999999995</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>10516.24</v>
+        <v>12554.900000000001</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -2969,11 +3014,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>44</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -2989,11 +3034,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>258678.93</v>
+        <v>268215.93</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>66321.070000000007</v>
+        <v>56784.070000000007</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3008,11 +3053,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3062.47</v>
+        <v>1123.7</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>4227.5300000000007</v>
+        <v>6166.3</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3046,11 +3091,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3066,11 +3111,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>239000.78999999995</v>
+        <v>242195.78999999995</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-79000.78999999995</v>
+        <v>-82195.78999999995</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3085,11 +3130,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2509.0800000000004</v>
+        <v>0</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>3410.9199999999996</v>
+        <v>5920</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3123,11 +3168,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>45</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3162,11 +3207,11 @@
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2848.92</v>
+        <v>1967.66</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>3841.08</v>
+        <v>4722.34</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3187,11 +3232,11 @@
       </c>
       <c r="V18" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="3"/>
-        <v>41</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3226,11 +3271,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5896.35</v>
+        <v>9866.0999999999985</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>5103.6499999999996</v>
+        <v>1133.9000000000015</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3259,11 +3304,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>57</v>
+        <v>-19</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3298,11 +3343,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>17938.599999999995</v>
+        <v>9428.2999999999993</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>-3078.5999999999949</v>
+        <v>5431.7000000000007</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3334,11 +3379,11 @@
       </c>
       <c r="V20" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="3"/>
-        <v>35</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3373,11 +3418,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>4099</v>
+        <v>2886.37</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>-389</v>
+        <v>823.63000000000011</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3390,11 +3435,11 @@
       </c>
       <c r="P21" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>623685.80999999982</v>
+        <v>623685.80999999971</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>-623685.80999999982</v>
+        <v>-623685.80999999971</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
@@ -3409,11 +3454,11 @@
       </c>
       <c r="V21" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S21,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="W21" s="4">
         <f t="shared" si="3"/>
-        <v>40</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3429,11 +3474,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>115679.6399999998</v>
+        <v>117647.29999999981</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>3820.3600000002043</v>
+        <v>1852.7000000001863</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3448,11 +3493,11 @@
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1610.95</v>
+        <v>6149.3000000000011</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>3909.05</v>
+        <v>-629.30000000000109</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3484,11 +3529,11 @@
       </c>
       <c r="V22" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S22,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W22" s="4">
         <f t="shared" si="3"/>
-        <v>40</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -3504,11 +3549,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>179836.22999999972</v>
+        <v>189702.3299999997</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>10163.770000000281</v>
+        <v>297.67000000030384</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3523,11 +3568,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2872.65</v>
+        <v>2246</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>2117.35</v>
+        <v>2744</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3540,11 +3585,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>0</v>
+        <v>13758.8</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>0</v>
+        <v>-13758.8</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3559,11 +3604,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>55</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3579,11 +3624,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>113177.64999999991</v>
+        <v>119326.94999999985</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>26822.350000000093</v>
+        <v>20673.050000000148</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3598,11 +3643,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5396.91</v>
+        <v>1255.0500000000002</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>-1596.9099999999999</v>
+        <v>2544.9499999999998</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3623,11 +3668,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>33</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3643,11 +3688,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>111494.7899999996</v>
+        <v>111934.48999999958</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>28505.210000000399</v>
+        <v>28065.510000000417</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3662,11 +3707,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1172.0600000000002</v>
+        <v>127.96</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>1727.9399999999998</v>
+        <v>2772.04</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3687,11 +3732,11 @@
       </c>
       <c r="V25" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S25,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="3"/>
-        <v>47</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -3707,11 +3752,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>58166.910000000113</v>
+        <v>58216.910000000113</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>31833.089999999887</v>
+        <v>31783.089999999887</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3726,11 +3771,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2387.7000000000007</v>
+        <v>0</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>1142.2999999999993</v>
+        <v>3530</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3751,11 +3796,11 @@
       </c>
       <c r="V26" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S26,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="3"/>
-        <v>31</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -3771,11 +3816,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>210407.45999999944</v>
+        <v>212205.35999999943</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>24592.540000000561</v>
+        <v>22794.640000000567</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3790,11 +3835,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>510.9</v>
+        <v>905.05</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>2349.1</v>
+        <v>1954.95</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3822,11 +3867,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>297412.17000000016</v>
+        <v>299954.80999999912</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>17587.829999999842</v>
+        <v>15045.190000000875</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -3868,11 +3913,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>155370.25999999998</v>
+        <v>156397.05999999997</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>11629.74000000002</v>
+        <v>10602.940000000031</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -3925,11 +3970,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>122958.22999999979</v>
+        <v>125752.37999999979</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>9041.7700000002078</v>
+        <v>6247.6200000002136</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -3942,11 +3987,11 @@
       </c>
       <c r="J30" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>663421.19500000414</v>
+        <v>663421.19500000367</v>
       </c>
       <c r="K30" s="7">
         <f>I30-J30</f>
-        <v>36578.80499999586</v>
+        <v>36578.804999996326</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -3985,11 +4030,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>142794.87999999989</v>
+        <v>143918.5799999999</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>24205.120000000112</v>
+        <v>23081.4200000001</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4002,11 +4047,11 @@
       </c>
       <c r="J31" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>656169.61500000302</v>
+        <v>656169.6150000029</v>
       </c>
       <c r="K31" s="7">
         <f t="shared" ref="K31:K33" si="4">I31-J31</f>
-        <v>43830.384999996983</v>
+        <v>43830.384999997099</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4045,11 +4090,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>255366.7399999997</v>
+        <v>268610.25999999978</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>-366.73999999969965</v>
+        <v>-13610.259999999776</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4062,11 +4107,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>638943.71500000253</v>
+        <v>639421.15500000201</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" si="4"/>
-        <v>61056.284999997471</v>
+        <v>60578.844999997993</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4085,11 +4130,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" ref="W32" si="5">U32-V32</f>
-        <v>185</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4105,11 +4150,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>69502.410000000033</v>
+        <v>69637.45000000007</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>30497.589999999967</v>
+        <v>30362.54999999993</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4122,11 +4167,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>0</v>
+        <v>61905.100000000035</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>700000</v>
+        <v>638094.89999999991</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4154,11 +4199,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>47169.730000000069</v>
+        <v>47176.690000000068</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>7830.2699999999313</v>
+        <v>7823.3099999999322</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4192,11 +4237,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>72817.384999999951</v>
+        <v>74072.434999999925</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>-2817.3849999999511</v>
+        <v>-4072.4349999999249</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4357,11 +4402,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1329222.1149999904</v>
+        <v>1329699.5549999904</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" si="6"/>
-        <v>48277.885000009555</v>
+        <v>47800.445000009611</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4393,11 +4438,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>0</v>
+        <v>75663.900000000023</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>1377500</v>
+        <v>1301836.1000000001</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 29/06/2026 11:01
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176EDCF5-9247-4B3E-865F-9EA65D383C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78454C2E-8BA3-4689-AA83-21C16F6278C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1011,7 +1011,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>905.05</v>
+            <v>2597.15</v>
           </cell>
         </row>
         <row r="6">
@@ -1019,13 +1019,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F6">
-            <v>53806.12999999999</v>
+            <v>55498.229999999981</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>5445.0999999999995</v>
+            <v>11519.449999999995</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1036,13 +1036,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>303072.33999999979</v>
+            <v>309146.68999999965</v>
           </cell>
           <cell r="H7" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>2246</v>
+            <v>2893.3999999999996</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1062,7 +1062,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>9428.2999999999993</v>
+            <v>13191.099999999993</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1076,13 +1076,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>79459.759999999835</v>
+            <v>80107.159999999829</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>2886.37</v>
+            <v>3696.97</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
@@ -1096,7 +1096,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>245781.73999999953</v>
+            <v>249544.53999999946</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE</v>
@@ -1108,7 +1108,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>43</v>
+            <v>44</v>
           </cell>
         </row>
         <row r="11">
@@ -1116,13 +1116,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>69283.180000000022</v>
+            <v>70093.780000000028</v>
           </cell>
           <cell r="H11" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>9866.0999999999985</v>
+            <v>11456.96</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1162,7 +1162,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>439.70000000000005</v>
+            <v>7425.8999999999969</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1176,19 +1176,19 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>779822.08000000007</v>
+            <v>788142.08000000007</v>
           </cell>
           <cell r="H14" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>1797.8999999999999</v>
+            <v>932.5</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>47</v>
+            <v>48</v>
           </cell>
         </row>
         <row r="15">
@@ -1199,10 +1199,10 @@
             <v>111572.95000000007</v>
           </cell>
           <cell r="H15" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>2394.44</v>
+            <v>7526.18</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1219,10 +1219,10 @@
             <v>531685.79000000039</v>
           </cell>
           <cell r="H16" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>2628.95</v>
+            <v>15086.365000000003</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1236,13 +1236,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>389719.22000000038</v>
+            <v>401853.62000000034</v>
           </cell>
           <cell r="H17" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I17">
-            <v>1123.7</v>
+            <v>2643.65</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1259,10 +1259,10 @@
             <v>117647.29999999981</v>
           </cell>
           <cell r="H18" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I18">
-            <v>13243.519999999997</v>
+            <v>3887.9</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1276,19 +1276,19 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>189702.3299999997</v>
+            <v>191293.18999999965</v>
           </cell>
           <cell r="H19" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I19">
-            <v>127.96</v>
+            <v>17269.02</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>76</v>
+            <v>77</v>
           </cell>
         </row>
         <row r="20">
@@ -1299,10 +1299,10 @@
             <v>119326.94999999985</v>
           </cell>
           <cell r="H20" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC</v>
           </cell>
           <cell r="I20">
-            <v>1255.0500000000002</v>
+            <v>2180.46</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
@@ -1316,13 +1316,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>111934.48999999958</v>
+            <v>118920.68999999955</v>
           </cell>
           <cell r="H21" t="str">
-            <v>Total Geral</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I21">
-            <v>61905.099999999984</v>
+            <v>1476.5000000000002</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
@@ -1336,7 +1336,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>58216.910000000113</v>
+            <v>59149.410000000113</v>
+          </cell>
+          <cell r="H22" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I22">
+            <v>5819.0099999999993</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
@@ -1350,7 +1356,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>212205.35999999943</v>
+            <v>217933.63999999937</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I23">
+            <v>117719.47500000003</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
@@ -1364,7 +1376,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>299954.80999999912</v>
+            <v>312646.7350000001</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
@@ -1384,7 +1396,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>713</v>
+            <v>716</v>
           </cell>
         </row>
         <row r="26">
@@ -1392,7 +1404,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>125752.37999999979</v>
+            <v>125767.0799999998</v>
           </cell>
         </row>
         <row r="27">
@@ -1400,7 +1412,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>143918.5799999999</v>
+            <v>146682.77999999988</v>
           </cell>
         </row>
         <row r="28">
@@ -1408,7 +1420,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>268610.25999999978</v>
+            <v>272635.7599999996</v>
           </cell>
         </row>
         <row r="29">
@@ -1416,7 +1428,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>69637.45000000007</v>
+            <v>71689.950000000041</v>
           </cell>
         </row>
         <row r="30">
@@ -1424,7 +1436,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>47176.690000000068</v>
+            <v>48653.190000000075</v>
           </cell>
         </row>
         <row r="31">
@@ -1432,7 +1444,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>74072.434999999925</v>
+            <v>78636.394999999931</v>
           </cell>
         </row>
         <row r="32">
@@ -1440,7 +1452,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>5070405.4449999304</v>
+            <v>5146674.2199999336</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2353,7 +2365,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>5070405.4449999975</v>
+        <v>5146674.2199999979</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2364,7 +2376,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>61905.100000000006</v>
+        <v>117719.47499999998</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2386,7 +2398,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2398,7 +2410,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>436594.5550000025</v>
+        <v>360325.78000000212</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2409,7 +2421,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>88114.9</v>
+        <v>32300.525000000023</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2431,7 +2443,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>-7</v>
+        <v>-10</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2443,7 +2455,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.92072007354276331</v>
+        <v>0.93456949700381298</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2454,7 +2466,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.41264564724703379</v>
+        <v>0.78469187441674426</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2476,7 +2488,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>1.0099150141643058</v>
+        <v>1.0141643059490084</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2575,11 +2587,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>53806.12999999999</v>
+        <v>55498.229999999981</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>10693.87000000001</v>
+        <v>9001.7700000000186</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2594,11 +2606,11 @@
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2394.44</v>
+        <v>15086.365000000003</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>12225.56</v>
+        <v>-466.36500000000342</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2649,11 +2661,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>303072.33999999979</v>
+        <v>309146.68999999965</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E35" si="0">C11-D11</f>
-        <v>16927.660000000207</v>
+        <v>10853.310000000347</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2668,11 +2680,11 @@
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1797.8999999999999</v>
+        <v>7526.18</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K27" si="1">I11-J11</f>
-        <v>15202.1</v>
+        <v>9473.82</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2745,11 +2757,11 @@
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2628.95</v>
+        <v>2643.65</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>3161.05</v>
+        <v>3146.35</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2783,11 +2795,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>-6</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2803,11 +2815,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>79459.759999999835</v>
+        <v>80107.159999999829</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>9540.2400000001653</v>
+        <v>8892.8400000001711</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2822,11 +2834,11 @@
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>13243.519999999997</v>
+        <v>17269.02</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>606.4800000000032</v>
+        <v>-3419.0200000000004</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2880,11 +2892,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>245781.73999999953</v>
+        <v>249544.53999999946</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>24218.260000000475</v>
+        <v>20455.460000000545</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2899,11 +2911,11 @@
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>439.70000000000005</v>
+        <v>7425.8999999999969</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>7250.3</v>
+        <v>264.10000000000309</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -2957,11 +2969,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>69283.180000000022</v>
+        <v>70093.780000000028</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>7716.8199999999779</v>
+        <v>6906.2199999999721</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2976,11 +2988,11 @@
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5445.0999999999995</v>
+        <v>11519.449999999995</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>12554.900000000001</v>
+        <v>6480.5500000000047</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3053,11 +3065,11 @@
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1123.7</v>
+        <v>3887.9</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>6166.3</v>
+        <v>3402.1</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3130,11 +3142,11 @@
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>932.5</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>5920</v>
+        <v>4987.5</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3168,11 +3180,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3188,11 +3200,11 @@
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>779822.08000000007</v>
+        <v>788142.08000000007</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>170177.91999999993</v>
+        <v>161857.91999999993</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3271,11 +3283,11 @@
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9866.0999999999985</v>
+        <v>11456.96</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>1133.9000000000015</v>
+        <v>-456.95999999999913</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3304,11 +3316,11 @@
       </c>
       <c r="V19" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="3"/>
-        <v>-19</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3343,11 +3355,11 @@
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>9428.2999999999993</v>
+        <v>13191.099999999993</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>5431.7000000000007</v>
+        <v>1668.9000000000069</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3399,11 +3411,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>389719.22000000038</v>
+        <v>401853.62000000034</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>20280.77999999962</v>
+        <v>8146.3799999996554</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3418,11 +3430,11 @@
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2886.37</v>
+        <v>3696.97</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>823.63000000000011</v>
+        <v>13.0300000000002</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3549,11 +3561,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>189702.3299999997</v>
+        <v>191293.18999999965</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>297.67000000030384</v>
+        <v>-1293.1899999996531</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3568,11 +3580,11 @@
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2246</v>
+        <v>2893.3999999999996</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>2744</v>
+        <v>2096.6000000000004</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3585,11 +3597,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>13758.8</v>
+        <v>34213.199999999997</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-13758.8</v>
+        <v>-34213.199999999997</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3643,11 +3655,11 @@
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1255.0500000000002</v>
+        <v>5819.0099999999993</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>2544.9499999999998</v>
+        <v>-2019.0099999999993</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3688,11 +3700,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>111934.48999999958</v>
+        <v>118920.68999999955</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>28065.510000000417</v>
+        <v>21079.310000000449</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3707,11 +3719,11 @@
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>127.96</v>
+        <v>2180.46</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>2772.04</v>
+        <v>719.54</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3752,11 +3764,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>58216.910000000113</v>
+        <v>59149.410000000113</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>31783.089999999887</v>
+        <v>30850.589999999887</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3771,11 +3783,11 @@
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>0</v>
+        <v>1476.5000000000002</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>3530</v>
+        <v>2053.5</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3816,11 +3828,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>212205.35999999943</v>
+        <v>217933.63999999937</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>22794.640000000567</v>
+        <v>17066.360000000626</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3835,11 +3847,11 @@
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>905.05</v>
+        <v>2597.15</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>1954.95</v>
+        <v>262.84999999999991</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3867,11 +3879,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>299954.80999999912</v>
+        <v>312646.7350000001</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>15045.190000000875</v>
+        <v>2353.2649999998976</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -3970,11 +3982,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>125752.37999999979</v>
+        <v>125767.0799999998</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>6247.6200000002136</v>
+        <v>6232.920000000202</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -3987,11 +3999,11 @@
       </c>
       <c r="J30" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>663421.19500000367</v>
+        <v>663421.19500000402</v>
       </c>
       <c r="K30" s="7">
         <f>I30-J30</f>
-        <v>36578.804999996326</v>
+        <v>36578.804999995977</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -4030,11 +4042,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>143918.5799999999</v>
+        <v>146682.77999999988</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>23081.4200000001</v>
+        <v>20317.220000000118</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4047,11 +4059,11 @@
       </c>
       <c r="J31" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>656169.6150000029</v>
+        <v>656169.61500000302</v>
       </c>
       <c r="K31" s="7">
         <f t="shared" ref="K31:K33" si="4">I31-J31</f>
-        <v>43830.384999997099</v>
+        <v>43830.384999996983</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4090,11 +4102,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>268610.25999999978</v>
+        <v>272635.7599999996</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>-13610.259999999776</v>
+        <v>-17635.759999999602</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4107,11 +4119,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>639421.15500000201</v>
+        <v>639421.15500000236</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" si="4"/>
-        <v>60578.844999997993</v>
+        <v>60578.844999997644</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4130,11 +4142,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" ref="W32" si="5">U32-V32</f>
-        <v>169</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4150,11 +4162,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>69637.45000000007</v>
+        <v>71689.950000000041</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>30362.54999999993</v>
+        <v>28310.049999999959</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4167,11 +4179,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>61905.100000000035</v>
+        <v>117719.47499999993</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>638094.89999999991</v>
+        <v>582280.52500000002</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4199,11 +4211,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>47176.690000000068</v>
+        <v>48653.190000000075</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>7823.3099999999322</v>
+        <v>6346.8099999999249</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4237,11 +4249,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>74072.434999999925</v>
+        <v>78636.394999999931</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>-4072.4349999999249</v>
+        <v>-8636.3949999999313</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4366,11 +4378,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1280088.9749999936</v>
+        <v>1280088.9749999931</v>
       </c>
       <c r="E39" s="7">
         <f t="shared" ref="E39:E41" si="6">C39-D39</f>
-        <v>97411.025000006426</v>
+        <v>97411.025000006892</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4402,11 +4414,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1329699.5549999904</v>
+        <v>1329699.5549999899</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" si="6"/>
-        <v>47800.445000009611</v>
+        <v>47800.445000010077</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4438,11 +4450,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>75663.900000000023</v>
+        <v>151932.67499999981</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>1301836.1000000001</v>
+        <v>1225567.3250000002</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 30/06/2026 11:22
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78454C2E-8BA3-4689-AA83-21C16F6278C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF2290D-B86A-4643-822C-D7DA763432B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-06-29T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-06-30T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -969,7 +969,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>29/06/2026</v>
+            <v>30/06/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1011,7 +1011,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>2597.15</v>
+            <v>2395.8999999999996</v>
           </cell>
         </row>
         <row r="6">
@@ -1019,13 +1019,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F6">
-            <v>55498.229999999981</v>
+            <v>57827.579999999987</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>11519.449999999995</v>
+            <v>11082.49</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1036,13 +1036,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>309146.68999999965</v>
+            <v>327909.82</v>
           </cell>
           <cell r="H7" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>2893.3999999999996</v>
+            <v>753.32999999999993</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1062,13 +1062,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>13191.099999999993</v>
+            <v>5101.7999999999993</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="N8">
-            <v>31</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="9">
@@ -1076,19 +1076,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>80107.159999999829</v>
+            <v>91188.049999999756</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>3696.97</v>
+            <v>5537.7</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>42</v>
+            <v>43</v>
           </cell>
         </row>
         <row r="10">
@@ -1096,19 +1096,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>249544.53999999946</v>
+            <v>261579.74999999942</v>
           </cell>
           <cell r="H10" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="I10">
-            <v>1967.66</v>
+            <v>4315.3400000000011</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>44</v>
+            <v>45</v>
           </cell>
         </row>
         <row r="11">
@@ -1116,19 +1116,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>70093.780000000028</v>
+            <v>77457.680000000008</v>
           </cell>
           <cell r="H11" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>11456.96</v>
+            <v>5515.67</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>57</v>
+            <v>59</v>
           </cell>
         </row>
         <row r="12">
@@ -1136,19 +1136,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>268215.93</v>
+            <v>294463.91000000003</v>
           </cell>
           <cell r="H12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>6149.3000000000011</v>
+            <v>4254.6000000000004</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N12">
-            <v>30</v>
+            <v>31</v>
           </cell>
         </row>
         <row r="13">
@@ -1156,19 +1156,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>242195.78999999995</v>
+            <v>260664.58999999985</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>7425.8999999999969</v>
+            <v>9172.1899999999969</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>40</v>
+            <v>45</v>
           </cell>
         </row>
         <row r="14">
@@ -1176,19 +1176,19 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>788142.08000000007</v>
+            <v>791214.48000000033</v>
           </cell>
           <cell r="H14" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>932.5</v>
+            <v>2764.650000000001</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>48</v>
+            <v>52</v>
           </cell>
         </row>
         <row r="15">
@@ -1196,13 +1196,13 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>111572.95000000007</v>
+            <v>145987.65000000005</v>
           </cell>
           <cell r="H15" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="I15">
-            <v>7526.18</v>
+            <v>5165.01</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1216,13 +1216,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>531685.79000000039</v>
+            <v>593931.99000000057</v>
           </cell>
           <cell r="H16" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I16">
-            <v>15086.365000000003</v>
+            <v>7109.83</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1236,19 +1236,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>401853.62000000034</v>
+            <v>421921.62000000034</v>
           </cell>
           <cell r="H17" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I17">
-            <v>2643.65</v>
+            <v>1663.0800000000002</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>35</v>
+            <v>36</v>
           </cell>
         </row>
         <row r="18">
@@ -1256,13 +1256,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>117647.29999999981</v>
+            <v>124398.08999999975</v>
           </cell>
           <cell r="H18" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I18">
-            <v>3887.9</v>
+            <v>7870.6399999999976</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -1276,13 +1276,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>191293.18999999965</v>
+            <v>202577.55999999959</v>
           </cell>
           <cell r="H19" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I19">
-            <v>17269.02</v>
+            <v>10082.51</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1296,19 +1296,19 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>119326.94999999985</v>
+            <v>129970.30999999981</v>
           </cell>
           <cell r="H20" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I20">
-            <v>2180.46</v>
+            <v>1513.7</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N20">
-            <v>36</v>
+            <v>39</v>
           </cell>
         </row>
         <row r="21">
@@ -1316,13 +1316,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>118920.68999999955</v>
+            <v>145768.56999999966</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SJC/VALE</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I21">
-            <v>1476.5000000000002</v>
+            <v>637.20000000000005</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
@@ -1336,19 +1336,19 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>59149.410000000113</v>
+            <v>65200.350000000108</v>
           </cell>
           <cell r="H22" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I22">
-            <v>5819.0099999999993</v>
+            <v>84935.640000000014</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
           </cell>
           <cell r="N22">
-            <v>43</v>
+            <v>44</v>
           </cell>
         </row>
         <row r="23">
@@ -1356,19 +1356,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>217933.63999999937</v>
-          </cell>
-          <cell r="H23" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I23">
-            <v>117719.47500000003</v>
+            <v>235429.209999999</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N23">
-            <v>30</v>
+            <v>33</v>
           </cell>
         </row>
         <row r="24">
@@ -1376,7 +1370,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>312646.7350000001</v>
+            <v>324357.91499999986</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
@@ -1390,13 +1384,13 @@
             <v>PIRACICABA</v>
           </cell>
           <cell r="F25">
-            <v>156397.05999999997</v>
+            <v>198284.66000000003</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>716</v>
+            <v>739</v>
           </cell>
         </row>
         <row r="26">
@@ -1404,7 +1398,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>125767.0799999998</v>
+            <v>131226.43999999974</v>
           </cell>
         </row>
         <row r="27">
@@ -1412,7 +1406,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>146682.77999999988</v>
+            <v>156981.61999999979</v>
           </cell>
         </row>
         <row r="28">
@@ -1420,7 +1414,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>272635.7599999996</v>
+            <v>288150.54999999981</v>
           </cell>
         </row>
         <row r="29">
@@ -1428,7 +1422,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>71689.950000000041</v>
+            <v>78085.370000000039</v>
           </cell>
         </row>
         <row r="30">
@@ -1436,7 +1430,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>48653.190000000075</v>
+            <v>49944.060000000078</v>
           </cell>
         </row>
         <row r="31">
@@ -1444,7 +1438,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>78636.394999999931</v>
+            <v>80321.314999999915</v>
           </cell>
         </row>
         <row r="32">
@@ -1452,7 +1446,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>5146674.2199999336</v>
+            <v>5536080.6699999217</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -1471,7 +1465,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="R35">
-            <v>49116.749999999993</v>
+            <v>49116.749999999985</v>
           </cell>
         </row>
         <row r="36">
@@ -2331,7 +2325,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>150020</v>
+        <v>250000</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -2365,7 +2359,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>5146674.2199999979</v>
+        <v>5536080.6699999981</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2376,7 +2370,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>117719.47499999998</v>
+        <v>84935.639999999985</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2398,7 +2392,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(Tabela11[ATINGIDO])</f>
-        <v>716</v>
+        <v>739</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2410,7 +2404,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>360325.78000000212</v>
+        <v>-29080.669999998063</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2421,7 +2415,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>32300.525000000023</v>
+        <v>165064.36000000002</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2443,7 +2437,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>-10</v>
+        <v>-33</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2455,7 +2449,7 @@
       </c>
       <c r="C7" s="3">
         <f>C5/C4</f>
-        <v>0.93456949700381298</v>
+        <v>1.0052806736880331</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2466,7 +2460,7 @@
       </c>
       <c r="I7" s="3">
         <f>I5/I4</f>
-        <v>0.78469187441674426</v>
+        <v>0.33974255999999992</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2488,7 +2482,7 @@
       </c>
       <c r="U7" s="3">
         <f>U5/U4</f>
-        <v>1.0141643059490084</v>
+        <v>1.046742209631728</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -2587,11 +2581,11 @@
       </c>
       <c r="D10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>55498.229999999981</v>
+        <v>57827.579999999987</v>
       </c>
       <c r="E10" s="7">
         <f>C10-D10</f>
-        <v>9001.7700000000186</v>
+        <v>6672.4200000000128</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
@@ -2602,15 +2596,15 @@
       </c>
       <c r="I10" s="2">
         <f>_xlfn.XLOOKUP(G10,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14620</v>
+        <v>21000</v>
       </c>
       <c r="J10" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G10,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>15086.365000000003</v>
+        <v>7109.83</v>
       </c>
       <c r="K10" s="7">
         <f>I10-J10</f>
-        <v>-466.36500000000342</v>
+        <v>13890.17</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -2641,11 +2635,11 @@
       </c>
       <c r="V10" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W10" s="4">
         <f>U10-V10</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -2661,11 +2655,11 @@
       </c>
       <c r="D11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>309146.68999999965</v>
+        <v>327909.82</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" ref="E11:E35" si="0">C11-D11</f>
-        <v>10853.310000000347</v>
+        <v>-7909.820000000007</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
@@ -2676,15 +2670,15 @@
       </c>
       <c r="I11" s="2">
         <f>_xlfn.XLOOKUP(G11,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>17000</v>
+        <v>11800</v>
       </c>
       <c r="J11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G11,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7526.18</v>
+        <v>5165.01</v>
       </c>
       <c r="K11" s="7">
         <f t="shared" ref="K11:K27" si="1">I11-J11</f>
-        <v>9473.82</v>
+        <v>6634.99</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -2718,11 +2712,11 @@
       </c>
       <c r="V11" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" ref="W11:W26" si="3">U11-V11</f>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2753,15 +2747,15 @@
       </c>
       <c r="I12" s="2">
         <f>_xlfn.XLOOKUP(G12,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5790</v>
+        <v>11500</v>
       </c>
       <c r="J12" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G12,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2643.65</v>
+        <v>1663.0800000000002</v>
       </c>
       <c r="K12" s="7">
         <f t="shared" si="1"/>
-        <v>3146.35</v>
+        <v>9836.92</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -2795,11 +2789,11 @@
       </c>
       <c r="V12" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="3"/>
-        <v>-7</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -2815,11 +2809,11 @@
       </c>
       <c r="D13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>80107.159999999829</v>
+        <v>91188.049999999756</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>8892.8400000001711</v>
+        <v>-2188.0499999997555</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
@@ -2830,15 +2824,15 @@
       </c>
       <c r="I13" s="2">
         <f>_xlfn.XLOOKUP(G13,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13850</v>
+        <v>18500</v>
       </c>
       <c r="J13" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G13,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>17269.02</v>
+        <v>10082.51</v>
       </c>
       <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v>-3419.0200000000004</v>
+        <v>8417.49</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -2872,11 +2866,11 @@
       </c>
       <c r="V13" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="3"/>
-        <v>-2</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -2892,11 +2886,11 @@
       </c>
       <c r="D14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>249544.53999999946</v>
+        <v>261579.74999999942</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>20455.460000000545</v>
+        <v>8420.2500000005821</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
@@ -2907,15 +2901,15 @@
       </c>
       <c r="I14" s="2">
         <f>_xlfn.XLOOKUP(G14,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>7690</v>
+        <v>9000</v>
       </c>
       <c r="J14" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G14,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>7425.8999999999969</v>
+        <v>9172.1899999999969</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>264.10000000000309</v>
+        <v>-172.18999999999687</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -2949,11 +2943,11 @@
       </c>
       <c r="V14" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="W14" s="4">
         <f>U14-V14</f>
-        <v>-7</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -2969,11 +2963,11 @@
       </c>
       <c r="D15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>70093.780000000028</v>
+        <v>77457.680000000008</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v>6906.2199999999721</v>
+        <v>-457.68000000000757</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
@@ -2984,15 +2978,15 @@
       </c>
       <c r="I15" s="2">
         <f>_xlfn.XLOOKUP(G15,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>18000</v>
+        <v>21000</v>
       </c>
       <c r="J15" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G15,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11519.449999999995</v>
+        <v>11082.49</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
-        <v>6480.5500000000047</v>
+        <v>9917.51</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3026,11 +3020,11 @@
       </c>
       <c r="V15" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3046,11 +3040,11 @@
       </c>
       <c r="D16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>268215.93</v>
+        <v>294463.91000000003</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v>56784.070000000007</v>
+        <v>30536.089999999967</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
@@ -3061,15 +3055,15 @@
       </c>
       <c r="I16" s="2">
         <f>_xlfn.XLOOKUP(G16,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>7290</v>
+        <v>18889</v>
       </c>
       <c r="J16" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G16,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3887.9</v>
+        <v>7870.6399999999976</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
-        <v>3402.1</v>
+        <v>11018.360000000002</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3103,11 +3097,11 @@
       </c>
       <c r="V16" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3123,11 +3117,11 @@
       </c>
       <c r="D17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>242195.78999999995</v>
+        <v>260664.58999999985</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>-82195.78999999995</v>
+        <v>-100664.58999999985</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
@@ -3138,15 +3132,15 @@
       </c>
       <c r="I17" s="2">
         <f>_xlfn.XLOOKUP(G17,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5920</v>
+        <v>28564</v>
       </c>
       <c r="J17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G17,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>932.5</v>
+        <v>2764.650000000001</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>4987.5</v>
+        <v>25799.35</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3161,11 +3155,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(Tabela8[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$P$34:$P$39,'[1]BASE PYTHON'!$R$34:$R$39),0)</f>
-        <v>49116.749999999993</v>
+        <v>49116.749999999985</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="2"/>
-        <v>-49116.749999999993</v>
+        <v>-49116.749999999985</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="4" t="s">
@@ -3180,11 +3174,11 @@
       </c>
       <c r="V17" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="3"/>
-        <v>-3</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3200,11 +3194,11 @@
       </c>
       <c r="D18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>788142.08000000007</v>
+        <v>791214.48000000033</v>
       </c>
       <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v>161857.91999999993</v>
+        <v>158785.51999999967</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
@@ -3215,15 +3209,15 @@
       </c>
       <c r="I18" s="2">
         <f>_xlfn.XLOOKUP(G18,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6690</v>
+        <v>6000</v>
       </c>
       <c r="J18" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G18,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1967.66</v>
+        <v>4315.3400000000011</v>
       </c>
       <c r="K18" s="7">
         <f t="shared" si="1"/>
-        <v>4722.34</v>
+        <v>1684.6599999999989</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3264,11 +3258,11 @@
       </c>
       <c r="D19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>111572.95000000007</v>
+        <v>145987.65000000005</v>
       </c>
       <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v>13427.04999999993</v>
+        <v>-20987.650000000052</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
@@ -3279,15 +3273,15 @@
       </c>
       <c r="I19" s="2">
         <f>_xlfn.XLOOKUP(G19,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11000</v>
+        <v>16200</v>
       </c>
       <c r="J19" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G19,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>11456.96</v>
+        <v>5515.67</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>-456.95999999999913</v>
+        <v>10684.33</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3336,11 +3330,11 @@
       </c>
       <c r="D20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>531685.79000000039</v>
+        <v>593931.99000000057</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="0"/>
-        <v>8314.2099999996135</v>
+        <v>-53931.990000000573</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
@@ -3351,15 +3345,15 @@
       </c>
       <c r="I20" s="2">
         <f>_xlfn.XLOOKUP(G20,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14860</v>
+        <v>14522</v>
       </c>
       <c r="J20" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G20,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>13191.099999999993</v>
+        <v>5101.7999999999993</v>
       </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>1668.9000000000069</v>
+        <v>9420.2000000000007</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3411,11 +3405,11 @@
       </c>
       <c r="D21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A21,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>401853.62000000034</v>
+        <v>421921.62000000034</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" si="0"/>
-        <v>8146.3799999996554</v>
+        <v>-11921.620000000345</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
@@ -3426,15 +3420,15 @@
       </c>
       <c r="I21" s="2">
         <f>_xlfn.XLOOKUP(G21,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3710</v>
+        <v>6080</v>
       </c>
       <c r="J21" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G21,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>3696.97</v>
+        <v>5537.7</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>13.0300000000002</v>
+        <v>542.30000000000018</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3466,11 +3460,11 @@
       </c>
       <c r="V21" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S21,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="W21" s="4">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3486,11 +3480,11 @@
       </c>
       <c r="D22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A22,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>117647.29999999981</v>
+        <v>124398.08999999975</v>
       </c>
       <c r="E22" s="7">
         <f t="shared" si="0"/>
-        <v>1852.7000000001863</v>
+        <v>-4898.0899999997491</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
@@ -3501,15 +3495,15 @@
       </c>
       <c r="I22" s="2">
         <f>_xlfn.XLOOKUP(G22,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5520</v>
+        <v>15284</v>
       </c>
       <c r="J22" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G22,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>6149.3000000000011</v>
+        <v>4254.6000000000004</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>-629.30000000000109</v>
+        <v>11029.4</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3561,11 +3555,11 @@
       </c>
       <c r="D23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A23,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>191293.18999999965</v>
+        <v>202577.55999999959</v>
       </c>
       <c r="E23" s="7">
         <f t="shared" si="0"/>
-        <v>-1293.1899999996531</v>
+        <v>-12577.55999999959</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
@@ -3576,15 +3570,15 @@
       </c>
       <c r="I23" s="2">
         <f>_xlfn.XLOOKUP(G23,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4990</v>
+        <v>5300</v>
       </c>
       <c r="J23" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G23,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2893.3999999999996</v>
+        <v>753.32999999999993</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>2096.6000000000004</v>
+        <v>4546.67</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -3597,11 +3591,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>34213.199999999997</v>
+        <v>240618.88000000024</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-34213.199999999997</v>
+        <v>-240618.88000000024</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
@@ -3616,11 +3610,11 @@
       </c>
       <c r="V23" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S23,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W23" s="4">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -3636,11 +3630,11 @@
       </c>
       <c r="D24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A24,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>119326.94999999985</v>
+        <v>129970.30999999981</v>
       </c>
       <c r="E24" s="7">
         <f t="shared" si="0"/>
-        <v>20673.050000000148</v>
+        <v>10029.690000000192</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
@@ -3651,15 +3645,15 @@
       </c>
       <c r="I24" s="2">
         <f>_xlfn.XLOOKUP(G24,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3800</v>
+        <v>5980</v>
       </c>
       <c r="J24" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G24,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>5819.0099999999993</v>
+        <v>637.20000000000005</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>-2019.0099999999993</v>
+        <v>5342.8</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -3680,11 +3674,11 @@
       </c>
       <c r="V24" s="4">
         <f>IFERROR(_xlfn.XLOOKUP(S24,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N),0)</f>
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -3700,11 +3694,11 @@
       </c>
       <c r="D25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A25,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>118920.68999999955</v>
+        <v>145768.56999999966</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
-        <v>21079.310000000449</v>
+        <v>-5768.5699999996577</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
@@ -3715,15 +3709,15 @@
       </c>
       <c r="I25" s="2">
         <f>_xlfn.XLOOKUP(G25,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2900</v>
+        <v>24428</v>
       </c>
       <c r="J25" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G25,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2180.46</v>
+        <v>1513.7</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
-        <v>719.54</v>
+        <v>22914.3</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -3764,11 +3758,11 @@
       </c>
       <c r="D26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A26,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>59149.410000000113</v>
+        <v>65200.350000000108</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="0"/>
-        <v>30850.589999999887</v>
+        <v>24799.649999999892</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
@@ -3779,15 +3773,15 @@
       </c>
       <c r="I26" s="2">
         <f>_xlfn.XLOOKUP(G26,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3530</v>
+        <v>6070</v>
       </c>
       <c r="J26" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G26,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>1476.5000000000002</v>
+        <v>0</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>2053.5</v>
+        <v>6070</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -3828,11 +3822,11 @@
       </c>
       <c r="D27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A27,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>217933.63999999937</v>
+        <v>235429.209999999</v>
       </c>
       <c r="E27" s="7">
         <f t="shared" si="0"/>
-        <v>17066.360000000626</v>
+        <v>-429.20999999900232</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
@@ -3843,15 +3837,15 @@
       </c>
       <c r="I27" s="2">
         <f>_xlfn.XLOOKUP(G27,[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2860</v>
+        <v>9883</v>
       </c>
       <c r="J27" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(G27,'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I),0)</f>
-        <v>2597.15</v>
+        <v>2395.8999999999996</v>
       </c>
       <c r="K27" s="7">
         <f t="shared" si="1"/>
-        <v>262.84999999999991</v>
+        <v>7487.1</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -3879,11 +3873,11 @@
       </c>
       <c r="D28" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A28,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>312646.7350000001</v>
+        <v>324357.91499999986</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="0"/>
-        <v>2353.2649999998976</v>
+        <v>-9357.9149999998626</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -3925,11 +3919,11 @@
       </c>
       <c r="D29" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A29,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>156397.05999999997</v>
+        <v>198284.66000000003</v>
       </c>
       <c r="E29" s="7">
         <f t="shared" si="0"/>
-        <v>10602.940000000031</v>
+        <v>-31284.660000000033</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -3982,11 +3976,11 @@
       </c>
       <c r="D30" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A30,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>125767.0799999998</v>
+        <v>131226.43999999974</v>
       </c>
       <c r="E30" s="7">
         <f t="shared" si="0"/>
-        <v>6232.920000000202</v>
+        <v>773.56000000025961</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -3999,11 +3993,11 @@
       </c>
       <c r="J30" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>663421.19500000402</v>
+        <v>663421.19500000391</v>
       </c>
       <c r="K30" s="7">
         <f>I30-J30</f>
-        <v>36578.804999995977</v>
+        <v>36578.804999996093</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -4042,11 +4036,11 @@
       </c>
       <c r="D31" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A31,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>146682.77999999988</v>
+        <v>156981.61999999979</v>
       </c>
       <c r="E31" s="7">
         <f t="shared" si="0"/>
-        <v>20317.220000000118</v>
+        <v>10018.380000000208</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4102,11 +4096,11 @@
       </c>
       <c r="D32" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A32,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>272635.7599999996</v>
+        <v>288150.54999999981</v>
       </c>
       <c r="E32" s="7">
         <f t="shared" si="0"/>
-        <v>-17635.759999999602</v>
+        <v>-33150.549999999814</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4119,11 +4113,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>639421.15500000236</v>
+        <v>638766.7150000023</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" si="4"/>
-        <v>60578.844999997644</v>
+        <v>61233.284999997704</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4142,11 +4136,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" ref="W32" si="5">U32-V32</f>
-        <v>152</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4162,11 +4156,11 @@
       </c>
       <c r="D33" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A33,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>71689.950000000041</v>
+        <v>78085.370000000039</v>
       </c>
       <c r="E33" s="7">
         <f t="shared" si="0"/>
-        <v>28310.049999999959</v>
+        <v>21914.629999999961</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4179,11 +4173,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>117719.47499999993</v>
+        <v>301374.68500000052</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>582280.52500000002</v>
+        <v>398625.31499999948</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4211,11 +4205,11 @@
       </c>
       <c r="D34" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A34,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>48653.190000000075</v>
+        <v>49944.060000000078</v>
       </c>
       <c r="E34" s="7">
         <f t="shared" si="0"/>
-        <v>6346.8099999999249</v>
+        <v>5055.9399999999223</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4249,11 +4243,11 @@
       </c>
       <c r="D35" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A35,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F),0)</f>
-        <v>78636.394999999931</v>
+        <v>80321.314999999915</v>
       </c>
       <c r="E35" s="7">
         <f t="shared" si="0"/>
-        <v>-8636.3949999999313</v>
+        <v>-10321.314999999915</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4414,11 +4408,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1329699.5549999899</v>
+        <v>1329045.11499999</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" si="6"/>
-        <v>47800.445000010077</v>
+        <v>48454.885000010021</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4450,11 +4444,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>151932.67499999981</v>
+        <v>541993.56500000076</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="6"/>
-        <v>1225567.3250000002</v>
+        <v>835506.43499999924</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 06/07/2026 10:55
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B93E0F-29DA-421E-B28D-7BA2A845041C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7BA505-5B8D-464A-A478-0BD9F627A8FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1717,13 +1717,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>6084.98</v>
+            <v>7480.3299999999981</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>624.20000000000005</v>
+            <v>2019.55</v>
           </cell>
         </row>
         <row r="6">
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>53838.940000000024</v>
+            <v>57626.830000000038</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>10193.949999999999</v>
+            <v>13981.84</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1754,7 +1754,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I7">
-            <v>6185.04</v>
+            <v>7553.6399999999994</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1771,16 +1771,16 @@
             <v>33.020000000000003</v>
           </cell>
           <cell r="H8" t="str">
-            <v>LESTE PENHA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I8">
-            <v>3232.7</v>
+            <v>6364.44</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N8">
-            <v>16</v>
+            <v>17</v>
           </cell>
         </row>
         <row r="9">
@@ -1791,10 +1791,10 @@
             <v>8818.9</v>
           </cell>
           <cell r="H9" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I9">
-            <v>369.85</v>
+            <v>2964</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
@@ -1808,19 +1808,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>24653.96000000001</v>
+            <v>26022.560000000009</v>
           </cell>
           <cell r="H10" t="str">
-            <v>PIRACICABA</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I10">
-            <v>3604.26</v>
+            <v>11331</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N10">
-            <v>5</v>
+            <v>6</v>
           </cell>
         </row>
         <row r="11">
@@ -1828,13 +1828,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>10197.16</v>
+            <v>16561.600000000006</v>
           </cell>
           <cell r="H11" t="str">
-            <v>PIRITUBA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>1247.8000000000002</v>
+            <v>4935.5999999999995</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
@@ -1851,10 +1851,10 @@
             <v>61613.220000000016</v>
           </cell>
           <cell r="H12" t="str">
-            <v>Total Geral</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>25457.80000000001</v>
+            <v>5429.5999999999995</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
@@ -1870,11 +1870,17 @@
           <cell r="F13">
             <v>70798.399999999994</v>
           </cell>
+          <cell r="H13" t="str">
+            <v>LESTE TATUAPE</v>
+          </cell>
+          <cell r="I13">
+            <v>3237.6700000000005</v>
+          </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>7</v>
+            <v>9</v>
           </cell>
         </row>
         <row r="14">
@@ -1884,6 +1890,12 @@
           <cell r="F14">
             <v>58605.799999999988</v>
           </cell>
+          <cell r="H14" t="str">
+            <v>MOGI</v>
+          </cell>
+          <cell r="I14">
+            <v>1302.75</v>
+          </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
@@ -1898,11 +1910,17 @@
           <cell r="F15">
             <v>4900.4000000000005</v>
           </cell>
+          <cell r="H15" t="str">
+            <v>OSASCO</v>
+          </cell>
+          <cell r="I15">
+            <v>9669.82</v>
+          </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>13</v>
+            <v>16</v>
           </cell>
         </row>
         <row r="16">
@@ -1910,13 +1928,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>12290.6</v>
+            <v>15254.599999999995</v>
+          </cell>
+          <cell r="H16" t="str">
+            <v>PIRACICABA</v>
+          </cell>
+          <cell r="I16">
+            <v>3604.26</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N16">
-            <v>9</v>
+            <v>11</v>
           </cell>
         </row>
         <row r="17">
@@ -1924,13 +1948,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>58426.400000000001</v>
+            <v>69757.400000000009</v>
+          </cell>
+          <cell r="H17" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="I17">
+            <v>2849.65</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>2</v>
+            <v>4</v>
           </cell>
         </row>
         <row r="18">
@@ -1940,6 +1970,12 @@
           <cell r="F18">
             <v>11856.740000000002</v>
           </cell>
+          <cell r="H18" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="I18">
+            <v>5653.2</v>
+          </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
           </cell>
@@ -1952,13 +1988,19 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>13716.539999999995</v>
+            <v>18652.140000000007</v>
+          </cell>
+          <cell r="H19" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="I19">
+            <v>384</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>84</v>
+            <v>95</v>
           </cell>
         </row>
         <row r="20">
@@ -1966,7 +2008,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>19291.289999999997</v>
+            <v>21488.189999999995</v>
+          </cell>
+          <cell r="H20" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I20">
+            <v>1513.29</v>
           </cell>
         </row>
         <row r="21">
@@ -1974,7 +2022,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>8124.8499999999985</v>
+            <v>10992.669999999998</v>
+          </cell>
+          <cell r="H21" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I21">
+            <v>7272.37</v>
           </cell>
         </row>
         <row r="22">
@@ -1982,7 +2036,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>5814.2699999999986</v>
+            <v>7117.0199999999968</v>
+          </cell>
+          <cell r="H22" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I22">
+            <v>90066.679999999935</v>
           </cell>
         </row>
         <row r="23">
@@ -1998,7 +2058,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>38256.229999999996</v>
+            <v>47926.050000000025</v>
           </cell>
         </row>
         <row r="25">
@@ -2014,7 +2074,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>15213.400000000001</v>
+            <v>16815.25</v>
           </cell>
         </row>
         <row r="27">
@@ -2022,7 +2082,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>14246.68</v>
+            <v>19899.88</v>
           </cell>
         </row>
         <row r="28">
@@ -2030,7 +2090,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>23149.339999999993</v>
+            <v>23533.34</v>
           </cell>
         </row>
         <row r="29">
@@ -2046,7 +2106,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>4535.3800000000019</v>
+            <v>6048.670000000001</v>
           </cell>
         </row>
         <row r="31">
@@ -2054,7 +2114,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>7861.4900000000007</v>
+            <v>15133.860000000004</v>
           </cell>
         </row>
         <row r="32">
@@ -2062,7 +2122,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>577505.65000000212</v>
+            <v>642114.53000000212</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2915,7 +2975,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>577430.52999999991</v>
+        <v>642039.41</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2926,7 +2986,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>21853.54</v>
+        <v>72167.42</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2937,7 +2997,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>3604.26</v>
+        <v>17899.260000000002</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -2948,7 +3008,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2960,7 +3020,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>5014069.47</v>
+        <v>4949460.59</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2971,7 +3031,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>278298.46000000002</v>
+        <v>227984.58000000002</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2982,7 +3042,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-3604.26</v>
+        <v>-17899.260000000002</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -2993,7 +3053,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>674</v>
+        <v>663</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3005,7 +3065,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.10326934275239208</v>
+        <v>0.11482418134668693</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3016,7 +3076,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>7.2808243823129559E-2</v>
+        <v>0.24043624563554455</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3038,7 +3098,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.1108179419525066</v>
+        <v>0.12532981530343013</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3137,11 +3197,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>6084.98</v>
+        <v>7480.3299999999981</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>58415.020000000004</v>
+        <v>57019.67</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3156,11 +3216,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>9669.82</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>34823</v>
+        <v>25153.18</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3211,11 +3271,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>53838.940000000024</v>
+        <v>57626.830000000038</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>271161.06</v>
+        <v>267373.17</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3268,11 +3328,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3306,11 +3366,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1247.8000000000002</v>
+        <v>2849.65</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11525.2</v>
+        <v>9923.35</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3383,11 +3443,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>384</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>29550</v>
+        <v>29166</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3402,11 +3462,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>11331</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>0</v>
+        <v>-11331</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3441,11 +3501,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>24653.96000000001</v>
+        <v>26022.560000000009</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>248346.03999999998</v>
+        <v>246977.44</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3460,11 +3520,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>369.85</v>
+        <v>3237.6700000000005</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>21339.15</v>
+        <v>18471.329999999998</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3498,11 +3558,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3518,11 +3578,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>10197.16</v>
+        <v>16561.600000000006</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>67802.84</v>
+        <v>61438.399999999994</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3537,11 +3597,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10193.949999999999</v>
+        <v>13981.84</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>22612.050000000003</v>
+        <v>18824.16</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3556,11 +3616,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>2964</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-2964</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3614,11 +3674,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>5653.2</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>16187</v>
+        <v>10533.8</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3691,11 +3751,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1302.75</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4976</v>
+        <v>3673.25</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3832,11 +3892,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4935.5999999999995</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>16828</v>
+        <v>11892.400000000001</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3853,11 +3913,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3873,11 +3933,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>12290.6</v>
+        <v>15254.599999999995</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>547709.4</v>
+        <v>544745.4</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3892,11 +3952,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6185.04</v>
+        <v>7553.6399999999994</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15059.96</v>
+        <v>13691.36</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3945,11 +4005,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>58426.400000000001</v>
+        <v>69757.400000000009</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>356573.6</v>
+        <v>345242.6</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -3964,11 +4024,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>6364.44</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6246</v>
+        <v>-118.4399999999996</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -3981,11 +4041,11 @@
       </c>
       <c r="P21" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>275241.61999999994</v>
+        <v>275241.61999999988</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>96349.28909090918</v>
+        <v>96349.289090909238</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="19" t="s">
@@ -4000,11 +4060,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -4039,11 +4099,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3232.7</v>
+        <v>5429.5999999999995</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11483.3</v>
+        <v>9286.4000000000015</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4056,11 +4116,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>3604.26</v>
+        <v>17899.259999999998</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>491850.28545454546</v>
+        <v>477555.28545454546</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4075,11 +4135,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4095,11 +4155,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>13716.539999999995</v>
+        <v>18652.140000000007</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>181283.46</v>
+        <v>176347.86</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4170,11 +4230,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>19291.289999999997</v>
+        <v>21488.189999999995</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>120708.71</v>
+        <v>118511.81</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4189,11 +4249,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>7272.37</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10474</v>
+        <v>3201.63</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4245,11 +4305,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>8124.8499999999985</v>
+        <v>10992.669999999998</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>134375.15</v>
+        <v>131507.33000000002</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4300,11 +4360,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4320,11 +4380,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>5814.2699999999986</v>
+        <v>7117.0199999999968</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>84185.73</v>
+        <v>82882.98000000001</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4339,11 +4399,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1513.29</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5351</v>
+        <v>3837.71</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4403,11 +4463,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>624.20000000000005</v>
+        <v>2019.55</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5591.8</v>
+        <v>4196.45</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4430,11 +4490,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>38256.229999999996</v>
+        <v>47926.050000000025</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>280243.77</v>
+        <v>270573.94999999995</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4509,11 +4569,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>15213.400000000001</v>
+        <v>16815.25</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>119286.6</v>
+        <v>117684.75</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4566,11 +4626,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>14246.68</v>
+        <v>19899.88</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>152753.32</v>
+        <v>147100.12</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4583,11 +4643,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>262981.55</v>
+        <v>262981.54999999987</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>127768.45000000001</v>
+        <v>127768.45000000013</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4606,11 +4666,11 @@
       </c>
       <c r="V31" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="3">U31-V31</f>
-        <v>134.81818181818181</v>
+        <v>123.81818181818181</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4626,11 +4686,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>23149.339999999993</v>
+        <v>23533.34</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>236850.66</v>
+        <v>236466.66</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4643,11 +4703,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>21853.540000000008</v>
+        <v>67231.819999999992</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>499146.45999999996</v>
+        <v>453768.18</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4746,11 +4806,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>4535.3800000000019</v>
+        <v>6048.670000000001</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50464.619999999995</v>
+        <v>48951.33</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4806,11 +4866,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>7861.4900000000007</v>
+        <v>15133.860000000004</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65138.51</v>
+        <v>57866.14</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4928,11 +4988,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>552047.85000000091</v>
+        <v>552047.85000000172</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>-161297.85000000091</v>
+        <v>-161297.85000000172</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -4964,11 +5024,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>25457.80000000001</v>
+        <v>90066.679999999935</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="5">C40-D40</f>
-        <v>495542.2</v>
+        <v>430933.32000000007</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 13/07/2026 08:58
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7BA505-5B8D-464A-A478-0BD9F627A8FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F647E5-6A8E-4828-8BBA-A4F097B736A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-06T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-13T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1681,7 +1681,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>06/07/2026</v>
+            <v>13/07/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1717,13 +1717,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>7480.3299999999981</v>
+            <v>16835.900000000001</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>2019.55</v>
+            <v>365.4</v>
           </cell>
         </row>
         <row r="6">
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>57626.830000000038</v>
+            <v>121640.54999999996</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>13981.84</v>
+            <v>12313.9</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1748,13 +1748,13 @@
             <v>ECOMMERCE</v>
           </cell>
           <cell r="F7">
-            <v>75.12</v>
+            <v>488.70000000000005</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INTERLAGOS</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I7">
-            <v>7553.6399999999994</v>
+            <v>810.09999999999991</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1768,19 +1768,19 @@
             <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F8">
-            <v>33.020000000000003</v>
+            <v>49.09</v>
           </cell>
           <cell r="H8" t="str">
-            <v>JUNDIAI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I8">
-            <v>6364.44</v>
+            <v>5677.7</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N8">
-            <v>17</v>
+            <v>31</v>
           </cell>
         </row>
         <row r="9">
@@ -1788,19 +1788,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>8818.9</v>
+            <v>21547.7</v>
           </cell>
           <cell r="H9" t="str">
-            <v>KEY SP</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I9">
-            <v>2964</v>
+            <v>184.85000000000002</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N9">
-            <v>8</v>
+            <v>17</v>
           </cell>
         </row>
         <row r="10">
@@ -1808,19 +1808,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>26022.560000000009</v>
+            <v>69777.699999999983</v>
           </cell>
           <cell r="H10" t="str">
-            <v>KEY ZL</v>
+            <v>PIRACICABA</v>
           </cell>
           <cell r="I10">
-            <v>11331</v>
+            <v>1505.5</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N10">
-            <v>6</v>
+            <v>12</v>
           </cell>
         </row>
         <row r="11">
@@ -1828,19 +1828,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>16561.600000000006</v>
+            <v>26771.370000000021</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE MOOCA</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I11">
-            <v>4935.5999999999995</v>
+            <v>20857.45</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N11">
-            <v>6</v>
+            <v>17</v>
           </cell>
         </row>
         <row r="12">
@@ -1848,19 +1848,13 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>61613.220000000016</v>
-          </cell>
-          <cell r="H12" t="str">
-            <v>LESTE PENHA</v>
-          </cell>
-          <cell r="I12">
-            <v>5429.5999999999995</v>
+            <v>118036.82000000002</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>5</v>
+            <v>9</v>
           </cell>
         </row>
         <row r="13">
@@ -1868,19 +1862,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>70798.399999999994</v>
-          </cell>
-          <cell r="H13" t="str">
-            <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="I13">
-            <v>3237.6700000000005</v>
+            <v>125944.45999999996</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>9</v>
+            <v>16</v>
           </cell>
         </row>
         <row r="14">
@@ -1888,19 +1876,13 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>58605.799999999988</v>
-          </cell>
-          <cell r="H14" t="str">
-            <v>MOGI</v>
-          </cell>
-          <cell r="I14">
-            <v>1302.75</v>
+            <v>335094.5</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>9</v>
+            <v>18</v>
           </cell>
         </row>
         <row r="15">
@@ -1908,19 +1890,13 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>4900.4000000000005</v>
-          </cell>
-          <cell r="H15" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="I15">
-            <v>9669.82</v>
+            <v>15117</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>16</v>
+            <v>29</v>
           </cell>
         </row>
         <row r="16">
@@ -1928,19 +1904,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>15254.599999999995</v>
-          </cell>
-          <cell r="H16" t="str">
-            <v>PIRACICABA</v>
-          </cell>
-          <cell r="I16">
-            <v>3604.26</v>
+            <v>68104.53</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N16">
-            <v>11</v>
+            <v>18</v>
           </cell>
         </row>
         <row r="17">
@@ -1948,19 +1918,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>69757.400000000009</v>
-          </cell>
-          <cell r="H17" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I17">
-            <v>2849.65</v>
+            <v>125699.9</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>4</v>
+            <v>16</v>
           </cell>
         </row>
         <row r="18">
@@ -1968,19 +1932,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>11856.740000000002</v>
-          </cell>
-          <cell r="H18" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I18">
-            <v>5653.2</v>
+            <v>32134.140000000014</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N18">
-            <v>4</v>
+            <v>15</v>
           </cell>
         </row>
         <row r="19">
@@ -1988,19 +1946,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>18652.140000000007</v>
-          </cell>
-          <cell r="H19" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I19">
-            <v>384</v>
+            <v>52316.990000000056</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>95</v>
+            <v>198</v>
           </cell>
         </row>
         <row r="20">
@@ -2008,13 +1960,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>21488.189999999995</v>
-          </cell>
-          <cell r="H20" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I20">
-            <v>1513.29</v>
+            <v>36923.840000000011</v>
           </cell>
         </row>
         <row r="21">
@@ -2022,13 +1968,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>10992.669999999998</v>
-          </cell>
-          <cell r="H21" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I21">
-            <v>7272.37</v>
+            <v>30978.680000000018</v>
           </cell>
         </row>
         <row r="22">
@@ -2036,13 +1976,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>7117.0199999999968</v>
-          </cell>
-          <cell r="H22" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I22">
-            <v>90066.679999999935</v>
+            <v>17403.189999999988</v>
           </cell>
         </row>
         <row r="23">
@@ -2050,7 +1984,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>27209.899999999998</v>
+            <v>75023.440000000031</v>
           </cell>
         </row>
         <row r="24">
@@ -2058,7 +1992,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>47926.050000000025</v>
+            <v>105944.97000000004</v>
           </cell>
         </row>
         <row r="25">
@@ -2066,7 +2000,7 @@
             <v>PIRACICABA</v>
           </cell>
           <cell r="F25">
-            <v>12211.059999999998</v>
+            <v>53478.660000000011</v>
           </cell>
         </row>
         <row r="26">
@@ -2074,7 +2008,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>16815.25</v>
+            <v>42891.429999999993</v>
           </cell>
         </row>
         <row r="27">
@@ -2082,7 +2016,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>19899.88</v>
+            <v>48489.55000000001</v>
           </cell>
         </row>
         <row r="28">
@@ -2090,7 +2024,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>23533.34</v>
+            <v>72774.290000000008</v>
           </cell>
         </row>
         <row r="29">
@@ -2098,7 +2032,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>5681.579999999999</v>
+            <v>24305.909999999985</v>
           </cell>
         </row>
         <row r="30">
@@ -2106,7 +2040,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>6048.670000000001</v>
+            <v>13522.699999999988</v>
           </cell>
         </row>
         <row r="31">
@@ -2114,7 +2048,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>15133.860000000004</v>
+            <v>25327.320000000003</v>
           </cell>
         </row>
         <row r="32">
@@ -2122,7 +2056,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>642114.53000000212</v>
+            <v>1676623.3299999835</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2941,7 +2875,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>300152</v>
+        <v>300104</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -2975,7 +2909,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>642039.41</v>
+        <v>1676134.63</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2986,7 +2920,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>72167.42</v>
+        <v>19351.949999999997</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2997,7 +2931,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>17899.260000000002</v>
+        <v>1505.5</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3008,7 +2942,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>95</v>
+        <v>198</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3020,7 +2954,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>4949460.59</v>
+        <v>3915365.37</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3031,7 +2965,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>227984.58000000002</v>
+        <v>280752.05</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3042,7 +2976,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-17899.260000000002</v>
+        <v>-1505.5</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3053,7 +2987,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>663</v>
+        <v>560</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3065,7 +2999,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.11482418134668693</v>
+        <v>0.2997647554323527</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3076,7 +3010,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.24043624563554455</v>
+        <v>6.4484145496228051E-2</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3098,7 +3032,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.12532981530343013</v>
+        <v>0.26121372031662271</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3197,11 +3131,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>7480.3299999999981</v>
+        <v>16835.900000000001</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>57019.67</v>
+        <v>47664.1</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3212,15 +3146,15 @@
       </c>
       <c r="I10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>34823</v>
+        <v>29150</v>
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9669.82</v>
+        <v>0</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>25153.18</v>
+        <v>29150</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3271,11 +3205,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>57626.830000000038</v>
+        <v>121640.54999999996</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>267373.17</v>
+        <v>203359.45000000004</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3286,7 +3220,7 @@
       </c>
       <c r="I11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>28168</v>
+        <v>26150</v>
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3294,7 +3228,7 @@
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>28168</v>
+        <v>26150</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3328,11 +3262,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>35</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3347,11 +3281,11 @@
       </c>
       <c r="D12" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>33.020000000000003</v>
+        <v>49.09</v>
       </c>
       <c r="E12" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>966.98</v>
+        <v>950.91</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="21" t="s">
@@ -3362,15 +3296,15 @@
       </c>
       <c r="I12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12773</v>
+        <v>12180</v>
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2849.65</v>
+        <v>0</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9923.35</v>
+        <v>12180</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3385,11 +3319,11 @@
       </c>
       <c r="P12" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3604.26</v>
+        <v>1505.5</v>
       </c>
       <c r="Q12" s="2">
         <f>O12-P12</f>
-        <v>-3604.26</v>
+        <v>-1505.5</v>
       </c>
       <c r="R12" s="2"/>
       <c r="S12" s="19" t="s">
@@ -3404,11 +3338,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3424,11 +3358,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>8818.9</v>
+        <v>21547.7</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>81181.100000000006</v>
+        <v>68452.3</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3439,15 +3373,15 @@
       </c>
       <c r="I13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>29550</v>
+        <v>24150</v>
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>384</v>
+        <v>0</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>29166</v>
+        <v>24150</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3462,11 +3396,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11331</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-11331</v>
+        <v>0</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3501,11 +3435,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>26022.560000000009</v>
+        <v>69777.699999999983</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>246977.44</v>
+        <v>203222.30000000002</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3516,15 +3450,15 @@
       </c>
       <c r="I14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>21709</v>
+        <v>22495</v>
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3237.6700000000005</v>
+        <v>5677.7</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>18471.329999999998</v>
+        <v>16817.3</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3558,11 +3492,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3578,11 +3512,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>16561.600000000006</v>
+        <v>26771.370000000021</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>61438.399999999994</v>
+        <v>51228.629999999976</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3593,15 +3527,15 @@
       </c>
       <c r="I15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>32806</v>
+        <v>25150</v>
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13981.84</v>
+        <v>12313.9</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>18824.16</v>
+        <v>12836.1</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3616,11 +3550,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2964</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-2964</v>
+        <v>0</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3635,11 +3569,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3655,11 +3589,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>61613.220000000016</v>
+        <v>118036.82000000002</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>263386.77999999997</v>
+        <v>206963.18</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3670,15 +3604,15 @@
       </c>
       <c r="I16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>16187</v>
+        <v>17150</v>
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5653.2</v>
+        <v>0</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10533.8</v>
+        <v>17150</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3732,11 +3666,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>70798.399999999994</v>
+        <v>125944.45999999996</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>99201.600000000006</v>
+        <v>44055.540000000037</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3747,15 +3681,15 @@
       </c>
       <c r="I17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4976</v>
+        <v>6701</v>
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1302.75</v>
+        <v>184.85000000000002</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3673.25</v>
+        <v>6516.15</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3809,11 +3743,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>58605.799999999988</v>
+        <v>335094.5</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>891394.2</v>
+        <v>614905.5</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3824,7 +3758,7 @@
       </c>
       <c r="I18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14530</v>
+        <v>15912</v>
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3832,7 +3766,7 @@
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>14530</v>
+        <v>15912</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3853,11 +3787,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3873,11 +3807,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>4900.4000000000005</v>
+        <v>15117</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>125099.6</v>
+        <v>114883</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3888,15 +3822,15 @@
       </c>
       <c r="I19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>16828</v>
+        <v>18150</v>
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4935.5999999999995</v>
+        <v>0</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11892.400000000001</v>
+        <v>18150</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3913,11 +3847,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3933,11 +3867,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>15254.599999999995</v>
+        <v>68104.53</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>544745.4</v>
+        <v>491895.47</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3948,15 +3882,15 @@
       </c>
       <c r="I20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>21245</v>
+        <v>20150</v>
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7553.6399999999994</v>
+        <v>0</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>13691.36</v>
+        <v>20150</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3985,11 +3919,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4005,11 +3939,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>69757.400000000009</v>
+        <v>125699.9</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>345242.6</v>
+        <v>289300.09999999998</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4020,15 +3954,15 @@
       </c>
       <c r="I21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6246</v>
+        <v>8150</v>
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6364.44</v>
+        <v>0</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-118.4399999999996</v>
+        <v>8150</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4041,11 +3975,11 @@
       </c>
       <c r="P21" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>275241.61999999988</v>
+        <v>275241.61999999976</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>96349.289090909238</v>
+        <v>96349.289090909355</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="19" t="s">
@@ -4060,11 +3994,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -4080,11 +4014,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>11856.740000000002</v>
+        <v>32134.140000000014</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>110143.26</v>
+        <v>89865.859999999986</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4095,15 +4029,15 @@
       </c>
       <c r="I22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14716</v>
+        <v>15870</v>
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5429.5999999999995</v>
+        <v>810.09999999999991</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9286.4000000000015</v>
+        <v>15059.9</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4116,11 +4050,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>17899.259999999998</v>
+        <v>564728.75000000047</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>477555.28545454546</v>
+        <v>-69274.204545454995</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4135,11 +4069,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4155,11 +4089,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>18652.140000000007</v>
+        <v>52316.990000000056</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>176347.86</v>
+        <v>142683.00999999995</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4170,7 +4104,7 @@
       </c>
       <c r="I23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12001</v>
+        <v>15604</v>
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4178,7 +4112,7 @@
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12001</v>
+        <v>15604</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4191,11 +4125,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>1505.5</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>619318.18181818188</v>
+        <v>617812.68181818188</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4230,11 +4164,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>21488.189999999995</v>
+        <v>36923.840000000011</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>118511.81</v>
+        <v>103076.15999999999</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4245,15 +4179,15 @@
       </c>
       <c r="I24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>10474</v>
+        <v>11650</v>
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7272.37</v>
+        <v>0</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3201.63</v>
+        <v>11650</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4285,11 +4219,11 @@
       </c>
       <c r="V24" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="W24" s="19">
         <f t="shared" si="2"/>
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -4305,11 +4239,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>10992.669999999998</v>
+        <v>30978.680000000018</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>131507.33000000002</v>
+        <v>111521.31999999998</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4320,7 +4254,7 @@
       </c>
       <c r="I25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11553</v>
+        <v>15130</v>
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4328,7 +4262,7 @@
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11553</v>
+        <v>15130</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4360,11 +4294,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4380,11 +4314,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>7117.0199999999968</v>
+        <v>17403.189999999988</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>82882.98000000001</v>
+        <v>72596.810000000012</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4395,15 +4329,15 @@
       </c>
       <c r="I26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5351</v>
+        <v>6925</v>
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1513.29</v>
+        <v>0</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3837.71</v>
+        <v>6925</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4444,11 +4378,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>27209.899999999998</v>
+        <v>75023.440000000031</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>210290.1</v>
+        <v>162476.55999999997</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4459,15 +4393,15 @@
       </c>
       <c r="I27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6216</v>
+        <v>9437</v>
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2019.55</v>
+        <v>365.4</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4196.45</v>
+        <v>9071.6</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4490,11 +4424,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>47926.050000000025</v>
+        <v>105944.97000000004</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>270573.94999999995</v>
+        <v>212555.02999999997</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4523,11 +4457,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>12211.059999999998</v>
+        <v>53478.660000000011</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>162788.94</v>
+        <v>121521.34</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4569,11 +4503,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>16815.25</v>
+        <v>42891.429999999993</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>117684.75</v>
+        <v>91608.57</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4606,11 +4540,11 @@
       </c>
       <c r="V30" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="W30" s="6">
         <f>U30-V30</f>
-        <v>22.36363636363636</v>
+        <v>24.36363636363636</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
@@ -4626,11 +4560,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>19899.88</v>
+        <v>48489.55000000001</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>147100.12</v>
+        <v>118510.44999999998</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4643,11 +4577,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>262981.54999999987</v>
+        <v>257833.44999999981</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>127768.45000000013</v>
+        <v>132916.55000000019</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4666,11 +4600,11 @@
       </c>
       <c r="V31" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>14</v>
+        <v>132</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="3">U31-V31</f>
-        <v>123.81818181818181</v>
+        <v>5.818181818181813</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4686,11 +4620,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>23533.34</v>
+        <v>72774.290000000008</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>236466.66</v>
+        <v>187225.71</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4703,11 +4637,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>67231.819999999992</v>
+        <v>505107.28000000294</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>453768.18</v>
+        <v>15892.719999997062</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4726,11 +4660,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>172.27272727272725</v>
+        <v>169.27272727272725</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4746,11 +4680,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>5681.579999999999</v>
+        <v>24305.909999999985</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>94318.42</v>
+        <v>75694.090000000011</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4763,11 +4697,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>19351.95</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>651250</v>
+        <v>631898.05000000005</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4806,11 +4740,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>6048.670000000001</v>
+        <v>13522.699999999988</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>48951.33</v>
+        <v>41477.30000000001</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4866,11 +4800,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>15133.860000000004</v>
+        <v>25327.320000000003</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>57866.14</v>
+        <v>47672.679999999993</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4988,11 +4922,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>552047.85000000172</v>
+        <v>546899.75000000163</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>-161297.85000000172</v>
+        <v>-156149.75000000163</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -5024,11 +4958,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>90066.679999999935</v>
+        <v>1108866.1299999962</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="5">C40-D40</f>
-        <v>430933.32000000007</v>
+        <v>-587866.12999999616</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -5060,11 +4994,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>20857.45</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="5"/>
-        <v>651250</v>
+        <v>630392.55000000005</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 13/07/2026 11:11
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F647E5-6A8E-4828-8BBA-A4F097B736A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1845FD-FA3A-4E34-8D10-EADB3AED4FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1717,13 +1717,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>16835.900000000001</v>
+            <v>17375.800000000003</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>365.4</v>
+            <v>905.3</v>
           </cell>
         </row>
         <row r="6">
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>121640.54999999996</v>
+            <v>129467.75999999995</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>12313.9</v>
+            <v>20141.109999999997</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1751,10 +1751,10 @@
             <v>488.70000000000005</v>
           </cell>
           <cell r="H7" t="str">
-            <v>LESTE PENHA</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>810.09999999999991</v>
+            <v>5055.8600000000006</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1771,10 +1771,10 @@
             <v>49.09</v>
           </cell>
           <cell r="H8" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>5677.7</v>
+            <v>8910.5999999999985</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -1788,19 +1788,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>21547.7</v>
+            <v>26603.559999999998</v>
           </cell>
           <cell r="H9" t="str">
-            <v>MOGI</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>184.85000000000002</v>
+            <v>864.5</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N9">
-            <v>17</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="10">
@@ -1808,13 +1808,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>69777.699999999983</v>
+            <v>78688.299999999974</v>
           </cell>
           <cell r="H10" t="str">
-            <v>PIRACICABA</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="I10">
-            <v>1505.5</v>
+            <v>8068.9999999999991</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
@@ -1828,13 +1828,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>26771.370000000021</v>
+            <v>27635.870000000021</v>
           </cell>
           <cell r="H11" t="str">
-            <v>Total Geral</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I11">
-            <v>20857.45</v>
+            <v>7328.6</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
@@ -1850,11 +1850,17 @@
           <cell r="F12">
             <v>118036.82000000002</v>
           </cell>
+          <cell r="H12" t="str">
+            <v>LESTE MOOCA</v>
+          </cell>
+          <cell r="I12">
+            <v>2291.1</v>
+          </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>9</v>
+            <v>10</v>
           </cell>
         </row>
         <row r="13">
@@ -1862,13 +1868,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>125944.45999999996</v>
+            <v>134013.46</v>
+          </cell>
+          <cell r="H13" t="str">
+            <v>LESTE PENHA</v>
+          </cell>
+          <cell r="I13">
+            <v>5696.4</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>16</v>
+            <v>17</v>
           </cell>
         </row>
         <row r="14">
@@ -1878,6 +1890,12 @@
           <cell r="F14">
             <v>335094.5</v>
           </cell>
+          <cell r="H14" t="str">
+            <v>LESTE TATUAPE</v>
+          </cell>
+          <cell r="I14">
+            <v>7604</v>
+          </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
@@ -1892,11 +1910,17 @@
           <cell r="F15">
             <v>15117</v>
           </cell>
+          <cell r="H15" t="str">
+            <v>MOGI</v>
+          </cell>
+          <cell r="I15">
+            <v>1267.6300000000001</v>
+          </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>29</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="16">
@@ -1906,6 +1930,12 @@
           <cell r="F16">
             <v>68104.53</v>
           </cell>
+          <cell r="H16" t="str">
+            <v>NORTE</v>
+          </cell>
+          <cell r="I16">
+            <v>6434.7999999999993</v>
+          </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
           </cell>
@@ -1918,7 +1948,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>125699.9</v>
+            <v>133028.49999999997</v>
+          </cell>
+          <cell r="H17" t="str">
+            <v>OSASCO</v>
+          </cell>
+          <cell r="I17">
+            <v>6578.51</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
@@ -1934,6 +1970,12 @@
           <cell r="F18">
             <v>32134.140000000014</v>
           </cell>
+          <cell r="H18" t="str">
+            <v>PIRACICABA</v>
+          </cell>
+          <cell r="I18">
+            <v>1505.5</v>
+          </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
           </cell>
@@ -1946,13 +1988,19 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>52316.990000000056</v>
+            <v>54478.090000000055</v>
+          </cell>
+          <cell r="H19" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="I19">
+            <v>2910.9500000000003</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>198</v>
+            <v>205</v>
           </cell>
         </row>
         <row r="20">
@@ -1960,7 +2008,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>36923.840000000011</v>
+            <v>41810.140000000007</v>
+          </cell>
+          <cell r="H20" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="I20">
+            <v>6333.9600000000009</v>
           </cell>
         </row>
         <row r="21">
@@ -1968,7 +2022,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>30978.680000000018</v>
+            <v>32904.980000000025</v>
+          </cell>
+          <cell r="H21" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="I21">
+            <v>14219.94</v>
           </cell>
         </row>
         <row r="22">
@@ -1976,7 +2036,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>17403.189999999988</v>
+            <v>18485.969999999994</v>
+          </cell>
+          <cell r="H22" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I22">
+            <v>4629.8</v>
           </cell>
         </row>
         <row r="23">
@@ -1984,7 +2050,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>75023.440000000031</v>
+            <v>81458.24000000002</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I23">
+            <v>1175.0900000000001</v>
           </cell>
         </row>
         <row r="24">
@@ -1992,7 +2064,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>105944.97000000004</v>
+            <v>112523.48000000005</v>
+          </cell>
+          <cell r="H24" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I24">
+            <v>1531.14</v>
           </cell>
         </row>
         <row r="25">
@@ -2002,13 +2080,19 @@
           <cell r="F25">
             <v>53478.660000000011</v>
           </cell>
+          <cell r="H25" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I25">
+            <v>113453.79</v>
+          </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>42891.429999999993</v>
+            <v>45802.37999999999</v>
           </cell>
         </row>
         <row r="27">
@@ -2016,7 +2100,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>48489.55000000001</v>
+            <v>54823.51</v>
           </cell>
         </row>
         <row r="28">
@@ -2024,7 +2108,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>72774.290000000008</v>
+            <v>86994.229999999938</v>
           </cell>
         </row>
         <row r="29">
@@ -2032,7 +2116,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>24305.909999999985</v>
+            <v>28935.709999999992</v>
           </cell>
         </row>
         <row r="30">
@@ -2040,7 +2124,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>13522.699999999988</v>
+            <v>14697.789999999988</v>
           </cell>
         </row>
         <row r="31">
@@ -2048,7 +2132,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>25327.320000000003</v>
+            <v>26858.460000000003</v>
           </cell>
         </row>
         <row r="32">
@@ -2056,7 +2140,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>1676623.3299999835</v>
+            <v>1769089.6699999834</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2909,7 +2993,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>1676134.63</v>
+        <v>1768600.9699999997</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2920,7 +3004,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>19351.949999999997</v>
+        <v>96550.69</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2931,7 +3015,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>1505.5</v>
+        <v>16903.099999999999</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -2942,7 +3026,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2954,7 +3038,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>3915365.37</v>
+        <v>3822899.0300000003</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2965,7 +3049,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>280752.05</v>
+        <v>203553.31</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2976,7 +3060,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-1505.5</v>
+        <v>-16903.099999999999</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -2987,7 +3071,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>560</v>
+        <v>553</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2999,7 +3083,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.2997647554323527</v>
+        <v>0.3163017025842797</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3010,7 +3094,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>6.4484145496228051E-2</v>
+        <v>0.32172410231119875</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3032,7 +3116,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.26121372031662271</v>
+        <v>0.27044854881266489</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3131,11 +3215,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>16835.900000000001</v>
+        <v>17375.800000000003</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>47664.1</v>
+        <v>47124.2</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3150,11 +3234,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>6578.51</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>29150</v>
+        <v>22571.489999999998</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3205,11 +3289,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>121640.54999999996</v>
+        <v>129467.75999999995</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>203359.45000000004</v>
+        <v>195532.24000000005</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3224,11 +3308,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>6434.7999999999993</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>26150</v>
+        <v>19715.2</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3300,11 +3384,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>2910.9500000000003</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12180</v>
+        <v>9269.0499999999993</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3338,11 +3422,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3358,11 +3442,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>21547.7</v>
+        <v>26603.559999999998</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>68452.3</v>
+        <v>63396.44</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3377,11 +3461,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>14219.94</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>24150</v>
+        <v>9930.06</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3396,11 +3480,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>7328.6</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>0</v>
+        <v>-7328.6</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3435,11 +3519,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>69777.699999999983</v>
+        <v>78688.299999999974</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>203222.30000000002</v>
+        <v>194311.7</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3454,11 +3538,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5677.7</v>
+        <v>7604</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>16817.3</v>
+        <v>14891</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3512,11 +3596,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>26771.370000000021</v>
+        <v>27635.870000000021</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>51228.629999999976</v>
+        <v>50364.129999999976</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3531,11 +3615,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>12313.9</v>
+        <v>20141.109999999997</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12836.1</v>
+        <v>5008.8900000000031</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3608,11 +3692,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>6333.9600000000009</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>17150</v>
+        <v>10816.039999999999</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3666,11 +3750,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>125944.45999999996</v>
+        <v>134013.46</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>44055.540000000037</v>
+        <v>35986.540000000008</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3685,11 +3769,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>184.85000000000002</v>
+        <v>1267.6300000000001</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6516.15</v>
+        <v>5433.37</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3704,11 +3788,11 @@
       </c>
       <c r="P17" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>8068.9999999999991</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-8068.9999999999991</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="19" t="s">
@@ -3826,11 +3910,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>2291.1</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>18150</v>
+        <v>15858.9</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3847,11 +3931,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3886,11 +3970,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>8910.5999999999985</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>20150</v>
+        <v>11239.400000000001</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3919,11 +4003,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3939,11 +4023,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>125699.9</v>
+        <v>133028.49999999997</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>289300.09999999998</v>
+        <v>281971.5</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -3958,11 +4042,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>864.5</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8150</v>
+        <v>7285.5</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4033,11 +4117,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>810.09999999999991</v>
+        <v>5696.4</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15059.9</v>
+        <v>10173.6</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4089,11 +4173,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52316.990000000056</v>
+        <v>54478.090000000055</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>142683.00999999995</v>
+        <v>140521.90999999995</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4108,11 +4192,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>5055.8600000000006</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15604</v>
+        <v>10548.14</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4125,11 +4209,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1505.5</v>
+        <v>16903.100000000006</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>617812.68181818188</v>
+        <v>602415.0818181819</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4164,11 +4248,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>36923.840000000011</v>
+        <v>41810.140000000007</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>103076.15999999999</v>
+        <v>98189.859999999986</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4183,11 +4267,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1531.14</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11650</v>
+        <v>10118.86</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4239,11 +4323,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>30978.680000000018</v>
+        <v>32904.980000000025</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>111521.31999999998</v>
+        <v>109595.01999999997</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4258,11 +4342,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4629.8</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15130</v>
+        <v>10500.2</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4294,11 +4378,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4314,11 +4398,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>17403.189999999988</v>
+        <v>18485.969999999994</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>72596.810000000012</v>
+        <v>71514.03</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4333,11 +4417,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1175.0900000000001</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6925</v>
+        <v>5749.91</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4378,11 +4462,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>75023.440000000031</v>
+        <v>81458.24000000002</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>162476.55999999997</v>
+        <v>156041.75999999998</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4397,11 +4481,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>365.4</v>
+        <v>905.3</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9071.6</v>
+        <v>8531.7000000000007</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4424,11 +4508,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>105944.97000000004</v>
+        <v>112523.48000000005</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>212555.02999999997</v>
+        <v>205976.51999999996</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4503,11 +4587,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>42891.429999999993</v>
+        <v>45802.37999999999</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>91608.57</v>
+        <v>88697.62000000001</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4560,11 +4644,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>48489.55000000001</v>
+        <v>54823.51</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>118510.44999999998</v>
+        <v>112176.48999999999</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4620,11 +4704,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>72774.290000000008</v>
+        <v>86994.229999999938</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>187225.71</v>
+        <v>173005.77000000008</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4660,11 +4744,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>169.27272727272725</v>
+        <v>155.27272727272725</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4680,11 +4764,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>24305.909999999985</v>
+        <v>28935.709999999992</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>75694.090000000011</v>
+        <v>71064.290000000008</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4697,11 +4781,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>19351.95</v>
+        <v>94259.589999999982</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>631898.05000000005</v>
+        <v>556990.41</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4740,11 +4824,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>13522.699999999988</v>
+        <v>14697.789999999988</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41477.30000000001</v>
+        <v>40302.210000000014</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4800,11 +4884,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>25327.320000000003</v>
+        <v>26858.460000000003</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>47672.679999999993</v>
+        <v>46141.539999999994</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4958,11 +5042,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1108866.1299999962</v>
+        <v>1108736.1299999962</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="5">C40-D40</f>
-        <v>-587866.12999999616</v>
+        <v>-587736.12999999616</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4994,11 +5078,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>20857.45</v>
+        <v>113453.79</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="5"/>
-        <v>630392.55000000005</v>
+        <v>537796.21</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 14/07/2026 09:50
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1845FD-FA3A-4E34-8D10-EADB3AED4FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7934FD57-6988-4266-8B7B-466900D4A361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-13T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-14T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1681,7 +1681,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>13/07/2026</v>
+            <v>14/07/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1717,13 +1717,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>17375.800000000003</v>
+            <v>19446.750000000004</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>905.3</v>
+            <v>1382.35</v>
           </cell>
         </row>
         <row r="6">
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>129467.75999999995</v>
+            <v>151882.9899999999</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>20141.109999999997</v>
+            <v>2591.6000000000004</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1748,13 +1748,13 @@
             <v>ECOMMERCE</v>
           </cell>
           <cell r="F7">
-            <v>488.70000000000005</v>
+            <v>828.94</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I7">
-            <v>5055.8600000000006</v>
+            <v>1440.91</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1771,16 +1771,16 @@
             <v>49.09</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I8">
-            <v>8910.5999999999985</v>
+            <v>1092</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N8">
-            <v>31</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="9">
@@ -1788,19 +1788,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>26603.559999999998</v>
+            <v>29329.179999999997</v>
           </cell>
           <cell r="H9" t="str">
-            <v>JUNDIAI</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I9">
-            <v>864.5</v>
+            <v>29751.200000000001</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N9">
-            <v>21</v>
+            <v>22</v>
           </cell>
         </row>
         <row r="10">
@@ -1808,13 +1808,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>78688.299999999974</v>
+            <v>88513.359999999971</v>
           </cell>
           <cell r="H10" t="str">
-            <v>KEY CASA</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I10">
-            <v>8068.9999999999991</v>
+            <v>14725.18</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
@@ -1828,19 +1828,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>27635.870000000021</v>
+            <v>31887.770000000026</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY ZL</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I11">
-            <v>7328.6</v>
+            <v>259.8</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N11">
-            <v>17</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="12">
@@ -1848,19 +1848,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>118036.82000000002</v>
+            <v>121733.92000000003</v>
           </cell>
           <cell r="H12" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I12">
-            <v>2291.1</v>
+            <v>2653.3</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>10</v>
+            <v>12</v>
           </cell>
         </row>
         <row r="13">
@@ -1868,19 +1868,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>134013.46</v>
+            <v>155213.56</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I13">
-            <v>5696.4</v>
+            <v>4077.82</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>17</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="14">
@@ -1888,19 +1888,19 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>335094.5</v>
+            <v>403983.90000000026</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>7604</v>
+            <v>604.70000000000005</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>18</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="15">
@@ -1908,19 +1908,19 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>15117</v>
+            <v>22426.3</v>
           </cell>
           <cell r="H15" t="str">
-            <v>MOGI</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I15">
-            <v>1267.6300000000001</v>
+            <v>627.6</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>30</v>
+            <v>38</v>
           </cell>
         </row>
         <row r="16">
@@ -1928,19 +1928,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>68104.53</v>
+            <v>127430.38</v>
           </cell>
           <cell r="H16" t="str">
-            <v>NORTE</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I16">
-            <v>6434.7999999999993</v>
+            <v>772.2</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N16">
-            <v>18</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="17">
@@ -1948,19 +1948,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>133028.49999999997</v>
+            <v>159429.97999999995</v>
           </cell>
           <cell r="H17" t="str">
-            <v>OSASCO</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I17">
-            <v>6578.51</v>
+            <v>839.76</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>16</v>
+            <v>17</v>
           </cell>
         </row>
         <row r="18">
@@ -1968,13 +1968,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>32134.140000000014</v>
+            <v>42575.060000000012</v>
           </cell>
           <cell r="H18" t="str">
-            <v>PIRACICABA</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I18">
-            <v>1505.5</v>
+            <v>60818.42000000002</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -1988,19 +1988,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>54478.090000000055</v>
-          </cell>
-          <cell r="H19" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I19">
-            <v>2910.9500000000003</v>
+            <v>73698.819999999992</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>205</v>
+            <v>228</v>
           </cell>
         </row>
         <row r="20">
@@ -2008,13 +2002,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>41810.140000000007</v>
-          </cell>
-          <cell r="H20" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I20">
-            <v>6333.9600000000009</v>
+            <v>52664.26</v>
           </cell>
         </row>
         <row r="21">
@@ -2022,13 +2010,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>32904.980000000025</v>
-          </cell>
-          <cell r="H21" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I21">
-            <v>14219.94</v>
+            <v>44701.440000000061</v>
           </cell>
         </row>
         <row r="22">
@@ -2036,13 +2018,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>18485.969999999994</v>
-          </cell>
-          <cell r="H22" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I22">
-            <v>4629.8</v>
+            <v>22225.860000000011</v>
           </cell>
         </row>
         <row r="23">
@@ -2050,13 +2026,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>81458.24000000002</v>
-          </cell>
-          <cell r="H23" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I23">
-            <v>1175.0900000000001</v>
+            <v>97946.510000000024</v>
           </cell>
         </row>
         <row r="24">
@@ -2064,13 +2034,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>112523.48000000005</v>
-          </cell>
-          <cell r="H24" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I24">
-            <v>1531.14</v>
+            <v>131615.06000000003</v>
           </cell>
         </row>
         <row r="25">
@@ -2080,19 +2044,13 @@
           <cell r="F25">
             <v>53478.660000000011</v>
           </cell>
-          <cell r="H25" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I25">
-            <v>113453.79</v>
-          </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>45802.37999999999</v>
+            <v>52551.639999999963</v>
           </cell>
         </row>
         <row r="27">
@@ -2100,7 +2058,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>54823.51</v>
+            <v>59936.180000000008</v>
           </cell>
         </row>
         <row r="28">
@@ -2108,7 +2066,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>86994.229999999938</v>
+            <v>94488.119999999893</v>
           </cell>
         </row>
         <row r="29">
@@ -2116,7 +2074,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>28935.709999999992</v>
+            <v>40132.44000000001</v>
           </cell>
         </row>
         <row r="30">
@@ -2124,7 +2082,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>14697.789999999988</v>
+            <v>17502.359999999986</v>
           </cell>
         </row>
         <row r="31">
@@ -2132,7 +2090,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>26858.460000000003</v>
+            <v>34782.590000000011</v>
           </cell>
         </row>
         <row r="32">
@@ -2140,7 +2098,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>1769089.6699999834</v>
+            <v>2130455.1199999726</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2959,7 +2917,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>300104</v>
+        <v>200027</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -2993,7 +2951,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>1768600.9699999997</v>
+        <v>2129626.1799999997</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3004,7 +2962,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>96550.69</v>
+        <v>16342.04</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3015,7 +2973,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>16903.099999999999</v>
+        <v>44476.380000000005</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3026,7 +2984,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>205</v>
+        <v>228</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3038,7 +2996,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>3822899.0300000003</v>
+        <v>3461873.8200000003</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3049,7 +3007,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>203553.31</v>
+        <v>183684.96</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3060,7 +3018,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-16903.099999999999</v>
+        <v>-44476.380000000005</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3071,7 +3029,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>553</v>
+        <v>530</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3083,7 +3041,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.3163017025842797</v>
+        <v>0.38086849324868099</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3094,7 +3052,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.32172410231119875</v>
+        <v>8.1699170611967409E-2</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3116,7 +3074,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.27044854881266489</v>
+        <v>0.30079155672823221</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3215,11 +3173,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>17375.800000000003</v>
+        <v>19446.750000000004</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>47124.2</v>
+        <v>45053.25</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3230,15 +3188,15 @@
       </c>
       <c r="I10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>29150</v>
+        <v>20000</v>
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6578.51</v>
+        <v>0</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>22571.489999999998</v>
+        <v>20000</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3289,11 +3247,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>129467.75999999995</v>
+        <v>151882.9899999999</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>195532.24000000005</v>
+        <v>173117.0100000001</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3304,15 +3262,15 @@
       </c>
       <c r="I11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>26150</v>
+        <v>13000</v>
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6434.7999999999993</v>
+        <v>0</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>19715.2</v>
+        <v>13000</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3346,11 +3304,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3380,15 +3338,15 @@
       </c>
       <c r="I12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12180</v>
+        <v>15390</v>
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2910.9500000000003</v>
+        <v>627.6</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9269.0499999999993</v>
+        <v>14762.4</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3403,11 +3361,11 @@
       </c>
       <c r="P12" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1505.5</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="2">
         <f>O12-P12</f>
-        <v>-1505.5</v>
+        <v>0</v>
       </c>
       <c r="R12" s="2"/>
       <c r="S12" s="19" t="s">
@@ -3422,11 +3380,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3442,11 +3400,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>26603.559999999998</v>
+        <v>29329.179999999997</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>63396.44</v>
+        <v>60670.820000000007</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3457,15 +3415,15 @@
       </c>
       <c r="I13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>24150</v>
+        <v>22000</v>
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14219.94</v>
+        <v>0</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9930.06</v>
+        <v>22000</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3480,11 +3438,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7328.6</v>
+        <v>14725.18</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-7328.6</v>
+        <v>-14725.18</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3519,11 +3477,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>78688.299999999974</v>
+        <v>88513.359999999971</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>194311.7</v>
+        <v>184486.64</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3534,15 +3492,15 @@
       </c>
       <c r="I14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>22495</v>
+        <v>11529</v>
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7604</v>
+        <v>0</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>14891</v>
+        <v>11529</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3596,11 +3554,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>27635.870000000021</v>
+        <v>31887.770000000026</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50364.129999999976</v>
+        <v>46112.229999999974</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3611,15 +3569,15 @@
       </c>
       <c r="I15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>25150</v>
+        <v>24000</v>
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>20141.109999999997</v>
+        <v>2591.6000000000004</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5008.8900000000031</v>
+        <v>21408.400000000001</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3634,11 +3592,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>29751.200000000001</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-29751.200000000001</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3653,11 +3611,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3673,11 +3631,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>118036.82000000002</v>
+        <v>121733.92000000003</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>206963.18</v>
+        <v>203266.07999999996</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3688,15 +3646,15 @@
       </c>
       <c r="I16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>17150</v>
+        <v>11000</v>
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6333.9600000000009</v>
+        <v>772.2</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10816.039999999999</v>
+        <v>10227.799999999999</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3750,11 +3708,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>134013.46</v>
+        <v>155213.56</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>35986.540000000008</v>
+        <v>14786.440000000002</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3765,15 +3723,15 @@
       </c>
       <c r="I17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6701</v>
+        <v>6888</v>
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1267.6300000000001</v>
+        <v>604.70000000000005</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5433.37</v>
+        <v>6283.3</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3788,11 +3746,11 @@
       </c>
       <c r="P17" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8068.9999999999991</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="1"/>
-        <v>-8068.9999999999991</v>
+        <v>0</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="19" t="s">
@@ -3827,11 +3785,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>335094.5</v>
+        <v>403983.90000000026</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>614905.5</v>
+        <v>546016.09999999974</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3842,15 +3800,15 @@
       </c>
       <c r="I18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15912</v>
+        <v>10191</v>
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>259.8</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15912</v>
+        <v>9931.2000000000007</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3871,11 +3829,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3891,11 +3849,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>15117</v>
+        <v>22426.3</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>114883</v>
+        <v>107573.7</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3906,15 +3864,15 @@
       </c>
       <c r="I19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>18150</v>
+        <v>11000</v>
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2291.1</v>
+        <v>2653.3</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15858.9</v>
+        <v>8346.7000000000007</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3931,11 +3889,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3951,11 +3909,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>68104.53</v>
+        <v>127430.38</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>491895.47</v>
+        <v>432569.62</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3966,15 +3924,15 @@
       </c>
       <c r="I20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>20150</v>
+        <v>12000</v>
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8910.5999999999985</v>
+        <v>1440.91</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11239.400000000001</v>
+        <v>10559.09</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4003,11 +3961,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4023,11 +3981,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>133028.49999999997</v>
+        <v>159429.97999999995</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>281971.5</v>
+        <v>255570.02000000005</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4038,15 +3996,15 @@
       </c>
       <c r="I21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>8150</v>
+        <v>7750</v>
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>864.5</v>
+        <v>1092</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7285.5</v>
+        <v>6658</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4059,11 +4017,11 @@
       </c>
       <c r="P21" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>275241.61999999976</v>
+        <v>275241.61999999988</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>96349.289090909355</v>
+        <v>96349.289090909238</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="19" t="s">
@@ -4078,11 +4036,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -4098,11 +4056,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>32134.140000000014</v>
+        <v>42575.060000000012</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>89865.859999999986</v>
+        <v>79424.939999999988</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4113,15 +4071,15 @@
       </c>
       <c r="I22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15870</v>
+        <v>10290</v>
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5696.4</v>
+        <v>4077.82</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10173.6</v>
+        <v>6212.18</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4134,11 +4092,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>564728.75000000047</v>
+        <v>564728.75000000023</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-69274.204545454995</v>
+        <v>-69274.204545454762</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4153,11 +4111,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4173,11 +4131,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>54478.090000000055</v>
+        <v>73698.819999999992</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>140521.90999999995</v>
+        <v>121301.18000000001</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4188,15 +4146,15 @@
       </c>
       <c r="I23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15604</v>
+        <v>7510</v>
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5055.8600000000006</v>
+        <v>0</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10548.14</v>
+        <v>7510</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4209,11 +4167,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>16903.100000000006</v>
+        <v>203726.33000000016</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>602415.0818181819</v>
+        <v>415591.85181818169</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4248,11 +4206,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>41810.140000000007</v>
+        <v>52664.26</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>98189.859999999986</v>
+        <v>87335.739999999991</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4263,15 +4221,15 @@
       </c>
       <c r="I24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11650</v>
+        <v>3930</v>
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1531.14</v>
+        <v>839.76</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10118.86</v>
+        <v>3090.24</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4323,11 +4281,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>32904.980000000025</v>
+        <v>44701.440000000061</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>109595.01999999997</v>
+        <v>97798.559999999939</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4338,15 +4296,15 @@
       </c>
       <c r="I25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15130</v>
+        <v>4760</v>
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4629.8</v>
+        <v>0</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10500.2</v>
+        <v>4760</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4378,11 +4336,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4398,11 +4356,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>18485.969999999994</v>
+        <v>22225.860000000011</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>71514.03</v>
+        <v>67774.139999999985</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4413,15 +4371,15 @@
       </c>
       <c r="I26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6925</v>
+        <v>3834</v>
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1175.0900000000001</v>
+        <v>0</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5749.91</v>
+        <v>3834</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4462,11 +4420,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>81458.24000000002</v>
+        <v>97946.510000000024</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>156041.75999999998</v>
+        <v>139553.49</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4477,15 +4435,15 @@
       </c>
       <c r="I27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>9437</v>
+        <v>4955</v>
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>905.3</v>
+        <v>1382.35</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8531.7000000000007</v>
+        <v>3572.65</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4508,11 +4466,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>112523.48000000005</v>
+        <v>131615.06000000003</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>205976.51999999996</v>
+        <v>186884.93999999997</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4587,11 +4545,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>45802.37999999999</v>
+        <v>52551.639999999963</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>88697.62000000001</v>
+        <v>81948.360000000044</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4644,11 +4602,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>54823.51</v>
+        <v>59936.180000000008</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>112176.48999999999</v>
+        <v>107063.81999999999</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4661,11 +4619,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>257833.44999999981</v>
+        <v>257463.44999999984</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>132916.55000000019</v>
+        <v>133286.55000000016</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4704,11 +4662,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>86994.229999999938</v>
+        <v>94488.119999999893</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>173005.77000000008</v>
+        <v>165511.88000000012</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4721,11 +4679,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>505107.28000000294</v>
+        <v>501987.34000000294</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>15892.719999997062</v>
+        <v>19012.659999997064</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4744,11 +4702,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>155.27272727272725</v>
+        <v>114.27272727272725</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4764,11 +4722,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>28935.709999999992</v>
+        <v>40132.44000000001</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>71064.290000000008</v>
+        <v>59867.55999999999</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4781,11 +4739,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>94259.589999999982</v>
+        <v>252730.7799999998</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>556990.41</v>
+        <v>398519.2200000002</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4824,11 +4782,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>14697.789999999988</v>
+        <v>17502.359999999986</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40302.210000000014</v>
+        <v>37497.640000000014</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4884,11 +4842,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>26858.460000000003</v>
+        <v>34782.590000000011</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>46141.539999999994</v>
+        <v>38217.409999999989</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5006,11 +4964,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>546899.75000000163</v>
+        <v>546529.75000000163</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>-156149.75000000163</v>
+        <v>-155779.75000000163</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -5042,11 +5000,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1108736.1299999962</v>
+        <v>1105616.189999996</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="5">C40-D40</f>
-        <v>-587736.12999999616</v>
+        <v>-584616.18999999599</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -5078,11 +5036,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>113453.79</v>
+        <v>478309.18000000156</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="5"/>
-        <v>537796.21</v>
+        <v>172940.81999999844</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 14/07/2026 14:34
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7934FD57-6988-4266-8B7B-466900D4A361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF41945-5C52-43A2-B1F9-42CE66258815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1717,13 +1717,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>19446.750000000004</v>
+            <v>23702.080000000009</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>1382.35</v>
+            <v>5637.6799999999994</v>
           </cell>
         </row>
         <row r="6">
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>151882.9899999999</v>
+            <v>163287.28999999989</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>2591.6000000000004</v>
+            <v>13995.9</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1751,10 +1751,10 @@
             <v>828.94</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>1440.91</v>
+            <v>2662.61</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1771,10 +1771,10 @@
             <v>49.09</v>
           </cell>
           <cell r="H8" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>1092</v>
+            <v>12584.929999999998</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -1788,19 +1788,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>29329.179999999997</v>
+            <v>31991.790000000008</v>
           </cell>
           <cell r="H9" t="str">
-            <v>KEY SP</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>29751.200000000001</v>
+            <v>5619.0999999999985</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N9">
-            <v>22</v>
+            <v>24</v>
           </cell>
         </row>
         <row r="10">
@@ -1808,19 +1808,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>88513.359999999971</v>
+            <v>99657.379999999888</v>
           </cell>
           <cell r="H10" t="str">
-            <v>KEY ZL</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="I10">
-            <v>14725.18</v>
+            <v>1771.4</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N10">
-            <v>12</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="11">
@@ -1828,19 +1828,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>31887.770000000026</v>
+            <v>36414.870000000024</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="I11">
-            <v>259.8</v>
+            <v>10001.5</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N11">
-            <v>19</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="12">
@@ -1848,19 +1848,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>121733.92000000003</v>
+            <v>121733.92000000001</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE MOOCA</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I12">
-            <v>2653.3</v>
+            <v>58720.200000000004</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>12</v>
+            <v>13</v>
           </cell>
         </row>
         <row r="13">
@@ -1871,16 +1871,16 @@
             <v>155213.56</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE PENHA</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I13">
-            <v>4077.82</v>
+            <v>32243.18</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>19</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="14">
@@ -1888,161 +1888,203 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>403983.90000000026</v>
+            <v>405755.30000000022</v>
           </cell>
           <cell r="H14" t="str">
-            <v>MOGI</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I14">
-            <v>604.70000000000005</v>
+            <v>3718.0800000000004</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>21</v>
+            <v>25</v>
           </cell>
         </row>
         <row r="15">
           <cell r="E15" t="str">
-            <v>KEY SJC</v>
+            <v>KEY PIRACICABA</v>
           </cell>
           <cell r="F15">
-            <v>22426.3</v>
+            <v>53478.660000000011</v>
           </cell>
           <cell r="H15" t="str">
-            <v>PIRITUBA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I15">
-            <v>627.6</v>
+            <v>7908.2999999999993</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>38</v>
+            <v>42</v>
           </cell>
         </row>
         <row r="16">
           <cell r="E16" t="str">
-            <v>KEY SP</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>127430.38</v>
+            <v>32427.8</v>
           </cell>
           <cell r="H16" t="str">
-            <v>SANTO ANDRE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I16">
-            <v>772.2</v>
+            <v>13546.770000000002</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N16">
-            <v>21</v>
+            <v>24</v>
           </cell>
         </row>
         <row r="17">
           <cell r="E17" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>159429.97999999995</v>
+            <v>156399.37999999995</v>
           </cell>
           <cell r="H17" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I17">
-            <v>839.76</v>
+            <v>3585.7000000000003</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>17</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
-            <v>LESTE</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>42575.060000000012</v>
+            <v>176947.97999999992</v>
           </cell>
           <cell r="H18" t="str">
-            <v>Total Geral</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I18">
-            <v>60818.42000000002</v>
+            <v>3941.8000000000006</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N18">
-            <v>15</v>
+            <v>17</v>
           </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>73698.819999999992</v>
+            <v>46037.240000000013</v>
+          </cell>
+          <cell r="H19" t="str">
+            <v>NORTE</v>
+          </cell>
+          <cell r="I19">
+            <v>6712.9299999999976</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>228</v>
+            <v>251</v>
           </cell>
         </row>
         <row r="20">
           <cell r="E20" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>52664.26</v>
+            <v>78953.819999999963</v>
+          </cell>
+          <cell r="H20" t="str">
+            <v>OSASCO</v>
+          </cell>
+          <cell r="I20">
+            <v>16027.849999999997</v>
           </cell>
         </row>
         <row r="21">
           <cell r="E21" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>44701.440000000061</v>
+            <v>62133.21</v>
+          </cell>
+          <cell r="H21" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="I21">
+            <v>4568.2299999999996</v>
           </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>22225.860000000011</v>
+            <v>48287.140000000087</v>
+          </cell>
+          <cell r="H22" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="I22">
+            <v>9675.2999999999993</v>
           </cell>
         </row>
         <row r="23">
           <cell r="E23" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>97946.510000000024</v>
+            <v>25582.760000000028</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="I23">
+            <v>15442.449999999999</v>
           </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>131615.06000000003</v>
+            <v>104659.43999999999</v>
+          </cell>
+          <cell r="H24" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I24">
+            <v>2336.44</v>
           </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
-            <v>PIRACICABA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>53478.660000000011</v>
+            <v>147657.61000000002</v>
+          </cell>
+          <cell r="H25" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I25">
+            <v>1169.45</v>
           </cell>
         </row>
         <row r="26">
@@ -2050,7 +2092,13 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>52551.639999999963</v>
+            <v>56494.369999999966</v>
+          </cell>
+          <cell r="H26" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I26">
+            <v>2290.3500000000004</v>
           </cell>
         </row>
         <row r="27">
@@ -2058,7 +2106,13 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>59936.180000000008</v>
+            <v>68839.279999999955</v>
+          </cell>
+          <cell r="H27" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I27">
+            <v>234160.14999999988</v>
           </cell>
         </row>
         <row r="28">
@@ -2066,7 +2120,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>94488.119999999893</v>
+            <v>109930.56999999991</v>
           </cell>
         </row>
         <row r="29">
@@ -2074,7 +2128,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>40132.44000000001</v>
+            <v>40401.58</v>
           </cell>
         </row>
         <row r="30">
@@ -2082,7 +2136,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>17502.359999999986</v>
+            <v>18671.809999999994</v>
           </cell>
         </row>
         <row r="31">
@@ -2090,7 +2144,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>34782.590000000011</v>
+            <v>36233.18</v>
           </cell>
         </row>
         <row r="32">
@@ -2098,7 +2152,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>2130455.1199999726</v>
+            <v>2301770.0499999654</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2951,7 +3005,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>2129626.1799999997</v>
+        <v>2247462.4500000002</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2962,7 +3016,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>16342.04</v>
+        <v>131423.87</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2973,7 +3027,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>44476.380000000005</v>
+        <v>102736.28</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -2984,7 +3038,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>228</v>
+        <v>251</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2996,7 +3050,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>3461873.8200000003</v>
+        <v>3344037.55</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3007,7 +3061,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>183684.96</v>
+        <v>68603.13</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3018,7 +3072,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-44476.380000000005</v>
+        <v>-102736.28</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3029,7 +3083,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>530</v>
+        <v>507</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3041,7 +3095,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.38086849324868099</v>
+        <v>0.4019426719127247</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3052,7 +3106,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>8.1699170611967409E-2</v>
+        <v>0.65703065086213353</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3074,7 +3128,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.30079155672823221</v>
+        <v>0.33113456464379942</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3173,11 +3227,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>19446.750000000004</v>
+        <v>23702.080000000009</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>45053.25</v>
+        <v>40797.919999999991</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3192,11 +3246,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>16027.849999999997</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>20000</v>
+        <v>3972.1500000000033</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3247,11 +3301,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>151882.9899999999</v>
+        <v>163287.28999999989</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>173117.0100000001</v>
+        <v>161712.71000000011</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3266,11 +3320,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>6712.9299999999976</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>13000</v>
+        <v>6287.0700000000024</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3342,11 +3396,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>627.6</v>
+        <v>4568.2299999999996</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>14762.4</v>
+        <v>10821.77</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3380,11 +3434,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3400,11 +3454,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29329.179999999997</v>
+        <v>31991.790000000008</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>60670.820000000007</v>
+        <v>58008.209999999992</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3419,11 +3473,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>15442.449999999999</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>22000</v>
+        <v>6557.5500000000011</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3438,11 +3492,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14725.18</v>
+        <v>32243.18</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-14725.18</v>
+        <v>-32243.18</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3477,11 +3531,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>88513.359999999971</v>
+        <v>99657.379999999888</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>184486.64</v>
+        <v>173342.62000000011</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3496,11 +3550,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>3585.7000000000003</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11529</v>
+        <v>7943.2999999999993</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3515,11 +3569,11 @@
       </c>
       <c r="P14" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1771.4</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-1771.4</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="19" t="s">
@@ -3534,11 +3588,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3554,11 +3608,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>31887.770000000026</v>
+        <v>36414.870000000024</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>46112.229999999974</v>
+        <v>41585.129999999976</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3573,11 +3627,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2591.6000000000004</v>
+        <v>13995.9</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>21408.400000000001</v>
+        <v>10004.1</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3592,11 +3646,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>29751.200000000001</v>
+        <v>58720.200000000004</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-29751.200000000001</v>
+        <v>-58720.200000000004</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3611,11 +3665,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3631,11 +3685,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>121733.92000000003</v>
+        <v>121733.92000000001</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>203266.07999999996</v>
+        <v>203266.08</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3650,11 +3704,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>772.2</v>
+        <v>9675.2999999999993</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10227.799999999999</v>
+        <v>1324.7000000000007</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3669,11 +3723,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>10001.5</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-10001.5</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3727,11 +3781,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>604.70000000000005</v>
+        <v>3941.8000000000006</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6283.3</v>
+        <v>2946.1999999999994</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3785,11 +3839,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>403983.90000000026</v>
+        <v>405755.30000000022</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>546016.09999999974</v>
+        <v>544244.69999999972</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3804,11 +3858,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>259.8</v>
+        <v>3718.0800000000004</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9931.2000000000007</v>
+        <v>6472.92</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3829,11 +3883,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3849,11 +3903,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>22426.3</v>
+        <v>32427.8</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>107573.7</v>
+        <v>97572.2</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3868,11 +3922,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2653.3</v>
+        <v>7908.2999999999993</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8346.7000000000007</v>
+        <v>3091.7000000000007</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3889,11 +3943,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3909,11 +3963,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>127430.38</v>
+        <v>156399.37999999995</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>432569.62</v>
+        <v>403600.62000000005</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3928,11 +3982,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1440.91</v>
+        <v>12584.929999999998</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10559.09</v>
+        <v>-584.92999999999847</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3961,11 +4015,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3981,11 +4035,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>159429.97999999995</v>
+        <v>176947.97999999992</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>255570.02000000005</v>
+        <v>238052.02000000008</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4000,11 +4054,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1092</v>
+        <v>5619.0999999999985</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6658</v>
+        <v>2130.9000000000015</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4017,11 +4071,11 @@
       </c>
       <c r="P21" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>275241.61999999988</v>
+        <v>266634.81999999995</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>96349.289090909238</v>
+        <v>104956.08909090917</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="19" t="s">
@@ -4036,11 +4090,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -4056,11 +4110,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>42575.060000000012</v>
+        <v>46037.240000000013</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>79424.939999999988</v>
+        <v>75962.75999999998</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4075,11 +4129,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4077.82</v>
+        <v>13546.770000000002</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6212.18</v>
+        <v>-3256.7700000000023</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4092,11 +4146,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>564728.75000000023</v>
+        <v>521362.39000000031</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-69274.204545454762</v>
+        <v>-25907.844545454835</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4111,11 +4165,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4131,11 +4185,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>73698.819999999992</v>
+        <v>78953.819999999963</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>121301.18000000001</v>
+        <v>116046.18000000004</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4150,11 +4204,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>2662.61</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7510</v>
+        <v>4847.3899999999994</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4167,11 +4221,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>203726.33000000016</v>
+        <v>260480.73000000019</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>415591.85181818169</v>
+        <v>358837.45181818167</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4206,11 +4260,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52664.26</v>
+        <v>62133.21</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>87335.739999999991</v>
+        <v>77866.790000000008</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4225,11 +4279,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>839.76</v>
+        <v>2290.3500000000004</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3090.24</v>
+        <v>1639.6499999999996</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4261,11 +4315,11 @@
       </c>
       <c r="V24" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="W24" s="19">
         <f t="shared" si="2"/>
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -4281,11 +4335,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>44701.440000000061</v>
+        <v>48287.140000000087</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>97798.559999999939</v>
+        <v>94212.859999999913</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4300,11 +4354,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>2336.44</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4760</v>
+        <v>2423.56</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4336,11 +4390,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4356,11 +4410,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>22225.860000000011</v>
+        <v>25582.760000000028</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>67774.139999999985</v>
+        <v>64417.239999999976</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4375,11 +4429,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1169.45</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3834</v>
+        <v>2664.55</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4420,11 +4474,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>97946.510000000024</v>
+        <v>104659.43999999999</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>139553.49</v>
+        <v>132840.56</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4439,11 +4493,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1382.35</v>
+        <v>5637.6799999999994</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3572.65</v>
+        <v>-682.67999999999938</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4466,11 +4520,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>131615.06000000003</v>
+        <v>147657.61000000002</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>186884.93999999997</v>
+        <v>170842.38999999998</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4499,11 +4553,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>53478.660000000011</v>
+        <v>0</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>121521.34</v>
+        <v>175000</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4545,11 +4599,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52551.639999999963</v>
+        <v>56494.369999999966</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>81948.360000000044</v>
+        <v>78005.630000000034</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4602,11 +4656,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>59936.180000000008</v>
+        <v>68839.279999999955</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>107063.81999999999</v>
+        <v>98160.720000000045</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4662,11 +4716,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>94488.119999999893</v>
+        <v>109930.56999999991</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>165511.88000000012</v>
+        <v>150069.43000000011</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4679,11 +4733,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>501987.34000000294</v>
+        <v>501987.34000000282</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>19012.659999997064</v>
+        <v>19012.65999999718</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4702,11 +4756,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>114.27272727272725</v>
+        <v>74.272727272727252</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4722,11 +4776,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>40132.44000000001</v>
+        <v>40401.58</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>59867.55999999999</v>
+        <v>59598.42</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4739,11 +4793,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>252730.7799999998</v>
+        <v>360530.81000000145</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>398519.2200000002</v>
+        <v>290719.18999999855</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4782,11 +4836,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>17502.359999999986</v>
+        <v>18671.809999999994</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>37497.640000000014</v>
+        <v>36328.19</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4842,11 +4896,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>34782.590000000011</v>
+        <v>36233.18</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>38217.409999999989</v>
+        <v>36766.82</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5036,11 +5090,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>478309.18000000156</v>
+        <v>649624.1100000015</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="5"/>
-        <v>172940.81999999844</v>
+        <v>1625.8899999985006</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 15/07/2026 10:43
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF41945-5C52-43A2-B1F9-42CE66258815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED691EA2-CBFE-45AF-822A-FDF60FBF7374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-14T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-15T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1681,7 +1681,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>14/07/2026</v>
+            <v>15/07/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1717,13 +1717,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>23702.080000000009</v>
+            <v>24454.740000000013</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>5637.6799999999994</v>
+            <v>752.66</v>
           </cell>
         </row>
         <row r="6">
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>163287.28999999989</v>
+            <v>167704.68999999997</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>13995.9</v>
+            <v>4417.3999999999996</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1754,7 +1754,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>2662.61</v>
+            <v>1821.55</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1774,7 +1774,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>12584.929999999998</v>
+            <v>2153.4100000000003</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -1788,19 +1788,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>31991.790000000008</v>
+            <v>33813.340000000011</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>5619.0999999999985</v>
+            <v>430.7</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N9">
-            <v>24</v>
+            <v>27</v>
           </cell>
         </row>
         <row r="10">
@@ -1808,19 +1808,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>99657.379999999888</v>
+            <v>101810.78999999988</v>
           </cell>
           <cell r="H10" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>1771.4</v>
+            <v>32482.3</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N10">
-            <v>14</v>
+            <v>15</v>
           </cell>
         </row>
         <row r="11">
@@ -1828,13 +1828,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>36414.870000000024</v>
+            <v>36845.570000000022</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY SJC</v>
+            <v>KEY PIRACICABA</v>
           </cell>
           <cell r="I11">
-            <v>10001.5</v>
+            <v>6603.5999999999995</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
@@ -1848,19 +1848,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>121733.92000000001</v>
+            <v>157577.22</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY SP</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I12">
-            <v>58720.200000000004</v>
+            <v>14711.1</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>13</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="13">
@@ -1871,16 +1871,16 @@
             <v>155213.56</v>
           </cell>
           <cell r="H13" t="str">
-            <v>KEY ZL</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I13">
-            <v>32243.18</v>
+            <v>3522.58</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>20</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="14">
@@ -1888,19 +1888,19 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>405755.30000000022</v>
+            <v>513142.70000000019</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I14">
-            <v>3718.0800000000004</v>
+            <v>1281.27</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>25</v>
+            <v>28</v>
           </cell>
         </row>
         <row r="15">
@@ -1908,13 +1908,13 @@
             <v>KEY PIRACICABA</v>
           </cell>
           <cell r="F15">
-            <v>53478.660000000011</v>
+            <v>60082.260000000017</v>
           </cell>
           <cell r="H15" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I15">
-            <v>7908.2999999999993</v>
+            <v>1057.27</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
@@ -1931,10 +1931,10 @@
             <v>32427.8</v>
           </cell>
           <cell r="H16" t="str">
-            <v>LESTE PENHA</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I16">
-            <v>13546.770000000002</v>
+            <v>1303.8999999999999</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -1948,19 +1948,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>156399.37999999995</v>
+            <v>169833.12000000005</v>
           </cell>
           <cell r="H17" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I17">
-            <v>3585.7000000000003</v>
+            <v>3292.2000000000003</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>19</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="18">
@@ -1968,13 +1968,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>176947.97999999992</v>
+            <v>191659.07999999996</v>
           </cell>
           <cell r="H18" t="str">
-            <v>MOGI</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I18">
-            <v>3941.8000000000006</v>
+            <v>5830.3999999999987</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -1988,19 +1988,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>46037.240000000013</v>
+            <v>46497.760000000017</v>
           </cell>
           <cell r="H19" t="str">
-            <v>NORTE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I19">
-            <v>6712.9299999999976</v>
+            <v>1084.3</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>251</v>
+            <v>261</v>
           </cell>
         </row>
         <row r="20">
@@ -2008,13 +2008,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>78953.819999999963</v>
+            <v>82493.399999999936</v>
           </cell>
           <cell r="H20" t="str">
-            <v>OSASCO</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I20">
-            <v>16027.849999999997</v>
+            <v>3827.7799999999997</v>
           </cell>
         </row>
         <row r="21">
@@ -2022,13 +2022,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>62133.21</v>
+            <v>63414.48000000001</v>
           </cell>
           <cell r="H21" t="str">
-            <v>PIRITUBA</v>
+            <v>SJC</v>
           </cell>
           <cell r="I21">
-            <v>4568.2299999999996</v>
+            <v>1411.48</v>
           </cell>
         </row>
         <row r="22">
@@ -2036,13 +2036,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>48287.140000000087</v>
+            <v>49344.410000000084</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SANTO ANDRE</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I22">
-            <v>9675.2999999999993</v>
+            <v>450</v>
           </cell>
         </row>
         <row r="23">
@@ -2050,13 +2050,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>25582.760000000028</v>
+            <v>27692.540000000045</v>
           </cell>
           <cell r="H23" t="str">
-            <v>SBC</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I23">
-            <v>15442.449999999999</v>
+            <v>86433.899999999965</v>
           </cell>
         </row>
         <row r="24">
@@ -2064,13 +2064,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>104659.43999999999</v>
-          </cell>
-          <cell r="H24" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I24">
-            <v>2336.44</v>
+            <v>107951.63999999998</v>
           </cell>
         </row>
         <row r="25">
@@ -2078,13 +2072,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>147657.61000000002</v>
-          </cell>
-          <cell r="H25" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I25">
-            <v>1169.45</v>
+            <v>153528.00999999989</v>
           </cell>
         </row>
         <row r="26">
@@ -2092,13 +2080,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>56494.369999999966</v>
-          </cell>
-          <cell r="H26" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I26">
-            <v>2290.3500000000004</v>
+            <v>59683.469999999965</v>
           </cell>
         </row>
         <row r="27">
@@ -2106,13 +2088,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>68839.279999999955</v>
-          </cell>
-          <cell r="H27" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I27">
-            <v>234160.14999999988</v>
+            <v>73953.459999999963</v>
           </cell>
         </row>
         <row r="28">
@@ -2120,7 +2096,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>109930.56999999991</v>
+            <v>110078.8099999999</v>
           </cell>
         </row>
         <row r="29">
@@ -2128,7 +2104,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>40401.58</v>
+            <v>41813.060000000027</v>
           </cell>
         </row>
         <row r="30">
@@ -2136,7 +2112,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>18671.809999999994</v>
+            <v>19234.969999999994</v>
           </cell>
         </row>
         <row r="31">
@@ -2144,7 +2120,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>36233.18</v>
+            <v>37192.940000000017</v>
           </cell>
         </row>
         <row r="32">
@@ -2152,7 +2128,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>2301770.0499999654</v>
+            <v>2518321.8499999698</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2971,7 +2947,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>200027</v>
+        <v>150013</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -3005,7 +2981,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>2247462.4500000002</v>
+        <v>2457410.65</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3016,7 +2992,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>131423.87</v>
+        <v>32636.9</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3027,7 +3003,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>102736.28</v>
+        <v>47193.4</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3038,7 +3014,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3050,7 +3026,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>3344037.55</v>
+        <v>3134089.35</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3061,7 +3037,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>68603.13</v>
+        <v>117376.1</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3072,7 +3048,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-102736.28</v>
+        <v>-47193.4</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3083,7 +3059,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>507</v>
+        <v>497</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3095,7 +3071,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.4019426719127247</v>
+        <v>0.43949041402128231</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3106,7 +3082,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.65703065086213353</v>
+        <v>0.21756047809189871</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3128,7 +3104,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.33113456464379942</v>
+        <v>0.34432717678100266</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3227,11 +3203,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>23702.080000000009</v>
+        <v>24454.740000000013</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40797.919999999991</v>
+        <v>40045.259999999987</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3242,15 +3218,15 @@
       </c>
       <c r="I10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>20000</v>
+        <v>17000</v>
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>16027.849999999997</v>
+        <v>5830.3999999999987</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3972.1500000000033</v>
+        <v>11169.600000000002</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3301,11 +3277,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>163287.28999999989</v>
+        <v>167704.68999999997</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>161712.71000000011</v>
+        <v>157295.31000000003</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3316,15 +3292,15 @@
       </c>
       <c r="I11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13000</v>
+        <v>11850</v>
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6712.9299999999976</v>
+        <v>3292.2000000000003</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6287.0700000000024</v>
+        <v>8557.7999999999993</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3339,11 +3315,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>32482.3</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>0</v>
+        <v>-32482.3</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3392,15 +3368,15 @@
       </c>
       <c r="I12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15390</v>
+        <v>9000</v>
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4568.2299999999996</v>
+        <v>1084.3</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10821.77</v>
+        <v>7915.7</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3434,11 +3410,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3454,11 +3430,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>31991.790000000008</v>
+        <v>33813.340000000011</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>58008.209999999992</v>
+        <v>56186.659999999989</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3469,15 +3445,15 @@
       </c>
       <c r="I13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>22000</v>
+        <v>15000</v>
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>15442.449999999999</v>
+        <v>0</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6557.5500000000011</v>
+        <v>15000</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3492,11 +3468,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>32243.18</v>
+        <v>14711.1</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-32243.18</v>
+        <v>-14711.1</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3531,11 +3507,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>99657.379999999888</v>
+        <v>101810.78999999988</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>173342.62000000011</v>
+        <v>171189.21000000014</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3546,15 +3522,15 @@
       </c>
       <c r="I14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11529</v>
+        <v>5324</v>
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3585.7000000000003</v>
+        <v>1057.27</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7943.2999999999993</v>
+        <v>4266.7299999999996</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3569,11 +3545,11 @@
       </c>
       <c r="P14" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1771.4</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" si="1"/>
-        <v>-1771.4</v>
+        <v>0</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="19" t="s">
@@ -3588,11 +3564,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3608,11 +3584,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>36414.870000000024</v>
+        <v>36845.570000000022</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41585.129999999976</v>
+        <v>41154.429999999978</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3623,15 +3599,15 @@
       </c>
       <c r="I15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>24000</v>
+        <v>16000</v>
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13995.9</v>
+        <v>4417.3999999999996</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10004.1</v>
+        <v>11582.6</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3646,11 +3622,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>58720.200000000004</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-58720.200000000004</v>
+        <v>0</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3685,11 +3661,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>121733.92000000001</v>
+        <v>157577.22</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>203266.08</v>
+        <v>167422.78</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3700,15 +3676,15 @@
       </c>
       <c r="I16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11000</v>
+        <v>12810</v>
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9675.2999999999993</v>
+        <v>3827.7799999999997</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1324.7000000000007</v>
+        <v>8982.2200000000012</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3723,11 +3699,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10001.5</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>-10001.5</v>
+        <v>0</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3777,15 +3753,15 @@
       </c>
       <c r="I17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6888</v>
+        <v>3144</v>
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3941.8000000000006</v>
+        <v>1303.8999999999999</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2946.1999999999994</v>
+        <v>1840.1000000000001</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3839,11 +3815,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>405755.30000000022</v>
+        <v>513142.70000000019</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>544244.69999999972</v>
+        <v>436857.29999999981</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3854,15 +3830,15 @@
       </c>
       <c r="I18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>10191</v>
+        <v>6216</v>
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3718.0800000000004</v>
+        <v>0</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6472.92</v>
+        <v>6216</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3883,11 +3859,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3918,15 +3894,15 @@
       </c>
       <c r="I19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11000</v>
+        <v>10870</v>
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7908.2999999999993</v>
+        <v>3522.58</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3091.7000000000007</v>
+        <v>7347.42</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3963,11 +3939,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>156399.37999999995</v>
+        <v>169833.12000000005</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>403600.62000000005</v>
+        <v>390166.87999999995</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3978,15 +3954,15 @@
       </c>
       <c r="I20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>12584.929999999998</v>
+        <v>2153.4100000000003</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-584.92999999999847</v>
+        <v>10846.59</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4015,11 +3991,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4035,11 +4011,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>176947.97999999992</v>
+        <v>191659.07999999996</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>238052.02000000008</v>
+        <v>223340.92000000004</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4050,15 +4026,15 @@
       </c>
       <c r="I21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>7750</v>
+        <v>5020</v>
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5619.0999999999985</v>
+        <v>430.7</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2130.9000000000015</v>
+        <v>4589.3</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4110,11 +4086,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>46037.240000000013</v>
+        <v>46497.760000000017</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>75962.75999999998</v>
+        <v>75502.239999999991</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4125,15 +4101,15 @@
       </c>
       <c r="I22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>10290</v>
+        <v>8104</v>
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13546.770000000002</v>
+        <v>1281.27</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-3256.7700000000023</v>
+        <v>6822.73</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4165,11 +4141,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4185,11 +4161,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>78953.819999999963</v>
+        <v>82493.399999999936</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>116046.18000000004</v>
+        <v>112506.60000000006</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4200,15 +4176,15 @@
       </c>
       <c r="I23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>7510</v>
+        <v>5255</v>
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2662.61</v>
+        <v>1821.55</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4847.3899999999994</v>
+        <v>3433.45</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4221,11 +4197,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>260480.73000000019</v>
+        <v>431856.27</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>358837.45181818167</v>
+        <v>187461.91181818186</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4260,11 +4236,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>62133.21</v>
+        <v>63414.48000000001</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>77866.790000000008</v>
+        <v>76585.51999999999</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4275,15 +4251,15 @@
       </c>
       <c r="I24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3930</v>
+        <v>3110</v>
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2290.3500000000004</v>
+        <v>450</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1639.6499999999996</v>
+        <v>2660</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4335,11 +4311,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>48287.140000000087</v>
+        <v>49344.410000000084</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>94212.859999999913</v>
+        <v>93155.589999999909</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4350,15 +4326,15 @@
       </c>
       <c r="I25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4760</v>
+        <v>3570</v>
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2336.44</v>
+        <v>1411.48</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2423.56</v>
+        <v>2158.52</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4390,11 +4366,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4410,11 +4386,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>25582.760000000028</v>
+        <v>27692.540000000045</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>64417.239999999976</v>
+        <v>62307.459999999955</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4425,15 +4401,15 @@
       </c>
       <c r="I26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3834</v>
+        <v>2442</v>
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1169.45</v>
+        <v>0</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2664.55</v>
+        <v>2442</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4474,11 +4450,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>104659.43999999999</v>
+        <v>107951.63999999998</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>132840.56</v>
+        <v>129548.36000000002</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4489,15 +4465,15 @@
       </c>
       <c r="I27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4955</v>
+        <v>2298</v>
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5637.6799999999994</v>
+        <v>752.66</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-682.67999999999938</v>
+        <v>1545.3400000000001</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4520,11 +4496,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>147657.61000000002</v>
+        <v>153528.00999999989</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>170842.38999999998</v>
+        <v>164971.99000000011</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4599,11 +4575,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>56494.369999999966</v>
+        <v>59683.469999999965</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>78005.630000000034</v>
+        <v>74816.530000000028</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4656,11 +4632,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>68839.279999999955</v>
+        <v>73953.459999999963</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>98160.720000000045</v>
+        <v>93046.540000000037</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4673,11 +4649,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>257463.44999999984</v>
+        <v>257463.44999999981</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>133286.55000000016</v>
+        <v>133286.55000000019</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4716,11 +4692,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>109930.56999999991</v>
+        <v>110078.8099999999</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>150069.43000000011</v>
+        <v>149921.19000000012</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4733,11 +4709,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>501987.34000000282</v>
+        <v>501987.34000000305</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>19012.65999999718</v>
+        <v>19012.659999996948</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4756,11 +4732,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>74.272727272727252</v>
+        <v>60.272727272727252</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4776,11 +4752,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>40401.58</v>
+        <v>41813.060000000027</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>59598.42</v>
+        <v>58186.939999999973</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4793,11 +4769,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>360530.81000000145</v>
+        <v>395563.89000000176</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>290719.18999999855</v>
+        <v>255686.10999999824</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4836,11 +4812,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>18671.809999999994</v>
+        <v>19234.969999999994</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>36328.19</v>
+        <v>35765.030000000006</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4896,11 +4872,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>36233.18</v>
+        <v>37192.940000000017</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>36766.82</v>
+        <v>35807.059999999983</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5090,11 +5066,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>649624.1100000015</v>
+        <v>866175.91000000038</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="5"/>
-        <v>1625.8899999985006</v>
+        <v>-214925.91000000038</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 16/07/2026 10:53
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED691EA2-CBFE-45AF-822A-FDF60FBF7374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E24D37A4-C358-402B-91D2-ED35B1899860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-15T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-16T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1681,7 +1681,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>15/07/2026</v>
+            <v>16/07/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1717,13 +1717,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>24454.740000000013</v>
+            <v>26930.750000000011</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>752.66</v>
+            <v>1304.31</v>
           </cell>
         </row>
         <row r="6">
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>167704.68999999997</v>
+            <v>181896.29</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>4417.3999999999996</v>
+            <v>6844.6999999999989</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1754,7 +1754,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>1821.55</v>
+            <v>2016.5</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1768,19 +1768,19 @@
             <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F8">
-            <v>49.09</v>
+            <v>100.09</v>
           </cell>
           <cell r="H8" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>2153.4100000000003</v>
+            <v>2353.0999999999995</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N8">
-            <v>32</v>
+            <v>34</v>
           </cell>
         </row>
         <row r="9">
@@ -1788,19 +1788,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>33813.340000000011</v>
+            <v>36891.44000000001</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>430.7</v>
+            <v>781.7600000000001</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N9">
-            <v>27</v>
+            <v>29</v>
           </cell>
         </row>
         <row r="10">
@@ -1808,19 +1808,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>101810.78999999988</v>
+            <v>111316.87999999987</v>
           </cell>
           <cell r="H10" t="str">
             <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>32482.3</v>
+            <v>13637.5</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N10">
-            <v>15</v>
+            <v>16</v>
           </cell>
         </row>
         <row r="11">
@@ -1828,19 +1828,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>36845.570000000022</v>
+            <v>40012.410000000025</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY PIRACICABA</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I11">
-            <v>6603.5999999999995</v>
+            <v>11566.400000000001</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N11">
-            <v>21</v>
+            <v>25</v>
           </cell>
         </row>
         <row r="12">
@@ -1848,19 +1848,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>157577.22</v>
+            <v>174575.71999999997</v>
           </cell>
           <cell r="H12" t="str">
             <v>KEY ZL</v>
           </cell>
           <cell r="I12">
-            <v>14711.1</v>
+            <v>3075.6</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>14</v>
+            <v>16</v>
           </cell>
         </row>
         <row r="13">
@@ -1868,19 +1868,19 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>155213.56</v>
+            <v>161197.35999999999</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I13">
-            <v>3522.58</v>
+            <v>856.4</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>21</v>
+            <v>23</v>
           </cell>
         </row>
         <row r="14">
@@ -1891,16 +1891,16 @@
             <v>513142.70000000019</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I14">
-            <v>1281.27</v>
+            <v>1293</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>28</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="15">
@@ -1911,16 +1911,16 @@
             <v>60082.260000000017</v>
           </cell>
           <cell r="H15" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I15">
-            <v>1057.27</v>
+            <v>996.34999999999991</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>42</v>
+            <v>45</v>
           </cell>
         </row>
         <row r="16">
@@ -1928,19 +1928,19 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>32427.8</v>
+            <v>36418.899999999994</v>
           </cell>
           <cell r="H16" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I16">
-            <v>1303.8999999999999</v>
+            <v>1434.75</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="N16">
-            <v>24</v>
+            <v>27</v>
           </cell>
         </row>
         <row r="17">
@@ -1948,19 +1948,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>169833.12000000005</v>
+            <v>181399.52000000014</v>
           </cell>
           <cell r="H17" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I17">
-            <v>3292.2000000000003</v>
+            <v>2197.6</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>20</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="18">
@@ -1968,19 +1968,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>191659.07999999996</v>
+            <v>206904.88</v>
           </cell>
           <cell r="H18" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I18">
-            <v>5830.3999999999987</v>
+            <v>9723</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N18">
-            <v>17</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="19">
@@ -1988,19 +1988,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>46497.760000000017</v>
+            <v>50153.310000000019</v>
           </cell>
           <cell r="H19" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I19">
-            <v>1084.3</v>
+            <v>3754.1</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>261</v>
+            <v>285</v>
           </cell>
         </row>
         <row r="20">
@@ -2008,13 +2008,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>82493.399999999936</v>
+            <v>88647.899999999878</v>
           </cell>
           <cell r="H20" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I20">
-            <v>3827.7799999999997</v>
+            <v>2872.3700000000003</v>
           </cell>
         </row>
         <row r="21">
@@ -2022,13 +2022,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>63414.48000000001</v>
+            <v>65392.23</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SJC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I21">
-            <v>1411.48</v>
+            <v>853.1</v>
           </cell>
         </row>
         <row r="22">
@@ -2036,13 +2036,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>49344.410000000084</v>
+            <v>53035.3100000001</v>
           </cell>
           <cell r="H22" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SBC</v>
           </cell>
           <cell r="I22">
-            <v>450</v>
+            <v>5748.5499999999984</v>
           </cell>
         </row>
         <row r="23">
@@ -2050,13 +2050,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>27692.540000000045</v>
+            <v>30794.440000000057</v>
           </cell>
           <cell r="H23" t="str">
-            <v>Total Geral</v>
+            <v>SJC</v>
           </cell>
           <cell r="I23">
-            <v>86433.899999999965</v>
+            <v>1202.75</v>
           </cell>
         </row>
         <row r="24">
@@ -2064,7 +2064,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>107951.63999999998</v>
+            <v>124836.28999999983</v>
+          </cell>
+          <cell r="H24" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I24">
+            <v>665.54</v>
           </cell>
         </row>
         <row r="25">
@@ -2072,7 +2078,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>153528.00999999989</v>
+            <v>165483.18</v>
+          </cell>
+          <cell r="H25" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I25">
+            <v>1040.82</v>
           </cell>
         </row>
         <row r="26">
@@ -2080,7 +2092,13 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>59683.469999999965</v>
+            <v>68864.489999999962</v>
+          </cell>
+          <cell r="H26" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I26">
+            <v>74218.2</v>
           </cell>
         </row>
         <row r="27">
@@ -2088,7 +2106,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>73953.459999999963</v>
+            <v>77338.629999999946</v>
           </cell>
         </row>
         <row r="28">
@@ -2096,7 +2114,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>110078.8099999999</v>
+            <v>126422.29999999987</v>
           </cell>
         </row>
         <row r="29">
@@ -2104,7 +2122,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>41813.060000000027</v>
+            <v>44063.920000000042</v>
           </cell>
         </row>
         <row r="30">
@@ -2112,7 +2130,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>19234.969999999994</v>
+            <v>20737.710000000003</v>
           </cell>
         </row>
         <row r="31">
@@ -2120,7 +2138,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>37192.940000000017</v>
+            <v>38431.760000000009</v>
           </cell>
         </row>
         <row r="32">
@@ -2128,7 +2146,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>2518321.8499999698</v>
+            <v>2685899.6099999631</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2981,7 +2999,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>2457410.65</v>
+        <v>2624988.4099999992</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2992,7 +3010,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>32636.9</v>
+        <v>45938.7</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3003,7 +3021,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>47193.4</v>
+        <v>28279.5</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3014,7 +3032,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>261</v>
+        <v>285</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3026,7 +3044,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>3134089.35</v>
+        <v>2966511.5900000008</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3037,7 +3055,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>117376.1</v>
+        <v>104074.3</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3048,7 +3066,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-47193.4</v>
+        <v>-28279.5</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3059,7 +3077,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>497</v>
+        <v>473</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3071,7 +3089,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.43949041402128231</v>
+        <v>0.46946050433693987</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3082,7 +3100,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.21756047809189871</v>
+        <v>0.30623145994013845</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3104,7 +3122,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.34432717678100266</v>
+        <v>0.37598944591029027</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3203,11 +3221,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>24454.740000000013</v>
+        <v>26930.750000000011</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40045.259999999987</v>
+        <v>37569.249999999985</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3222,11 +3240,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5830.3999999999987</v>
+        <v>3754.1</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11169.600000000002</v>
+        <v>13245.9</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3277,11 +3295,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>167704.68999999997</v>
+        <v>181896.29</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>157295.31000000003</v>
+        <v>143103.71</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3296,11 +3314,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3292.2000000000003</v>
+        <v>9723</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8557.7999999999993</v>
+        <v>2127</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3315,11 +3333,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>32482.3</v>
+        <v>13637.5</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>-32482.3</v>
+        <v>-13637.5</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3334,11 +3352,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3353,11 +3371,11 @@
       </c>
       <c r="D12" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>49.09</v>
+        <v>100.09</v>
       </c>
       <c r="E12" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>950.91</v>
+        <v>899.91</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="21" t="s">
@@ -3372,11 +3390,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1084.3</v>
+        <v>2872.3700000000003</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7915.7</v>
+        <v>6127.6299999999992</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3410,11 +3428,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3430,11 +3448,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>33813.340000000011</v>
+        <v>36891.44000000001</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>56186.659999999989</v>
+        <v>53108.55999999999</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3449,11 +3467,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>5748.5499999999984</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15000</v>
+        <v>9251.4500000000007</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3468,11 +3486,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14711.1</v>
+        <v>3075.6</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-14711.1</v>
+        <v>-3075.6</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3507,11 +3525,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>101810.78999999988</v>
+        <v>111316.87999999987</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>171189.21000000014</v>
+        <v>161683.12000000011</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3526,11 +3544,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1057.27</v>
+        <v>1434.75</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4266.7299999999996</v>
+        <v>3889.25</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3564,11 +3582,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3584,11 +3602,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>36845.570000000022</v>
+        <v>40012.410000000025</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41154.429999999978</v>
+        <v>37987.589999999975</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3603,11 +3621,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4417.3999999999996</v>
+        <v>6844.6999999999989</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11582.6</v>
+        <v>9155.3000000000011</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3622,11 +3640,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>11566.400000000001</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-11566.400000000001</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3641,11 +3659,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3661,11 +3679,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>157577.22</v>
+        <v>174575.71999999997</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>167422.78</v>
+        <v>150424.28000000003</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3680,11 +3698,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3827.7799999999997</v>
+        <v>853.1</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8982.2200000000012</v>
+        <v>11956.9</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3738,11 +3756,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>155213.56</v>
+        <v>161197.35999999999</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>14786.440000000002</v>
+        <v>8802.640000000014</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3757,11 +3775,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1303.8999999999999</v>
+        <v>2197.6</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1840.1000000000001</v>
+        <v>946.40000000000009</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3834,11 +3852,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>856.4</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6216</v>
+        <v>5359.6</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3859,11 +3877,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3879,11 +3897,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>32427.8</v>
+        <v>36418.899999999994</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>97572.2</v>
+        <v>93581.1</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3898,11 +3916,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3522.58</v>
+        <v>1293</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7347.42</v>
+        <v>9577</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3919,11 +3937,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3939,11 +3957,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>169833.12000000005</v>
+        <v>181399.52000000014</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>390166.87999999995</v>
+        <v>378600.47999999986</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3958,11 +3976,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2153.4100000000003</v>
+        <v>2353.0999999999995</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10846.59</v>
+        <v>10646.900000000001</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3991,11 +4009,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4011,11 +4029,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>191659.07999999996</v>
+        <v>206904.88</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>223340.92000000004</v>
+        <v>208095.12</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4030,11 +4048,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>430.7</v>
+        <v>781.7600000000001</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4589.3</v>
+        <v>4238.24</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4047,11 +4065,11 @@
       </c>
       <c r="P21" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>266634.81999999995</v>
+        <v>266634.81999999983</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>104956.08909090917</v>
+        <v>104956.08909090929</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="19" t="s">
@@ -4066,11 +4084,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -4086,11 +4104,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>46497.760000000017</v>
+        <v>50153.310000000019</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>75502.239999999991</v>
+        <v>71846.689999999973</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4105,11 +4123,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1281.27</v>
+        <v>996.34999999999991</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6822.73</v>
+        <v>7107.65</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4122,11 +4140,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>521362.39000000031</v>
+        <v>520408.39000000031</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-25907.844545454835</v>
+        <v>-24953.844545454835</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4141,11 +4159,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4161,11 +4179,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>82493.399999999936</v>
+        <v>88647.899999999878</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>112506.60000000006</v>
+        <v>106352.10000000012</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4180,11 +4198,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1821.55</v>
+        <v>2016.5</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3433.45</v>
+        <v>3238.5</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4197,11 +4215,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>431856.27</v>
+        <v>486595.86999999976</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>187461.91181818186</v>
+        <v>132722.31181818212</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4236,11 +4254,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>63414.48000000001</v>
+        <v>65392.23</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>76585.51999999999</v>
+        <v>74607.76999999999</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4255,11 +4273,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>450</v>
+        <v>1040.82</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2660</v>
+        <v>2069.1800000000003</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4291,11 +4309,11 @@
       </c>
       <c r="V24" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W24" s="19">
         <f t="shared" si="2"/>
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -4311,11 +4329,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>49344.410000000084</v>
+        <v>53035.3100000001</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>93155.589999999909</v>
+        <v>89464.6899999999</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4330,11 +4348,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1411.48</v>
+        <v>1202.75</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2158.52</v>
+        <v>2367.25</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4366,11 +4384,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4386,11 +4404,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>27692.540000000045</v>
+        <v>30794.440000000057</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>62307.459999999955</v>
+        <v>59205.559999999939</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4405,11 +4423,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>665.54</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2442</v>
+        <v>1776.46</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4450,11 +4468,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>107951.63999999998</v>
+        <v>124836.28999999983</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>129548.36000000002</v>
+        <v>112663.71000000017</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4469,11 +4487,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>752.66</v>
+        <v>1304.31</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1545.3400000000001</v>
+        <v>993.69</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4496,11 +4514,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>153528.00999999989</v>
+        <v>165483.18</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>164971.99000000011</v>
+        <v>153016.82</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4575,11 +4593,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>59683.469999999965</v>
+        <v>68864.489999999962</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>74816.530000000028</v>
+        <v>65635.510000000038</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4632,11 +4650,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>73953.459999999963</v>
+        <v>77338.629999999946</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>93046.540000000037</v>
+        <v>89661.370000000054</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4649,11 +4667,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>257463.44999999981</v>
+        <v>256807.39999999982</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>133286.55000000019</v>
+        <v>133942.60000000018</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4692,11 +4710,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>110078.8099999999</v>
+        <v>126422.29999999987</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>149921.19000000012</v>
+        <v>133577.70000000013</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4709,11 +4727,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>501987.34000000305</v>
+        <v>501987.34000000299</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>19012.659999996948</v>
+        <v>19012.659999997006</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4732,11 +4750,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>60.272727272727252</v>
+        <v>27.272727272727252</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4752,11 +4770,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>41813.060000000027</v>
+        <v>44063.920000000042</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>58186.939999999973</v>
+        <v>55936.079999999958</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4769,11 +4787,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>395563.89000000176</v>
+        <v>503806.60000000341</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>255686.10999999824</v>
+        <v>147443.39999999659</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4812,11 +4830,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>19234.969999999994</v>
+        <v>20737.710000000003</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>35765.030000000006</v>
+        <v>34262.289999999994</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4872,11 +4890,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>37192.940000000017</v>
+        <v>38431.760000000009</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>35807.059999999983</v>
+        <v>34568.239999999991</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4994,11 +5012,11 @@
       </c>
       <c r="D39" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>546529.75000000163</v>
+        <v>545873.70000000158</v>
       </c>
       <c r="E39" s="7">
         <f>C39-D39</f>
-        <v>-155779.75000000163</v>
+        <v>-155123.70000000158</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -5030,11 +5048,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1105616.189999996</v>
+        <v>1104662.189999996</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="5">C40-D40</f>
-        <v>-584616.18999999599</v>
+        <v>-583662.18999999599</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -5066,11 +5084,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>866175.91000000038</v>
+        <v>1035363.7200000017</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="5"/>
-        <v>-214925.91000000038</v>
+        <v>-384113.72000000172</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 16/07/2026 10:59
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E24D37A4-C358-402B-91D2-ED35B1899860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523F3A00-42F7-41D0-8F02-318644F30C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1653,11 +1653,11 @@
       <sheetName val="BASE PYTHON"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">

</xml_diff>

<commit_message>
Dados atualizados em 16/07/2026 11:12
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523F3A00-42F7-41D0-8F02-318644F30C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80BB754-168F-4AE0-B070-0AE48CF8C55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>181896.29</v>
+            <v>183405.49</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>6844.6999999999989</v>
+            <v>8353.8999999999978</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1754,7 +1754,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>2016.5</v>
+            <v>2265.44</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1774,7 +1774,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>2353.0999999999995</v>
+            <v>3766.8999999999996</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -1788,13 +1788,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>36891.44000000001</v>
+            <v>37140.380000000012</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>781.7600000000001</v>
+            <v>791.7600000000001</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
@@ -1808,7 +1808,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>111316.87999999987</v>
+            <v>112730.67999999986</v>
           </cell>
           <cell r="H10" t="str">
             <v>KEY ABC</v>
@@ -1828,13 +1828,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>40012.410000000025</v>
+            <v>40022.410000000025</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY SP</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="I11">
-            <v>11566.400000000001</v>
+            <v>4337</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
@@ -1851,10 +1851,10 @@
             <v>174575.71999999997</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I12">
-            <v>3075.6</v>
+            <v>11566.400000000001</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
@@ -1871,10 +1871,10 @@
             <v>161197.35999999999</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I13">
-            <v>856.4</v>
+            <v>3075.6</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
@@ -1891,10 +1891,10 @@
             <v>513142.70000000019</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I14">
-            <v>1293</v>
+            <v>856.4</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
@@ -1911,10 +1911,10 @@
             <v>60082.260000000017</v>
           </cell>
           <cell r="H15" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I15">
-            <v>996.34999999999991</v>
+            <v>1293</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
@@ -1928,13 +1928,13 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>36418.899999999994</v>
+            <v>40755.899999999994</v>
           </cell>
           <cell r="H16" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I16">
-            <v>1434.75</v>
+            <v>2052.5499999999997</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -1951,16 +1951,16 @@
             <v>181399.52000000014</v>
           </cell>
           <cell r="H17" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I17">
-            <v>2197.6</v>
+            <v>1434.75</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>21</v>
+            <v>22</v>
           </cell>
         </row>
         <row r="18">
@@ -1971,10 +1971,10 @@
             <v>206904.88</v>
           </cell>
           <cell r="H18" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I18">
-            <v>9723</v>
+            <v>2197.6</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -1991,16 +1991,16 @@
             <v>50153.310000000019</v>
           </cell>
           <cell r="H19" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I19">
-            <v>3754.1</v>
+            <v>11377.999999999998</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>285</v>
+            <v>286</v>
           </cell>
         </row>
         <row r="20">
@@ -2011,10 +2011,10 @@
             <v>88647.899999999878</v>
           </cell>
           <cell r="H20" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I20">
-            <v>2872.3700000000003</v>
+            <v>3754.1</v>
           </cell>
         </row>
         <row r="21">
@@ -2022,13 +2022,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>65392.23</v>
+            <v>66448.430000000008</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I21">
-            <v>853.1</v>
+            <v>2872.3700000000003</v>
           </cell>
         </row>
         <row r="22">
@@ -2039,10 +2039,10 @@
             <v>53035.3100000001</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I22">
-            <v>5748.5499999999984</v>
+            <v>2181.6</v>
           </cell>
         </row>
         <row r="23">
@@ -2053,10 +2053,10 @@
             <v>30794.440000000057</v>
           </cell>
           <cell r="H23" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I23">
-            <v>1202.75</v>
+            <v>5748.5499999999984</v>
           </cell>
         </row>
         <row r="24">
@@ -2064,13 +2064,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>124836.28999999983</v>
+            <v>126491.28999999985</v>
           </cell>
           <cell r="H24" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
           </cell>
           <cell r="I24">
-            <v>665.54</v>
+            <v>1222.75</v>
           </cell>
         </row>
         <row r="25">
@@ -2081,10 +2081,10 @@
             <v>165483.18</v>
           </cell>
           <cell r="H25" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I25">
-            <v>1040.82</v>
+            <v>665.54</v>
           </cell>
         </row>
         <row r="26">
@@ -2095,10 +2095,10 @@
             <v>68864.489999999962</v>
           </cell>
           <cell r="H26" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I26">
-            <v>74218.2</v>
+            <v>1040.82</v>
           </cell>
         </row>
         <row r="27">
@@ -2106,7 +2106,13 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>77338.629999999946</v>
+            <v>78667.129999999946</v>
+          </cell>
+          <cell r="H27" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I27">
+            <v>85796.839999999982</v>
           </cell>
         </row>
         <row r="28">
@@ -2122,7 +2128,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>44063.920000000042</v>
+            <v>44083.920000000042</v>
           </cell>
         </row>
         <row r="30">
@@ -2146,7 +2152,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>2685899.6099999631</v>
+            <v>2697478.2499999623</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2999,7 +3005,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>2624988.4099999992</v>
+        <v>2696649.3099999996</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3010,7 +3016,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>45938.7</v>
+        <v>53180.340000000004</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3021,7 +3027,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>28279.5</v>
+        <v>32616.5</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3032,7 +3038,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3044,7 +3050,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>2966511.5900000008</v>
+        <v>2894850.6900000004</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3055,7 +3061,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>104074.3</v>
+        <v>96832.66</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3066,7 +3072,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-28279.5</v>
+        <v>-32616.5</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3077,7 +3083,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3089,7 +3095,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.46946050433693987</v>
+        <v>0.4822765465438611</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3100,7 +3106,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.30623145994013845</v>
+        <v>0.3545048762440588</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3122,7 +3128,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.37598944591029027</v>
+        <v>0.37730870712401055</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3295,11 +3301,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>181896.29</v>
+        <v>183405.49</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>143103.71</v>
+        <v>141594.51</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3314,11 +3320,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9723</v>
+        <v>11377.999999999998</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2127</v>
+        <v>472.00000000000182</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3448,11 +3454,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>36891.44000000001</v>
+        <v>37140.380000000012</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>53108.55999999999</v>
+        <v>52859.619999999988</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3525,11 +3531,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>111316.87999999987</v>
+        <v>112730.67999999986</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>161683.12000000011</v>
+        <v>160269.32000000012</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3602,11 +3608,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>40012.410000000025</v>
+        <v>40022.410000000025</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>37987.589999999975</v>
+        <v>37977.589999999975</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3621,11 +3627,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6844.6999999999989</v>
+        <v>8353.8999999999978</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9155.3000000000011</v>
+        <v>7646.1000000000022</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3698,11 +3704,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>853.1</v>
+        <v>2181.6</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11956.9</v>
+        <v>10628.4</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3717,11 +3723,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4337</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-4337</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3897,11 +3903,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>36418.899999999994</v>
+        <v>40755.899999999994</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>93581.1</v>
+        <v>89244.1</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3976,11 +3982,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2353.0999999999995</v>
+        <v>3766.8999999999996</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10646.900000000001</v>
+        <v>9233.1</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4048,11 +4054,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>781.7600000000001</v>
+        <v>791.7600000000001</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4238.24</v>
+        <v>4228.24</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4123,11 +4129,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>996.34999999999991</v>
+        <v>2052.5499999999997</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7107.65</v>
+        <v>6051.4500000000007</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4159,11 +4165,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4198,11 +4204,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2016.5</v>
+        <v>2265.44</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3238.5</v>
+        <v>2989.56</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4215,11 +4221,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>486595.86999999976</v>
+        <v>490932.8699999997</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>132722.31181818212</v>
+        <v>128385.31181818218</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4254,11 +4260,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>65392.23</v>
+        <v>66448.430000000008</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>74607.76999999999</v>
+        <v>73551.569999999992</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4348,11 +4354,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1202.75</v>
+        <v>1222.75</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2367.25</v>
+        <v>2347.25</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4468,11 +4474,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>124836.28999999983</v>
+        <v>126491.28999999985</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>112663.71000000017</v>
+        <v>111008.71000000015</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4536,7 +4542,7 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="B29" s="16" t="s">
         <v>27</v>
@@ -4547,11 +4553,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>0</v>
+        <v>60082.260000000017</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>175000</v>
+        <v>114917.73999999999</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4650,11 +4656,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>77338.629999999946</v>
+        <v>78667.129999999946</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>89661.370000000054</v>
+        <v>88332.870000000054</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4750,11 +4756,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>27.272727272727252</v>
+        <v>24.272727272727252</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4770,11 +4776,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>44063.920000000042</v>
+        <v>44083.920000000042</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>55936.079999999958</v>
+        <v>55916.079999999958</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4787,11 +4793,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>503806.60000000341</v>
+        <v>511048.24000000337</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>147443.39999999659</v>
+        <v>140201.75999999663</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -5084,11 +5090,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1035363.7200000017</v>
+        <v>1046942.3600000022</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="5"/>
-        <v>-384113.72000000172</v>
+        <v>-395692.3600000022</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 16/07/2026 13:08
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80BB754-168F-4AE0-B070-0AE48CF8C55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2758DB46-397C-4047-A984-2248904272AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1731,13 +1731,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>183405.49</v>
+            <v>184286.28999999998</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>8353.8999999999978</v>
+            <v>9234.6999999999989</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1751,10 +1751,10 @@
             <v>828.94</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
+            <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="I7">
-            <v>2265.44</v>
+            <v>51</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1768,13 +1768,13 @@
             <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F8">
-            <v>100.09</v>
+            <v>151.09</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I8">
-            <v>3766.8999999999996</v>
+            <v>3491.37</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -1788,19 +1788,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>37140.380000000012</v>
+            <v>38366.310000000005</v>
           </cell>
           <cell r="H9" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I9">
-            <v>791.7600000000001</v>
+            <v>9450.7000000000007</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N9">
-            <v>29</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="10">
@@ -1808,13 +1808,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>112730.67999999986</v>
+            <v>118414.47999999986</v>
           </cell>
           <cell r="H10" t="str">
-            <v>KEY ABC</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I10">
-            <v>13637.5</v>
+            <v>1664.94</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
@@ -1828,13 +1828,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>40022.410000000025</v>
+            <v>40895.590000000033</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY SJC</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="I11">
-            <v>4337</v>
+            <v>13637.5</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
@@ -1851,10 +1851,10 @@
             <v>174575.71999999997</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY SP</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="I12">
-            <v>11566.400000000001</v>
+            <v>315.2</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
@@ -1868,13 +1868,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>161197.35999999999</v>
+            <v>161512.55999999997</v>
           </cell>
           <cell r="H13" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="I13">
-            <v>3075.6</v>
+            <v>5897</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
@@ -1891,16 +1891,16 @@
             <v>513142.70000000019</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I14">
-            <v>856.4</v>
+            <v>11566.400000000001</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>30</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="15">
@@ -1911,16 +1911,16 @@
             <v>60082.260000000017</v>
           </cell>
           <cell r="H15" t="str">
-            <v>LESTE MOOCA</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I15">
-            <v>1293</v>
+            <v>3075.6</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>45</v>
+            <v>47</v>
           </cell>
         </row>
         <row r="16">
@@ -1928,13 +1928,13 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>40755.899999999994</v>
+            <v>42315.899999999994</v>
           </cell>
           <cell r="H16" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I16">
-            <v>2052.5499999999997</v>
+            <v>2208.2500000000005</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -1951,10 +1951,10 @@
             <v>181399.52000000014</v>
           </cell>
           <cell r="H17" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I17">
-            <v>1434.75</v>
+            <v>2613.5</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
@@ -1971,10 +1971,10 @@
             <v>206904.88</v>
           </cell>
           <cell r="H18" t="str">
-            <v>MOGI</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I18">
-            <v>2197.6</v>
+            <v>2052.5499999999997</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -1988,19 +1988,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>50153.310000000019</v>
+            <v>51505.160000000018</v>
           </cell>
           <cell r="H19" t="str">
-            <v>NORTE</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I19">
-            <v>11377.999999999998</v>
+            <v>1434.75</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>286</v>
+            <v>291</v>
           </cell>
         </row>
         <row r="20">
@@ -2008,13 +2008,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>88647.899999999878</v>
+            <v>89968.399999999907</v>
           </cell>
           <cell r="H20" t="str">
-            <v>OSASCO</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I20">
-            <v>3754.1</v>
+            <v>3111.8</v>
           </cell>
         </row>
         <row r="21">
@@ -2025,10 +2025,10 @@
             <v>66448.430000000008</v>
           </cell>
           <cell r="H21" t="str">
-            <v>PIRITUBA</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I21">
-            <v>2872.3700000000003</v>
+            <v>15172.779999999995</v>
           </cell>
         </row>
         <row r="22">
@@ -2039,10 +2039,10 @@
             <v>53035.3100000001</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SANTO ANDRE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I22">
-            <v>2181.6</v>
+            <v>15225.139999999994</v>
           </cell>
         </row>
         <row r="23">
@@ -2050,13 +2050,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>30794.440000000057</v>
+            <v>31708.640000000058</v>
           </cell>
           <cell r="H23" t="str">
-            <v>SBC</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I23">
-            <v>5748.5499999999984</v>
+            <v>2872.3700000000003</v>
           </cell>
         </row>
         <row r="24">
@@ -2064,13 +2064,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>126491.28999999985</v>
+            <v>130286.06999999985</v>
           </cell>
           <cell r="H24" t="str">
-            <v>SJC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I24">
-            <v>1222.75</v>
+            <v>3766.4500000000003</v>
           </cell>
         </row>
         <row r="25">
@@ -2078,13 +2078,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>165483.18</v>
+            <v>176954.21999999994</v>
           </cell>
           <cell r="H25" t="str">
-            <v>SJC/VALE</v>
+            <v>SBC</v>
           </cell>
           <cell r="I25">
-            <v>665.54</v>
+            <v>5748.5499999999984</v>
           </cell>
         </row>
         <row r="26">
@@ -2095,10 +2095,10 @@
             <v>68864.489999999962</v>
           </cell>
           <cell r="H26" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC</v>
           </cell>
           <cell r="I26">
-            <v>1040.82</v>
+            <v>1597.3100000000002</v>
           </cell>
         </row>
         <row r="27">
@@ -2106,13 +2106,13 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>78667.129999999946</v>
+            <v>80251.979999999952</v>
           </cell>
           <cell r="H27" t="str">
-            <v>Total Geral</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I27">
-            <v>85796.839999999982</v>
+            <v>665.54</v>
           </cell>
         </row>
         <row r="28">
@@ -2122,13 +2122,25 @@
           <cell r="F28">
             <v>126422.29999999987</v>
           </cell>
+          <cell r="H28" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I28">
+            <v>1040.82</v>
+          </cell>
         </row>
         <row r="29">
           <cell r="E29" t="str">
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>44083.920000000042</v>
+            <v>44458.48000000004</v>
+          </cell>
+          <cell r="H29" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I29">
+            <v>117198.52999999978</v>
           </cell>
         </row>
         <row r="30">
@@ -2144,7 +2156,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>38431.760000000009</v>
+            <v>37456.760000000017</v>
           </cell>
         </row>
         <row r="32">
@@ -2152,7 +2164,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>2697478.2499999623</v>
+            <v>2727904.9399999613</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3005,7 +3017,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D35)</f>
-        <v>2696649.3099999996</v>
+        <v>2727075.9999999991</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3016,7 +3028,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>53180.340000000004</v>
+        <v>82655.829999999987</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3027,7 +3039,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>32616.5</v>
+        <v>34491.699999999997</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3038,7 +3050,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3050,7 +3062,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>2894850.6900000004</v>
+        <v>2864424.0000000009</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3061,7 +3073,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>96832.66</v>
+        <v>67357.170000000013</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3072,7 +3084,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-32616.5</v>
+        <v>-34491.699999999997</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3083,7 +3095,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3095,7 +3107,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.4822765465438611</v>
+        <v>0.48771814361083776</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3106,7 +3118,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.3545048762440588</v>
+        <v>0.55099111410344426</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3128,7 +3140,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.37730870712401055</v>
+        <v>0.38390501319261217</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3246,11 +3258,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3754.1</v>
+        <v>15225.139999999994</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>13245.9</v>
+        <v>1774.860000000006</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3301,11 +3313,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>183405.49</v>
+        <v>184286.28999999998</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>141594.51</v>
+        <v>140713.71000000002</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3320,11 +3332,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11377.999999999998</v>
+        <v>15172.779999999995</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>472.00000000000182</v>
+        <v>-3322.7799999999952</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3377,11 +3389,11 @@
       </c>
       <c r="D12" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>100.09</v>
+        <v>151.09</v>
       </c>
       <c r="E12" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>899.91</v>
+        <v>848.91</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="21" t="s">
@@ -3434,11 +3446,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3454,11 +3466,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>37140.380000000012</v>
+        <v>38366.310000000005</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>52859.619999999988</v>
+        <v>51633.689999999995</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3531,11 +3543,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>112730.67999999986</v>
+        <v>118414.47999999986</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>160269.32000000012</v>
+        <v>154585.52000000014</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3608,11 +3620,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>40022.410000000025</v>
+        <v>40895.590000000033</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>37977.589999999975</v>
+        <v>37104.409999999967</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3627,11 +3639,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8353.8999999999978</v>
+        <v>9234.6999999999989</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7646.1000000000022</v>
+        <v>6765.3000000000011</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3704,11 +3716,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2181.6</v>
+        <v>3766.4500000000003</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10628.4</v>
+        <v>9043.5499999999993</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3723,11 +3735,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4337</v>
+        <v>5897</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>-4337</v>
+        <v>-5897</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3762,11 +3774,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>161197.35999999999</v>
+        <v>161512.55999999997</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>8802.640000000014</v>
+        <v>8487.4400000000314</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3781,11 +3793,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2197.6</v>
+        <v>3111.8</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>946.40000000000009</v>
+        <v>32.199999999999818</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3800,11 +3812,11 @@
       </c>
       <c r="P17" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>315.2</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-315.2</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="19" t="s">
@@ -3858,11 +3870,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>856.4</v>
+        <v>2208.2500000000005</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5359.6</v>
+        <v>4007.7499999999995</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3883,11 +3895,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3903,11 +3915,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>40755.899999999994</v>
+        <v>42315.899999999994</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>89244.1</v>
+        <v>87684.1</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3922,11 +3934,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1293</v>
+        <v>2613.5</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9577</v>
+        <v>8256.5</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3943,11 +3955,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3982,11 +3994,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3766.8999999999996</v>
+        <v>9450.7000000000007</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9233.1</v>
+        <v>3549.2999999999993</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4054,11 +4066,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>791.7600000000001</v>
+        <v>1664.94</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4228.24</v>
+        <v>3355.06</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4110,11 +4122,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>50153.310000000019</v>
+        <v>51505.160000000018</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>71846.689999999973</v>
+        <v>70494.839999999982</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4185,11 +4197,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>88647.899999999878</v>
+        <v>89968.399999999907</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>106352.10000000012</v>
+        <v>105031.60000000009</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4204,11 +4216,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2265.44</v>
+        <v>3491.37</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2989.56</v>
+        <v>1763.63</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4221,11 +4233,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>490932.8699999997</v>
+        <v>492808.06999999977</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>128385.31181818218</v>
+        <v>126510.11181818211</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4354,11 +4366,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1222.75</v>
+        <v>1597.3100000000002</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2347.25</v>
+        <v>1972.6899999999998</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4410,11 +4422,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>30794.440000000057</v>
+        <v>31708.640000000058</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>59205.559999999939</v>
+        <v>58291.359999999942</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4474,11 +4486,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>126491.28999999985</v>
+        <v>130286.06999999985</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>111008.71000000015</v>
+        <v>107213.93000000015</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4520,11 +4532,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>165483.18</v>
+        <v>176954.21999999994</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>153016.82</v>
+        <v>141545.78000000006</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4656,11 +4668,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>78667.129999999946</v>
+        <v>80251.979999999952</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>88332.870000000054</v>
+        <v>86748.020000000048</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4733,11 +4745,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>501987.34000000299</v>
+        <v>501687.34000000299</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>19012.659999997006</v>
+        <v>19312.659999997006</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4756,11 +4768,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>24.272727272727252</v>
+        <v>17.272727272727252</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4776,11 +4788,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>44083.920000000042</v>
+        <v>44458.48000000004</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>55916.079999999958</v>
+        <v>55541.51999999996</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4793,11 +4805,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>511048.24000000337</v>
+        <v>538528.23000000359</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>140201.75999999663</v>
+        <v>112721.76999999641</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4896,11 +4908,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>38431.760000000009</v>
+        <v>37456.760000000017</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>34568.239999999991</v>
+        <v>35543.239999999983</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5054,11 +5066,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1104662.189999996</v>
+        <v>1104362.189999996</v>
       </c>
       <c r="E40" s="7">
         <f t="shared" ref="E40:E42" si="5">C40-D40</f>
-        <v>-583662.18999999599</v>
+        <v>-583362.18999999599</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -5090,11 +5102,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1046942.3600000022</v>
+        <v>1077669.0499999991</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" si="5"/>
-        <v>-395692.3600000022</v>
+        <v>-426419.04999999912</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 16/07/2026 14:06
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2758DB46-397C-4047-A984-2248904272AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4810163-3EDF-42F4-9206-8C681188A47E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="54">
   <si>
     <t>META DIA</t>
   </si>
@@ -424,7 +424,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -508,6 +508,18 @@
     <xf numFmtId="44" fontId="3" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Moeda" xfId="2" builtinId="4"/>
@@ -518,7 +530,17 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="78">
+  <dxfs count="79">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -538,11 +560,15 @@
       </font>
       <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
-        <top/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -564,6 +590,32 @@
       </font>
       <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
@@ -674,7 +726,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
@@ -764,35 +815,6 @@
         <right/>
         <top/>
         <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1731,13 +1753,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>184286.28999999998</v>
+            <v>186540.97</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>9234.6999999999989</v>
+            <v>11489.379999999997</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1794,7 +1816,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I9">
-            <v>9450.7000000000007</v>
+            <v>13467.2</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
@@ -1808,7 +1830,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>118414.47999999986</v>
+            <v>122430.97999999985</v>
           </cell>
           <cell r="H10" t="str">
             <v>JUNDIAI</v>
@@ -1860,7 +1882,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>16</v>
+            <v>17</v>
           </cell>
         </row>
         <row r="13">
@@ -1880,7 +1902,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>23</v>
+            <v>24</v>
           </cell>
         </row>
         <row r="14">
@@ -1894,13 +1916,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="I14">
-            <v>11566.400000000001</v>
+            <v>20532.100000000002</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>32</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="15">
@@ -1934,7 +1956,7 @@
             <v>LESTE</v>
           </cell>
           <cell r="I16">
-            <v>2208.2500000000005</v>
+            <v>2980.05</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -1948,13 +1970,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>181399.52000000014</v>
+            <v>190365.22000000015</v>
           </cell>
           <cell r="H17" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I17">
-            <v>2613.5</v>
+            <v>3987.1200000000003</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
@@ -1974,7 +1996,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I18">
-            <v>2052.5499999999997</v>
+            <v>2362.75</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -1988,19 +2010,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>51505.160000000018</v>
+            <v>52276.960000000021</v>
           </cell>
           <cell r="H19" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I19">
-            <v>1434.75</v>
+            <v>2359.1500000000005</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>291</v>
+            <v>296</v>
           </cell>
         </row>
         <row r="20">
@@ -2008,13 +2030,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>89968.399999999907</v>
+            <v>91342.019999999902</v>
           </cell>
           <cell r="H20" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="I20">
-            <v>3111.8</v>
+            <v>5852.5499999999993</v>
           </cell>
         </row>
         <row r="21">
@@ -2022,13 +2044,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>66448.430000000008</v>
+            <v>66758.630000000019</v>
           </cell>
           <cell r="H21" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="I21">
-            <v>15172.779999999995</v>
+            <v>16318.529999999995</v>
           </cell>
         </row>
         <row r="22">
@@ -2036,7 +2058,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>53035.3100000001</v>
+            <v>53959.710000000101</v>
           </cell>
           <cell r="H22" t="str">
             <v>OSASCO</v>
@@ -2050,13 +2072,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>31708.640000000058</v>
+            <v>34449.390000000058</v>
           </cell>
           <cell r="H23" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I23">
-            <v>2872.3700000000003</v>
+            <v>3452.3699999999994</v>
           </cell>
         </row>
         <row r="24">
@@ -2064,13 +2086,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>130286.06999999985</v>
+            <v>131431.81999999983</v>
           </cell>
           <cell r="H24" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I24">
-            <v>3766.4500000000003</v>
+            <v>6695.95</v>
           </cell>
         </row>
         <row r="25">
@@ -2084,7 +2106,7 @@
             <v>SBC</v>
           </cell>
           <cell r="I25">
-            <v>5748.5499999999984</v>
+            <v>7824.8499999999967</v>
           </cell>
         </row>
         <row r="26">
@@ -2092,7 +2114,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>68864.489999999962</v>
+            <v>69444.489999999962</v>
           </cell>
           <cell r="H26" t="str">
             <v>SJC</v>
@@ -2106,13 +2128,13 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>80251.979999999952</v>
+            <v>83181.479999999952</v>
           </cell>
           <cell r="H27" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I27">
-            <v>665.54</v>
+            <v>1783.7000000000005</v>
           </cell>
         </row>
         <row r="28">
@@ -2120,7 +2142,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>126422.29999999987</v>
+            <v>128498.59999999985</v>
           </cell>
           <cell r="H28" t="str">
             <v>VENDEDOR INTERNO 1</v>
@@ -2140,7 +2162,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="I29">
-            <v>117198.52999999978</v>
+            <v>146405.88999999966</v>
           </cell>
         </row>
         <row r="30">
@@ -2148,7 +2170,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>20737.710000000003</v>
+            <v>21855.87</v>
           </cell>
         </row>
         <row r="31">
@@ -2164,7 +2186,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>2727904.9399999613</v>
+            <v>2757112.2999999598</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2330,17 +2352,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C97E85A-DD10-4825-81C1-53CD3989178B}" name="Tabela1" displayName="Tabela1" ref="B4:C7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C97E85A-DD10-4825-81C1-53CD3989178B}" name="Tabela1" displayName="Tabela1" ref="B4:C7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{3308613D-E7FC-469E-B078-C5AC910E183B}" name="Coluna1" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{C994D666-6174-475E-AE71-1F12062A5225}" name="Coluna2" headerRowDxfId="74" dataDxfId="73" dataCellStyle="Moeda"/>
+    <tableColumn id="1" xr3:uid="{3308613D-E7FC-469E-B078-C5AC910E183B}" name="Coluna1" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{C994D666-6174-475E-AE71-1F12062A5225}" name="Coluna2" headerRowDxfId="75" dataDxfId="74" dataCellStyle="Moeda"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{874935CD-63EE-45D7-AA45-CFFFE79EAC7D}" name="Tabela2" displayName="Tabela2" ref="S9:W26" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26" tableBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{874935CD-63EE-45D7-AA45-CFFFE79EAC7D}" name="Tabela2" displayName="Tabela2" ref="S9:W26" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27" tableBorderDxfId="26">
   <autoFilter ref="S9:W26" xr:uid="{874935CD-63EE-45D7-AA45-CFFFE79EAC7D}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2349,15 +2371,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{96702934-C966-496F-B51E-ADD7BF9BB7D8}" name="VENDEDOR" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{E2D85F5C-4525-4FA4-B813-A1322F5C254D}" name="REFERENCIA" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{53C55BB3-DDD4-47EF-87D5-552E4D02B5BA}" name="META A" dataDxfId="22">
+    <tableColumn id="1" xr3:uid="{96702934-C966-496F-B51E-ADD7BF9BB7D8}" name="VENDEDOR" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{E2D85F5C-4525-4FA4-B813-A1322F5C254D}" name="REFERENCIA" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{53C55BB3-DDD4-47EF-87D5-552E4D02B5BA}" name="META A" dataDxfId="23">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],[1]!Tabela5[VENDEDOR],[1]!Tabela5[META A])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{018C7BF7-4C79-4668-95B2-CBF2E10B657D}" name="ATINGIDO" dataDxfId="21">
+    <tableColumn id="4" xr3:uid="{018C7BF7-4C79-4668-95B2-CBF2E10B657D}" name="ATINGIDO" dataDxfId="22">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{37E12533-09AB-4B65-AEC8-6BB07B5CC2B1}" name="FALTA" dataDxfId="20">
+    <tableColumn id="5" xr3:uid="{37E12533-09AB-4B65-AEC8-6BB07B5CC2B1}" name="FALTA" dataDxfId="21">
       <calculatedColumnFormula>U10-V10</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2366,18 +2388,18 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E3745920-1197-4A81-B558-958DBAB19EA3}" name="Tabela5" displayName="Tabela5" ref="G9:K27" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E3745920-1197-4A81-B558-958DBAB19EA3}" name="Tabela5" displayName="Tabela5" ref="G9:K27" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="G9:K27" xr:uid="{E3745920-1197-4A81-B558-958DBAB19EA3}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D324C7DB-F877-4A7E-BC26-EF8905C85433}" name="VENDEDOR" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{A71A6478-3B31-4F54-A10C-E6EC00E95E0B}" name="REFERENCIA" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{9F5EDCDD-D442-4FBE-9C74-26084F24EFCB}" name="COMPROMISSO" dataDxfId="14" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{D324C7DB-F877-4A7E-BC26-EF8905C85433}" name="VENDEDOR" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{A71A6478-3B31-4F54-A10C-E6EC00E95E0B}" name="REFERENCIA" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{9F5EDCDD-D442-4FBE-9C74-26084F24EFCB}" name="COMPROMISSO" dataDxfId="15" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2E4F9793-0E4B-42F0-B595-748F8481D0D0}" name="ATINGIDO" dataDxfId="13" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{2E4F9793-0E4B-42F0-B595-748F8481D0D0}" name="ATINGIDO" dataDxfId="14" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{3CEFD09C-EF55-4119-A139-BD17682D2B73}" name="FALTA" dataDxfId="12">
+    <tableColumn id="5" xr3:uid="{3CEFD09C-EF55-4119-A139-BD17682D2B73}" name="FALTA" dataDxfId="13">
       <calculatedColumnFormula>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2386,8 +2408,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{3A7104A0-4D5E-4CED-9364-119005653576}" name="Tabela13" displayName="Tabela13" ref="A9:E35" headerRowDxfId="11" tableBorderDxfId="10">
-  <autoFilter ref="A9:E35" xr:uid="{3A7104A0-4D5E-4CED-9364-119005653576}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{3A7104A0-4D5E-4CED-9364-119005653576}" name="Tabela13" displayName="Tabela13" ref="A9:E36" headerRowDxfId="12" tableBorderDxfId="11">
+  <autoFilter ref="A9:E36" xr:uid="{3A7104A0-4D5E-4CED-9364-119005653576}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -2395,15 +2417,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{50EE0FE5-ADD7-4A3A-9DF8-D52FFFCF08DA}" name="VENDEDOR" totalsRowLabel="Total" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{4F0BAF4D-D0FC-4B7C-8FF4-8DDD6505FDA1}" name="REFERENCIA" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{CCB341E8-8BC2-4209-AEA0-D6F26BFCB356}" name="META A" dataDxfId="5" totalsRowDxfId="4" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{50EE0FE5-ADD7-4A3A-9DF8-D52FFFCF08DA}" name="VENDEDOR" totalsRowLabel="Total" dataDxfId="9" totalsRowDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{4F0BAF4D-D0FC-4B7C-8FF4-8DDD6505FDA1}" name="REFERENCIA" dataDxfId="7" totalsRowDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{CCB341E8-8BC2-4209-AEA0-D6F26BFCB356}" name="META A" dataDxfId="5" totalsRowDxfId="6" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],[1]!Tabela2[VENDEDOR],[1]!Tabela2[META A])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{9AA985E6-33FD-40FD-9473-5AF6B4D03030}" name="ATINGIDO" dataDxfId="3" totalsRowDxfId="2" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{9AA985E6-33FD-40FD-9473-5AF6B4D03030}" name="ATINGIDO" dataDxfId="3" totalsRowDxfId="4" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7B8A46E1-DE6F-44C0-A6C8-83887563A4C0}" name="FALTA" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
+    <tableColumn id="5" xr3:uid="{7B8A46E1-DE6F-44C0-A6C8-83887563A4C0}" name="FALTA" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="2">
       <calculatedColumnFormula>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2412,23 +2434,21 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}" name="Tabela3" displayName="Tabela3" ref="B38:E43" totalsRowShown="0" headerRowDxfId="72" dataDxfId="71">
-  <autoFilter ref="B38:E43" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}" name="Tabela3" displayName="Tabela3" ref="B39:E44" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
+  <autoFilter ref="B39:E44" xr:uid="{A3157CCA-AE81-44E6-8AC3-6B69E02394E0}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D5CFA35F-1C13-42CF-B05C-430BF14AC2B0}" name="SEMANAL" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{06063E15-5C9E-4303-B5F6-B9D0B178DB82}" name="META" dataDxfId="69" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{D5CFA35F-1C13-42CF-B05C-430BF14AC2B0}" name="SEMANAL" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{06063E15-5C9E-4303-B5F6-B9D0B178DB82}" name="META" dataDxfId="70" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{425F53BB-8CBB-40E8-9773-1C7C39906AD7}" name="REALIZADO" dataDxfId="68" dataCellStyle="Moeda">
-      <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{A18F5082-185F-44C4-B163-8A3CBDDA6732}" name="FALTA" dataDxfId="67">
-      <calculatedColumnFormula>C39-D39</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{425F53BB-8CBB-40E8-9773-1C7C39906AD7}" name="REALIZADO" dataDxfId="69" dataCellStyle="Moeda"/>
+    <tableColumn id="4" xr3:uid="{A18F5082-185F-44C4-B163-8A3CBDDA6732}" name="FALTA" dataDxfId="68">
+      <calculatedColumnFormula>C40-D40</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2436,17 +2456,17 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BA69D712-8843-4CBF-AD2F-C801E56B1CFC}" name="Tabela4" displayName="Tabela4" ref="H4:I7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="66" dataDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BA69D712-8843-4CBF-AD2F-C801E56B1CFC}" name="Tabela4" displayName="Tabela4" ref="H4:I7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C661D03F-A79A-4D24-86FD-3574B6E5537D}" name="Coluna1" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{7EF7A574-C8A3-4CB7-9C98-86948FE130EB}" name="Coluna2" headerRowDxfId="63" dataDxfId="62"/>
+    <tableColumn id="1" xr3:uid="{C661D03F-A79A-4D24-86FD-3574B6E5537D}" name="Coluna1" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{7EF7A574-C8A3-4CB7-9C98-86948FE130EB}" name="Coluna2" headerRowDxfId="64" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}" name="Tabela6" displayName="Tabela6" ref="H30:K35" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}" name="Tabela6" displayName="Tabela6" ref="H30:K35" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
   <autoFilter ref="H30:K35" xr:uid="{A75040F9-F863-450B-ACF9-7CEC08A64AB4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2454,14 +2474,14 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{14E3BD3B-54B0-47BF-931C-064E12741C86}" name="SEMANAL" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{67CE9FE2-AA11-4BD4-9F34-EDC9123EA89F}" name="META" dataDxfId="58" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{14E3BD3B-54B0-47BF-931C-064E12741C86}" name="SEMANAL" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{67CE9FE2-AA11-4BD4-9F34-EDC9123EA89F}" name="META" dataDxfId="59" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(Tabela6[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{14D3AA11-9DFC-420F-8F5A-5002E14D4AAA}" name="REALIZADO" dataDxfId="57">
+    <tableColumn id="3" xr3:uid="{14D3AA11-9DFC-420F-8F5A-5002E14D4AAA}" name="REALIZADO" dataDxfId="58">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{16DC2DF3-76D8-4A80-B29C-E276BB17D8FF}" name="FALTA" dataDxfId="56">
+    <tableColumn id="4" xr3:uid="{16DC2DF3-76D8-4A80-B29C-E276BB17D8FF}" name="FALTA" dataDxfId="57">
       <calculatedColumnFormula>I31-J31</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2470,17 +2490,17 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9D5C0B8F-3138-4FD4-9A83-375E8D4AC464}" name="Tabela7" displayName="Tabela7" ref="N4:O7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9D5C0B8F-3138-4FD4-9A83-375E8D4AC464}" name="Tabela7" displayName="Tabela7" ref="N4:O7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{0139F26F-4C9F-4E96-9F64-C5C5B271DCA9}" name="Coluna1" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{1DA3E17F-38EB-4042-B2F0-3DFB7629A3F5}" name="Coluna2" headerRowDxfId="52" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{0139F26F-4C9F-4E96-9F64-C5C5B271DCA9}" name="Coluna1" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{1DA3E17F-38EB-4042-B2F0-3DFB7629A3F5}" name="Coluna2" headerRowDxfId="53" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{87A5A608-D233-46F9-8E75-B1963DE71BC6}" name="Tabela8" displayName="Tabela8" ref="M10:Q17" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49" dataCellStyle="Moeda">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{87A5A608-D233-46F9-8E75-B1963DE71BC6}" name="Tabela8" displayName="Tabela8" ref="M10:Q17" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50" dataCellStyle="Moeda">
   <autoFilter ref="M10:Q17" xr:uid="{87A5A608-D233-46F9-8E75-B1963DE71BC6}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2489,15 +2509,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{EE89D966-6315-4DB4-9927-EEB09B51F44E}" name="VENDEDOR" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{0B55D821-52F8-4CE2-9F16-C5BCDBCE53AC}" name="REFERENCIA" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{B5D24BF0-392E-420D-BB1D-3FED1D3383B5}" name="COMPROMISSO" dataDxfId="46" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{EE89D966-6315-4DB4-9927-EEB09B51F44E}" name="VENDEDOR" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{0B55D821-52F8-4CE2-9F16-C5BCDBCE53AC}" name="REFERENCIA" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{B5D24BF0-392E-420D-BB1D-3FED1D3383B5}" name="COMPROMISSO" dataDxfId="47" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">IFERROR(_xlfn.XLOOKUP(M11,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{92C88D8B-4724-4B0F-86B9-CEB8CCE813E5}" name="ATINGIDO" dataDxfId="45" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{92C88D8B-4724-4B0F-86B9-CEB8CCE813E5}" name="ATINGIDO" dataDxfId="46" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{CA195FA3-3822-41FA-8A93-2D86914C048E}" name="FALTA" dataDxfId="44" dataCellStyle="Moeda">
+    <tableColumn id="5" xr3:uid="{CA195FA3-3822-41FA-8A93-2D86914C048E}" name="FALTA" dataDxfId="45" dataCellStyle="Moeda">
       <calculatedColumnFormula>O11-P11</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2506,7 +2526,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{3D6BA5FD-BBE8-4A7A-9B76-3F3F6D1F10E9}" name="Tabela9" displayName="Tabela9" ref="N20:Q25" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{3D6BA5FD-BBE8-4A7A-9B76-3F3F6D1F10E9}" name="Tabela9" displayName="Tabela9" ref="N20:Q25" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="N20:Q25" xr:uid="{3D6BA5FD-BBE8-4A7A-9B76-3F3F6D1F10E9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2514,12 +2534,12 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{985251B0-0E07-4E60-9774-18D0D763437D}" name="SEMANAL" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{7B11DBA8-6FBD-4B67-BDA9-6624DF753EFD}" name="META" dataDxfId="40" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{985251B0-0E07-4E60-9774-18D0D763437D}" name="SEMANAL" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{7B11DBA8-6FBD-4B67-BDA9-6624DF753EFD}" name="META" dataDxfId="41" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(Tabela9[[#This Row],[SEMANAL]],[1]!Tabela10[[#All],[Coluna1]],[1]!Tabela10[[#All],[Coluna2]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0B727490-D536-4FC5-B857-CD92C459F1FB}" name="REALIZADO" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{84544AF4-5466-4CAC-A349-7B2C804BDA05}" name="FALTA" dataDxfId="38">
+    <tableColumn id="3" xr3:uid="{0B727490-D536-4FC5-B857-CD92C459F1FB}" name="REALIZADO" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{84544AF4-5466-4CAC-A349-7B2C804BDA05}" name="FALTA" dataDxfId="39">
       <calculatedColumnFormula>O21-P21</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2528,17 +2548,17 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7AAFC688-3718-400A-9213-0DC213191E8B}" name="Tabela10" displayName="Tabela10" ref="T4:U7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7AAFC688-3718-400A-9213-0DC213191E8B}" name="Tabela10" displayName="Tabela10" ref="T4:U7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{870B59CA-1EA4-4CA9-BDCF-4A342A313131}" name="Coluna1" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{6FE31DF2-1DB4-4D4B-8783-48EA07B43B53}" name="Coluna2" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{870B59CA-1EA4-4CA9-BDCF-4A342A313131}" name="Coluna1" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{6FE31DF2-1DB4-4D4B-8783-48EA07B43B53}" name="Coluna2" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}" name="Tabela12" displayName="Tabela12" ref="T29:W34" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}" name="Tabela12" displayName="Tabela12" ref="T29:W34" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="T29:W34" xr:uid="{A15FC431-91F7-4B09-9000-61CB68A149E7}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2546,14 +2566,14 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{65A441BB-28F2-4C4D-8CD8-F9F9788A0656}" name="SEMANAL" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{B849FCBC-ED0F-47D9-B4E7-149FFE3500D9}" name="META" dataDxfId="30" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{65A441BB-28F2-4C4D-8CD8-F9F9788A0656}" name="SEMANAL" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{B849FCBC-ED0F-47D9-B4E7-149FFE3500D9}" name="META" dataDxfId="31" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(Tabela12[[#This Row],[SEMANAL]],[1]!Tabela11[[#All],[Coluna1]],[1]!Tabela11[[#All],[Coluna2]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A81AB4FC-EF49-4A93-8229-1B0CBFC88744}" name="REALIZADO" dataDxfId="29">
+    <tableColumn id="3" xr3:uid="{A81AB4FC-EF49-4A93-8229-1B0CBFC88744}" name="REALIZADO" dataDxfId="30">
       <calculatedColumnFormula>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[PARAMETRO]","[Intervalo 2].[PARAMETRO].&amp;[DIA]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{13865A0A-FFF3-4F90-A201-753948DC8E26}" name="FALTA" dataDxfId="28">
+    <tableColumn id="4" xr3:uid="{13865A0A-FFF3-4F90-A201-753948DC8E26}" name="FALTA" dataDxfId="29">
       <calculatedColumnFormula>U30-V30</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2858,7 +2878,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47C29905-7DAF-4BE5-BDE6-DF5442C33639}">
-  <dimension ref="A1:W43"/>
+  <dimension ref="A1:W63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" bestFit="1" customWidth="1"/>
@@ -2971,8 +2991,8 @@
         <v>38</v>
       </c>
       <c r="C4" s="2">
-        <f>SUM(C10:C35)</f>
-        <v>5591500</v>
+        <f>SUM(C10:C36)</f>
+        <v>5592500</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="4"/>
@@ -3016,8 +3036,8 @@
         <v>1</v>
       </c>
       <c r="C5" s="2">
-        <f>SUM(D10:D35)</f>
-        <v>2727075.9999999991</v>
+        <f>SUM(D10:D36)</f>
+        <v>2757112.3</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3028,7 +3048,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>82655.829999999987</v>
+        <v>102897.48999999998</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3039,7 +3059,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>34491.699999999997</v>
+        <v>43457.399999999994</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3050,7 +3070,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3062,7 +3082,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>2864424.0000000009</v>
+        <v>2835387.7</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3073,7 +3093,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>67357.170000000013</v>
+        <v>47115.510000000024</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3084,7 +3104,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-34491.699999999997</v>
+        <v>-43457.399999999994</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3095,7 +3115,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3107,7 +3127,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.48771814361083776</v>
+        <v>0.49300175234689314</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3118,7 +3138,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.55099111410344426</v>
+        <v>0.68592381993560547</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3140,7 +3160,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.38390501319261217</v>
+        <v>0.39050131926121368</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3313,11 +3333,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>184286.28999999998</v>
+        <v>186540.97</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>140713.71000000002</v>
+        <v>138459.03</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3332,11 +3352,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>15172.779999999995</v>
+        <v>16318.529999999995</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-3322.7799999999952</v>
+        <v>-4468.5299999999952</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3408,11 +3428,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2872.3700000000003</v>
+        <v>3452.3699999999994</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6127.6299999999992</v>
+        <v>5547.630000000001</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3485,11 +3505,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5748.5499999999984</v>
+        <v>7824.8499999999967</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9251.4500000000007</v>
+        <v>7175.1500000000033</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3543,11 +3563,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>118414.47999999986</v>
+        <v>122430.97999999985</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>154585.52000000014</v>
+        <v>150569.02000000014</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3562,11 +3582,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1434.75</v>
+        <v>2359.1500000000005</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3889.25</v>
+        <v>2964.8499999999995</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3639,11 +3659,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9234.6999999999989</v>
+        <v>11489.379999999997</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6765.3000000000011</v>
+        <v>4510.6200000000026</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3658,11 +3678,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11566.400000000001</v>
+        <v>20532.100000000002</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-11566.400000000001</v>
+        <v>-20532.100000000002</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3716,11 +3736,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3766.4500000000003</v>
+        <v>6695.95</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9043.5499999999993</v>
+        <v>6114.05</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3793,11 +3813,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3111.8</v>
+        <v>5852.5499999999993</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>32.199999999999818</v>
+        <v>-2708.5499999999993</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3870,11 +3890,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2208.2500000000005</v>
+        <v>2980.05</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4007.7499999999995</v>
+        <v>3235.95</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3895,11 +3915,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3934,11 +3954,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2613.5</v>
+        <v>3987.1200000000003</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8256.5</v>
+        <v>6882.8799999999992</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3975,11 +3995,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>181399.52000000014</v>
+        <v>190365.22000000015</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>378600.47999999986</v>
+        <v>369634.77999999985</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3994,11 +4014,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9450.7000000000007</v>
+        <v>13467.2</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3549.2999999999993</v>
+        <v>-467.20000000000073</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4027,11 +4047,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4122,11 +4142,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51505.160000000018</v>
+        <v>52276.960000000021</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>70494.839999999982</v>
+        <v>69723.039999999979</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4141,11 +4161,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2052.5499999999997</v>
+        <v>2362.75</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6051.4500000000007</v>
+        <v>5741.25</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4197,11 +4217,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>89968.399999999907</v>
+        <v>91342.019999999902</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>105031.60000000009</v>
+        <v>103657.9800000001</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4233,11 +4253,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>492808.06999999977</v>
+        <v>501773.76999999979</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>126510.11181818211</v>
+        <v>117544.4118181821</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4272,11 +4292,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>66448.430000000008</v>
+        <v>66758.630000000019</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>73551.569999999992</v>
+        <v>73241.369999999981</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4347,11 +4367,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>53035.3100000001</v>
+        <v>53959.710000000101</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>89464.6899999999</v>
+        <v>88540.289999999892</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4402,11 +4422,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4422,11 +4442,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>31708.640000000058</v>
+        <v>34449.390000000058</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>58291.359999999942</v>
+        <v>55550.609999999942</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4441,11 +4461,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>665.54</v>
+        <v>1783.7000000000005</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1776.46</v>
+        <v>658.2999999999995</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4486,11 +4506,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>130286.06999999985</v>
+        <v>131431.81999999983</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>107213.93000000015</v>
+        <v>106068.18000000017</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4611,11 +4631,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>68864.489999999962</v>
+        <v>69444.489999999962</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65635.510000000038</v>
+        <v>65055.510000000038</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4668,11 +4688,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>80251.979999999952</v>
+        <v>83181.479999999952</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>86748.020000000048</v>
+        <v>83818.520000000048</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4728,11 +4748,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>126422.29999999987</v>
+        <v>128498.59999999985</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>133577.70000000013</v>
+        <v>131501.40000000014</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4768,11 +4788,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>17.272727272727252</v>
+        <v>9.2727272727272521</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4805,11 +4825,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>538528.23000000359</v>
+        <v>557396.27000000444</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>112721.76999999641</v>
+        <v>93853.729999995558</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4848,11 +4868,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>20737.710000000003</v>
+        <v>21855.87</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>34262.289999999994</v>
+        <v>33144.130000000005</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4945,8 +4965,24 @@
       <c r="W35" s="4"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="C36"/>
-      <c r="D36"/>
+      <c r="A36" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="31">
+        <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],[1]!Tabela2[VENDEDOR],[1]!Tabela2[META A])</f>
+        <v>1000</v>
+      </c>
+      <c r="D36" s="31">
+        <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
+        <v>828.94</v>
+      </c>
+      <c r="E36" s="32">
+        <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
+        <v>171.05999999999995</v>
+      </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -4967,6 +5003,7 @@
       <c r="W36" s="4"/>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A37" s="29"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -4987,19 +5024,7 @@
       <c r="W37" s="4"/>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>2</v>
-      </c>
+      <c r="A38" s="29"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -5020,21 +5045,18 @@
       <c r="W38" s="4"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A39" s="4"/>
+      <c r="A39" s="29"/>
       <c r="B39" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C39" s="2" cm="1">
-        <f t="array" ref="C39">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
-        <v>390750</v>
-      </c>
-      <c r="D39" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>545873.70000000158</v>
-      </c>
-      <c r="E39" s="7">
-        <f>C39-D39</f>
-        <v>-155123.70000000158</v>
+        <v>47</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>2</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -5056,21 +5078,21 @@
       <c r="W39" s="4"/>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A40" s="4"/>
+      <c r="A40" s="29"/>
       <c r="B40" s="4" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="C40" s="2" cm="1">
         <f t="array" ref="C40">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
-        <v>521000</v>
+        <v>390750</v>
       </c>
       <c r="D40" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1104362.189999996</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
+        <v>545873.70000000158</v>
       </c>
       <c r="E40" s="7">
-        <f t="shared" ref="E40:E42" si="5">C40-D40</f>
-        <v>-583362.18999999599</v>
+        <f>C40-D40</f>
+        <v>-155123.70000000158</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -5092,21 +5114,21 @@
       <c r="W40" s="4"/>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A41" s="4"/>
+      <c r="A41" s="29"/>
       <c r="B41" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C41" s="2" cm="1">
         <f t="array" ref="C41">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
-        <v>651250</v>
+        <v>521000</v>
       </c>
       <c r="D41" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1077669.0499999991</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
+        <v>1104362.189999996</v>
       </c>
       <c r="E41" s="7">
-        <f t="shared" si="5"/>
-        <v>-426419.04999999912</v>
+        <f t="shared" ref="E41:E43" si="5">C41-D41</f>
+        <v>-583362.18999999599</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -5128,21 +5150,21 @@
       <c r="W41" s="4"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="4"/>
+      <c r="A42" s="29"/>
       <c r="B42" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C42" s="2" cm="1">
         <f t="array" ref="C42">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
         <v>651250</v>
       </c>
       <c r="D42" s="2">
-        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
+        <v>1106876.4099999981</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>651250</v>
+        <v>-455626.40999999805</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -5164,25 +5186,103 @@
       <c r="W42" s="4"/>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A43" s="4"/>
+      <c r="A43" s="29"/>
       <c r="B43" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C43" s="2" cm="1">
         <f t="array" ref="C43">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
         <v>651250</v>
       </c>
       <c r="D43" s="2">
+        <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E43" s="7">
+        <f t="shared" si="5"/>
+        <v>651250</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A44" s="29"/>
+      <c r="B44" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C44" s="2" cm="1">
+        <f t="array" ref="C44">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
+        <v>651250</v>
+      </c>
+      <c r="D44" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
         <v>0</v>
       </c>
-      <c r="E43" s="7">
-        <f t="shared" ref="E43" si="6">C43-D43</f>
+      <c r="E44" s="7">
+        <f t="shared" ref="E44" si="6">C44-D44</f>
         <v>651250</v>
       </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A45" s="29"/>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A46" s="29"/>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A47" s="29"/>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A48" s="29"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="29"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="29"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="29"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="29"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="29"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="29"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="29"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="29"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="29"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="29"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="29"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="29"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="29"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="29"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="29"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="12">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Dados atualizados em 17/07/2026 10:54
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4810163-3EDF-42F4-9206-8C681188A47E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098102FB-0048-4D4A-B24F-725C9F230EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-16T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-17T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -424,7 +424,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -511,15 +511,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Moeda" xfId="2" builtinId="4"/>
@@ -560,15 +551,11 @@
       </font>
       <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
+        <top/>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -590,6 +577,36 @@
       </font>
       <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
@@ -700,7 +717,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
@@ -790,31 +806,6 @@
         <bottom/>
         <vertical/>
         <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -1703,7 +1694,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>16/07/2026</v>
+            <v>17/07/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1739,13 +1730,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>26930.750000000011</v>
+            <v>28954.370000000006</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>1304.31</v>
+            <v>2023.62</v>
           </cell>
         </row>
         <row r="6">
@@ -1753,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>186540.97</v>
+            <v>192119.4199999999</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>11489.379999999997</v>
+            <v>5016.05</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1773,10 +1764,10 @@
             <v>828.94</v>
           </cell>
           <cell r="H7" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>51</v>
+            <v>1325.15</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1793,16 +1784,16 @@
             <v>151.09</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INDAIATUBA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>3491.37</v>
+            <v>5399.95</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N8">
-            <v>34</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="9">
@@ -1810,13 +1801,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>38366.310000000005</v>
+            <v>39691.460000000014</v>
           </cell>
           <cell r="H9" t="str">
-            <v>INTERLAGOS</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>13467.2</v>
+            <v>1699</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
@@ -1830,13 +1821,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>122430.97999999985</v>
+            <v>130910.1299999999</v>
           </cell>
           <cell r="H10" t="str">
-            <v>JUNDIAI</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I10">
-            <v>1664.94</v>
+            <v>2006.24</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
@@ -1850,13 +1841,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>40895.590000000033</v>
+            <v>42594.590000000047</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY ABC</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I11">
-            <v>13637.5</v>
+            <v>529.79999999999995</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
@@ -1870,19 +1861,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>174575.71999999997</v>
+            <v>189681.72</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY CASA</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I12">
-            <v>315.2</v>
+            <v>913.27</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>17</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="13">
@@ -1893,16 +1884,16 @@
             <v>161512.55999999997</v>
           </cell>
           <cell r="H13" t="str">
-            <v>KEY SJC</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I13">
-            <v>5897</v>
+            <v>5336</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>24</v>
+            <v>25</v>
           </cell>
         </row>
         <row r="14">
@@ -1913,10 +1904,10 @@
             <v>513142.70000000019</v>
           </cell>
           <cell r="H14" t="str">
-            <v>KEY SP</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I14">
-            <v>20532.100000000002</v>
+            <v>1356.2900000000002</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
@@ -1933,16 +1924,16 @@
             <v>60082.260000000017</v>
           </cell>
           <cell r="H15" t="str">
-            <v>KEY ZL</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I15">
-            <v>3075.6</v>
+            <v>1760.92</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>47</v>
+            <v>49</v>
           </cell>
         </row>
         <row r="16">
@@ -1953,10 +1944,10 @@
             <v>42315.899999999994</v>
           </cell>
           <cell r="H16" t="str">
-            <v>LESTE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I16">
-            <v>2980.05</v>
+            <v>139.9</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -1970,13 +1961,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>190365.22000000015</v>
+            <v>193562.72000000015</v>
           </cell>
           <cell r="H17" t="str">
-            <v>LESTE MOOCA</v>
+            <v>SBC</v>
           </cell>
           <cell r="I17">
-            <v>3987.1200000000003</v>
+            <v>6275.3</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
@@ -1990,13 +1981,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>206904.88</v>
+            <v>208911.12</v>
           </cell>
           <cell r="H18" t="str">
-            <v>LESTE PENHA</v>
+            <v>SJC</v>
           </cell>
           <cell r="I18">
-            <v>2362.75</v>
+            <v>1462.54</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -2010,19 +2001,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>52276.960000000021</v>
+            <v>52276.960000000014</v>
           </cell>
           <cell r="H19" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I19">
-            <v>2359.1500000000005</v>
+            <v>529.79999999999995</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>296</v>
+            <v>302</v>
           </cell>
         </row>
         <row r="20">
@@ -2030,13 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>91342.019999999902</v>
+            <v>92187.919999999882</v>
           </cell>
           <cell r="H20" t="str">
-            <v>MOGI</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I20">
-            <v>5852.5499999999993</v>
+            <v>2193.2399999999998</v>
           </cell>
         </row>
         <row r="21">
@@ -2044,13 +2035,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>66758.630000000019</v>
+            <v>67671.900000000009</v>
           </cell>
           <cell r="H21" t="str">
-            <v>NORTE</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I21">
-            <v>16318.529999999995</v>
+            <v>37967.07</v>
           </cell>
         </row>
         <row r="22">
@@ -2058,13 +2049,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>53959.710000000101</v>
-          </cell>
-          <cell r="H22" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="I22">
-            <v>15225.139999999994</v>
+            <v>59295.710000000094</v>
           </cell>
         </row>
         <row r="23">
@@ -2072,13 +2057,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>34449.390000000058</v>
-          </cell>
-          <cell r="H23" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I23">
-            <v>3452.3699999999994</v>
+            <v>35615.780000000057</v>
           </cell>
         </row>
         <row r="24">
@@ -2088,25 +2067,13 @@
           <cell r="F24">
             <v>131431.81999999983</v>
           </cell>
-          <cell r="H24" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I24">
-            <v>6695.95</v>
-          </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>176954.21999999994</v>
-          </cell>
-          <cell r="H25" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I25">
-            <v>7824.8499999999967</v>
+            <v>178715.14000000004</v>
           </cell>
         </row>
         <row r="26">
@@ -2114,13 +2081,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>69444.489999999962</v>
-          </cell>
-          <cell r="H26" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I26">
-            <v>1597.3100000000002</v>
+            <v>69584.389999999956</v>
           </cell>
         </row>
         <row r="27">
@@ -2128,13 +2089,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>83181.479999999952</v>
-          </cell>
-          <cell r="H27" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I27">
-            <v>1783.7000000000005</v>
+            <v>84980.229999999967</v>
           </cell>
         </row>
         <row r="28">
@@ -2142,13 +2097,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>128498.59999999985</v>
-          </cell>
-          <cell r="H28" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I28">
-            <v>1040.82</v>
+            <v>134773.89999999985</v>
           </cell>
         </row>
         <row r="29">
@@ -2156,13 +2105,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>44458.48000000004</v>
-          </cell>
-          <cell r="H29" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I29">
-            <v>146405.88999999966</v>
+            <v>45921.020000000055</v>
           </cell>
         </row>
         <row r="30">
@@ -2170,7 +2113,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>21855.87</v>
+            <v>22385.670000000002</v>
           </cell>
         </row>
         <row r="31">
@@ -2178,7 +2121,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>37456.760000000017</v>
+            <v>39650.000000000015</v>
           </cell>
         </row>
         <row r="32">
@@ -2186,7 +2129,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>2757112.2999999598</v>
+            <v>2818949.4199999906</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2417,15 +2360,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{50EE0FE5-ADD7-4A3A-9DF8-D52FFFCF08DA}" name="VENDEDOR" totalsRowLabel="Total" dataDxfId="9" totalsRowDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{4F0BAF4D-D0FC-4B7C-8FF4-8DDD6505FDA1}" name="REFERENCIA" dataDxfId="7" totalsRowDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{CCB341E8-8BC2-4209-AEA0-D6F26BFCB356}" name="META A" dataDxfId="5" totalsRowDxfId="6" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{50EE0FE5-ADD7-4A3A-9DF8-D52FFFCF08DA}" name="VENDEDOR" totalsRowLabel="Total" dataDxfId="10" totalsRowDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{4F0BAF4D-D0FC-4B7C-8FF4-8DDD6505FDA1}" name="REFERENCIA" dataDxfId="8" totalsRowDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{CCB341E8-8BC2-4209-AEA0-D6F26BFCB356}" name="META A" dataDxfId="6" totalsRowDxfId="5" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],[1]!Tabela2[VENDEDOR],[1]!Tabela2[META A])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{9AA985E6-33FD-40FD-9473-5AF6B4D03030}" name="ATINGIDO" dataDxfId="3" totalsRowDxfId="4" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{9AA985E6-33FD-40FD-9473-5AF6B4D03030}" name="ATINGIDO" dataDxfId="4" totalsRowDxfId="3" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7B8A46E1-DE6F-44C0-A6C8-83887563A4C0}" name="FALTA" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="2">
+    <tableColumn id="5" xr3:uid="{7B8A46E1-DE6F-44C0-A6C8-83887563A4C0}" name="FALTA" totalsRowFunction="sum" dataDxfId="2" totalsRowDxfId="1">
       <calculatedColumnFormula>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3003,7 +2946,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>150013</v>
+        <v>130000</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -3037,7 +2980,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>2757112.3</v>
+        <v>2818949.4200000004</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3048,7 +2991,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>102897.48999999998</v>
+        <v>35960.830000000009</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3059,7 +3002,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>43457.399999999994</v>
+        <v>2006.24</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3070,7 +3013,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3082,7 +3025,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>2835387.7</v>
+        <v>2773550.5799999996</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3093,7 +3036,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>47115.510000000024</v>
+        <v>94039.169999999984</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3104,7 +3047,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-43457.399999999994</v>
+        <v>-2006.24</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3115,7 +3058,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3127,7 +3070,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.49300175234689314</v>
+        <v>0.50405890388913732</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3138,7 +3081,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.68592381993560547</v>
+        <v>0.27662176923076931</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3160,7 +3103,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.39050131926121368</v>
+        <v>0.39841688654353558</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3259,11 +3202,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>26930.750000000011</v>
+        <v>28954.370000000006</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>37569.249999999985</v>
+        <v>35545.62999999999</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3274,15 +3217,15 @@
       </c>
       <c r="I10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>17000</v>
+        <v>13500</v>
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>15225.139999999994</v>
+        <v>1760.92</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1774.860000000006</v>
+        <v>11739.08</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3333,11 +3276,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>186540.97</v>
+        <v>192119.4199999999</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>138459.03</v>
+        <v>132880.5800000001</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3348,15 +3291,15 @@
       </c>
       <c r="I11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11850</v>
+        <v>6500</v>
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>16318.529999999995</v>
+        <v>0</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-4468.5299999999952</v>
+        <v>6500</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3371,11 +3314,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13637.5</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>-13637.5</v>
+        <v>0</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3390,11 +3333,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3424,15 +3367,15 @@
       </c>
       <c r="I12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>9000</v>
+        <v>4520</v>
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3452.3699999999994</v>
+        <v>139.9</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5547.630000000001</v>
+        <v>4380.1000000000004</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3486,11 +3429,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>38366.310000000005</v>
+        <v>39691.460000000014</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>51633.689999999995</v>
+        <v>50308.539999999986</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3501,15 +3444,15 @@
       </c>
       <c r="I13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15000</v>
+        <v>7850</v>
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7824.8499999999967</v>
+        <v>6275.3</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7175.1500000000033</v>
+        <v>1574.6999999999998</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3524,11 +3467,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3075.6</v>
+        <v>2006.24</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-3075.6</v>
+        <v>-2006.24</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3563,11 +3506,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>122430.97999999985</v>
+        <v>130910.1299999999</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>150569.02000000014</v>
+        <v>142089.87000000011</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3578,15 +3521,15 @@
       </c>
       <c r="I14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5324</v>
+        <v>6500</v>
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2359.1500000000005</v>
+        <v>5336</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2964.8499999999995</v>
+        <v>1164</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3640,11 +3583,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>40895.590000000033</v>
+        <v>42594.590000000047</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>37104.409999999967</v>
+        <v>35405.409999999953</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3655,15 +3598,15 @@
       </c>
       <c r="I15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>16000</v>
+        <v>12500</v>
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11489.379999999997</v>
+        <v>5016.05</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4510.6200000000026</v>
+        <v>7483.95</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3678,11 +3621,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>20532.100000000002</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-20532.100000000002</v>
+        <v>0</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3717,11 +3660,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>174575.71999999997</v>
+        <v>189681.72</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>150424.28000000003</v>
+        <v>135318.28</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3732,15 +3675,15 @@
       </c>
       <c r="I16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12810</v>
+        <v>4240</v>
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6695.95</v>
+        <v>0</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6114.05</v>
+        <v>4240</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3755,11 +3698,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5897</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>-5897</v>
+        <v>0</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3809,15 +3752,15 @@
       </c>
       <c r="I17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3144</v>
+        <v>8290</v>
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5852.5499999999993</v>
+        <v>1356.2900000000002</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-2708.5499999999993</v>
+        <v>6933.71</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3832,11 +3775,11 @@
       </c>
       <c r="P17" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>315.2</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="1"/>
-        <v>-315.2</v>
+        <v>0</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="19" t="s">
@@ -3886,15 +3829,15 @@
       </c>
       <c r="I18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6216</v>
+        <v>8500</v>
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2980.05</v>
+        <v>0</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3235.95</v>
+        <v>8500</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3950,15 +3893,15 @@
       </c>
       <c r="I19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>10870</v>
+        <v>8500</v>
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3987.1200000000003</v>
+        <v>529.79999999999995</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6882.8799999999992</v>
+        <v>7970.2</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3975,11 +3918,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3995,11 +3938,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>190365.22000000015</v>
+        <v>193562.72000000015</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>369634.77999999985</v>
+        <v>366437.27999999985</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -4010,15 +3953,15 @@
       </c>
       <c r="I20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13000</v>
+        <v>11500</v>
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13467.2</v>
+        <v>5399.95</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-467.20000000000073</v>
+        <v>6100.05</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4047,11 +3990,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4067,11 +4010,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>206904.88</v>
+        <v>208911.12</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>208095.12</v>
+        <v>206088.88</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4082,15 +4025,15 @@
       </c>
       <c r="I21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5020</v>
+        <v>5500</v>
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1664.94</v>
+        <v>1699</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3355.06</v>
+        <v>3801</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4142,7 +4085,7 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52276.960000000021</v>
+        <v>52276.960000000014</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
@@ -4157,15 +4100,15 @@
       </c>
       <c r="I22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>8104</v>
+        <v>4000</v>
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2362.75</v>
+        <v>913.27</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5741.25</v>
+        <v>3086.73</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4178,11 +4121,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>520408.39000000031</v>
+        <v>519801.59000000026</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-24953.844545454835</v>
+        <v>-24347.044545454788</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4217,11 +4160,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>91342.019999999902</v>
+        <v>92187.919999999882</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>103657.9800000001</v>
+        <v>102812.08000000012</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4232,15 +4175,15 @@
       </c>
       <c r="I23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5255</v>
+        <v>5500</v>
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3491.37</v>
+        <v>1325.15</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1763.63</v>
+        <v>4174.8500000000004</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4253,11 +4196,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>501773.76999999979</v>
+        <v>522690.31</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>117544.4118181821</v>
+        <v>96627.871818181884</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4292,11 +4235,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>66758.630000000019</v>
+        <v>67671.900000000009</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>73241.369999999981</v>
+        <v>72328.099999999991</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4307,15 +4250,15 @@
       </c>
       <c r="I24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3110</v>
+        <v>4700</v>
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1040.82</v>
+        <v>2193.2399999999998</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2069.1800000000003</v>
+        <v>2506.7600000000002</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4367,11 +4310,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>53959.710000000101</v>
+        <v>59295.710000000094</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>88540.289999999892</v>
+        <v>83204.289999999906</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4382,15 +4325,15 @@
       </c>
       <c r="I25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3570</v>
+        <v>6080</v>
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1597.3100000000002</v>
+        <v>1462.54</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1972.6899999999998</v>
+        <v>4617.46</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4422,11 +4365,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4442,11 +4385,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>34449.390000000058</v>
+        <v>35615.780000000057</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>55550.609999999942</v>
+        <v>54384.219999999943</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4457,15 +4400,15 @@
       </c>
       <c r="I26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2442</v>
+        <v>5500</v>
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1783.7000000000005</v>
+        <v>529.79999999999995</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>658.2999999999995</v>
+        <v>4970.2</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4521,15 +4464,15 @@
       </c>
       <c r="I27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2298</v>
+        <v>6320</v>
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1304.31</v>
+        <v>2023.62</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>993.69</v>
+        <v>4296.38</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4552,11 +4495,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>176954.21999999994</v>
+        <v>178715.14000000004</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>141545.78000000006</v>
+        <v>139784.85999999996</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4631,11 +4574,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>69444.489999999962</v>
+        <v>69584.389999999956</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65055.510000000038</v>
+        <v>64915.610000000044</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4688,11 +4631,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>83181.479999999952</v>
+        <v>84980.229999999967</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>83818.520000000048</v>
+        <v>82019.770000000033</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4705,11 +4648,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>256807.39999999982</v>
+        <v>256617.49999999983</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>133942.60000000018</v>
+        <v>134132.50000000017</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4748,11 +4691,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>128498.59999999985</v>
+        <v>134773.89999999985</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>131501.40000000014</v>
+        <v>125226.10000000015</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4765,11 +4708,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>501687.34000000299</v>
+        <v>501687.34000000305</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>19312.659999997006</v>
+        <v>19312.659999996948</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4788,11 +4731,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>9.2727272727272521</v>
+        <v>1.2727272727272521</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4808,11 +4751,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>44458.48000000004</v>
+        <v>45921.020000000055</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>55541.51999999996</v>
+        <v>54078.979999999945</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4825,11 +4768,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>557396.27000000444</v>
+        <v>598267.65000000386</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>93853.729999995558</v>
+        <v>52982.349999996135</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4868,11 +4811,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>21855.87</v>
+        <v>22385.670000000002</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>33144.130000000005</v>
+        <v>32614.329999999998</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4928,11 +4871,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>37456.760000000017</v>
+        <v>39650.000000000015</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>35543.239999999983</v>
+        <v>33349.999999999985</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4965,21 +4908,21 @@
       <c r="W35" s="4"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A36" s="30" t="s">
+      <c r="A36" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="30" t="s">
+      <c r="B36" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="31">
+      <c r="C36" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],[1]!Tabela2[VENDEDOR],[1]!Tabela2[META A])</f>
         <v>1000</v>
       </c>
-      <c r="D36" s="31">
+      <c r="D36" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
         <v>828.94</v>
       </c>
-      <c r="E36" s="32">
+      <c r="E36" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
         <v>171.05999999999995</v>
       </c>
@@ -5088,11 +5031,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>545873.70000000158</v>
+        <v>545683.80000000156</v>
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>-155123.70000000158</v>
+        <v>-154933.80000000156</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -5124,11 +5067,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1104362.189999996</v>
+        <v>1103755.3899999959</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="5">C41-D41</f>
-        <v>-583362.18999999599</v>
+        <v>-582755.38999999594</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -5160,11 +5103,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1106876.4099999981</v>
+        <v>1169510.229999996</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>-455626.40999999805</v>
+        <v>-518260.22999999602</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 07:32
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098102FB-0048-4D4A-B24F-725C9F230EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE4B821-55C4-4629-B841-4C90615F5945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-17T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1694,7 +1694,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>17/07/2026</v>
+            <v/>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1730,13 +1730,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>28954.370000000006</v>
-          </cell>
-          <cell r="H5" t="str">
-            <v>CAMPINAS</v>
-          </cell>
-          <cell r="I5">
-            <v>2023.62</v>
+            <v>35170.719999999994</v>
           </cell>
         </row>
         <row r="6">
@@ -1744,13 +1738,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>192119.4199999999</v>
-          </cell>
-          <cell r="H6" t="str">
-            <v>CENTRO</v>
-          </cell>
-          <cell r="I6">
-            <v>5016.05</v>
+            <v>250121.85999999967</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1761,19 +1749,10 @@
             <v>ECOMMERCE</v>
           </cell>
           <cell r="F7">
-            <v>828.94</v>
-          </cell>
-          <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
-          </cell>
-          <cell r="I7">
-            <v>1325.15</v>
+            <v>1082.83</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
-          </cell>
-          <cell r="N7" t="str">
-            <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
@@ -1783,17 +1762,8 @@
           <cell r="F8">
             <v>151.09</v>
           </cell>
-          <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
-          </cell>
-          <cell r="I8">
-            <v>5399.95</v>
-          </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
-          </cell>
-          <cell r="N8">
-            <v>35</v>
           </cell>
         </row>
         <row r="9">
@@ -1801,19 +1771,10 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>39691.460000000014</v>
-          </cell>
-          <cell r="H9" t="str">
-            <v>JUNDIAI</v>
-          </cell>
-          <cell r="I9">
-            <v>1699</v>
+            <v>49046.209999999985</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
-          </cell>
-          <cell r="N9">
-            <v>30</v>
           </cell>
         </row>
         <row r="10">
@@ -1821,19 +1782,10 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>130910.1299999999</v>
-          </cell>
-          <cell r="H10" t="str">
-            <v>KEY ZL</v>
-          </cell>
-          <cell r="I10">
-            <v>2006.24</v>
+            <v>170499.18999999986</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
-          </cell>
-          <cell r="N10">
-            <v>16</v>
           </cell>
         </row>
         <row r="11">
@@ -1841,19 +1793,10 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>42594.590000000047</v>
-          </cell>
-          <cell r="H11" t="str">
-            <v>LESTE MOOCA</v>
-          </cell>
-          <cell r="I11">
-            <v>529.79999999999995</v>
+            <v>48386.230000000061</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
-          </cell>
-          <cell r="N11">
-            <v>25</v>
           </cell>
         </row>
         <row r="12">
@@ -1861,19 +1804,10 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>189681.72</v>
-          </cell>
-          <cell r="H12" t="str">
-            <v>LESTE PENHA</v>
-          </cell>
-          <cell r="I12">
-            <v>913.27</v>
+            <v>209220.31999999995</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
-          </cell>
-          <cell r="N12">
-            <v>19</v>
           </cell>
         </row>
         <row r="13">
@@ -1881,19 +1815,10 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>161512.55999999997</v>
-          </cell>
-          <cell r="H13" t="str">
-            <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="I13">
-            <v>5336</v>
+            <v>263985.40000000084</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="N13">
-            <v>25</v>
           </cell>
         </row>
         <row r="14">
@@ -1901,19 +1826,10 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>513142.70000000019</v>
-          </cell>
-          <cell r="H14" t="str">
-            <v>MOGI</v>
-          </cell>
-          <cell r="I14">
-            <v>1356.2900000000002</v>
+            <v>516869.3000000001</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
-          </cell>
-          <cell r="N14">
-            <v>35</v>
           </cell>
         </row>
         <row r="15">
@@ -1921,19 +1837,10 @@
             <v>KEY PIRACICABA</v>
           </cell>
           <cell r="F15">
-            <v>60082.260000000017</v>
-          </cell>
-          <cell r="H15" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="I15">
-            <v>1760.92</v>
+            <v>87483.25999999998</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
-          </cell>
-          <cell r="N15">
-            <v>49</v>
           </cell>
         </row>
         <row r="16">
@@ -1941,19 +1848,10 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>42315.899999999994</v>
-          </cell>
-          <cell r="H16" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I16">
-            <v>139.9</v>
+            <v>90046.200000000041</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
-          </cell>
-          <cell r="N16">
-            <v>27</v>
           </cell>
         </row>
         <row r="17">
@@ -1961,19 +1859,10 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>193562.72000000015</v>
-          </cell>
-          <cell r="H17" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I17">
-            <v>6275.3</v>
+            <v>263197.75</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="N17">
-            <v>22</v>
           </cell>
         </row>
         <row r="18">
@@ -1981,19 +1870,10 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>208911.12</v>
-          </cell>
-          <cell r="H18" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I18">
-            <v>1462.54</v>
+            <v>258438.59999999986</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
-          </cell>
-          <cell r="N18">
-            <v>19</v>
           </cell>
         </row>
         <row r="19">
@@ -2001,19 +1881,10 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>52276.960000000014</v>
-          </cell>
-          <cell r="H19" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I19">
-            <v>529.79999999999995</v>
+            <v>68920.430000000037</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
-          </cell>
-          <cell r="N19">
-            <v>302</v>
           </cell>
         </row>
         <row r="20">
@@ -2021,13 +1892,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>92187.919999999882</v>
-          </cell>
-          <cell r="H20" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I20">
-            <v>2193.2399999999998</v>
+            <v>124383.96499999975</v>
           </cell>
         </row>
         <row r="21">
@@ -2035,13 +1900,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>67671.900000000009</v>
-          </cell>
-          <cell r="H21" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I21">
-            <v>37967.07</v>
+            <v>90030.500000000029</v>
           </cell>
         </row>
         <row r="22">
@@ -2049,7 +1908,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>59295.710000000094</v>
+            <v>81708.579999999885</v>
           </cell>
         </row>
         <row r="23">
@@ -2057,7 +1916,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>35615.780000000057</v>
+            <v>45589.900000000074</v>
           </cell>
         </row>
         <row r="24">
@@ -2065,7 +1924,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>131431.81999999983</v>
+            <v>155921.10999999987</v>
           </cell>
         </row>
         <row r="25">
@@ -2073,7 +1932,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>178715.14000000004</v>
+            <v>228769.10999999967</v>
           </cell>
         </row>
         <row r="26">
@@ -2081,7 +1940,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>69584.389999999956</v>
+            <v>88801.109999999913</v>
           </cell>
         </row>
         <row r="27">
@@ -2089,7 +1948,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>84980.229999999967</v>
+            <v>104847.86999999995</v>
           </cell>
         </row>
         <row r="28">
@@ -2097,7 +1956,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>134773.89999999985</v>
+            <v>169078.53999999986</v>
           </cell>
         </row>
         <row r="29">
@@ -2105,7 +1964,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>45921.020000000055</v>
+            <v>56024.890000000094</v>
           </cell>
         </row>
         <row r="30">
@@ -2113,7 +1972,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>22385.670000000002</v>
+            <v>29659.220000000012</v>
           </cell>
         </row>
         <row r="31">
@@ -2121,7 +1980,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>39650.000000000015</v>
+            <v>51511.549999999988</v>
           </cell>
         </row>
         <row r="32">
@@ -2129,7 +1988,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>2818949.4199999906</v>
+            <v>3538945.7349999724</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2946,7 +2805,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>130000</v>
+        <v>150000</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -2980,7 +2839,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>2818949.4200000004</v>
+        <v>3538945.7349999999</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2991,7 +2850,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>35960.830000000009</v>
+        <v>0</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3002,7 +2861,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>2006.24</v>
+        <v>0</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3013,7 +2872,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>302</v>
+        <v>0</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3025,7 +2884,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>2773550.5799999996</v>
+        <v>2053554.2650000001</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3036,7 +2895,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>94039.169999999984</v>
+        <v>150000</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3047,7 +2906,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-2006.24</v>
+        <v>0</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3058,7 +2917,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>456</v>
+        <v>758</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3070,7 +2929,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.50405890388913732</v>
+        <v>0.6328020983459991</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3081,7 +2940,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.27662176923076931</v>
+        <v>0</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3103,7 +2962,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.39841688654353558</v>
+        <v>0</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3202,11 +3061,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>28954.370000000006</v>
+        <v>35170.719999999994</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>35545.62999999999</v>
+        <v>29329.280000000006</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3217,15 +3076,15 @@
       </c>
       <c r="I10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13500</v>
+        <v>17000</v>
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1760.92</v>
+        <v>0</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11739.08</v>
+        <v>17000</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3276,11 +3135,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>192119.4199999999</v>
+        <v>250121.85999999967</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>132880.5800000001</v>
+        <v>74878.140000000334</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3291,7 +3150,7 @@
       </c>
       <c r="I11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6500</v>
+        <v>11960</v>
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3299,7 +3158,7 @@
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6500</v>
+        <v>11960</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3333,11 +3192,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>17</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3367,15 +3226,15 @@
       </c>
       <c r="I12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4520</v>
+        <v>9110</v>
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>139.9</v>
+        <v>0</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4380.1000000000004</v>
+        <v>9110</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3409,11 +3268,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3429,11 +3288,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>39691.460000000014</v>
+        <v>49046.209999999985</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50308.539999999986</v>
+        <v>40953.790000000015</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3444,15 +3303,15 @@
       </c>
       <c r="I13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>7850</v>
+        <v>15000</v>
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6275.3</v>
+        <v>0</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1574.6999999999998</v>
+        <v>15000</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3467,11 +3326,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2006.24</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-2006.24</v>
+        <v>0</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3506,11 +3365,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>130910.1299999999</v>
+        <v>170499.18999999986</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>142089.87000000011</v>
+        <v>102500.81000000014</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3521,15 +3380,15 @@
       </c>
       <c r="I14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6500</v>
+        <v>4280</v>
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5336</v>
+        <v>0</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1164</v>
+        <v>4280</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3563,11 +3422,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3583,11 +3442,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>42594.590000000047</v>
+        <v>48386.230000000061</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>35405.409999999953</v>
+        <v>29613.769999999939</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3598,15 +3457,15 @@
       </c>
       <c r="I15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5016.05</v>
+        <v>0</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7483.95</v>
+        <v>15000</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3640,11 +3499,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>23</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3660,11 +3519,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>189681.72</v>
+        <v>209220.31999999995</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>135318.28</v>
+        <v>115779.68000000005</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3675,7 +3534,7 @@
       </c>
       <c r="I16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4240</v>
+        <v>13470</v>
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3683,7 +3542,7 @@
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4240</v>
+        <v>13470</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3737,11 +3596,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>161512.55999999997</v>
+        <v>263985.40000000084</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>8487.4400000000314</v>
+        <v>-93985.400000000838</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3752,15 +3611,15 @@
       </c>
       <c r="I17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>8290</v>
+        <v>2530</v>
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1356.2900000000002</v>
+        <v>0</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6933.71</v>
+        <v>2530</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3814,11 +3673,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>513142.70000000019</v>
+        <v>516869.3000000001</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>436857.29999999981</v>
+        <v>433130.6999999999</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3829,7 +3688,7 @@
       </c>
       <c r="I18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>8500</v>
+        <v>6840</v>
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3837,7 +3696,7 @@
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8500</v>
+        <v>6840</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3858,11 +3717,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3878,11 +3737,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>42315.899999999994</v>
+        <v>90046.200000000041</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>87684.1</v>
+        <v>39953.799999999959</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3893,15 +3752,15 @@
       </c>
       <c r="I19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>8500</v>
+        <v>10910</v>
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>529.79999999999995</v>
+        <v>0</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7970.2</v>
+        <v>10910</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3918,11 +3777,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3938,11 +3797,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>193562.72000000015</v>
+        <v>263197.75</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>366437.27999999985</v>
+        <v>296802.25</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3953,15 +3812,15 @@
       </c>
       <c r="I20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11500</v>
+        <v>13000</v>
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5399.95</v>
+        <v>0</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6100.05</v>
+        <v>13000</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3990,11 +3849,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4010,11 +3869,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>208911.12</v>
+        <v>258438.59999999986</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>206088.88</v>
+        <v>156561.40000000014</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4025,15 +3884,15 @@
       </c>
       <c r="I21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5500</v>
+        <v>5490</v>
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1699</v>
+        <v>0</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3801</v>
+        <v>5490</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4046,11 +3905,11 @@
       </c>
       <c r="P21" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>266634.81999999983</v>
+        <v>266634.81999999995</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>104956.08909090929</v>
+        <v>104956.08909090917</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="19" t="s">
@@ -4065,11 +3924,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -4085,11 +3944,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52276.960000000014</v>
+        <v>68920.430000000037</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>69723.039999999979</v>
+        <v>53079.569999999963</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4100,15 +3959,15 @@
       </c>
       <c r="I22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4000</v>
+        <v>7350</v>
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>913.27</v>
+        <v>0</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3086.73</v>
+        <v>7350</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4140,11 +3999,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>18</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4160,11 +4019,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>92187.919999999882</v>
+        <v>124383.96499999975</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>102812.08000000012</v>
+        <v>70616.035000000251</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4175,15 +4034,15 @@
       </c>
       <c r="I23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5500</v>
+        <v>5290</v>
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1325.15</v>
+        <v>0</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4174.8500000000004</v>
+        <v>5290</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4196,11 +4055,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>522690.31</v>
+        <v>661756.44999999937</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>96627.871818181884</v>
+        <v>-42438.26818181749</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4235,11 +4094,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>67671.900000000009</v>
+        <v>90030.500000000029</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>72328.099999999991</v>
+        <v>49969.499999999971</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4250,15 +4109,15 @@
       </c>
       <c r="I24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4700</v>
+        <v>3540</v>
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2193.2399999999998</v>
+        <v>0</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2506.7600000000002</v>
+        <v>3540</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4271,11 +4130,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>153564.71</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>619318.18181818188</v>
+        <v>465753.47181818192</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4290,11 +4149,11 @@
       </c>
       <c r="V24" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="W24" s="19">
         <f t="shared" si="2"/>
-        <v>18</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -4310,11 +4169,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>59295.710000000094</v>
+        <v>81708.579999999885</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>83204.289999999906</v>
+        <v>60791.420000000115</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4325,15 +4184,15 @@
       </c>
       <c r="I25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6080</v>
+        <v>3900</v>
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1462.54</v>
+        <v>0</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4617.46</v>
+        <v>3900</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4365,11 +4224,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>26</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4385,11 +4244,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>35615.780000000057</v>
+        <v>45589.900000000074</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>54384.219999999943</v>
+        <v>44410.099999999926</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4400,15 +4259,15 @@
       </c>
       <c r="I26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5500</v>
+        <v>2780</v>
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>529.79999999999995</v>
+        <v>0</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4970.2</v>
+        <v>2780</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4449,11 +4308,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>131431.81999999983</v>
+        <v>155921.10999999987</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>106068.18000000017</v>
+        <v>81578.89000000013</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4464,15 +4323,15 @@
       </c>
       <c r="I27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6320</v>
+        <v>2550</v>
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2023.62</v>
+        <v>0</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4296.38</v>
+        <v>2550</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4495,11 +4354,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>178715.14000000004</v>
+        <v>228769.10999999967</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>139784.85999999996</v>
+        <v>89730.890000000334</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4528,11 +4387,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>60082.260000000017</v>
+        <v>87483.25999999998</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>114917.73999999999</v>
+        <v>87516.74000000002</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4574,11 +4433,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>69584.389999999956</v>
+        <v>88801.109999999913</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>64915.610000000044</v>
+        <v>45698.890000000087</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4631,11 +4490,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>84980.229999999967</v>
+        <v>104847.86999999995</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>82019.770000000033</v>
+        <v>62152.130000000048</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4691,11 +4550,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>134773.89999999985</v>
+        <v>169078.53999999986</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>125226.10000000015</v>
+        <v>90921.460000000137</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4708,11 +4567,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>501687.34000000305</v>
+        <v>501687.34000000299</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>19312.659999996948</v>
+        <v>19312.659999997006</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4731,11 +4590,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>1.2727272727272521</v>
+        <v>-16.727272727272748</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4751,11 +4610,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>45921.020000000055</v>
+        <v>56024.890000000094</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>54078.979999999945</v>
+        <v>43975.109999999906</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4768,11 +4627,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>598267.65000000386</v>
+        <v>656209.83000000252</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>52982.349999996135</v>
+        <v>-4959.8300000025192</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4791,11 +4650,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>172.27272727272725</v>
+        <v>91.272727272727252</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4811,11 +4670,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>22385.670000000002</v>
+        <v>29659.220000000012</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>32614.329999999998</v>
+        <v>25340.779999999988</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4828,11 +4687,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>309572.35000000085</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>651250</v>
+        <v>341677.64999999915</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4871,11 +4730,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>39650.000000000015</v>
+        <v>51511.549999999988</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>33349.999999999985</v>
+        <v>21488.450000000012</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4920,11 +4779,11 @@
       </c>
       <c r="D36" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>828.94</v>
+        <v>1082.83</v>
       </c>
       <c r="E36" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>171.05999999999995</v>
+        <v>-82.829999999999927</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -5067,11 +4926,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1103755.3899999959</v>
+        <v>1103755.3899999962</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="5">C41-D41</f>
-        <v>-582755.38999999594</v>
+        <v>-582755.38999999617</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -5103,11 +4962,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1169510.229999996</v>
+        <v>1392309.7799999886</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>-518260.22999999602</v>
+        <v>-741059.77999998862</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -5139,11 +4998,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>497196.76500000083</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>651250</v>
+        <v>154053.23499999917</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 08:39
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE4B821-55C4-4629-B841-4C90615F5945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC4ACA97-E5DA-4CE0-9F67-36F85D27D6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-22T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1694,7 +1694,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v/>
+            <v>22/07/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1730,7 +1730,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>35170.719999999994</v>
+            <v>36967.219999999994</v>
+          </cell>
+          <cell r="H5" t="str">
+            <v>CAMPINAS</v>
+          </cell>
+          <cell r="I5">
+            <v>1796.4999999999998</v>
           </cell>
         </row>
         <row r="6">
@@ -1738,7 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>250121.85999999967</v>
+            <v>251896.55999999962</v>
+          </cell>
+          <cell r="H6" t="str">
+            <v>CENTRO</v>
+          </cell>
+          <cell r="I6">
+            <v>1774.7</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1751,8 +1763,17 @@
           <cell r="F7">
             <v>1082.83</v>
           </cell>
+          <cell r="H7" t="str">
+            <v>INTERLAGOS</v>
+          </cell>
+          <cell r="I7">
+            <v>169.9</v>
+          </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
+          </cell>
+          <cell r="N7" t="str">
+            <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
@@ -1762,8 +1783,17 @@
           <cell r="F8">
             <v>151.09</v>
           </cell>
+          <cell r="H8" t="str">
+            <v>LESTE</v>
+          </cell>
+          <cell r="I8">
+            <v>430.15</v>
+          </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
+          </cell>
+          <cell r="N8">
+            <v>40</v>
           </cell>
         </row>
         <row r="9">
@@ -1771,10 +1801,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>49046.209999999985</v>
+            <v>49046.209999999992</v>
+          </cell>
+          <cell r="H9" t="str">
+            <v>LESTE MOOCA</v>
+          </cell>
+          <cell r="I9">
+            <v>2834.6</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
+          </cell>
+          <cell r="N9">
+            <v>31</v>
           </cell>
         </row>
         <row r="10">
@@ -1782,10 +1821,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>170499.18999999986</v>
+            <v>170669.08999999985</v>
+          </cell>
+          <cell r="H10" t="str">
+            <v>LESTE PENHA</v>
+          </cell>
+          <cell r="I10">
+            <v>625.89</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
+          </cell>
+          <cell r="N10">
+            <v>18</v>
           </cell>
         </row>
         <row r="11">
@@ -1795,8 +1843,17 @@
           <cell r="F11">
             <v>48386.230000000061</v>
           </cell>
+          <cell r="H11" t="str">
+            <v>MOGI</v>
+          </cell>
+          <cell r="I11">
+            <v>608.20000000000005</v>
+          </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
+          </cell>
+          <cell r="N11">
+            <v>27</v>
           </cell>
         </row>
         <row r="12">
@@ -1806,8 +1863,17 @@
           <cell r="F12">
             <v>209220.31999999995</v>
           </cell>
+          <cell r="H12" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="I12">
+            <v>664.59999999999991</v>
+          </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
+          </cell>
+          <cell r="N12">
+            <v>23</v>
           </cell>
         </row>
         <row r="13">
@@ -1817,8 +1883,17 @@
           <cell r="F13">
             <v>263985.40000000084</v>
           </cell>
+          <cell r="H13" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I13">
+            <v>809</v>
+          </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
+          </cell>
+          <cell r="N13">
+            <v>33</v>
           </cell>
         </row>
         <row r="14">
@@ -1828,8 +1903,17 @@
           <cell r="F14">
             <v>516869.3000000001</v>
           </cell>
+          <cell r="H14" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I14">
+            <v>75</v>
+          </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
+          </cell>
+          <cell r="N14">
+            <v>38</v>
           </cell>
         </row>
         <row r="15">
@@ -1837,10 +1921,19 @@
             <v>KEY PIRACICABA</v>
           </cell>
           <cell r="F15">
-            <v>87483.25999999998</v>
+            <v>87483.259999999951</v>
+          </cell>
+          <cell r="H15" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I15">
+            <v>9788.5399999999972</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
+          </cell>
+          <cell r="N15">
+            <v>58</v>
           </cell>
         </row>
         <row r="16">
@@ -1853,6 +1946,9 @@
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
           </cell>
+          <cell r="N16">
+            <v>27</v>
+          </cell>
         </row>
         <row r="17">
           <cell r="E17" t="str">
@@ -1864,6 +1960,9 @@
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
+          <cell r="N17">
+            <v>24</v>
+          </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
@@ -1875,16 +1974,22 @@
           <cell r="K18" t="str">
             <v>SJC</v>
           </cell>
+          <cell r="N18">
+            <v>21</v>
+          </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>68920.430000000037</v>
+            <v>69350.580000000045</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
+          </cell>
+          <cell r="N19">
+            <v>340</v>
           </cell>
         </row>
         <row r="20">
@@ -1892,7 +1997,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>124383.96499999975</v>
+            <v>127218.56499999974</v>
           </cell>
         </row>
         <row r="21">
@@ -1900,7 +2005,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>90030.500000000029</v>
+            <v>90656.390000000029</v>
           </cell>
         </row>
         <row r="22">
@@ -1916,7 +2021,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>45589.900000000074</v>
+            <v>46198.100000000079</v>
           </cell>
         </row>
         <row r="24">
@@ -1924,7 +2029,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>155921.10999999987</v>
+            <v>155921.10999999984</v>
           </cell>
         </row>
         <row r="25">
@@ -1940,7 +2045,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>88801.109999999913</v>
+            <v>89465.709999999919</v>
           </cell>
         </row>
         <row r="27">
@@ -1956,7 +2061,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>169078.53999999986</v>
+            <v>169078.53999999989</v>
           </cell>
         </row>
         <row r="29">
@@ -1964,7 +2069,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>56024.890000000094</v>
+            <v>56833.890000000094</v>
           </cell>
         </row>
         <row r="30">
@@ -1980,7 +2085,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>51511.549999999988</v>
+            <v>51586.549999999988</v>
           </cell>
         </row>
         <row r="32">
@@ -1988,7 +2093,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>3538945.7349999724</v>
+            <v>3548734.2749999715</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2839,7 +2944,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>3538945.7349999999</v>
+        <v>3548734.2750000004</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2850,7 +2955,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>0</v>
+        <v>9788.5399999999991</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2872,7 +2977,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>0</v>
+        <v>340</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2884,7 +2989,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>2053554.2650000001</v>
+        <v>2043765.7249999996</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2895,7 +3000,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>150000</v>
+        <v>140211.46</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2917,7 +3022,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>758</v>
+        <v>418</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2929,7 +3034,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.6328020983459991</v>
+        <v>0.6345523960661601</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2940,7 +3045,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0</v>
+        <v>6.5256933333333378E-2</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2962,7 +3067,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0</v>
+        <v>0.44854881266490765</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3061,11 +3166,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>35170.719999999994</v>
+        <v>36967.219999999994</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>29329.280000000006</v>
+        <v>27532.780000000006</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3135,11 +3240,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>250121.85999999967</v>
+        <v>251896.55999999962</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>74878.140000000334</v>
+        <v>73103.440000000381</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3192,11 +3297,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>52</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3230,11 +3335,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>664.59999999999991</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9110</v>
+        <v>8445.4</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3268,11 +3373,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>41</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3288,11 +3393,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>49046.209999999985</v>
+        <v>49046.209999999992</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40953.790000000015</v>
+        <v>40953.790000000008</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3365,11 +3470,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>170499.18999999986</v>
+        <v>170669.08999999985</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>102500.81000000014</v>
+        <v>102330.91000000015</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3422,11 +3527,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3461,11 +3566,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1774.7</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15000</v>
+        <v>13225.3</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3499,11 +3604,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3615,11 +3720,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>608.20000000000005</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2530</v>
+        <v>1921.8</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3692,11 +3797,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>430.15</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6840</v>
+        <v>6409.85</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3717,11 +3822,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3756,11 +3861,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>2834.6</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10910</v>
+        <v>8075.4</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3777,11 +3882,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>61</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3816,11 +3921,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>169.9</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>13000</v>
+        <v>12830.1</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3849,11 +3954,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3905,11 +4010,11 @@
       </c>
       <c r="P21" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>266634.81999999995</v>
+        <v>266634.81999999989</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>104956.08909090917</v>
+        <v>104956.08909090923</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="19" t="s">
@@ -3924,11 +4029,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>44</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3944,11 +4049,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>68920.430000000037</v>
+        <v>69350.580000000045</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>53079.569999999963</v>
+        <v>52649.419999999955</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -3963,11 +4068,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>625.89</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7350</v>
+        <v>6724.11</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -3999,11 +4104,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>40</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4019,11 +4124,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>124383.96499999975</v>
+        <v>127218.56499999974</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>70616.035000000251</v>
+        <v>67781.43500000026</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4055,11 +4160,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>661756.44999999937</v>
+        <v>661756.44999999925</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-42438.26818181749</v>
+        <v>-42438.268181817373</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4094,11 +4199,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>90030.500000000029</v>
+        <v>90656.390000000029</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>49969.499999999971</v>
+        <v>49343.609999999971</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4113,11 +4218,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3540</v>
+        <v>3465</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4149,11 +4254,11 @@
       </c>
       <c r="V24" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="W24" s="19">
         <f t="shared" si="2"/>
-        <v>37</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -4188,11 +4293,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>809</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3900</v>
+        <v>3091</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4224,11 +4329,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>51</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4244,11 +4349,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>45589.900000000074</v>
+        <v>46198.100000000079</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>44410.099999999926</v>
+        <v>43801.899999999921</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4308,11 +4413,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>155921.10999999987</v>
+        <v>155921.10999999984</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>81578.89000000013</v>
+        <v>81578.890000000159</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4327,11 +4432,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1796.4999999999998</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2550</v>
+        <v>753.50000000000023</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4387,11 +4492,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>87483.25999999998</v>
+        <v>87483.259999999951</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>87516.74000000002</v>
+        <v>87516.740000000049</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4433,11 +4538,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>88801.109999999913</v>
+        <v>89465.709999999919</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>45698.890000000087</v>
+        <v>45034.290000000081</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4550,11 +4655,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>169078.53999999986</v>
+        <v>169078.53999999989</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>90921.460000000137</v>
+        <v>90921.460000000108</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4610,11 +4715,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>56024.890000000094</v>
+        <v>56833.890000000094</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>43975.109999999906</v>
+        <v>43166.109999999906</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4627,11 +4732,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>656209.83000000252</v>
+        <v>656209.83000000194</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>-4959.8300000025192</v>
+        <v>-4959.8300000019372</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4650,11 +4755,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>91.272727272727252</v>
+        <v>90.272727272727252</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4687,11 +4792,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>309572.35000000085</v>
+        <v>316526.29000000103</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>341677.64999999915</v>
+        <v>334723.70999999897</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4730,11 +4835,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51511.549999999988</v>
+        <v>51586.549999999988</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>21488.450000000012</v>
+        <v>21413.450000000012</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4962,11 +5067,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1392309.7799999886</v>
+        <v>1392309.7799999909</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>-741059.77999998862</v>
+        <v>-741059.77999999095</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -4998,11 +5103,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>497196.76500000083</v>
+        <v>506985.30500000098</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>154053.23499999917</v>
+        <v>144264.69499999902</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 08:49
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC4ACA97-E5DA-4CE0-9F67-36F85D27D6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B5B1C6-12CA-46FC-95CE-D7765EDD1DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -4010,11 +4010,11 @@
       </c>
       <c r="P21" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>266634.81999999989</v>
+        <v>275241.61999999988</v>
       </c>
       <c r="Q21" s="7">
         <f>O21-P21</f>
-        <v>104956.08909090923</v>
+        <v>96349.289090909238</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="19" t="s">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>519801.59000000026</v>
+        <v>563167.95000000019</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-24347.044545454788</v>
+        <v>-67713.404545454716</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>661756.44999999925</v>
+        <v>691799.54999999935</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-42438.268181817373</v>
+        <v>-72481.368181817466</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4235,11 +4235,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>153564.71</v>
+        <v>159031.71</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>465753.47181818192</v>
+        <v>460286.47181818192</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4612,11 +4612,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>256617.49999999983</v>
+        <v>270334.04000000004</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>134132.50000000017</v>
+        <v>120415.95999999996</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4672,11 +4672,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>501687.34000000299</v>
+        <v>540157.7900000033</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>19312.659999997006</v>
+        <v>-19157.790000003297</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4732,11 +4732,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>656209.83000000194</v>
+        <v>700067.9900000022</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>-4959.8300000019372</v>
+        <v>-48817.990000002203</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4792,11 +4792,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>316526.29000000103</v>
+        <v>347699.70500000124</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>334723.70999999897</v>
+        <v>303550.29499999876</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 10:45
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B5B1C6-12CA-46FC-95CE-D7765EDD1DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A812A6F6-50CE-49B7-BA3C-A13441478DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1730,13 +1730,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>36967.219999999994</v>
+            <v>38432.729999999974</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>1796.4999999999998</v>
+            <v>3262.0099999999998</v>
           </cell>
         </row>
         <row r="6">
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>251896.55999999962</v>
+            <v>253523.69999999958</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>1774.7</v>
+            <v>3401.8400000000006</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1764,10 +1764,10 @@
             <v>1082.83</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>169.9</v>
+            <v>1865.2</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1784,10 +1784,10 @@
             <v>151.09</v>
           </cell>
           <cell r="H8" t="str">
-            <v>LESTE</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>430.15</v>
+            <v>1218.9000000000001</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -1801,19 +1801,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>49046.209999999992</v>
+            <v>50911.409999999996</v>
           </cell>
           <cell r="H9" t="str">
-            <v>LESTE MOOCA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>2834.6</v>
+            <v>2111</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N9">
-            <v>31</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="10">
@@ -1821,13 +1821,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>170669.08999999985</v>
+            <v>171718.08999999985</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE PENHA</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I10">
-            <v>625.89</v>
+            <v>1755.6</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
@@ -1841,19 +1841,19 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>48386.230000000061</v>
+            <v>50497.230000000061</v>
           </cell>
           <cell r="H11" t="str">
-            <v>MOGI</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I11">
-            <v>608.20000000000005</v>
+            <v>19933.399999999991</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="N11">
-            <v>27</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="12">
@@ -1864,16 +1864,16 @@
             <v>209220.31999999995</v>
           </cell>
           <cell r="H12" t="str">
-            <v>PIRITUBA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I12">
-            <v>664.59999999999991</v>
+            <v>3049.08</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="N12">
-            <v>23</v>
+            <v>24</v>
           </cell>
         </row>
         <row r="13">
@@ -1884,16 +1884,16 @@
             <v>263985.40000000084</v>
           </cell>
           <cell r="H13" t="str">
-            <v>SJC</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I13">
-            <v>809</v>
+            <v>4393.3999999999996</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>33</v>
+            <v>34</v>
           </cell>
         </row>
         <row r="14">
@@ -1904,16 +1904,16 @@
             <v>516869.3000000001</v>
           </cell>
           <cell r="H14" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I14">
-            <v>75</v>
+            <v>2026.69</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>38</v>
+            <v>39</v>
           </cell>
         </row>
         <row r="15">
@@ -1924,16 +1924,16 @@
             <v>87483.259999999951</v>
           </cell>
           <cell r="H15" t="str">
-            <v>Total Geral</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I15">
-            <v>9788.5399999999972</v>
+            <v>1089.3000000000002</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="N15">
-            <v>58</v>
+            <v>60</v>
           </cell>
         </row>
         <row r="16">
@@ -1943,6 +1943,12 @@
           <cell r="F16">
             <v>90046.200000000041</v>
           </cell>
+          <cell r="H16" t="str">
+            <v>MOGI</v>
+          </cell>
+          <cell r="I16">
+            <v>2802.23</v>
+          </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
           </cell>
@@ -1955,13 +1961,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>263197.75</v>
+            <v>264953.34999999998</v>
+          </cell>
+          <cell r="H17" t="str">
+            <v>NORTE</v>
+          </cell>
+          <cell r="I17">
+            <v>1391.6</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>24</v>
+            <v>25</v>
           </cell>
         </row>
         <row r="18">
@@ -1969,7 +1981,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>258438.59999999986</v>
+            <v>278371.99999999994</v>
+          </cell>
+          <cell r="H18" t="str">
+            <v>OSASCO</v>
+          </cell>
+          <cell r="I18">
+            <v>3163.2</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -1983,13 +2001,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>69350.580000000045</v>
+            <v>71969.509999999995</v>
+          </cell>
+          <cell r="H19" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="I19">
+            <v>944.40000000000009</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>340</v>
+            <v>350</v>
           </cell>
         </row>
         <row r="20">
@@ -1997,7 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>127218.56499999974</v>
+            <v>128777.36499999973</v>
+          </cell>
+          <cell r="H20" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="I20">
+            <v>4797.5999999999995</v>
           </cell>
         </row>
         <row r="21">
@@ -2005,7 +2035,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>90656.390000000029</v>
+            <v>92057.190000000046</v>
+          </cell>
+          <cell r="H21" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="I21">
+            <v>3032.0400000000004</v>
           </cell>
         </row>
         <row r="22">
@@ -2013,7 +2049,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>81708.579999999885</v>
+            <v>82797.879999999874</v>
+          </cell>
+          <cell r="H22" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I22">
+            <v>2083.1800000000003</v>
           </cell>
         </row>
         <row r="23">
@@ -2021,7 +2063,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>46198.100000000079</v>
+            <v>48392.130000000092</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I23">
+            <v>75</v>
           </cell>
         </row>
         <row r="24">
@@ -2029,7 +2077,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>155921.10999999984</v>
+            <v>157312.70999999982</v>
+          </cell>
+          <cell r="H24" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I24">
+            <v>62395.67</v>
           </cell>
         </row>
         <row r="25">
@@ -2037,7 +2091,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>228769.10999999967</v>
+            <v>231932.30999999968</v>
           </cell>
         </row>
         <row r="26">
@@ -2045,7 +2099,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>89465.709999999919</v>
+            <v>89745.509999999907</v>
           </cell>
         </row>
         <row r="27">
@@ -2053,7 +2107,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>104847.86999999995</v>
+            <v>109645.46999999996</v>
           </cell>
         </row>
         <row r="28">
@@ -2061,7 +2115,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>169078.53999999989</v>
+            <v>172110.57999999987</v>
           </cell>
         </row>
         <row r="29">
@@ -2069,7 +2123,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>56833.890000000094</v>
+            <v>58108.070000000094</v>
           </cell>
         </row>
         <row r="30">
@@ -2085,7 +2139,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>51586.549999999988</v>
+            <v>51586.549999999996</v>
           </cell>
         </row>
         <row r="32">
@@ -2093,7 +2147,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>3548734.2749999715</v>
+            <v>3601341.4049999751</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2944,7 +2998,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>3548734.2750000004</v>
+        <v>3601341.4049999989</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2955,7 +3009,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>9788.5399999999991</v>
+        <v>40706.670000000006</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2966,7 +3020,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>0</v>
+        <v>21688.999999999989</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -2977,7 +3031,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2989,7 +3043,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>2043765.7249999996</v>
+        <v>1991158.5950000011</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3000,7 +3054,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>140211.46</v>
+        <v>109293.32999999999</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3011,7 +3065,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>0</v>
+        <v>-21688.999999999989</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3022,7 +3076,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>418</v>
+        <v>408</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3034,7 +3088,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.6345523960661601</v>
+        <v>0.64395912472060779</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3045,7 +3099,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>6.5256933333333378E-2</v>
+        <v>0.27137780000000011</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3067,7 +3121,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.44854881266490765</v>
+        <v>0.46174142480211078</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3166,11 +3220,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>36967.219999999994</v>
+        <v>38432.729999999974</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>27532.780000000006</v>
+        <v>26067.270000000026</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3185,11 +3239,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>3163.2</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>17000</v>
+        <v>13836.8</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3240,11 +3294,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>251896.55999999962</v>
+        <v>253523.69999999958</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>73103.440000000381</v>
+        <v>71476.300000000425</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3259,11 +3313,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1391.6</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11960</v>
+        <v>10568.4</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3335,11 +3389,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>664.59999999999991</v>
+        <v>944.40000000000009</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8445.4</v>
+        <v>8165.6</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3373,11 +3427,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3393,11 +3447,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>49046.209999999992</v>
+        <v>50911.409999999996</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40953.790000000008</v>
+        <v>39088.590000000004</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3412,11 +3466,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>3032.0400000000004</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15000</v>
+        <v>11967.96</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3431,11 +3485,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>19933.399999999991</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>0</v>
+        <v>-19933.399999999991</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3470,11 +3524,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>170669.08999999985</v>
+        <v>171718.08999999985</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>102330.91000000015</v>
+        <v>101281.91000000015</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3489,11 +3543,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1089.3000000000002</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4280</v>
+        <v>3190.7</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3547,11 +3601,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>48386.230000000061</v>
+        <v>50497.230000000061</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>29613.769999999939</v>
+        <v>27502.769999999939</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3566,11 +3620,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1774.7</v>
+        <v>3401.8400000000006</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>13225.3</v>
+        <v>11598.16</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3585,11 +3639,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1755.6</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-1755.6</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3604,11 +3658,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3643,11 +3697,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4797.5999999999995</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>13470</v>
+        <v>8672.4000000000015</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3720,11 +3774,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>608.20000000000005</v>
+        <v>2802.23</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1921.8</v>
+        <v>-272.23</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3797,11 +3851,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>430.15</v>
+        <v>3049.08</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6409.85</v>
+        <v>3790.92</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3822,11 +3876,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3861,11 +3915,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2834.6</v>
+        <v>4393.3999999999996</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8075.4</v>
+        <v>6516.6</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3882,11 +3936,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3902,11 +3956,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>263197.75</v>
+        <v>264953.34999999998</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>296802.25</v>
+        <v>295046.65000000002</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3921,11 +3975,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>169.9</v>
+        <v>1218.9000000000001</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12830.1</v>
+        <v>11781.1</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3954,11 +4008,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3974,11 +4028,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>258438.59999999986</v>
+        <v>278371.99999999994</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>156561.40000000014</v>
+        <v>136628.00000000006</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -3993,11 +4047,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>2111</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5490</v>
+        <v>3379</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4049,11 +4103,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>69350.580000000045</v>
+        <v>71969.509999999995</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>52649.419999999955</v>
+        <v>50030.490000000005</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4068,11 +4122,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>625.89</v>
+        <v>2026.69</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6724.11</v>
+        <v>5323.3099999999995</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4104,11 +4158,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4124,11 +4178,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>127218.56499999974</v>
+        <v>128777.36499999973</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>67781.43500000026</v>
+        <v>66222.635000000271</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4143,11 +4197,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1865.2</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5290</v>
+        <v>3424.8</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4199,11 +4253,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>90656.390000000029</v>
+        <v>92057.190000000046</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>49343.609999999971</v>
+        <v>47942.809999999954</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4235,11 +4289,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>159031.71</v>
+        <v>180720.71000000008</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>460286.47181818192</v>
+        <v>438597.4718181818</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4274,11 +4328,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>81708.579999999885</v>
+        <v>82797.879999999874</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>60791.420000000115</v>
+        <v>59702.120000000126</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4293,11 +4347,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>809</v>
+        <v>2083.1800000000003</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3091</v>
+        <v>1816.8199999999997</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4329,11 +4383,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4349,11 +4403,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>46198.100000000079</v>
+        <v>48392.130000000092</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>43801.899999999921</v>
+        <v>41607.869999999908</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4413,11 +4467,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>155921.10999999984</v>
+        <v>157312.70999999982</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>81578.890000000159</v>
+        <v>80187.290000000183</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4432,11 +4486,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1796.4999999999998</v>
+        <v>3262.0099999999998</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>753.50000000000023</v>
+        <v>-712.00999999999976</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4459,11 +4513,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>228769.10999999967</v>
+        <v>231932.30999999968</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>89730.890000000334</v>
+        <v>86567.690000000322</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4538,11 +4592,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>89465.709999999919</v>
+        <v>89745.509999999907</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>45034.290000000081</v>
+        <v>44754.490000000093</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4595,11 +4649,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>104847.86999999995</v>
+        <v>109645.46999999996</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>62152.130000000048</v>
+        <v>57354.530000000042</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4655,11 +4709,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>169078.53999999989</v>
+        <v>172110.57999999987</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>90921.460000000108</v>
+        <v>87889.420000000129</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4715,11 +4769,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>56833.890000000094</v>
+        <v>58108.070000000094</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>43166.109999999906</v>
+        <v>41891.929999999906</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4732,11 +4786,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>700067.9900000022</v>
+        <v>700067.99000000232</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>-48817.990000002203</v>
+        <v>-48817.990000002319</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4755,11 +4809,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>90.272727272727252</v>
+        <v>73.272727272727252</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4792,11 +4846,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>347699.70500000124</v>
+        <v>378617.83500000124</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>303550.29499999876</v>
+        <v>272632.16499999876</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4835,11 +4889,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51586.549999999988</v>
+        <v>51586.549999999996</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>21413.450000000012</v>
+        <v>21413.450000000004</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5103,11 +5157,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>506985.30500000098</v>
+        <v>559592.43500000192</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>144264.69499999902</v>
+        <v>91657.564999998081</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 11:36
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A812A6F6-50CE-49B7-BA3C-A13441478DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E186EB74-E1E8-447C-B244-D89B7323B36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>253523.69999999958</v>
+            <v>255196.99999999956</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>3401.8400000000006</v>
+            <v>5075.1400000000003</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1781,13 +1781,13 @@
             <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F8">
-            <v>151.09</v>
+            <v>4733.2199999999993</v>
           </cell>
           <cell r="H8" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>1218.9000000000001</v>
+            <v>1582.6</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -1821,7 +1821,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>171718.08999999985</v>
+            <v>172081.78999999986</v>
           </cell>
           <cell r="H10" t="str">
             <v>KEY SP</v>
@@ -1867,7 +1867,7 @@
             <v>LESTE</v>
           </cell>
           <cell r="I12">
-            <v>3049.08</v>
+            <v>3369.5499999999997</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
@@ -1881,13 +1881,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>263985.40000000084</v>
+            <v>262775.00000000081</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I13">
-            <v>4393.3999999999996</v>
+            <v>6579.7000000000007</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
@@ -1901,13 +1901,13 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>516869.3000000001</v>
+            <v>518079.70000000013</v>
           </cell>
           <cell r="H14" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I14">
-            <v>2026.69</v>
+            <v>2531.9900000000002</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
@@ -1927,7 +1927,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I15">
-            <v>1089.3000000000002</v>
+            <v>2119.7999999999997</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
@@ -1947,7 +1947,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="I16">
-            <v>2802.23</v>
+            <v>3106.9800000000005</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -1967,13 +1967,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="I17">
-            <v>1391.6</v>
+            <v>1671.3999999999999</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N17">
-            <v>25</v>
+            <v>26</v>
           </cell>
         </row>
         <row r="18">
@@ -2001,19 +2001,19 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>71969.509999999995</v>
+            <v>72289.98</v>
           </cell>
           <cell r="H19" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I19">
-            <v>944.40000000000009</v>
+            <v>1555.4</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>350</v>
+            <v>351</v>
           </cell>
         </row>
         <row r="20">
@@ -2021,13 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>128777.36499999973</v>
+            <v>126381.53499999977</v>
           </cell>
           <cell r="H20" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I20">
-            <v>4797.5999999999995</v>
+            <v>6084.99</v>
           </cell>
         </row>
         <row r="21">
@@ -2035,13 +2035,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>92057.190000000046</v>
+            <v>92562.490000000049</v>
           </cell>
           <cell r="H21" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I21">
-            <v>3032.0400000000004</v>
+            <v>10282.75</v>
           </cell>
         </row>
         <row r="22">
@@ -2049,7 +2049,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>82797.879999999874</v>
+            <v>83828.379999999845</v>
           </cell>
           <cell r="H22" t="str">
             <v>SJC</v>
@@ -2063,13 +2063,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>48392.130000000092</v>
+            <v>48696.880000000092</v>
           </cell>
           <cell r="H23" t="str">
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I23">
-            <v>75</v>
+            <v>695.4</v>
           </cell>
         </row>
         <row r="24">
@@ -2077,13 +2077,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>157312.70999999982</v>
+            <v>157592.50999999983</v>
           </cell>
           <cell r="H24" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I24">
-            <v>62395.67</v>
+            <v>78829.290000000008</v>
           </cell>
         </row>
         <row r="25">
@@ -2099,7 +2099,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>89745.509999999907</v>
+            <v>90356.509999999907</v>
           </cell>
         </row>
         <row r="27">
@@ -2107,7 +2107,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>109645.46999999996</v>
+            <v>110932.85999999996</v>
           </cell>
         </row>
         <row r="28">
@@ -2115,7 +2115,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>172110.57999999987</v>
+            <v>179361.28999999983</v>
           </cell>
         </row>
         <row r="29">
@@ -2139,7 +2139,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>51586.549999999996</v>
+            <v>52206.95</v>
           </cell>
         </row>
         <row r="32">
@@ -2147,7 +2147,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>3601341.4049999751</v>
+            <v>3617775.0249999752</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>3601341.4049999989</v>
+        <v>3617775.0249999994</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>40706.670000000006</v>
+        <v>57140.29</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3043,7 +3043,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1991158.5950000011</v>
+        <v>1974724.9750000006</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>109293.32999999999</v>
+        <v>92859.709999999992</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.64395912472060779</v>
+        <v>0.64689763522574872</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.27137780000000011</v>
+        <v>0.38093526666666677</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.46174142480211078</v>
+        <v>0.46306068601583117</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3294,11 +3294,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>253523.69999999958</v>
+        <v>255196.99999999956</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>71476.300000000425</v>
+        <v>69803.000000000437</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3313,11 +3313,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1391.6</v>
+        <v>1671.3999999999999</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10568.4</v>
+        <v>10288.6</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3370,11 +3370,11 @@
       </c>
       <c r="D12" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>151.09</v>
+        <v>4733.2199999999993</v>
       </c>
       <c r="E12" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>848.91</v>
+        <v>-3733.2199999999993</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="21" t="s">
@@ -3389,11 +3389,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>944.40000000000009</v>
+        <v>1555.4</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8165.6</v>
+        <v>7554.6</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3466,11 +3466,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3032.0400000000004</v>
+        <v>10282.75</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11967.96</v>
+        <v>4717.25</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3524,11 +3524,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>171718.08999999985</v>
+        <v>172081.78999999986</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>101281.91000000015</v>
+        <v>100918.21000000014</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3543,11 +3543,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1089.3000000000002</v>
+        <v>2119.7999999999997</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3190.7</v>
+        <v>2160.2000000000003</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3620,11 +3620,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3401.8400000000006</v>
+        <v>5075.1400000000003</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11598.16</v>
+        <v>9924.86</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3697,11 +3697,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4797.5999999999995</v>
+        <v>6084.99</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8672.4000000000015</v>
+        <v>7385.01</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>263985.40000000084</v>
+        <v>262775.00000000081</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-93985.400000000838</v>
+        <v>-92775.000000000815</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3774,11 +3774,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2802.23</v>
+        <v>3106.9800000000005</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-272.23</v>
+        <v>-576.98000000000047</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3832,11 +3832,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>516869.3000000001</v>
+        <v>518079.70000000013</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>433130.6999999999</v>
+        <v>431920.29999999987</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3851,11 +3851,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3049.08</v>
+        <v>3369.5499999999997</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3790.92</v>
+        <v>3470.4500000000003</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3915,11 +3915,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4393.3999999999996</v>
+        <v>6579.7000000000007</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6516.6</v>
+        <v>4330.2999999999993</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3975,11 +3975,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1218.9000000000001</v>
+        <v>1582.6</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11781.1</v>
+        <v>11417.4</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4103,11 +4103,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>71969.509999999995</v>
+        <v>72289.98</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50030.490000000005</v>
+        <v>49710.020000000004</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4122,11 +4122,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2026.69</v>
+        <v>2531.9900000000002</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5323.3099999999995</v>
+        <v>4818.01</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4158,11 +4158,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4178,11 +4178,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>128777.36499999973</v>
+        <v>126381.53499999977</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>66222.635000000271</v>
+        <v>68618.465000000229</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>92057.190000000046</v>
+        <v>92562.490000000049</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>47942.809999999954</v>
+        <v>47437.509999999951</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4272,11 +4272,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>75</v>
+        <v>695.4</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3465</v>
+        <v>2844.6</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4328,11 +4328,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>82797.879999999874</v>
+        <v>83828.379999999845</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>59702.120000000126</v>
+        <v>58671.620000000155</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4403,11 +4403,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>48392.130000000092</v>
+        <v>48696.880000000092</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41607.869999999908</v>
+        <v>41303.119999999908</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4467,11 +4467,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>157312.70999999982</v>
+        <v>157592.50999999983</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>80187.290000000183</v>
+        <v>79907.490000000165</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4592,11 +4592,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>89745.509999999907</v>
+        <v>90356.509999999907</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>44754.490000000093</v>
+        <v>44143.490000000093</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4649,11 +4649,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>109645.46999999996</v>
+        <v>110932.85999999996</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>57354.530000000042</v>
+        <v>56067.140000000043</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4666,11 +4666,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>270334.04000000004</v>
+        <v>265751.90999999992</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>120415.95999999996</v>
+        <v>124998.09000000008</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4709,11 +4709,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>172110.57999999987</v>
+        <v>179361.28999999983</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>87889.420000000129</v>
+        <v>80638.710000000166</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4786,11 +4786,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>700067.99000000232</v>
+        <v>700067.9900000022</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>-48817.990000002319</v>
+        <v>-48817.990000002203</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4809,11 +4809,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>73.272727272727252</v>
+        <v>70.272727272727252</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4846,11 +4846,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>378617.83500000124</v>
+        <v>395051.4550000013</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>272632.16499999876</v>
+        <v>256198.5449999987</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4889,11 +4889,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51586.549999999996</v>
+        <v>52206.95</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>21413.450000000004</v>
+        <v>20793.050000000003</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5157,11 +5157,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>559592.43500000192</v>
+        <v>576026.05500000238</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>91657.564999998081</v>
+        <v>75223.94499999762</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 12:08
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E186EB74-E1E8-447C-B244-D89B7323B36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90367404-D61C-4999-BDB8-67BAE3132CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>255196.99999999956</v>
+            <v>257828.3999999995</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>5075.1400000000003</v>
+            <v>7706.54</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1781,19 +1781,19 @@
             <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F8">
-            <v>4733.2199999999993</v>
+            <v>151.09</v>
           </cell>
           <cell r="H8" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>1582.6</v>
+            <v>3277.1499999999996</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N8">
-            <v>40</v>
+            <v>41</v>
           </cell>
         </row>
         <row r="9">
@@ -1801,13 +1801,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>50911.409999999996</v>
+            <v>50911.409999999989</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>2111</v>
+            <v>2894.05</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
@@ -1821,7 +1821,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>172081.78999999986</v>
+            <v>173776.33999999985</v>
           </cell>
           <cell r="H10" t="str">
             <v>KEY SP</v>
@@ -1841,7 +1841,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>50497.230000000061</v>
+            <v>51280.280000000064</v>
           </cell>
           <cell r="H11" t="str">
             <v>KEY ZL</v>
@@ -1881,13 +1881,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>262775.00000000081</v>
+            <v>263985.40000000084</v>
           </cell>
           <cell r="H13" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I13">
-            <v>6579.7000000000007</v>
+            <v>7110.35</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
@@ -1901,7 +1901,7 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>518079.70000000013</v>
+            <v>516869.3000000001</v>
           </cell>
           <cell r="H14" t="str">
             <v>LESTE PENHA</v>
@@ -1961,7 +1961,7 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>264953.34999999998</v>
+            <v>264953.35000000003</v>
           </cell>
           <cell r="H17" t="str">
             <v>NORTE</v>
@@ -2013,7 +2013,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>351</v>
+            <v>352</v>
           </cell>
         </row>
         <row r="20">
@@ -2021,13 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>126381.53499999977</v>
+            <v>131494.31499999971</v>
           </cell>
           <cell r="H20" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I20">
-            <v>6084.99</v>
+            <v>8505.1899999999987</v>
           </cell>
         </row>
         <row r="21">
@@ -2069,7 +2069,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I23">
-            <v>695.4</v>
+            <v>1031.8499999999999</v>
           </cell>
         </row>
         <row r="24">
@@ -2083,7 +2083,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="I24">
-            <v>78829.290000000008</v>
+            <v>87225.590000000011</v>
           </cell>
         </row>
         <row r="25">
@@ -2107,7 +2107,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>110932.85999999996</v>
+            <v>113353.05999999997</v>
           </cell>
         </row>
         <row r="28">
@@ -2139,7 +2139,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>52206.95</v>
+            <v>52543.399999999994</v>
           </cell>
         </row>
         <row r="32">
@@ -2147,7 +2147,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>3617775.0249999752</v>
+            <v>3626171.324999975</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>3617775.0249999994</v>
+        <v>3626171.3249999997</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>57140.29</v>
+        <v>65536.59</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3043,7 +3043,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1974724.9750000006</v>
+        <v>1966328.6750000003</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>92859.709999999992</v>
+        <v>84463.41</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.64689763522574872</v>
+        <v>0.64839898524810002</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.38093526666666677</v>
+        <v>0.43691059999999993</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.46306068601583117</v>
+        <v>0.46437994722955145</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3294,11 +3294,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>255196.99999999956</v>
+        <v>257828.3999999995</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>69803.000000000437</v>
+        <v>67171.600000000501</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3351,11 +3351,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3370,11 +3370,11 @@
       </c>
       <c r="D12" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>4733.2199999999993</v>
+        <v>151.09</v>
       </c>
       <c r="E12" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-3733.2199999999993</v>
+        <v>848.91</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="21" t="s">
@@ -3447,11 +3447,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>50911.409999999996</v>
+        <v>50911.409999999989</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>39088.590000000004</v>
+        <v>39088.590000000011</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3524,11 +3524,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>172081.78999999986</v>
+        <v>173776.33999999985</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>100918.21000000014</v>
+        <v>99223.660000000149</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3601,11 +3601,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>50497.230000000061</v>
+        <v>51280.280000000064</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>27502.769999999939</v>
+        <v>26719.719999999936</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3620,11 +3620,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5075.1400000000003</v>
+        <v>7706.54</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9924.86</v>
+        <v>7293.46</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3697,11 +3697,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6084.99</v>
+        <v>8505.1899999999987</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7385.01</v>
+        <v>4964.8100000000013</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>262775.00000000081</v>
+        <v>263985.40000000084</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-92775.000000000815</v>
+        <v>-93985.400000000838</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3832,11 +3832,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>518079.70000000013</v>
+        <v>516869.3000000001</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>431920.29999999987</v>
+        <v>433130.6999999999</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3915,11 +3915,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6579.7000000000007</v>
+        <v>7110.35</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4330.2999999999993</v>
+        <v>3799.6499999999996</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3956,11 +3956,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>264953.34999999998</v>
+        <v>264953.35000000003</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>295046.65000000002</v>
+        <v>295046.64999999997</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3975,11 +3975,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1582.6</v>
+        <v>3277.1499999999996</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11417.4</v>
+        <v>9722.85</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4047,11 +4047,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2111</v>
+        <v>2894.05</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3379</v>
+        <v>2595.9499999999998</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4139,11 +4139,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>563167.95000000019</v>
+        <v>563167.95000000042</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-67713.404545454716</v>
+        <v>-67713.404545454949</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4178,11 +4178,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>126381.53499999977</v>
+        <v>131494.31499999971</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>68618.465000000229</v>
+        <v>63505.685000000289</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4272,11 +4272,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>695.4</v>
+        <v>1031.8499999999999</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2844.6</v>
+        <v>2508.15</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4649,11 +4649,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>110932.85999999996</v>
+        <v>113353.05999999997</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>56067.140000000043</v>
+        <v>53646.940000000031</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4666,11 +4666,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>265751.90999999992</v>
+        <v>270334.04000000004</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>124998.09000000008</v>
+        <v>120415.95999999996</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4809,11 +4809,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>70.272727272727252</v>
+        <v>66.272727272727252</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4846,11 +4846,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>395051.4550000013</v>
+        <v>403447.7550000014</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>256198.5449999987</v>
+        <v>247802.2449999986</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4889,11 +4889,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52206.95</v>
+        <v>52543.399999999994</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>20793.050000000003</v>
+        <v>20456.600000000006</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5157,11 +5157,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>576026.05500000238</v>
+        <v>584422.35500000231</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>75223.94499999762</v>
+        <v>66827.64499999769</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 13:26
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90367404-D61C-4999-BDB8-67BAE3132CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF65049-B623-490E-BCD3-50F82B622B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>257828.3999999995</v>
+            <v>258498.57999999952</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>7706.54</v>
+            <v>8376.7199999999993</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1767,7 +1767,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>1865.2</v>
+            <v>2152</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1801,13 +1801,13 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>50911.409999999989</v>
+            <v>51198.209999999992</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>2894.05</v>
+            <v>3373.65</v>
           </cell>
           <cell r="K9" t="str">
             <v>INDAIATUBA</v>
@@ -1821,19 +1821,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>173776.33999999985</v>
+            <v>173776.33999999988</v>
           </cell>
           <cell r="H10" t="str">
-            <v>KEY SP</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="I10">
-            <v>1755.6</v>
+            <v>201849.3</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N10">
-            <v>18</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="11">
@@ -1841,13 +1841,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>51280.280000000064</v>
+            <v>51759.880000000063</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I11">
-            <v>19933.399999999991</v>
+            <v>3715.6000000000004</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
@@ -1864,10 +1864,10 @@
             <v>209220.31999999995</v>
           </cell>
           <cell r="H12" t="str">
-            <v>LESTE</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I12">
-            <v>3369.5499999999997</v>
+            <v>19933.399999999991</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
@@ -1884,16 +1884,16 @@
             <v>263985.40000000084</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I13">
-            <v>7110.35</v>
+            <v>3369.5499999999997</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N13">
-            <v>34</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="14">
@@ -1901,13 +1901,13 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>516869.3000000001</v>
+            <v>718718.60000000021</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I14">
-            <v>2531.9900000000002</v>
+            <v>8547</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
@@ -1924,10 +1924,10 @@
             <v>87483.259999999951</v>
           </cell>
           <cell r="H15" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I15">
-            <v>2119.7999999999997</v>
+            <v>3880.9900000000007</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
@@ -1944,10 +1944,10 @@
             <v>90046.200000000041</v>
           </cell>
           <cell r="H16" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I16">
-            <v>3106.9800000000005</v>
+            <v>2704.6000000000004</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -1961,13 +1961,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>264953.35000000003</v>
+            <v>266913.34999999992</v>
           </cell>
           <cell r="H17" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I17">
-            <v>1671.3999999999999</v>
+            <v>3106.9800000000005</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
@@ -1984,10 +1984,10 @@
             <v>278371.99999999994</v>
           </cell>
           <cell r="H18" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I18">
-            <v>3163.2</v>
+            <v>4877.2700000000004</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -2004,16 +2004,16 @@
             <v>72289.98</v>
           </cell>
           <cell r="H19" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I19">
-            <v>1555.4</v>
+            <v>7032.4399999999987</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>352</v>
+            <v>354</v>
           </cell>
         </row>
         <row r="20">
@@ -2021,13 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>131494.31499999971</v>
+            <v>132930.96499999968</v>
           </cell>
           <cell r="H20" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I20">
-            <v>8505.1899999999987</v>
+            <v>3180.72</v>
           </cell>
         </row>
         <row r="21">
@@ -2035,13 +2035,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>92562.490000000049</v>
+            <v>93911.490000000063</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I21">
-            <v>10282.75</v>
+            <v>8505.1899999999987</v>
           </cell>
         </row>
         <row r="22">
@@ -2049,13 +2049,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>83828.379999999845</v>
+            <v>84413.179999999847</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I22">
-            <v>2083.1800000000003</v>
+            <v>10282.75</v>
           </cell>
         </row>
         <row r="23">
@@ -2066,10 +2066,10 @@
             <v>48696.880000000092</v>
           </cell>
           <cell r="H23" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC</v>
           </cell>
           <cell r="I23">
-            <v>1031.8499999999999</v>
+            <v>2083.1800000000003</v>
           </cell>
         </row>
         <row r="24">
@@ -2077,13 +2077,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>157592.50999999983</v>
+            <v>160798.37999999977</v>
           </cell>
           <cell r="H24" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I24">
-            <v>87225.590000000011</v>
+            <v>1031.8499999999999</v>
           </cell>
         </row>
         <row r="25">
@@ -2091,7 +2091,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>231932.30999999968</v>
+            <v>235801.54999999964</v>
+          </cell>
+          <cell r="H25" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I25">
+            <v>304542.34999999992</v>
           </cell>
         </row>
         <row r="26">
@@ -2099,7 +2105,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>90356.509999999907</v>
+            <v>91981.829999999944</v>
           </cell>
         </row>
         <row r="27">
@@ -2139,7 +2145,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>52543.399999999994</v>
+            <v>52543.4</v>
           </cell>
         </row>
         <row r="32">
@@ -2147,7 +2153,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>3626171.324999975</v>
+            <v>3843488.0849999674</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2998,7 +3004,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>3626171.3249999997</v>
+        <v>3843488.085</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3009,7 +3015,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>65536.59</v>
+        <v>79044.05</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3020,7 +3026,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>21688.999999999989</v>
+        <v>225498.3</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3031,7 +3037,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3043,7 +3049,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1966328.6750000003</v>
+        <v>1749011.915</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3054,7 +3060,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>84463.41</v>
+        <v>70955.95</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3065,7 +3071,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-21688.999999999989</v>
+        <v>-225498.3</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3076,7 +3082,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3088,7 +3094,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.64839898524810002</v>
+        <v>0.68725759231113104</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3099,7 +3105,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.43691059999999993</v>
+        <v>0.52696033333333336</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3121,7 +3127,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.46437994722955145</v>
+        <v>0.46701846965699212</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3239,11 +3245,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3163.2</v>
+        <v>7032.4399999999987</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>13836.8</v>
+        <v>9967.5600000000013</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3294,11 +3300,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>257828.3999999995</v>
+        <v>258498.57999999952</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>67171.600000000501</v>
+        <v>66501.420000000478</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3313,11 +3319,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1671.3999999999999</v>
+        <v>4877.2700000000004</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10288.6</v>
+        <v>7082.73</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3389,11 +3395,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1555.4</v>
+        <v>3180.72</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7554.6</v>
+        <v>5929.2800000000007</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3447,11 +3453,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>50911.409999999989</v>
+        <v>51198.209999999992</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>39088.590000000011</v>
+        <v>38801.790000000008</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3524,11 +3530,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>173776.33999999985</v>
+        <v>173776.33999999988</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>99223.660000000149</v>
+        <v>99223.66000000012</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3543,11 +3549,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2119.7999999999997</v>
+        <v>2704.6000000000004</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2160.2000000000003</v>
+        <v>1575.3999999999996</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3562,11 +3568,11 @@
       </c>
       <c r="P14" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>201849.3</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-201849.3</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="19" t="s">
@@ -3581,11 +3587,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3601,11 +3607,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51280.280000000064</v>
+        <v>51759.880000000063</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>26719.719999999936</v>
+        <v>26240.119999999937</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3620,11 +3626,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7706.54</v>
+        <v>8376.7199999999993</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7293.46</v>
+        <v>6623.2800000000007</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3639,11 +3645,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1755.6</v>
+        <v>3715.6000000000004</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-1755.6</v>
+        <v>-3715.6000000000004</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3832,11 +3838,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>516869.3000000001</v>
+        <v>718718.60000000021</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>433130.6999999999</v>
+        <v>231281.39999999979</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3915,11 +3921,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7110.35</v>
+        <v>8547</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3799.6499999999996</v>
+        <v>2363</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3956,11 +3962,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>264953.35000000003</v>
+        <v>266913.34999999992</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>295046.64999999997</v>
+        <v>293086.65000000008</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -4047,11 +4053,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2894.05</v>
+        <v>3373.65</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2595.9499999999998</v>
+        <v>2116.35</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4122,11 +4128,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2531.9900000000002</v>
+        <v>3880.9900000000007</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4818.01</v>
+        <v>3469.0099999999993</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4178,11 +4184,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>131494.31499999971</v>
+        <v>132930.96499999968</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>63505.685000000289</v>
+        <v>62069.035000000324</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4197,11 +4203,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1865.2</v>
+        <v>2152</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3424.8</v>
+        <v>3138</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4253,11 +4259,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>92562.490000000049</v>
+        <v>93911.490000000063</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>47437.509999999951</v>
+        <v>46088.509999999937</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4289,11 +4295,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>180720.71000000008</v>
+        <v>384530.01</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>438597.4718181818</v>
+        <v>234788.17181818187</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4328,11 +4334,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>83828.379999999845</v>
+        <v>84413.179999999847</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>58671.620000000155</v>
+        <v>58086.820000000153</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4383,11 +4389,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4467,11 +4473,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>157592.50999999983</v>
+        <v>160798.37999999977</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>79907.490000000165</v>
+        <v>76701.620000000228</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4513,11 +4519,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>231932.30999999968</v>
+        <v>235801.54999999964</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>86567.690000000322</v>
+        <v>82698.450000000361</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4592,11 +4598,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>90356.509999999907</v>
+        <v>91981.829999999944</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>44143.490000000093</v>
+        <v>42518.170000000056</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4809,11 +4815,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>66.272727272727252</v>
+        <v>62.272727272727252</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4846,11 +4852,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>403447.7550000014</v>
+        <v>416955.21500000142</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>247802.2449999986</v>
+        <v>234294.78499999858</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4889,11 +4895,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52543.399999999994</v>
+        <v>52543.4</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>20456.600000000006</v>
+        <v>20456.599999999999</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5157,11 +5163,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>584422.35500000231</v>
+        <v>801739.1150000015</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>66827.64499999769</v>
+        <v>-150489.1150000015</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 14:26
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF65049-B623-490E-BCD3-50F82B622B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29265D4B-486E-4B17-AFE5-F63E9223CAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1730,13 +1730,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>38432.729999999974</v>
+            <v>39246.379999999976</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>3262.0099999999998</v>
+            <v>4075.6599999999994</v>
           </cell>
         </row>
         <row r="6">
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>258498.57999999952</v>
+            <v>260146.47999999952</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>8376.7199999999993</v>
+            <v>10024.619999999999</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1787,7 +1787,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>3277.1499999999996</v>
+            <v>4951.3</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
@@ -1821,13 +1821,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>173776.33999999988</v>
+            <v>175450.48999999985</v>
           </cell>
           <cell r="H10" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>201849.3</v>
+            <v>2409.6999999999998</v>
           </cell>
           <cell r="K10" t="str">
             <v>JUNDIAI</v>
@@ -1844,10 +1844,10 @@
             <v>51759.880000000063</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY SP</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="I11">
-            <v>3715.6000000000004</v>
+            <v>334524.09999999998</v>
           </cell>
           <cell r="K11" t="str">
             <v>LESTE</v>
@@ -1861,13 +1861,13 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>209220.31999999995</v>
+            <v>211630.01999999996</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="I12">
-            <v>19933.399999999991</v>
+            <v>20600.599999999999</v>
           </cell>
           <cell r="K12" t="str">
             <v>LESTE PENHA</v>
@@ -1884,10 +1884,10 @@
             <v>263985.40000000084</v>
           </cell>
           <cell r="H13" t="str">
-            <v>LESTE</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I13">
-            <v>3369.5499999999997</v>
+            <v>3715.6000000000004</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE TATUAPE</v>
@@ -1901,19 +1901,19 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>718718.60000000021</v>
+            <v>851393.40000000026</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE MOOCA</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I14">
-            <v>8547</v>
+            <v>19933.399999999991</v>
           </cell>
           <cell r="K14" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N14">
-            <v>39</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="15">
@@ -1924,10 +1924,10 @@
             <v>87483.259999999951</v>
           </cell>
           <cell r="H15" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I15">
-            <v>3880.9900000000007</v>
+            <v>3369.5499999999997</v>
           </cell>
           <cell r="K15" t="str">
             <v>OSASCO</v>
@@ -1941,13 +1941,13 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>90046.200000000041</v>
+            <v>110646.80000000005</v>
           </cell>
           <cell r="H16" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I16">
-            <v>2704.6000000000004</v>
+            <v>9469.7999999999975</v>
           </cell>
           <cell r="K16" t="str">
             <v>PIRITUBA</v>
@@ -1964,10 +1964,10 @@
             <v>266913.34999999992</v>
           </cell>
           <cell r="H17" t="str">
-            <v>MOGI</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I17">
-            <v>3106.9800000000005</v>
+            <v>6244.4900000000007</v>
           </cell>
           <cell r="K17" t="str">
             <v>SANTO ANDRE</v>
@@ -1984,10 +1984,10 @@
             <v>278371.99999999994</v>
           </cell>
           <cell r="H18" t="str">
-            <v>NORTE</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I18">
-            <v>4877.2700000000004</v>
+            <v>2844.5000000000005</v>
           </cell>
           <cell r="K18" t="str">
             <v>SJC</v>
@@ -2004,16 +2004,16 @@
             <v>72289.98</v>
           </cell>
           <cell r="H19" t="str">
-            <v>OSASCO</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I19">
-            <v>7032.4399999999987</v>
+            <v>3561.78</v>
           </cell>
           <cell r="K19" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N19">
-            <v>354</v>
+            <v>355</v>
           </cell>
         </row>
         <row r="20">
@@ -2021,13 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>132930.96499999968</v>
+            <v>133853.76499999966</v>
           </cell>
           <cell r="H20" t="str">
-            <v>PIRITUBA</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I20">
-            <v>3180.72</v>
+            <v>6785.7699999999995</v>
           </cell>
         </row>
         <row r="21">
@@ -2035,13 +2035,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>93911.490000000063</v>
+            <v>96274.990000000063</v>
           </cell>
           <cell r="H21" t="str">
-            <v>SANTO ANDRE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I21">
-            <v>8505.1899999999987</v>
+            <v>7423.8599999999988</v>
           </cell>
         </row>
         <row r="22">
@@ -2049,13 +2049,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>84413.179999999847</v>
+            <v>84553.079999999842</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SBC</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I22">
-            <v>10282.75</v>
+            <v>3907.3199999999997</v>
           </cell>
         </row>
         <row r="23">
@@ -2063,13 +2063,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>48696.880000000092</v>
+            <v>49151.680000000095</v>
           </cell>
           <cell r="H23" t="str">
-            <v>SJC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I23">
-            <v>2083.1800000000003</v>
+            <v>10826.189999999999</v>
           </cell>
         </row>
         <row r="24">
@@ -2077,13 +2077,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>160798.37999999977</v>
+            <v>162706.87999999977</v>
           </cell>
           <cell r="H24" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SBC</v>
           </cell>
           <cell r="I24">
-            <v>1031.8499999999999</v>
+            <v>10432.15</v>
           </cell>
         </row>
         <row r="25">
@@ -2091,13 +2091,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>235801.54999999964</v>
+            <v>236192.96999999977</v>
           </cell>
           <cell r="H25" t="str">
-            <v>Total Geral</v>
+            <v>SJC</v>
           </cell>
           <cell r="I25">
-            <v>304542.34999999992</v>
+            <v>2312.58</v>
           </cell>
         </row>
         <row r="26">
@@ -2105,7 +2105,13 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>91981.829999999944</v>
+            <v>92708.429999999935</v>
+          </cell>
+          <cell r="H26" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I26">
+            <v>1031.8499999999999</v>
           </cell>
         </row>
         <row r="27">
@@ -2113,7 +2119,13 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>113353.05999999997</v>
+            <v>115674.05999999995</v>
+          </cell>
+          <cell r="H27" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I27">
+            <v>473970.4700000002</v>
           </cell>
         </row>
         <row r="28">
@@ -2121,7 +2133,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>179361.28999999983</v>
+            <v>179510.68999999983</v>
           </cell>
         </row>
         <row r="29">
@@ -2129,7 +2141,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>58108.070000000094</v>
+            <v>58337.470000000103</v>
           </cell>
         </row>
         <row r="30">
@@ -2145,7 +2157,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>52543.4</v>
+            <v>52543.400000000009</v>
           </cell>
         </row>
         <row r="32">
@@ -2153,7 +2165,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>3843488.0849999674</v>
+            <v>4012916.2049999516</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3004,7 +3016,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>3843488.085</v>
+        <v>4012916.2050000005</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3015,7 +3027,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>79044.05</v>
+        <v>92787.070000000022</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3026,7 +3038,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>225498.3</v>
+        <v>381183.39999999991</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3037,7 +3049,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3049,7 +3061,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1749011.915</v>
+        <v>1579583.7949999995</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3060,7 +3072,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>70955.95</v>
+        <v>57212.929999999978</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3071,7 +3083,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-225498.3</v>
+        <v>-381183.39999999991</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3082,7 +3094,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3094,7 +3106,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.68725759231113104</v>
+        <v>0.71755318819848024</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3105,7 +3117,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.52696033333333336</v>
+        <v>0.61858046666666677</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3127,7 +3139,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.46701846965699212</v>
+        <v>0.4683377308707124</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3226,11 +3238,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>38432.729999999974</v>
+        <v>39246.379999999976</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>26067.270000000026</v>
+        <v>25253.620000000024</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3245,11 +3257,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7032.4399999999987</v>
+        <v>7423.8599999999988</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9967.5600000000013</v>
+        <v>9576.1400000000012</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3300,11 +3312,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>258498.57999999952</v>
+        <v>260146.47999999952</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>66501.420000000478</v>
+        <v>64853.520000000484</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3319,11 +3331,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4877.2700000000004</v>
+        <v>6785.7699999999995</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7082.73</v>
+        <v>5174.2300000000005</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3338,11 +3350,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>2409.6999999999998</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>0</v>
+        <v>-2409.6999999999998</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3395,11 +3407,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3180.72</v>
+        <v>3907.3199999999997</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5929.2800000000007</v>
+        <v>5202.68</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3472,11 +3484,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10282.75</v>
+        <v>10432.15</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4717.25</v>
+        <v>4567.8500000000004</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3530,11 +3542,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>173776.33999999988</v>
+        <v>175450.48999999985</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>99223.66000000012</v>
+        <v>97549.510000000155</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3549,11 +3561,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2704.6000000000004</v>
+        <v>2844.5000000000005</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1575.3999999999996</v>
+        <v>1435.4999999999995</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3568,11 +3580,11 @@
       </c>
       <c r="P14" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>201849.3</v>
+        <v>334524.09999999998</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" si="1"/>
-        <v>-201849.3</v>
+        <v>-334524.09999999998</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="19" t="s">
@@ -3626,11 +3638,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8376.7199999999993</v>
+        <v>10024.619999999999</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6623.2800000000007</v>
+        <v>4975.380000000001</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3684,11 +3696,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>209220.31999999995</v>
+        <v>211630.01999999996</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>115779.68000000005</v>
+        <v>113369.98000000004</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3703,11 +3715,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8505.1899999999987</v>
+        <v>10826.189999999999</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4964.8100000000013</v>
+        <v>2643.8100000000013</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3722,11 +3734,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>20600.599999999999</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-20600.599999999999</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3780,11 +3792,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3106.9800000000005</v>
+        <v>3561.78</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-576.98000000000047</v>
+        <v>-1031.7800000000002</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3838,11 +3850,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>718718.60000000021</v>
+        <v>851393.40000000026</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>231281.39999999979</v>
+        <v>98606.599999999744</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3882,11 +3894,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3902,11 +3914,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>90046.200000000041</v>
+        <v>110646.80000000005</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>39953.799999999959</v>
+        <v>19353.199999999953</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3921,11 +3933,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8547</v>
+        <v>9469.7999999999975</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2363</v>
+        <v>1440.2000000000025</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3981,11 +3993,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3277.1499999999996</v>
+        <v>4951.3</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9722.85</v>
+        <v>8048.7</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4128,11 +4140,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3880.9900000000007</v>
+        <v>6244.4900000000007</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3469.0099999999993</v>
+        <v>1105.5099999999993</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4184,11 +4196,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>132930.96499999968</v>
+        <v>133853.76499999966</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>62069.035000000324</v>
+        <v>61146.235000000335</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4259,11 +4271,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>93911.490000000063</v>
+        <v>96274.990000000063</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>46088.509999999937</v>
+        <v>43725.009999999937</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4295,11 +4307,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>384530.01</v>
+        <v>540215.10999999964</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>234788.17181818187</v>
+        <v>79103.071818182245</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4334,11 +4346,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>84413.179999999847</v>
+        <v>84553.079999999842</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>58086.820000000153</v>
+        <v>57946.920000000158</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4353,11 +4365,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2083.1800000000003</v>
+        <v>2312.58</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1816.8199999999997</v>
+        <v>1587.42</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4409,11 +4421,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>48696.880000000092</v>
+        <v>49151.680000000095</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41303.119999999908</v>
+        <v>40848.319999999905</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4473,11 +4485,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>160798.37999999977</v>
+        <v>162706.87999999977</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>76701.620000000228</v>
+        <v>74793.120000000228</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4492,11 +4504,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3262.0099999999998</v>
+        <v>4075.6599999999994</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-712.00999999999976</v>
+        <v>-1525.6599999999994</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4519,11 +4531,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>235801.54999999964</v>
+        <v>236192.96999999977</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>82698.450000000361</v>
+        <v>82307.030000000232</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4598,11 +4610,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>91981.829999999944</v>
+        <v>92708.429999999935</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>42518.170000000056</v>
+        <v>41791.570000000065</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4655,11 +4667,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>113353.05999999997</v>
+        <v>115674.05999999995</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>53646.940000000031</v>
+        <v>51325.940000000046</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4715,11 +4727,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>179361.28999999983</v>
+        <v>179510.68999999983</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>80638.710000000166</v>
+        <v>80489.310000000172</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4732,11 +4744,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>540157.7900000033</v>
+        <v>540157.79000000341</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>-19157.790000003297</v>
+        <v>-19157.790000003413</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4775,11 +4787,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>58108.070000000094</v>
+        <v>58337.470000000103</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41891.929999999906</v>
+        <v>41662.529999999897</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4815,11 +4827,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>62.272727272727252</v>
+        <v>60.272727272727252</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4852,11 +4864,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>416955.21500000142</v>
+        <v>430698.23500000173</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>234294.78499999858</v>
+        <v>220551.76499999827</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4895,11 +4907,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52543.4</v>
+        <v>52543.400000000009</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>20456.599999999999</v>
+        <v>20456.599999999991</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5163,11 +5175,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>801739.1150000015</v>
+        <v>971167.23500000197</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-150489.1150000015</v>
+        <v>-319917.23500000197</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 14:52
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29265D4B-486E-4B17-AFE5-F63E9223CAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6295783-5E0F-490A-8880-39A6728FB101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>260146.47999999952</v>
+            <v>260716.2799999995</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>10024.619999999999</v>
+            <v>10594.419999999998</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1787,13 +1787,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>4951.3</v>
+            <v>4951.2999999999993</v>
           </cell>
           <cell r="K8" t="str">
-            <v>CENTRO</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="N8">
-            <v>41</v>
+            <v>23</v>
           </cell>
         </row>
         <row r="9">
@@ -1810,10 +1810,10 @@
             <v>3373.65</v>
           </cell>
           <cell r="K9" t="str">
-            <v>INDAIATUBA</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>32</v>
+            <v>41</v>
           </cell>
         </row>
         <row r="10">
@@ -1830,10 +1830,10 @@
             <v>2409.6999999999998</v>
           </cell>
           <cell r="K10" t="str">
-            <v>JUNDIAI</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>19</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="11">
@@ -1850,10 +1850,10 @@
             <v>334524.09999999998</v>
           </cell>
           <cell r="K11" t="str">
-            <v>LESTE</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>30</v>
+            <v>50</v>
           </cell>
         </row>
         <row r="12">
@@ -1870,10 +1870,10 @@
             <v>20600.599999999999</v>
           </cell>
           <cell r="K12" t="str">
-            <v>LESTE PENHA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="N12">
-            <v>24</v>
+            <v>19</v>
           </cell>
         </row>
         <row r="13">
@@ -1890,10 +1890,10 @@
             <v>3715.6000000000004</v>
           </cell>
           <cell r="K13" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>35</v>
+            <v>30</v>
           </cell>
         </row>
         <row r="14">
@@ -1910,10 +1910,10 @@
             <v>19933.399999999991</v>
           </cell>
           <cell r="K14" t="str">
-            <v>NORTE</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>40</v>
+            <v>48</v>
           </cell>
         </row>
         <row r="15">
@@ -1927,13 +1927,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="I15">
-            <v>3369.5499999999997</v>
+            <v>3541.45</v>
           </cell>
           <cell r="K15" t="str">
-            <v>OSASCO</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="N15">
-            <v>60</v>
+            <v>24</v>
           </cell>
         </row>
         <row r="16">
@@ -1950,10 +1950,10 @@
             <v>9469.7999999999975</v>
           </cell>
           <cell r="K16" t="str">
-            <v>PIRITUBA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>27</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="17">
@@ -1970,10 +1970,10 @@
             <v>6244.4900000000007</v>
           </cell>
           <cell r="K17" t="str">
-            <v>SANTO ANDRE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>26</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="18">
@@ -1990,10 +1990,10 @@
             <v>2844.5000000000005</v>
           </cell>
           <cell r="K18" t="str">
-            <v>SJC</v>
+            <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>21</v>
+            <v>40</v>
           </cell>
         </row>
         <row r="19">
@@ -2001,7 +2001,7 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>72289.98</v>
+            <v>72461.88</v>
           </cell>
           <cell r="H19" t="str">
             <v>MOGI</v>
@@ -2010,10 +2010,10 @@
             <v>3561.78</v>
           </cell>
           <cell r="K19" t="str">
-            <v>Total Geral</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="N19">
-            <v>355</v>
+            <v>60</v>
           </cell>
         </row>
         <row r="20">
@@ -2027,7 +2027,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="I20">
-            <v>6785.7699999999995</v>
+            <v>7244.07</v>
+          </cell>
+          <cell r="K20" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="N20">
+            <v>27</v>
           </cell>
         </row>
         <row r="21">
@@ -2043,6 +2049,12 @@
           <cell r="I21">
             <v>7423.8599999999988</v>
           </cell>
+          <cell r="K21" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="N21">
+            <v>26</v>
+          </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
@@ -2057,6 +2069,12 @@
           <cell r="I22">
             <v>3907.3199999999997</v>
           </cell>
+          <cell r="K22" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="N22">
+            <v>36</v>
+          </cell>
         </row>
         <row r="23">
           <cell r="E23" t="str">
@@ -2071,19 +2089,31 @@
           <cell r="I23">
             <v>10826.189999999999</v>
           </cell>
+          <cell r="K23" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="N23">
+            <v>21</v>
+          </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>162706.87999999977</v>
+            <v>163165.17999999976</v>
           </cell>
           <cell r="H24" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I24">
             <v>10432.15</v>
+          </cell>
+          <cell r="K24" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="N24">
+            <v>23</v>
           </cell>
         </row>
         <row r="25">
@@ -2091,13 +2121,19 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>236192.96999999977</v>
+            <v>236192.96999999959</v>
           </cell>
           <cell r="H25" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I25">
             <v>2312.58</v>
+          </cell>
+          <cell r="K25" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="N25">
+            <v>570</v>
           </cell>
         </row>
         <row r="26">
@@ -2125,7 +2161,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="I27">
-            <v>473970.4700000002</v>
+            <v>475170.47000000032</v>
           </cell>
         </row>
         <row r="28">
@@ -2141,7 +2177,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>58337.470000000103</v>
+            <v>58337.470000000096</v>
           </cell>
         </row>
         <row r="30">
@@ -2165,7 +2201,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4012916.2049999516</v>
+            <v>4014116.2049999516</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3016,7 +3052,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4012916.2050000005</v>
+        <v>4014116.2049999996</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3027,7 +3063,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>92787.070000000022</v>
+        <v>93987.07</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3049,7 +3085,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>355</v>
+        <v>570</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3061,7 +3097,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1579583.7949999995</v>
+        <v>1578383.7950000004</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3072,7 +3108,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>57212.929999999978</v>
+        <v>56012.929999999993</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3094,7 +3130,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>403</v>
+        <v>188</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3106,7 +3142,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.71755318819848024</v>
+        <v>0.71776776128743847</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3117,7 +3153,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.61858046666666677</v>
+        <v>0.62658046666666678</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3139,7 +3175,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.4683377308707124</v>
+        <v>0.75197889182058053</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3292,11 +3328,11 @@
       </c>
       <c r="V10" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="W10" s="19">
         <f>U10-V10</f>
-        <v>36</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -3312,11 +3348,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>260146.47999999952</v>
+        <v>260716.2799999995</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>64853.520000000484</v>
+        <v>64283.720000000496</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3331,11 +3367,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6785.7699999999995</v>
+        <v>7244.07</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5174.2300000000005</v>
+        <v>4715.93</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3522,11 +3558,11 @@
       </c>
       <c r="V13" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="W13" s="19">
         <f t="shared" si="0"/>
-        <v>59</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -3638,11 +3674,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10024.619999999999</v>
+        <v>10594.419999999998</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4975.380000000001</v>
+        <v>4405.5800000000017</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3753,11 +3789,11 @@
       </c>
       <c r="V16" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W16" s="19">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3830,11 +3866,11 @@
       </c>
       <c r="V17" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="W17" s="19">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3869,11 +3905,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3369.5499999999997</v>
+        <v>3541.45</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3470.4500000000003</v>
+        <v>3298.55</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3993,11 +4029,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4951.3</v>
+        <v>4951.2999999999993</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8048.7</v>
+        <v>8048.7000000000007</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4121,11 +4157,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>72289.98</v>
+        <v>72461.88</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>49710.020000000004</v>
+        <v>49538.119999999995</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4251,11 +4287,11 @@
       </c>
       <c r="V23" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="W23" s="19">
         <f t="shared" si="2"/>
-        <v>55</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -4465,11 +4501,11 @@
       </c>
       <c r="V26" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="W26" s="19">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -4485,11 +4521,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>162706.87999999977</v>
+        <v>163165.17999999976</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>74793.120000000228</v>
+        <v>74334.82000000024</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4531,11 +4567,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>236192.96999999977</v>
+        <v>236192.96999999959</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>82307.030000000232</v>
+        <v>82307.030000000406</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4647,11 +4683,11 @@
       </c>
       <c r="V30" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="W30" s="6">
         <f>U30-V30</f>
-        <v>24.36363636363636</v>
+        <v>-15.63636363636364</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
@@ -4707,11 +4743,11 @@
       </c>
       <c r="V31" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>132</v>
+        <v>214</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="3">U31-V31</f>
-        <v>5.818181818181813</v>
+        <v>-76.181818181818187</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4744,11 +4780,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>540157.79000000341</v>
+        <v>540157.7900000033</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>-19157.790000003413</v>
+        <v>-19157.790000003297</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4767,11 +4803,11 @@
       </c>
       <c r="V32" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>189</v>
+        <v>294</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="3"/>
-        <v>-16.727272727272748</v>
+        <v>-121.72727272727275</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -4787,11 +4823,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>58337.470000000103</v>
+        <v>58337.470000000096</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41662.529999999897</v>
+        <v>41662.529999999904</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4827,11 +4863,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>112</v>
+        <v>183</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>60.272727272727252</v>
+        <v>-10.727272727272748</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4864,11 +4900,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>430698.23500000173</v>
+        <v>431898.23500000179</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>220551.76499999827</v>
+        <v>219351.76499999821</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -5103,11 +5139,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1103755.3899999962</v>
+        <v>1103755.3899999959</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="5">C41-D41</f>
-        <v>-582755.38999999617</v>
+        <v>-582755.38999999594</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -5175,11 +5211,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>971167.23500000197</v>
+        <v>972367.23500000208</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-319917.23500000197</v>
+        <v>-321117.23500000208</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 22/07/2026 16:15
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6295783-5E0F-490A-8880-39A6728FB101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D599799-BA6C-46B7-9655-866F7B11587F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1787,7 +1787,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>4951.2999999999993</v>
+            <v>4953.2</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1821,7 +1821,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>175450.48999999985</v>
+            <v>175452.38999999984</v>
           </cell>
           <cell r="H10" t="str">
             <v>KEY ABC</v>
@@ -1864,10 +1864,10 @@
             <v>211630.01999999996</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY SJC</v>
+            <v>KEY PIRACICABA</v>
           </cell>
           <cell r="I12">
-            <v>20600.599999999999</v>
+            <v>5892</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1884,10 +1884,10 @@
             <v>263985.40000000084</v>
           </cell>
           <cell r="H13" t="str">
-            <v>KEY SP</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="I13">
-            <v>3715.6000000000004</v>
+            <v>22599.599999999999</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1904,10 +1904,10 @@
             <v>851393.40000000026</v>
           </cell>
           <cell r="H14" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I14">
-            <v>19933.399999999991</v>
+            <v>4033.8200000000006</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1924,10 +1924,10 @@
             <v>87483.259999999951</v>
           </cell>
           <cell r="H15" t="str">
-            <v>LESTE</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I15">
-            <v>3541.45</v>
+            <v>19933.399999999991</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1944,10 +1944,10 @@
             <v>110646.80000000005</v>
           </cell>
           <cell r="H16" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I16">
-            <v>9469.7999999999975</v>
+            <v>3543.95</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1964,10 +1964,10 @@
             <v>266913.34999999992</v>
           </cell>
           <cell r="H17" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I17">
-            <v>6244.4900000000007</v>
+            <v>9469.7999999999975</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1984,10 +1984,10 @@
             <v>278371.99999999994</v>
           </cell>
           <cell r="H18" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I18">
-            <v>2844.5000000000005</v>
+            <v>6244.4900000000007</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -2001,13 +2001,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>72461.88</v>
+            <v>72464.38</v>
           </cell>
           <cell r="H19" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I19">
-            <v>3561.78</v>
+            <v>2844.5000000000005</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -2024,10 +2024,10 @@
             <v>133853.76499999966</v>
           </cell>
           <cell r="H20" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I20">
-            <v>7244.07</v>
+            <v>3569.1000000000004</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
@@ -2044,16 +2044,16 @@
             <v>96274.990000000063</v>
           </cell>
           <cell r="H21" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I21">
-            <v>7423.8599999999988</v>
+            <v>7244.07</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N21">
-            <v>26</v>
+            <v>27</v>
           </cell>
         </row>
         <row r="22">
@@ -2064,16 +2064,16 @@
             <v>84553.079999999842</v>
           </cell>
           <cell r="H22" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I22">
-            <v>3907.3199999999997</v>
+            <v>7588.8599999999988</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
           </cell>
           <cell r="N22">
-            <v>36</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="23">
@@ -2081,13 +2081,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>49151.680000000095</v>
+            <v>49159.000000000095</v>
           </cell>
           <cell r="H23" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I23">
-            <v>10826.189999999999</v>
+            <v>3907.3199999999997</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
@@ -2104,10 +2104,10 @@
             <v>163165.17999999976</v>
           </cell>
           <cell r="H24" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I24">
-            <v>10432.15</v>
+            <v>11473.039999999997</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
@@ -2124,10 +2124,10 @@
             <v>236192.96999999959</v>
           </cell>
           <cell r="H25" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I25">
-            <v>2312.58</v>
+            <v>10432.39</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
@@ -2144,10 +2144,10 @@
             <v>92708.429999999935</v>
           </cell>
           <cell r="H26" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC</v>
           </cell>
           <cell r="I26">
-            <v>1031.8499999999999</v>
+            <v>2316.5</v>
           </cell>
         </row>
         <row r="27">
@@ -2155,13 +2155,13 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>115674.05999999995</v>
+            <v>116320.90999999995</v>
           </cell>
           <cell r="H27" t="str">
-            <v>Total Geral</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I27">
-            <v>475170.47000000032</v>
+            <v>36.6</v>
           </cell>
         </row>
         <row r="28">
@@ -2169,7 +2169,13 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>179510.68999999983</v>
+            <v>179510.92999999985</v>
+          </cell>
+          <cell r="H28" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I28">
+            <v>1031.8499999999999</v>
           </cell>
         </row>
         <row r="29">
@@ -2177,7 +2183,13 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>58337.470000000096</v>
+            <v>58341.390000000094</v>
+          </cell>
+          <cell r="H29" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I29">
+            <v>484244.02000000025</v>
           </cell>
         </row>
         <row r="30">
@@ -2185,7 +2197,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>29659.220000000012</v>
+            <v>29667.840000000015</v>
           </cell>
         </row>
         <row r="31">
@@ -2201,7 +2213,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4014116.2049999516</v>
+            <v>4014787.5549999522</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3052,7 +3064,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4014116.2049999996</v>
+        <v>4014787.5549999988</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3063,7 +3075,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>93987.07</v>
+        <v>94851.4</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3074,7 +3086,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>381183.39999999991</v>
+        <v>383500.61999999994</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3097,7 +3109,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1578383.7950000004</v>
+        <v>1577712.4450000012</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3108,7 +3120,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>56012.929999999993</v>
+        <v>55148.600000000006</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3119,7 +3131,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-381183.39999999991</v>
+        <v>-383500.61999999994</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3142,7 +3154,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.71776776128743847</v>
+        <v>0.71788780599016522</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3153,7 +3165,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.62658046666666678</v>
+        <v>0.63234266666666661</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3293,11 +3305,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7423.8599999999988</v>
+        <v>7588.8599999999988</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9576.1400000000012</v>
+        <v>9411.1400000000012</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3520,11 +3532,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10432.15</v>
+        <v>10432.39</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4567.8500000000004</v>
+        <v>4567.6100000000006</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3578,11 +3590,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>175450.48999999985</v>
+        <v>175452.38999999984</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>97549.510000000155</v>
+        <v>97547.610000000161</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3693,11 +3705,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3715.6000000000004</v>
+        <v>4033.8200000000006</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-3715.6000000000004</v>
+        <v>-4033.8200000000006</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3751,11 +3763,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10826.189999999999</v>
+        <v>11473.039999999997</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2643.8100000000013</v>
+        <v>1996.9600000000028</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3770,11 +3782,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>20600.599999999999</v>
+        <v>22599.599999999999</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>-20600.599999999999</v>
+        <v>-22599.599999999999</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3828,11 +3840,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3561.78</v>
+        <v>3569.1000000000004</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1031.7800000000002</v>
+        <v>-1039.1000000000004</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3905,11 +3917,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3541.45</v>
+        <v>3543.95</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3298.55</v>
+        <v>3296.05</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -4029,11 +4041,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4951.2999999999993</v>
+        <v>4953.2</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8048.7000000000007</v>
+        <v>8046.8</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4157,11 +4169,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>72461.88</v>
+        <v>72464.38</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>49538.119999999995</v>
+        <v>49535.619999999995</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4193,11 +4205,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>563167.95000000042</v>
+        <v>563167.95000000019</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-67713.404545454949</v>
+        <v>-67713.404545454716</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4212,11 +4224,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4268,11 +4280,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>691799.54999999935</v>
+        <v>685907.54999999935</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-72481.368181817466</v>
+        <v>-66589.368181817466</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4287,11 +4299,11 @@
       </c>
       <c r="V23" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="W23" s="19">
         <f t="shared" si="2"/>
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -4343,11 +4355,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>540215.10999999964</v>
+        <v>546107.10999999964</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>79103.071818182245</v>
+        <v>73211.071818182245</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4401,11 +4413,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2312.58</v>
+        <v>2316.5</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1587.42</v>
+        <v>1583.5</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4457,11 +4469,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>49151.680000000095</v>
+        <v>49159.000000000095</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40848.319999999905</v>
+        <v>40840.999999999905</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4476,11 +4488,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>36.6</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2780</v>
+        <v>2743.4</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4703,11 +4715,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>115674.05999999995</v>
+        <v>116320.90999999995</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>51325.940000000046</v>
+        <v>50679.090000000055</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4763,11 +4775,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>179510.68999999983</v>
+        <v>179510.92999999985</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>80489.310000000172</v>
+        <v>80489.070000000153</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4823,11 +4835,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>58337.470000000096</v>
+        <v>58341.390000000094</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41662.529999999904</v>
+        <v>41658.609999999906</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4863,11 +4875,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>-10.727272727272748</v>
+        <v>-11.727272727272748</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4883,11 +4895,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29659.220000000012</v>
+        <v>29667.840000000015</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>25340.779999999988</v>
+        <v>25332.159999999985</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4900,11 +4912,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>431898.23500000179</v>
+        <v>432569.58500000188</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>219351.76499999821</v>
+        <v>218680.41499999812</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -5175,11 +5187,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1392309.7799999909</v>
+        <v>1386417.7799999914</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>-741059.77999999095</v>
+        <v>-735167.77999999141</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -5211,11 +5223,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>972367.23500000208</v>
+        <v>978930.58500000194</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-321117.23500000208</v>
+        <v>-327680.58500000194</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 23/07/2026 07:21
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D599799-BA6C-46B7-9655-866F7B11587F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D47A0C-67AD-4897-9464-9061CE778270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1772,9 +1772,6 @@
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
           </cell>
-          <cell r="N7" t="str">
-            <v>Total Geral</v>
-          </cell>
         </row>
         <row r="8">
           <cell r="E8" t="str">
@@ -1792,9 +1789,6 @@
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
-          <cell r="N8">
-            <v>23</v>
-          </cell>
         </row>
         <row r="9">
           <cell r="E9" t="str">
@@ -1812,9 +1806,6 @@
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
-          <cell r="N9">
-            <v>41</v>
-          </cell>
         </row>
         <row r="10">
           <cell r="E10" t="str">
@@ -1832,9 +1823,6 @@
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
-          <cell r="N10">
-            <v>32</v>
-          </cell>
         </row>
         <row r="11">
           <cell r="E11" t="str">
@@ -1852,9 +1840,6 @@
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
-          <cell r="N11">
-            <v>50</v>
-          </cell>
         </row>
         <row r="12">
           <cell r="E12" t="str">
@@ -1872,9 +1857,6 @@
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
-          <cell r="N12">
-            <v>19</v>
-          </cell>
         </row>
         <row r="13">
           <cell r="E13" t="str">
@@ -1887,13 +1869,10 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="I13">
-            <v>22599.599999999999</v>
+            <v>26173.7</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
-          </cell>
-          <cell r="N13">
-            <v>30</v>
           </cell>
         </row>
         <row r="14">
@@ -1912,16 +1891,13 @@
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
-          <cell r="N14">
-            <v>48</v>
-          </cell>
         </row>
         <row r="15">
           <cell r="E15" t="str">
             <v>KEY PIRACICABA</v>
           </cell>
           <cell r="F15">
-            <v>87483.259999999951</v>
+            <v>87483.25999999998</v>
           </cell>
           <cell r="H15" t="str">
             <v>KEY ZL</v>
@@ -1931,9 +1907,6 @@
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
-          </cell>
-          <cell r="N15">
-            <v>24</v>
           </cell>
         </row>
         <row r="16">
@@ -1941,7 +1914,7 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>110646.80000000005</v>
+            <v>114220.90000000004</v>
           </cell>
           <cell r="H16" t="str">
             <v>LESTE</v>
@@ -1951,9 +1924,6 @@
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="N16">
-            <v>35</v>
           </cell>
         </row>
         <row r="17">
@@ -1972,9 +1942,6 @@
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
-          <cell r="N17">
-            <v>35</v>
-          </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
@@ -1992,9 +1959,6 @@
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
-          <cell r="N18">
-            <v>40</v>
-          </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
@@ -2012,16 +1976,13 @@
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
-          <cell r="N19">
-            <v>60</v>
-          </cell>
         </row>
         <row r="20">
           <cell r="E20" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>133853.76499999966</v>
+            <v>133853.76499999964</v>
           </cell>
           <cell r="H20" t="str">
             <v>MOGI</v>
@@ -2031,9 +1992,6 @@
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
-          </cell>
-          <cell r="N20">
-            <v>27</v>
           </cell>
         </row>
         <row r="21">
@@ -2052,9 +2010,6 @@
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
           </cell>
-          <cell r="N21">
-            <v>27</v>
-          </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
@@ -2067,13 +2022,10 @@
             <v>OSASCO</v>
           </cell>
           <cell r="I22">
-            <v>7588.8599999999988</v>
+            <v>7588.86</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
-          </cell>
-          <cell r="N22">
-            <v>35</v>
           </cell>
         </row>
         <row r="23">
@@ -2092,9 +2044,6 @@
           <cell r="K23" t="str">
             <v>SJC</v>
           </cell>
-          <cell r="N23">
-            <v>21</v>
-          </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
@@ -2112,16 +2061,13 @@
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
           </cell>
-          <cell r="N24">
-            <v>23</v>
-          </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>236192.96999999959</v>
+            <v>236192.97000000015</v>
           </cell>
           <cell r="H25" t="str">
             <v>SBC</v>
@@ -2131,9 +2077,6 @@
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
-          </cell>
-          <cell r="N25">
-            <v>570</v>
           </cell>
         </row>
         <row r="26">
@@ -2155,7 +2098,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>116320.90999999995</v>
+            <v>116320.90999999996</v>
           </cell>
           <cell r="H27" t="str">
             <v>SJC/VALE</v>
@@ -2175,7 +2118,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I28">
-            <v>1031.8499999999999</v>
+            <v>1333.2999999999997</v>
           </cell>
         </row>
         <row r="29">
@@ -2183,13 +2126,13 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>58341.390000000094</v>
+            <v>58341.390000000087</v>
           </cell>
           <cell r="H29" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I29">
-            <v>484244.02000000025</v>
+            <v>488119.57000000012</v>
           </cell>
         </row>
         <row r="30">
@@ -2205,7 +2148,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>52543.400000000009</v>
+            <v>52844.85</v>
           </cell>
         </row>
         <row r="32">
@@ -2213,7 +2156,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4014787.5549999522</v>
+            <v>4018663.1049999632</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3030,7 +2973,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>150000</v>
+        <v>130000</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -3064,7 +3007,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4014787.5549999988</v>
+        <v>4018663.1050000004</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3075,7 +3018,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>94851.4</v>
+        <v>95152.849999999991</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3086,7 +3029,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>383500.61999999994</v>
+        <v>387074.72</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3097,7 +3040,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>570</v>
+        <v>0</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3109,7 +3052,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1577712.4450000012</v>
+        <v>1573836.8949999996</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3120,7 +3063,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>55148.600000000006</v>
+        <v>34847.150000000009</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3131,7 +3074,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-383500.61999999994</v>
+        <v>-387074.72</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3142,7 +3085,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>188</v>
+        <v>758</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3154,7 +3097,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.71788780599016522</v>
+        <v>0.71858079660259278</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3165,7 +3108,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.63234266666666661</v>
+        <v>0.73194499999999996</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3187,7 +3130,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.75197889182058053</v>
+        <v>0</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3301,15 +3244,15 @@
       </c>
       <c r="I10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>17000</v>
+        <v>12090</v>
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7588.8599999999988</v>
+        <v>7588.86</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9411.1400000000012</v>
+        <v>4501.1400000000003</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3340,11 +3283,11 @@
       </c>
       <c r="V10" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="W10" s="19">
         <f>U10-V10</f>
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -3375,7 +3318,7 @@
       </c>
       <c r="I11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11960</v>
+        <v>11000</v>
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3383,7 +3326,7 @@
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4715.93</v>
+        <v>3755.9300000000003</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3417,11 +3360,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3451,7 +3394,7 @@
       </c>
       <c r="I12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>9110</v>
+        <v>5400</v>
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3459,7 +3402,7 @@
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5202.68</v>
+        <v>1492.6800000000003</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3493,11 +3436,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3528,7 +3471,7 @@
       </c>
       <c r="I13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15000</v>
+        <v>13000</v>
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3536,7 +3479,7 @@
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4567.6100000000006</v>
+        <v>2567.6100000000006</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3570,11 +3513,11 @@
       </c>
       <c r="V13" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="W13" s="19">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -3605,7 +3548,7 @@
       </c>
       <c r="I14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4280</v>
+        <v>3840</v>
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3613,7 +3556,7 @@
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1435.4999999999995</v>
+        <v>995.49999999999955</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3647,11 +3590,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3724,11 +3667,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3759,7 +3702,7 @@
       </c>
       <c r="I16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13470</v>
+        <v>9840</v>
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3767,7 +3710,7 @@
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1996.9600000000028</v>
+        <v>-1633.0399999999972</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3782,11 +3725,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>22599.599999999999</v>
+        <v>26173.7</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>-22599.599999999999</v>
+        <v>-26173.7</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3801,11 +3744,11 @@
       </c>
       <c r="V16" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="W16" s="19">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3836,7 +3779,7 @@
       </c>
       <c r="I17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2530</v>
+        <v>4850</v>
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3844,7 +3787,7 @@
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1039.1000000000004</v>
+        <v>1280.8999999999996</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3878,11 +3821,11 @@
       </c>
       <c r="V17" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="W17" s="19">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3942,11 +3885,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3962,11 +3905,11 @@
       </c>
       <c r="D19" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>110646.80000000005</v>
+        <v>114220.90000000004</v>
       </c>
       <c r="E19" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>19353.199999999953</v>
+        <v>15779.099999999962</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="21" t="s">
@@ -3977,7 +3920,7 @@
       </c>
       <c r="I19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>10910</v>
+        <v>7120</v>
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -3985,7 +3928,7 @@
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1440.2000000000025</v>
+        <v>-2349.7999999999975</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -4002,11 +3945,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -4037,7 +3980,7 @@
       </c>
       <c r="I20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13000</v>
+        <v>15000</v>
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4045,7 +3988,7 @@
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8046.8</v>
+        <v>10046.799999999999</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4074,11 +4017,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4109,7 +4052,7 @@
       </c>
       <c r="I21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5490</v>
+        <v>5100</v>
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4117,7 +4060,7 @@
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2116.35</v>
+        <v>1726.35</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4149,11 +4092,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -4184,7 +4127,7 @@
       </c>
       <c r="I22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>7350</v>
+        <v>3320</v>
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4192,7 +4135,7 @@
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1105.5099999999993</v>
+        <v>-2924.4900000000007</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4205,11 +4148,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>563167.95000000019</v>
+        <v>563167.95000000042</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-67713.404545454716</v>
+        <v>-67713.404545454949</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="19" t="s">
@@ -4224,11 +4167,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>13</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4244,11 +4187,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>133853.76499999966</v>
+        <v>133853.76499999964</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>61146.235000000335</v>
+        <v>61146.235000000364</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4259,7 +4202,7 @@
       </c>
       <c r="I23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5290</v>
+        <v>4010</v>
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4267,7 +4210,7 @@
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3138</v>
+        <v>1858</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4280,11 +4223,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>685907.54999999935</v>
+        <v>685907.54999999946</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-66589.368181817466</v>
+        <v>-66589.368181817583</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4299,11 +4242,11 @@
       </c>
       <c r="V23" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="W23" s="19">
         <f t="shared" si="2"/>
-        <v>20</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -4334,15 +4277,15 @@
       </c>
       <c r="I24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3540</v>
+        <v>4700</v>
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1031.8499999999999</v>
+        <v>1333.2999999999997</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2508.15</v>
+        <v>3366.7000000000003</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4355,11 +4298,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>546107.10999999964</v>
+        <v>549681.20999999973</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>73211.071818182245</v>
+        <v>69636.971818182152</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4374,11 +4317,11 @@
       </c>
       <c r="V24" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="W24" s="19">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -4409,7 +4352,7 @@
       </c>
       <c r="I25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3900</v>
+        <v>2690</v>
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4417,7 +4360,7 @@
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1583.5</v>
+        <v>373.5</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4449,11 +4392,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4484,7 +4427,7 @@
       </c>
       <c r="I26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2780</v>
+        <v>3530</v>
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4492,7 +4435,7 @@
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2743.4</v>
+        <v>3493.4</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4513,11 +4456,11 @@
       </c>
       <c r="V26" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="W26" s="19">
         <f t="shared" si="2"/>
-        <v>12</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -4548,7 +4491,7 @@
       </c>
       <c r="I27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2550</v>
+        <v>2670</v>
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -4556,7 +4499,7 @@
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1525.6599999999994</v>
+        <v>-1405.6599999999994</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4579,11 +4522,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>236192.96999999959</v>
+        <v>236192.97000000015</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>82307.030000000406</v>
+        <v>82307.029999999853</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4612,11 +4555,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>87483.259999999951</v>
+        <v>87483.25999999998</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>87516.740000000049</v>
+        <v>87516.74000000002</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4715,11 +4658,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>116320.90999999995</v>
+        <v>116320.90999999996</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50679.090000000055</v>
+        <v>50679.09000000004</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4732,11 +4675,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>270334.04000000004</v>
+        <v>270334.03999999998</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>120415.95999999996</v>
+        <v>120415.96000000002</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4792,11 +4735,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>540157.7900000033</v>
+        <v>540157.79000000341</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>-19157.790000003297</v>
+        <v>-19157.790000003413</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4835,11 +4778,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>58341.390000000094</v>
+        <v>58341.390000000087</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41658.609999999906</v>
+        <v>41658.609999999913</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4852,11 +4795,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>700067.9900000022</v>
+        <v>700067.99000000325</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>-48817.990000002203</v>
+        <v>-48817.99000000325</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4912,11 +4855,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>432569.58500000188</v>
+        <v>432871.03500000184</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>218680.41499999812</v>
+        <v>218378.96499999816</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4955,11 +4898,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52543.400000000009</v>
+        <v>52844.85</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>20456.599999999991</v>
+        <v>20155.150000000001</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5115,11 +5058,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>545683.80000000156</v>
+        <v>545683.80000000168</v>
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>-154933.80000000156</v>
+        <v>-154933.80000000168</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -5151,11 +5094,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1103755.3899999959</v>
+        <v>1103755.3899999962</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="5">C41-D41</f>
-        <v>-582755.38999999594</v>
+        <v>-582755.38999999617</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -5187,11 +5130,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1386417.7799999914</v>
+        <v>1386417.7799999891</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>-735167.77999999141</v>
+        <v>-735167.77999998908</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -5223,11 +5166,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>978930.58500000194</v>
+        <v>982806.13500000234</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-327680.58500000194</v>
+        <v>-331556.13500000234</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 23/07/2026 07:36
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D47A0C-67AD-4897-9464-9061CE778270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E4DAFE7-AEE9-4803-8D95-12CE3BE4A4B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-22T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1666,11 +1666,11 @@
       <sheetName val="BASE PYTHON"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
@@ -1694,7 +1694,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>22/07/2026</v>
+            <v/>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1732,12 +1732,6 @@
           <cell r="F5">
             <v>39246.379999999976</v>
           </cell>
-          <cell r="H5" t="str">
-            <v>CAMPINAS</v>
-          </cell>
-          <cell r="I5">
-            <v>4075.6599999999994</v>
-          </cell>
         </row>
         <row r="6">
           <cell r="E6" t="str">
@@ -1746,12 +1740,6 @@
           <cell r="F6">
             <v>260716.2799999995</v>
           </cell>
-          <cell r="H6" t="str">
-            <v>CENTRO</v>
-          </cell>
-          <cell r="I6">
-            <v>10594.419999999998</v>
-          </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
           </cell>
@@ -1763,12 +1751,6 @@
           <cell r="F7">
             <v>1082.83</v>
           </cell>
-          <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
-          </cell>
-          <cell r="I7">
-            <v>2152</v>
-          </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
           </cell>
@@ -1780,12 +1762,6 @@
           <cell r="F8">
             <v>151.09</v>
           </cell>
-          <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
-          </cell>
-          <cell r="I8">
-            <v>4953.2</v>
-          </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
@@ -1797,12 +1773,6 @@
           <cell r="F9">
             <v>51198.209999999992</v>
           </cell>
-          <cell r="H9" t="str">
-            <v>JUNDIAI</v>
-          </cell>
-          <cell r="I9">
-            <v>3373.65</v>
-          </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
@@ -1814,12 +1784,6 @@
           <cell r="F10">
             <v>175452.38999999984</v>
           </cell>
-          <cell r="H10" t="str">
-            <v>KEY ABC</v>
-          </cell>
-          <cell r="I10">
-            <v>2409.6999999999998</v>
-          </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
@@ -1831,12 +1795,6 @@
           <cell r="F11">
             <v>51759.880000000063</v>
           </cell>
-          <cell r="H11" t="str">
-            <v>KEY INTERIOR</v>
-          </cell>
-          <cell r="I11">
-            <v>334524.09999999998</v>
-          </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
@@ -1848,12 +1806,6 @@
           <cell r="F12">
             <v>211630.01999999996</v>
           </cell>
-          <cell r="H12" t="str">
-            <v>KEY PIRACICABA</v>
-          </cell>
-          <cell r="I12">
-            <v>5892</v>
-          </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
@@ -1865,12 +1817,6 @@
           <cell r="F13">
             <v>263985.40000000084</v>
           </cell>
-          <cell r="H13" t="str">
-            <v>KEY SJC</v>
-          </cell>
-          <cell r="I13">
-            <v>26173.7</v>
-          </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
@@ -1882,12 +1828,6 @@
           <cell r="F14">
             <v>851393.40000000026</v>
           </cell>
-          <cell r="H14" t="str">
-            <v>KEY SP</v>
-          </cell>
-          <cell r="I14">
-            <v>4033.8200000000006</v>
-          </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
@@ -1899,12 +1839,6 @@
           <cell r="F15">
             <v>87483.25999999998</v>
           </cell>
-          <cell r="H15" t="str">
-            <v>KEY ZL</v>
-          </cell>
-          <cell r="I15">
-            <v>19933.399999999991</v>
-          </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
@@ -1916,12 +1850,6 @@
           <cell r="F16">
             <v>114220.90000000004</v>
           </cell>
-          <cell r="H16" t="str">
-            <v>LESTE</v>
-          </cell>
-          <cell r="I16">
-            <v>3543.95</v>
-          </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
@@ -1933,12 +1861,6 @@
           <cell r="F17">
             <v>266913.34999999992</v>
           </cell>
-          <cell r="H17" t="str">
-            <v>LESTE MOOCA</v>
-          </cell>
-          <cell r="I17">
-            <v>9469.7999999999975</v>
-          </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
@@ -1950,12 +1872,6 @@
           <cell r="F18">
             <v>278371.99999999994</v>
           </cell>
-          <cell r="H18" t="str">
-            <v>LESTE PENHA</v>
-          </cell>
-          <cell r="I18">
-            <v>6244.4900000000007</v>
-          </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
@@ -1967,12 +1883,6 @@
           <cell r="F19">
             <v>72464.38</v>
           </cell>
-          <cell r="H19" t="str">
-            <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="I19">
-            <v>2844.5000000000005</v>
-          </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
@@ -1984,12 +1894,6 @@
           <cell r="F20">
             <v>133853.76499999964</v>
           </cell>
-          <cell r="H20" t="str">
-            <v>MOGI</v>
-          </cell>
-          <cell r="I20">
-            <v>3569.1000000000004</v>
-          </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
           </cell>
@@ -2001,12 +1905,6 @@
           <cell r="F21">
             <v>96274.990000000063</v>
           </cell>
-          <cell r="H21" t="str">
-            <v>NORTE</v>
-          </cell>
-          <cell r="I21">
-            <v>7244.07</v>
-          </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
           </cell>
@@ -2018,12 +1916,6 @@
           <cell r="F22">
             <v>84553.079999999842</v>
           </cell>
-          <cell r="H22" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="I22">
-            <v>7588.86</v>
-          </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
           </cell>
@@ -2035,12 +1927,6 @@
           <cell r="F23">
             <v>49159.000000000095</v>
           </cell>
-          <cell r="H23" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I23">
-            <v>3907.3199999999997</v>
-          </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
           </cell>
@@ -2052,12 +1938,6 @@
           <cell r="F24">
             <v>163165.17999999976</v>
           </cell>
-          <cell r="H24" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I24">
-            <v>11473.039999999997</v>
-          </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
           </cell>
@@ -2069,12 +1949,6 @@
           <cell r="F25">
             <v>236192.97000000015</v>
           </cell>
-          <cell r="H25" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I25">
-            <v>10432.39</v>
-          </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
@@ -2086,12 +1960,6 @@
           <cell r="F26">
             <v>92708.429999999935</v>
           </cell>
-          <cell r="H26" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I26">
-            <v>2316.5</v>
-          </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
@@ -2100,12 +1968,6 @@
           <cell r="F27">
             <v>116320.90999999996</v>
           </cell>
-          <cell r="H27" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I27">
-            <v>36.6</v>
-          </cell>
         </row>
         <row r="28">
           <cell r="E28" t="str">
@@ -2114,12 +1976,6 @@
           <cell r="F28">
             <v>179510.92999999985</v>
           </cell>
-          <cell r="H28" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I28">
-            <v>1333.2999999999997</v>
-          </cell>
         </row>
         <row r="29">
           <cell r="E29" t="str">
@@ -2127,12 +1983,6 @@
           </cell>
           <cell r="F29">
             <v>58341.390000000087</v>
-          </cell>
-          <cell r="H29" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I29">
-            <v>488119.57000000012</v>
           </cell>
         </row>
         <row r="30">
@@ -3018,7 +2868,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>95152.849999999991</v>
+        <v>0</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3029,7 +2879,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>387074.72</v>
+        <v>0</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3063,7 +2913,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>34847.150000000009</v>
+        <v>130000</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3074,7 +2924,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-387074.72</v>
+        <v>0</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3108,7 +2958,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.73194499999999996</v>
+        <v>0</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3248,11 +3098,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7588.86</v>
+        <v>0</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4501.1400000000003</v>
+        <v>12090</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3322,11 +3172,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7244.07</v>
+        <v>0</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3755.9300000000003</v>
+        <v>11000</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3341,11 +3191,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2409.6999999999998</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>-2409.6999999999998</v>
+        <v>0</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3398,11 +3248,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3907.3199999999997</v>
+        <v>0</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1492.6800000000003</v>
+        <v>5400</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3475,11 +3325,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10432.39</v>
+        <v>0</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2567.6100000000006</v>
+        <v>13000</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3494,11 +3344,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>19933.399999999991</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-19933.399999999991</v>
+        <v>0</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3552,11 +3402,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2844.5000000000005</v>
+        <v>0</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>995.49999999999955</v>
+        <v>3840</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3571,11 +3421,11 @@
       </c>
       <c r="P14" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>334524.09999999998</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" si="1"/>
-        <v>-334524.09999999998</v>
+        <v>0</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="19" t="s">
@@ -3629,11 +3479,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10594.419999999998</v>
+        <v>0</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4405.5800000000017</v>
+        <v>15000</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3648,11 +3498,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4033.8200000000006</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-4033.8200000000006</v>
+        <v>0</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3706,11 +3556,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11473.039999999997</v>
+        <v>0</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1633.0399999999972</v>
+        <v>9840</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3725,11 +3575,11 @@
       </c>
       <c r="P16" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>26173.7</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="1"/>
-        <v>-26173.7</v>
+        <v>0</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="19" t="s">
@@ -3783,11 +3633,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3569.1000000000004</v>
+        <v>0</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1280.8999999999996</v>
+        <v>4850</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3860,11 +3710,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3543.95</v>
+        <v>0</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3296.05</v>
+        <v>6840</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3924,11 +3774,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9469.7999999999975</v>
+        <v>0</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-2349.7999999999975</v>
+        <v>7120</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3984,11 +3834,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4953.2</v>
+        <v>0</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10046.799999999999</v>
+        <v>15000</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4056,11 +3906,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3373.65</v>
+        <v>0</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1726.35</v>
+        <v>5100</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4131,11 +3981,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6244.4900000000007</v>
+        <v>0</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-2924.4900000000007</v>
+        <v>3320</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4206,11 +4056,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2152</v>
+        <v>0</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1858</v>
+        <v>4010</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4281,11 +4131,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1333.2999999999997</v>
+        <v>0</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3366.7000000000003</v>
+        <v>4700</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4356,11 +4206,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2316.5</v>
+        <v>0</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>373.5</v>
+        <v>2690</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4431,11 +4281,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>36.6</v>
+        <v>0</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3493.4</v>
+        <v>3530</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4495,11 +4345,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4075.6599999999994</v>
+        <v>0</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1405.6599999999994</v>
+        <v>2670</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 23/07/2026 08:37
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E4DAFE7-AEE9-4803-8D95-12CE3BE4A4B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F98E042-6379-462D-AB8A-CD0DE687FABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-23T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1666,11 +1666,11 @@
       <sheetName val="BASE PYTHON"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
@@ -1694,7 +1694,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v/>
+            <v>23/07/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1732,6 +1732,12 @@
           <cell r="F5">
             <v>39246.379999999976</v>
           </cell>
+          <cell r="H5" t="str">
+            <v>INDAIATUBA</v>
+          </cell>
+          <cell r="I5">
+            <v>119.9</v>
+          </cell>
         </row>
         <row r="6">
           <cell r="E6" t="str">
@@ -1740,6 +1746,12 @@
           <cell r="F6">
             <v>260716.2799999995</v>
           </cell>
+          <cell r="H6" t="str">
+            <v>INTERLAGOS</v>
+          </cell>
+          <cell r="I6">
+            <v>158</v>
+          </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
           </cell>
@@ -1751,8 +1763,17 @@
           <cell r="F7">
             <v>1082.83</v>
           </cell>
+          <cell r="H7" t="str">
+            <v>KEY ABC</v>
+          </cell>
+          <cell r="I7">
+            <v>1217.5999999999999</v>
+          </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
+          </cell>
+          <cell r="N7" t="str">
+            <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
@@ -1762,8 +1783,17 @@
           <cell r="F8">
             <v>151.09</v>
           </cell>
+          <cell r="H8" t="str">
+            <v>LESTE</v>
+          </cell>
+          <cell r="I8">
+            <v>1019.85</v>
+          </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
+          </cell>
+          <cell r="N8">
+            <v>23</v>
           </cell>
         </row>
         <row r="9">
@@ -1771,10 +1801,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>51198.209999999992</v>
+            <v>51318.109999999993</v>
+          </cell>
+          <cell r="H9" t="str">
+            <v>LESTE MOOCA</v>
+          </cell>
+          <cell r="I9">
+            <v>349.75</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
+          </cell>
+          <cell r="N9">
+            <v>41</v>
           </cell>
         </row>
         <row r="10">
@@ -1782,10 +1821,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>175452.38999999984</v>
+            <v>175610.38999999984</v>
+          </cell>
+          <cell r="H10" t="str">
+            <v>LESTE PENHA</v>
+          </cell>
+          <cell r="I10">
+            <v>299.8</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
+          </cell>
+          <cell r="N10">
+            <v>33</v>
           </cell>
         </row>
         <row r="11">
@@ -1795,8 +1843,17 @@
           <cell r="F11">
             <v>51759.880000000063</v>
           </cell>
+          <cell r="H11" t="str">
+            <v>LESTE TATUAPE</v>
+          </cell>
+          <cell r="I11">
+            <v>313.10000000000002</v>
+          </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
+          </cell>
+          <cell r="N11">
+            <v>50</v>
           </cell>
         </row>
         <row r="12">
@@ -1804,10 +1861,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>211630.01999999996</v>
+            <v>212847.61999999997</v>
+          </cell>
+          <cell r="H12" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I12">
+            <v>649.5</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
+          </cell>
+          <cell r="N12">
+            <v>19</v>
           </cell>
         </row>
         <row r="13">
@@ -1817,8 +1883,17 @@
           <cell r="F13">
             <v>263985.40000000084</v>
           </cell>
+          <cell r="H13" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I13">
+            <v>4127.5</v>
+          </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
+          </cell>
+          <cell r="N13">
+            <v>30</v>
           </cell>
         </row>
         <row r="14">
@@ -1831,16 +1906,22 @@
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
+          <cell r="N14">
+            <v>48</v>
+          </cell>
         </row>
         <row r="15">
           <cell r="E15" t="str">
             <v>KEY PIRACICABA</v>
           </cell>
           <cell r="F15">
-            <v>87483.25999999998</v>
+            <v>87483.259999999951</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
+          </cell>
+          <cell r="N15">
+            <v>25</v>
           </cell>
         </row>
         <row r="16">
@@ -1853,6 +1934,9 @@
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
+          <cell r="N16">
+            <v>36</v>
+          </cell>
         </row>
         <row r="17">
           <cell r="E17" t="str">
@@ -1864,6 +1948,9 @@
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
+          <cell r="N17">
+            <v>35</v>
+          </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
@@ -1875,16 +1962,22 @@
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
+          <cell r="N18">
+            <v>40</v>
+          </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>72464.38</v>
+            <v>73484.23</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
+          </cell>
+          <cell r="N19">
+            <v>60</v>
           </cell>
         </row>
         <row r="20">
@@ -1892,10 +1985,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>133853.76499999964</v>
+            <v>134203.51499999966</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
+          </cell>
+          <cell r="N20">
+            <v>27</v>
           </cell>
         </row>
         <row r="21">
@@ -1903,10 +1999,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>96274.990000000063</v>
+            <v>96574.790000000066</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="N21">
+            <v>27</v>
           </cell>
         </row>
         <row r="22">
@@ -1914,10 +2013,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>84553.079999999842</v>
+            <v>84866.179999999833</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
+          </cell>
+          <cell r="N22">
+            <v>35</v>
           </cell>
         </row>
         <row r="23">
@@ -1930,6 +2032,9 @@
           <cell r="K23" t="str">
             <v>SJC</v>
           </cell>
+          <cell r="N23">
+            <v>21</v>
+          </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
@@ -1941,16 +2046,22 @@
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
           </cell>
+          <cell r="N24">
+            <v>23</v>
+          </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>236192.97000000015</v>
+            <v>236192.96999999977</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
+          </cell>
+          <cell r="N25">
+            <v>573</v>
           </cell>
         </row>
         <row r="26">
@@ -1966,7 +2077,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>116320.90999999996</v>
+            <v>116320.90999999995</v>
           </cell>
         </row>
         <row r="28">
@@ -1982,7 +2093,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>58341.390000000087</v>
+            <v>58990.890000000087</v>
           </cell>
         </row>
         <row r="30">
@@ -1998,7 +2109,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>52844.85</v>
+            <v>52844.850000000006</v>
           </cell>
         </row>
         <row r="32">
@@ -2006,7 +2117,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4018663.1049999632</v>
+            <v>4022790.604999952</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2857,7 +2968,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4018663.1050000004</v>
+        <v>4022790.6049999995</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2868,7 +2979,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>0</v>
+        <v>2909.9</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2879,7 +2990,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>0</v>
+        <v>1217.5999999999999</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -2890,7 +3001,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>0</v>
+        <v>573</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2902,7 +3013,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1573836.8949999996</v>
+        <v>1569709.3950000005</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -2913,7 +3024,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>130000</v>
+        <v>127090.1</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2924,7 +3035,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>0</v>
+        <v>-1217.5999999999999</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -2935,7 +3046,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>758</v>
+        <v>185</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -2947,7 +3058,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.71858079660259278</v>
+        <v>0.71931883862315593</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -2958,7 +3069,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0</v>
+        <v>2.2383846153846143E-2</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2980,7 +3091,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0</v>
+        <v>0.75593667546174137</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3133,11 +3244,11 @@
       </c>
       <c r="V10" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="W10" s="19">
         <f>U10-V10</f>
-        <v>36</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -3191,11 +3302,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1217.5999999999999</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>0</v>
+        <v>-1217.5999999999999</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3210,11 +3321,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>52</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3286,11 +3397,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>41</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3306,11 +3417,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51198.209999999992</v>
+        <v>51318.109999999993</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>38801.790000000008</v>
+        <v>38681.890000000007</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3363,11 +3474,11 @@
       </c>
       <c r="V13" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="W13" s="19">
         <f t="shared" si="0"/>
-        <v>59</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -3383,11 +3494,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>175452.38999999984</v>
+        <v>175610.38999999984</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>97547.610000000161</v>
+        <v>97389.610000000161</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3402,11 +3513,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>313.10000000000002</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3840</v>
+        <v>3526.9</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3440,11 +3551,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3517,11 +3628,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3537,11 +3648,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>211630.01999999996</v>
+        <v>212847.61999999997</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>113369.98000000004</v>
+        <v>112152.38000000003</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3594,11 +3705,11 @@
       </c>
       <c r="V16" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W16" s="19">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3671,11 +3782,11 @@
       </c>
       <c r="V17" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="W17" s="19">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3710,11 +3821,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1019.85</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6840</v>
+        <v>5820.15</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3735,11 +3846,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3774,11 +3885,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>349.75</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7120</v>
+        <v>6770.25</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3795,11 +3906,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>61</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -3834,11 +3945,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>158</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15000</v>
+        <v>14842</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3867,11 +3978,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -3942,11 +4053,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>44</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -3962,11 +4073,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>72464.38</v>
+        <v>73484.23</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>49535.619999999995</v>
+        <v>48515.770000000004</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -3981,11 +4092,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>299.8</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3320</v>
+        <v>3020.2</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4017,11 +4128,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4037,11 +4148,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>133853.76499999964</v>
+        <v>134203.51499999966</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>61146.235000000364</v>
+        <v>60796.485000000335</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4056,11 +4167,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>119.9</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4010</v>
+        <v>3890.1</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4092,11 +4203,11 @@
       </c>
       <c r="V23" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W23" s="19">
         <f t="shared" si="2"/>
-        <v>55</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -4112,11 +4223,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>96274.990000000063</v>
+        <v>96574.790000000066</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>43725.009999999937</v>
+        <v>43425.209999999934</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4148,11 +4259,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>549681.20999999973</v>
+        <v>550898.80999999971</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>69636.971818182152</v>
+        <v>68419.371818182175</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4167,11 +4278,11 @@
       </c>
       <c r="V24" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="W24" s="19">
         <f t="shared" si="2"/>
-        <v>37</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -4187,11 +4298,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>84553.079999999842</v>
+        <v>84866.179999999833</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>57946.920000000158</v>
+        <v>57633.820000000167</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4206,11 +4317,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>649.5</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2690</v>
+        <v>2040.5</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4242,11 +4353,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>51</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4306,11 +4417,11 @@
       </c>
       <c r="V26" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="W26" s="19">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -4372,11 +4483,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>236192.97000000015</v>
+        <v>236192.96999999977</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>82307.029999999853</v>
+        <v>82307.030000000232</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4405,11 +4516,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>87483.25999999998</v>
+        <v>87483.259999999951</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>87516.74000000002</v>
+        <v>87516.740000000049</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4508,11 +4619,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>116320.90999999996</v>
+        <v>116320.90999999995</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50679.09000000004</v>
+        <v>50679.090000000055</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4525,11 +4636,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>270334.03999999998</v>
+        <v>270334.04000000004</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>120415.96000000002</v>
+        <v>120415.95999999996</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -4628,11 +4739,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>58341.390000000087</v>
+        <v>58990.890000000087</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41658.609999999913</v>
+        <v>41009.109999999913</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4645,11 +4756,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>700067.99000000325</v>
+        <v>700067.9900000022</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>-48817.99000000325</v>
+        <v>-48817.990000002203</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4668,11 +4779,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>-11.727272727272748</v>
+        <v>-15.727272727272748</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4705,11 +4816,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>432871.03500000184</v>
+        <v>435780.93500000192</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>218378.96499999816</v>
+        <v>215469.06499999808</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4748,11 +4859,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52844.85</v>
+        <v>52844.850000000006</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>20155.150000000001</v>
+        <v>20155.149999999994</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -4908,11 +5019,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>545683.80000000168</v>
+        <v>545683.80000000156</v>
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>-154933.80000000168</v>
+        <v>-154933.80000000156</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -4980,11 +5091,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1386417.7799999891</v>
+        <v>1386417.7799999914</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>-735167.77999998908</v>
+        <v>-735167.77999999141</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -5016,11 +5127,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>982806.13500000234</v>
+        <v>986933.63500000199</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-331556.13500000234</v>
+        <v>-335683.63500000199</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 23/07/2026 10:42
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F98E042-6379-462D-AB8A-CD0DE687FABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527F4460-41A3-4906-A5C4-F1A616BC9DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1730,13 +1730,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>39246.379999999976</v>
+            <v>39704.279999999977</v>
           </cell>
           <cell r="H5" t="str">
-            <v>INDAIATUBA</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>119.9</v>
+            <v>457.9</v>
           </cell>
         </row>
         <row r="6">
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>260716.2799999995</v>
+            <v>265155.72999999957</v>
           </cell>
           <cell r="H6" t="str">
-            <v>INTERLAGOS</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>158</v>
+            <v>4439.45</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1764,10 +1764,10 @@
             <v>1082.83</v>
           </cell>
           <cell r="H7" t="str">
-            <v>KEY ABC</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>1217.5999999999999</v>
+            <v>602.70000000000005</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1784,16 +1784,16 @@
             <v>151.09</v>
           </cell>
           <cell r="H8" t="str">
-            <v>LESTE</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>1019.85</v>
+            <v>4897.0999999999995</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="N8">
-            <v>23</v>
+            <v>24</v>
           </cell>
         </row>
         <row r="9">
@@ -1801,19 +1801,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>51318.109999999993</v>
+            <v>51800.909999999996</v>
           </cell>
           <cell r="H9" t="str">
-            <v>LESTE MOOCA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>349.75</v>
+            <v>509.6</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>41</v>
+            <v>44</v>
           </cell>
         </row>
         <row r="10">
@@ -1821,19 +1821,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>175610.38999999984</v>
+            <v>179685.48999999987</v>
           </cell>
           <cell r="H10" t="str">
-            <v>LESTE PENHA</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>299.8</v>
+            <v>15911.699999999997</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>33</v>
+            <v>34</v>
           </cell>
         </row>
         <row r="11">
@@ -1841,13 +1841,13 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>51759.880000000063</v>
+            <v>52269.480000000069</v>
           </cell>
           <cell r="H11" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>KEY PIRACICABA</v>
           </cell>
           <cell r="I11">
-            <v>313.10000000000002</v>
+            <v>16526.2</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1861,19 +1861,19 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>212847.61999999997</v>
+            <v>227541.71999999991</v>
           </cell>
           <cell r="H12" t="str">
-            <v>SJC</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I12">
-            <v>649.5</v>
+            <v>4583.4400000000005</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="N12">
-            <v>19</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="13">
@@ -1884,10 +1884,10 @@
             <v>263985.40000000084</v>
           </cell>
           <cell r="H13" t="str">
-            <v>Total Geral</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I13">
-            <v>4127.5</v>
+            <v>3534.2</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1903,11 +1903,17 @@
           <cell r="F14">
             <v>851393.40000000026</v>
           </cell>
+          <cell r="H14" t="str">
+            <v>LESTE</v>
+          </cell>
+          <cell r="I14">
+            <v>1019.85</v>
+          </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>48</v>
+            <v>49</v>
           </cell>
         </row>
         <row r="15">
@@ -1915,7 +1921,13 @@
             <v>KEY PIRACICABA</v>
           </cell>
           <cell r="F15">
-            <v>87483.259999999951</v>
+            <v>104009.45999999996</v>
+          </cell>
+          <cell r="H15" t="str">
+            <v>LESTE MOOCA</v>
+          </cell>
+          <cell r="I15">
+            <v>553.65</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1931,6 +1943,12 @@
           <cell r="F16">
             <v>114220.90000000004</v>
           </cell>
+          <cell r="H16" t="str">
+            <v>LESTE PENHA</v>
+          </cell>
+          <cell r="I16">
+            <v>607.15</v>
+          </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
@@ -1943,13 +1961,19 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>266913.34999999992</v>
+            <v>271496.78999999992</v>
+          </cell>
+          <cell r="H17" t="str">
+            <v>LESTE TATUAPE</v>
+          </cell>
+          <cell r="I17">
+            <v>313.10000000000002</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="N17">
-            <v>35</v>
+            <v>36</v>
           </cell>
         </row>
         <row r="18">
@@ -1957,13 +1981,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>278371.99999999994</v>
+            <v>281906.1999999999</v>
+          </cell>
+          <cell r="H18" t="str">
+            <v>MOGI</v>
+          </cell>
+          <cell r="I18">
+            <v>1194.25</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>40</v>
+            <v>42</v>
           </cell>
         </row>
         <row r="19">
@@ -1971,7 +2001,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>73484.23</v>
+            <v>73484.229999999981</v>
+          </cell>
+          <cell r="H19" t="str">
+            <v>NORTE</v>
+          </cell>
+          <cell r="I19">
+            <v>8708.3000000000011</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -1985,7 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>134203.51499999966</v>
+            <v>134407.41499999966</v>
+          </cell>
+          <cell r="H20" t="str">
+            <v>OSASCO</v>
+          </cell>
+          <cell r="I20">
+            <v>4072.88</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
@@ -1999,7 +2041,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>96574.790000000066</v>
+            <v>96686.940000000075</v>
+          </cell>
+          <cell r="H21" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="I21">
+            <v>1483.2</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
@@ -2015,6 +2063,12 @@
           <cell r="F22">
             <v>84866.179999999833</v>
           </cell>
+          <cell r="H22" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="I22">
+            <v>1028.2</v>
+          </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
           </cell>
@@ -2027,7 +2081,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>49159.000000000095</v>
+            <v>50130.750000000102</v>
+          </cell>
+          <cell r="H23" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I23">
+            <v>1072.3</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
@@ -2041,7 +2101,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>163165.17999999976</v>
+            <v>171873.47999999969</v>
+          </cell>
+          <cell r="H24" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I24">
+            <v>521.16000000000008</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
@@ -2055,13 +2121,19 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>236192.96999999977</v>
+            <v>240265.84999999945</v>
+          </cell>
+          <cell r="H25" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I25">
+            <v>72036.330000000031</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>573</v>
+            <v>584</v>
           </cell>
         </row>
         <row r="26">
@@ -2069,7 +2141,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>92708.429999999935</v>
+            <v>94191.629999999932</v>
           </cell>
         </row>
         <row r="27">
@@ -2085,7 +2157,7 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>179510.92999999985</v>
+            <v>179510.92999999982</v>
           </cell>
         </row>
         <row r="29">
@@ -2093,7 +2165,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>58990.890000000087</v>
+            <v>59369.590000000084</v>
           </cell>
         </row>
         <row r="30">
@@ -2101,7 +2173,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>29667.840000000015</v>
+            <v>30740.140000000014</v>
           </cell>
         </row>
         <row r="31">
@@ -2109,7 +2181,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>52844.850000000006</v>
+            <v>53366.009999999995</v>
           </cell>
         </row>
         <row r="32">
@@ -2117,7 +2189,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4022790.604999952</v>
+            <v>4089617.73499995</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -2968,7 +3040,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4022790.6049999995</v>
+        <v>4089617.734999998</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -2979,7 +3051,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>2909.9</v>
+        <v>31480.79</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -2990,7 +3062,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>1217.5999999999999</v>
+        <v>24029.339999999997</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3001,7 +3073,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>573</v>
+        <v>584</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3013,7 +3085,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1569709.3950000005</v>
+        <v>1502882.265000002</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3024,7 +3096,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>127090.1</v>
+        <v>98519.209999999992</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3035,7 +3107,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-1217.5999999999999</v>
+        <v>-24029.339999999997</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3046,7 +3118,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3058,7 +3130,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.71931883862315593</v>
+        <v>0.7312682583817609</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3069,7 +3141,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>2.2383846153846143E-2</v>
+        <v>0.24215992307692313</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3091,7 +3163,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.75593667546174137</v>
+        <v>0.77044854881266489</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3190,11 +3262,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>39246.379999999976</v>
+        <v>39704.279999999977</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>25253.620000000024</v>
+        <v>24795.720000000023</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3209,11 +3281,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4072.88</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12090</v>
+        <v>8017.12</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3244,11 +3316,11 @@
       </c>
       <c r="V10" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W10" s="19">
         <f>U10-V10</f>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -3264,11 +3336,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>260716.2799999995</v>
+        <v>265155.72999999957</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>64283.720000000496</v>
+        <v>59844.270000000426</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3283,11 +3355,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>8708.3000000000011</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11000</v>
+        <v>2291.6999999999989</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3302,11 +3374,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1217.5999999999999</v>
+        <v>15911.699999999997</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>-1217.5999999999999</v>
+        <v>-15911.699999999997</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3321,11 +3393,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3359,11 +3431,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1483.2</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5400</v>
+        <v>3916.8</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3397,11 +3469,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3417,11 +3489,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51318.109999999993</v>
+        <v>51800.909999999996</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>38681.890000000007</v>
+        <v>38199.090000000004</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3455,11 +3527,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>3534.2</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>0</v>
+        <v>-3534.2</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3494,11 +3566,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>175610.38999999984</v>
+        <v>179685.48999999987</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>97389.610000000161</v>
+        <v>93314.510000000126</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3551,11 +3623,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3571,11 +3643,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51759.880000000063</v>
+        <v>52269.480000000069</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>26240.119999999937</v>
+        <v>25730.519999999931</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3590,11 +3662,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4439.45</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15000</v>
+        <v>10560.55</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3609,11 +3681,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4583.4400000000005</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-4583.4400000000005</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3648,11 +3720,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>212847.61999999997</v>
+        <v>227541.71999999991</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>112152.38000000003</v>
+        <v>97458.280000000086</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3705,11 +3777,11 @@
       </c>
       <c r="V16" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W16" s="19">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3744,11 +3816,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1194.25</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4850</v>
+        <v>3655.75</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3782,11 +3854,11 @@
       </c>
       <c r="V17" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="W17" s="19">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3846,11 +3918,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3885,11 +3957,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>349.75</v>
+        <v>553.65</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6770.25</v>
+        <v>6566.35</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3926,11 +3998,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>266913.34999999992</v>
+        <v>271496.78999999992</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>293086.65000000008</v>
+        <v>288503.21000000008</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -3945,11 +4017,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>158</v>
+        <v>4897.0999999999995</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>14842</v>
+        <v>10102.900000000001</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -3998,11 +4070,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>278371.99999999994</v>
+        <v>281906.1999999999</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>136628.00000000006</v>
+        <v>133093.8000000001</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4017,11 +4089,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>509.6</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5100</v>
+        <v>4590.3999999999996</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4073,11 +4145,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>73484.23</v>
+        <v>73484.229999999981</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>48515.770000000004</v>
+        <v>48515.770000000019</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4092,11 +4164,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>299.8</v>
+        <v>607.15</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3020.2</v>
+        <v>2712.85</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4148,11 +4220,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>134203.51499999966</v>
+        <v>134407.41499999966</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>60796.485000000335</v>
+        <v>60592.585000000341</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4167,11 +4239,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>119.9</v>
+        <v>602.70000000000005</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3890.1</v>
+        <v>3407.3</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4184,11 +4256,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>685907.54999999946</v>
+        <v>685907.54999999935</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-66589.368181817583</v>
+        <v>-66589.368181817466</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4223,11 +4295,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>96574.790000000066</v>
+        <v>96686.940000000075</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>43425.209999999934</v>
+        <v>43313.059999999925</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4242,11 +4314,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>521.16000000000008</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4700</v>
+        <v>4178.84</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4259,11 +4331,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>550898.80999999971</v>
+        <v>590236.74999999977</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>68419.371818182175</v>
+        <v>29081.431818182115</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4317,11 +4389,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>649.5</v>
+        <v>1028.2</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2040.5</v>
+        <v>1661.8</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4373,11 +4445,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>49159.000000000095</v>
+        <v>50130.750000000102</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40840.999999999905</v>
+        <v>39869.249999999898</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4392,11 +4464,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>1072.3</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3530</v>
+        <v>2457.6999999999998</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4437,11 +4509,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>163165.17999999976</v>
+        <v>171873.47999999969</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>74334.82000000024</v>
+        <v>65626.52000000031</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4456,11 +4528,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>457.9</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2670</v>
+        <v>2212.1</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4483,11 +4555,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>236192.96999999977</v>
+        <v>240265.84999999945</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>82307.030000000232</v>
+        <v>78234.150000000547</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4516,11 +4588,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>87483.259999999951</v>
+        <v>104009.45999999996</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>87516.740000000049</v>
+        <v>70990.540000000037</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4562,11 +4634,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>92708.429999999935</v>
+        <v>94191.629999999932</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41791.570000000065</v>
+        <v>40308.370000000068</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4679,11 +4751,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>179510.92999999985</v>
+        <v>179510.92999999982</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>80489.070000000153</v>
+        <v>80489.070000000182</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4696,11 +4768,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>540157.79000000341</v>
+        <v>539962.59000000334</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="4">I32-J32</f>
-        <v>-19157.790000003413</v>
+        <v>-18962.590000003343</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -4739,11 +4811,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>58990.890000000087</v>
+        <v>59369.590000000084</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>41009.109999999913</v>
+        <v>40630.409999999916</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4756,11 +4828,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>700067.9900000022</v>
+        <v>699181.49000000209</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>-48817.990000002203</v>
+        <v>-47931.490000002086</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4779,11 +4851,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>-15.727272727272748</v>
+        <v>-29.727272727272748</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4799,11 +4871,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29667.840000000015</v>
+        <v>30740.140000000014</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>25332.159999999985</v>
+        <v>24259.859999999986</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4816,11 +4888,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>435780.93500000192</v>
+        <v>464351.82500000199</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>215469.06499999808</v>
+        <v>186898.17499999801</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4859,11 +4931,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52844.850000000006</v>
+        <v>53366.009999999995</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>20155.149999999994</v>
+        <v>19633.990000000005</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5055,11 +5127,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1103755.3899999962</v>
+        <v>1103560.1899999958</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="5">C41-D41</f>
-        <v>-582755.38999999617</v>
+        <v>-582560.18999999575</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -5091,11 +5163,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1386417.7799999914</v>
+        <v>1385531.2799999914</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>-735167.77999999141</v>
+        <v>-734281.27999999141</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -5127,11 +5199,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>986933.63500000199</v>
+        <v>1054842.4650000024</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-335683.63500000199</v>
+        <v>-403592.46500000241</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 23/07/2026 11:57
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527F4460-41A3-4906-A5C4-F1A616BC9DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DDD1AB1-829A-454D-BB39-CCF1FE331BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>265155.72999999957</v>
+            <v>267402.02999999956</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>4439.45</v>
+            <v>6685.7500000000009</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1787,7 +1787,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>4897.0999999999995</v>
+            <v>7772.1999999999989</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1801,7 +1801,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>51800.909999999996</v>
+            <v>51909.509999999995</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
@@ -1821,7 +1821,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>179685.48999999987</v>
+            <v>182570.58999999982</v>
           </cell>
           <cell r="H10" t="str">
             <v>KEY ABC</v>
@@ -1844,16 +1844,16 @@
             <v>52269.480000000069</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY PIRACICABA</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="I11">
-            <v>16526.2</v>
+            <v>4507.2</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="N11">
-            <v>50</v>
+            <v>52</v>
           </cell>
         </row>
         <row r="12">
@@ -1864,10 +1864,10 @@
             <v>227541.71999999991</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY SP</v>
+            <v>KEY PIRACICABA</v>
           </cell>
           <cell r="I12">
-            <v>4583.4400000000005</v>
+            <v>16526.2</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1881,13 +1881,13 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>263985.40000000084</v>
+            <v>267282.20000000083</v>
           </cell>
           <cell r="H13" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I13">
-            <v>3534.2</v>
+            <v>16606.490000000002</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -1904,10 +1904,10 @@
             <v>851393.40000000026</v>
           </cell>
           <cell r="H14" t="str">
-            <v>LESTE</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I14">
-            <v>1019.85</v>
+            <v>3534.2</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
@@ -1924,10 +1924,10 @@
             <v>104009.45999999996</v>
           </cell>
           <cell r="H15" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I15">
-            <v>553.65</v>
+            <v>1030.8499999999999</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1944,10 +1944,10 @@
             <v>114220.90000000004</v>
           </cell>
           <cell r="H16" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I16">
-            <v>607.15</v>
+            <v>553.65</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1961,13 +1961,13 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>271496.78999999992</v>
+            <v>283519.83999999997</v>
           </cell>
           <cell r="H17" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I17">
-            <v>313.10000000000002</v>
+            <v>966.94999999999993</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1984,10 +1984,10 @@
             <v>281906.1999999999</v>
           </cell>
           <cell r="H18" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I18">
-            <v>1194.25</v>
+            <v>932.7</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -2001,13 +2001,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>73484.229999999981</v>
+            <v>73495.229999999981</v>
           </cell>
           <cell r="H19" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I19">
-            <v>8708.3000000000011</v>
+            <v>2622.35</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -2021,13 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>134407.41499999966</v>
+            <v>134433.21499999968</v>
           </cell>
           <cell r="H20" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I20">
-            <v>4072.88</v>
+            <v>10871.329999999998</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
@@ -2041,13 +2041,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>96686.940000000075</v>
+            <v>97046.740000000093</v>
           </cell>
           <cell r="H21" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I21">
-            <v>1483.2</v>
+            <v>6088.8799999999992</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
@@ -2061,13 +2061,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>84866.179999999833</v>
+            <v>85485.779999999824</v>
           </cell>
           <cell r="H22" t="str">
-            <v>SJC</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I22">
-            <v>1028.2</v>
+            <v>1646.5</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
@@ -2081,19 +2081,19 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>50130.750000000102</v>
+            <v>51458.900000000111</v>
           </cell>
           <cell r="H23" t="str">
-            <v>SJC/VALE</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I23">
-            <v>1072.3</v>
+            <v>4445.28</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
           </cell>
           <cell r="N23">
-            <v>21</v>
+            <v>22</v>
           </cell>
         </row>
         <row r="24">
@@ -2101,13 +2101,13 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>171873.47999999969</v>
+            <v>174036.50999999969</v>
           </cell>
           <cell r="H24" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SBC</v>
           </cell>
           <cell r="I24">
-            <v>521.16000000000008</v>
+            <v>3647.91</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
@@ -2121,19 +2121,19 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>240265.84999999945</v>
+            <v>242282.50999999946</v>
           </cell>
           <cell r="H25" t="str">
-            <v>Total Geral</v>
+            <v>SJC</v>
           </cell>
           <cell r="I25">
-            <v>72036.330000000031</v>
+            <v>2136.54</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>584</v>
+            <v>587</v>
           </cell>
         </row>
         <row r="26">
@@ -2141,7 +2141,13 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>94191.629999999932</v>
+            <v>94354.929999999935</v>
+          </cell>
+          <cell r="H26" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="I26">
+            <v>1072.3</v>
           </cell>
         </row>
         <row r="27">
@@ -2149,7 +2155,13 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>116320.90999999995</v>
+            <v>120766.18999999997</v>
+          </cell>
+          <cell r="H27" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="I27">
+            <v>521.16000000000008</v>
           </cell>
         </row>
         <row r="28">
@@ -2157,7 +2169,13 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>179510.92999999982</v>
+            <v>183158.83999999976</v>
+          </cell>
+          <cell r="H28" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I28">
+            <v>109650.34000000003</v>
           </cell>
         </row>
         <row r="29">
@@ -2165,7 +2183,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>59369.590000000084</v>
+            <v>60477.930000000088</v>
           </cell>
         </row>
         <row r="30">
@@ -2181,7 +2199,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>53366.009999999995</v>
+            <v>53366.01</v>
           </cell>
         </row>
         <row r="32">
@@ -2189,7 +2207,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4089617.73499995</v>
+            <v>4126066.4549999475</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3040,7 +3058,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4089617.734999998</v>
+        <v>4126066.4549999996</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3051,7 +3069,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>31480.79</v>
+        <v>52564.549999999996</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3062,7 +3080,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>24029.339999999997</v>
+        <v>40559.589999999997</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3073,7 +3091,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3085,7 +3103,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1502882.265000002</v>
+        <v>1466433.5450000004</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3096,7 +3114,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>98519.209999999992</v>
+        <v>77435.450000000012</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3107,7 +3125,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-24029.339999999997</v>
+        <v>-40559.589999999997</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3118,7 +3136,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3130,7 +3148,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.7312682583817609</v>
+        <v>0.73778568708091186</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3141,7 +3159,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.24215992307692313</v>
+        <v>0.40434269230769226</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3163,7 +3181,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.77044854881266489</v>
+        <v>0.77440633245382584</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3281,11 +3299,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4072.88</v>
+        <v>6088.8799999999992</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8017.12</v>
+        <v>6001.1200000000008</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3336,11 +3354,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>265155.72999999957</v>
+        <v>267402.02999999956</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>59844.270000000426</v>
+        <v>57597.970000000438</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3355,11 +3373,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8708.3000000000011</v>
+        <v>10871.329999999998</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2291.6999999999989</v>
+        <v>128.67000000000189</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3431,11 +3449,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1483.2</v>
+        <v>1646.5</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3916.8</v>
+        <v>3753.5</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3489,11 +3507,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51800.909999999996</v>
+        <v>51909.509999999995</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>38199.090000000004</v>
+        <v>38090.490000000005</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3508,11 +3526,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>3647.91</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>13000</v>
+        <v>9352.09</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3546,11 +3564,11 @@
       </c>
       <c r="V13" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="W13" s="19">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -3566,11 +3584,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>179685.48999999987</v>
+        <v>182570.58999999982</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>93314.510000000126</v>
+        <v>90429.410000000178</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3585,11 +3603,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>313.10000000000002</v>
+        <v>932.7</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3526.9</v>
+        <v>2907.3</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3662,11 +3680,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4439.45</v>
+        <v>6685.7500000000009</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10560.55</v>
+        <v>8314.25</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3681,11 +3699,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4583.4400000000005</v>
+        <v>16606.490000000002</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-4583.4400000000005</v>
+        <v>-16606.490000000002</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3739,11 +3757,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4445.28</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9840</v>
+        <v>5394.72</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3797,11 +3815,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>263985.40000000084</v>
+        <v>267282.20000000083</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-93985.400000000838</v>
+        <v>-97282.200000000827</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3816,11 +3834,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1194.25</v>
+        <v>2622.35</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3655.75</v>
+        <v>2227.65</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3835,11 +3853,11 @@
       </c>
       <c r="P17" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>0</v>
+        <v>4507.2</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-4507.2</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="19" t="s">
@@ -3893,11 +3911,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1019.85</v>
+        <v>1030.8499999999999</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5820.15</v>
+        <v>5809.15</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3998,11 +4016,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>271496.78999999992</v>
+        <v>283519.83999999997</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>288503.21000000008</v>
+        <v>276480.16000000003</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -4017,11 +4035,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4897.0999999999995</v>
+        <v>7772.1999999999989</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10102.900000000001</v>
+        <v>7227.8000000000011</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4145,11 +4163,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>73484.229999999981</v>
+        <v>73495.229999999981</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>48515.770000000019</v>
+        <v>48504.770000000019</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4164,11 +4182,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>607.15</v>
+        <v>966.94999999999993</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2712.85</v>
+        <v>2353.0500000000002</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4220,11 +4238,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>134407.41499999966</v>
+        <v>134433.21499999968</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>60592.585000000341</v>
+        <v>60566.785000000324</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4256,11 +4274,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>685907.54999999935</v>
+        <v>684697.14999999932</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>-66589.368181817466</v>
+        <v>-65378.968181817443</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="19" t="s">
@@ -4295,11 +4313,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>96686.940000000075</v>
+        <v>97046.740000000093</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>43313.059999999925</v>
+        <v>42953.259999999907</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4331,11 +4349,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>590236.74999999977</v>
+        <v>606766.99999999977</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>29081.431818182115</v>
+        <v>12551.181818182115</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4350,11 +4368,11 @@
       </c>
       <c r="V24" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W24" s="19">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -4370,11 +4388,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>84866.179999999833</v>
+        <v>85485.779999999824</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>57633.820000000167</v>
+        <v>57014.220000000176</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4389,11 +4407,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1028.2</v>
+        <v>2136.54</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1661.8</v>
+        <v>553.46</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4445,11 +4463,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>50130.750000000102</v>
+        <v>51458.900000000111</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>39869.249999999898</v>
+        <v>38541.099999999889</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4509,11 +4527,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>171873.47999999969</v>
+        <v>174036.50999999969</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65626.52000000031</v>
+        <v>63463.490000000311</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4555,11 +4573,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>240265.84999999945</v>
+        <v>242282.50999999946</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>78234.150000000547</v>
+        <v>76217.490000000544</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4634,11 +4652,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>94191.629999999932</v>
+        <v>94354.929999999935</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40308.370000000068</v>
+        <v>40145.070000000065</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4691,11 +4709,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>116320.90999999995</v>
+        <v>120766.18999999997</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50679.090000000055</v>
+        <v>46233.810000000027</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4751,11 +4769,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>179510.92999999982</v>
+        <v>183158.83999999976</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>80489.070000000182</v>
+        <v>76841.160000000236</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4811,11 +4829,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>59369.590000000084</v>
+        <v>60477.930000000088</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40630.409999999916</v>
+        <v>39522.069999999912</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4828,11 +4846,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>699181.49000000209</v>
+        <v>699081.54000000213</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="4"/>
-        <v>-47931.490000002086</v>
+        <v>-47831.540000002133</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -4851,11 +4869,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>-29.727272727272748</v>
+        <v>-39.727272727272748</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4888,11 +4906,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>464351.82500000199</v>
+        <v>485580.64500000241</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>186898.17499999801</v>
+        <v>165669.35499999759</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4931,11 +4949,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>53366.009999999995</v>
+        <v>53366.01</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>19633.990000000005</v>
+        <v>19633.989999999998</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5163,11 +5181,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>1385531.2799999914</v>
+        <v>1384220.9299999916</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="5"/>
-        <v>-734281.27999999141</v>
+        <v>-732970.92999999155</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -5199,11 +5217,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1054842.4650000024</v>
+        <v>1092601.5350000008</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-403592.46500000241</v>
+        <v>-441351.53500000085</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 23/07/2026 13:31
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DDD1AB1-829A-454D-BB39-CCF1FE331BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38BAB39-E347-47E9-892C-61C0AAB0B2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1730,13 +1730,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>39704.279999999977</v>
+            <v>41266.429999999978</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>457.9</v>
+            <v>2020.05</v>
           </cell>
         </row>
         <row r="6">
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>267402.02999999956</v>
+            <v>272023.67999999953</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>6685.7500000000009</v>
+            <v>11307.4</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1787,13 +1787,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>7772.1999999999989</v>
+            <v>11574.8</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="N8">
-            <v>24</v>
+            <v>25</v>
           </cell>
         </row>
         <row r="9">
@@ -1801,19 +1801,19 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>51909.509999999995</v>
+            <v>51909.51</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>509.6</v>
+            <v>1261.6000000000001</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="N9">
-            <v>44</v>
+            <v>45</v>
           </cell>
         </row>
         <row r="10">
@@ -1821,13 +1821,13 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>182570.58999999982</v>
+            <v>186373.18999999983</v>
           </cell>
           <cell r="H10" t="str">
             <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>15911.699999999997</v>
+            <v>30672.1</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1841,7 +1841,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>52269.480000000069</v>
+            <v>53021.480000000069</v>
           </cell>
           <cell r="H11" t="str">
             <v>KEY CASA</v>
@@ -1861,13 +1861,13 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>227541.71999999991</v>
+            <v>242302.11999999994</v>
           </cell>
           <cell r="H12" t="str">
             <v>KEY PIRACICABA</v>
           </cell>
           <cell r="I12">
-            <v>16526.2</v>
+            <v>18252.82</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
@@ -1881,7 +1881,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>267282.20000000083</v>
+            <v>267282.20000000024</v>
           </cell>
           <cell r="H13" t="str">
             <v>KEY SP</v>
@@ -1893,7 +1893,7 @@
             <v>LESTE</v>
           </cell>
           <cell r="N13">
-            <v>30</v>
+            <v>31</v>
           </cell>
         </row>
         <row r="14">
@@ -1907,13 +1907,13 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="I14">
-            <v>3534.2</v>
+            <v>9288.7000000000007</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="N14">
-            <v>49</v>
+            <v>50</v>
           </cell>
         </row>
         <row r="15">
@@ -1921,13 +1921,13 @@
             <v>KEY PIRACICABA</v>
           </cell>
           <cell r="F15">
-            <v>104009.45999999996</v>
+            <v>105736.07999999996</v>
           </cell>
           <cell r="H15" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="I15">
-            <v>1030.8499999999999</v>
+            <v>1709.3500000000001</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1947,13 +1947,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I16">
-            <v>553.65</v>
+            <v>2753.39</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="N16">
-            <v>36</v>
+            <v>38</v>
           </cell>
         </row>
         <row r="17">
@@ -1981,19 +1981,19 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>281906.1999999999</v>
+            <v>287660.6999999999</v>
           </cell>
           <cell r="H18" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I18">
-            <v>932.7</v>
+            <v>1628.2500000000002</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="N18">
-            <v>42</v>
+            <v>43</v>
           </cell>
         </row>
         <row r="19">
@@ -2001,13 +2001,13 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>73495.229999999981</v>
+            <v>74173.729999999981</v>
           </cell>
           <cell r="H19" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="I19">
-            <v>2622.35</v>
+            <v>2791.9200000000005</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
@@ -2021,13 +2021,13 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>134433.21499999968</v>
+            <v>136632.95499999967</v>
           </cell>
           <cell r="H20" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="I20">
-            <v>10871.329999999998</v>
+            <v>14091.089999999997</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
@@ -2047,13 +2047,13 @@
             <v>OSASCO</v>
           </cell>
           <cell r="I21">
-            <v>6088.8799999999992</v>
+            <v>8158.1999999999971</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="N21">
-            <v>27</v>
+            <v>28</v>
           </cell>
         </row>
         <row r="22">
@@ -2061,19 +2061,19 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>85485.779999999824</v>
+            <v>86181.329999999798</v>
           </cell>
           <cell r="H22" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I22">
-            <v>1646.5</v>
+            <v>2935.4000000000005</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
           </cell>
           <cell r="N22">
-            <v>35</v>
+            <v>36</v>
           </cell>
         </row>
         <row r="23">
@@ -2081,13 +2081,13 @@
             <v>MOGI</v>
           </cell>
           <cell r="F23">
-            <v>51458.900000000111</v>
+            <v>51628.47000000011</v>
           </cell>
           <cell r="H23" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I23">
-            <v>4445.28</v>
+            <v>6971.079999999999</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
@@ -2101,19 +2101,19 @@
             <v>NORTE</v>
           </cell>
           <cell r="F24">
-            <v>174036.50999999969</v>
+            <v>177256.26999999961</v>
           </cell>
           <cell r="H24" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I24">
-            <v>3647.91</v>
+            <v>5803.97</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="N24">
-            <v>23</v>
+            <v>25</v>
           </cell>
         </row>
         <row r="25">
@@ -2121,19 +2121,19 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>242282.50999999946</v>
+            <v>244351.82999999938</v>
           </cell>
           <cell r="H25" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I25">
-            <v>2136.54</v>
+            <v>2448.94</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>587</v>
+            <v>598</v>
           </cell>
         </row>
         <row r="26">
@@ -2141,13 +2141,13 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>94354.929999999935</v>
+            <v>95643.829999999944</v>
           </cell>
           <cell r="H26" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I26">
-            <v>1072.3</v>
+            <v>1615.8200000000004</v>
           </cell>
         </row>
         <row r="27">
@@ -2155,7 +2155,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>120766.18999999997</v>
+            <v>123291.98999999996</v>
           </cell>
           <cell r="H27" t="str">
             <v>VENDEDOR INTERNO 1</v>
@@ -2169,13 +2169,13 @@
             <v>SBC</v>
           </cell>
           <cell r="F28">
-            <v>183158.83999999976</v>
+            <v>185314.89999999973</v>
           </cell>
           <cell r="H28" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I28">
-            <v>109650.34000000003</v>
+            <v>158489.38</v>
           </cell>
         </row>
         <row r="29">
@@ -2183,7 +2183,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>60477.930000000088</v>
+            <v>60790.330000000104</v>
           </cell>
         </row>
         <row r="30">
@@ -2191,7 +2191,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>30740.140000000014</v>
+            <v>31283.660000000022</v>
           </cell>
         </row>
         <row r="31">
@@ -2207,7 +2207,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4126066.4549999475</v>
+            <v>4174905.4949999442</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4126066.4549999996</v>
+        <v>4174905.4949999982</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>52564.549999999996</v>
+        <v>79162.070000000007</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>40559.589999999997</v>
+        <v>61074.490000000005</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>587</v>
+        <v>598</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1466433.5450000004</v>
+        <v>1417594.5050000018</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>77435.450000000012</v>
+        <v>50837.929999999993</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-40559.589999999997</v>
+        <v>-61074.490000000005</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.73778568708091186</v>
+        <v>0.74651864014304836</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.40434269230769226</v>
+        <v>0.60893900000000012</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.77440633245382584</v>
+        <v>0.78891820580474936</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3280,11 +3280,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>39704.279999999977</v>
+        <v>41266.429999999978</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>24795.720000000023</v>
+        <v>23233.570000000022</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3299,11 +3299,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6088.8799999999992</v>
+        <v>8158.1999999999971</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6001.1200000000008</v>
+        <v>3931.8000000000029</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3334,11 +3334,11 @@
       </c>
       <c r="V10" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="W10" s="19">
         <f>U10-V10</f>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -3354,11 +3354,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>267402.02999999956</v>
+        <v>272023.67999999953</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>57597.970000000438</v>
+        <v>52976.320000000473</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3373,11 +3373,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10871.329999999998</v>
+        <v>14091.089999999997</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>128.67000000000189</v>
+        <v>-3091.0899999999965</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3392,11 +3392,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>15911.699999999997</v>
+        <v>30672.1</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>-15911.699999999997</v>
+        <v>-30672.1</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3411,11 +3411,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3449,11 +3449,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1646.5</v>
+        <v>2935.4000000000005</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3753.5</v>
+        <v>2464.5999999999995</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3507,11 +3507,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51909.509999999995</v>
+        <v>51909.51</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>38090.490000000005</v>
+        <v>38090.49</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3526,11 +3526,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3647.91</v>
+        <v>5803.97</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9352.09</v>
+        <v>7196.03</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3534.2</v>
+        <v>9288.7000000000007</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-3534.2</v>
+        <v>-9288.7000000000007</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3584,11 +3584,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>182570.58999999982</v>
+        <v>186373.18999999983</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>90429.410000000178</v>
+        <v>86626.810000000172</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3603,11 +3603,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>932.7</v>
+        <v>1628.2500000000002</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2907.3</v>
+        <v>2211.75</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3661,11 +3661,11 @@
       </c>
       <c r="D15" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52269.480000000069</v>
+        <v>53021.480000000069</v>
       </c>
       <c r="E15" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>25730.519999999931</v>
+        <v>24978.519999999931</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="21" t="s">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6685.7500000000009</v>
+        <v>11307.4</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>8314.25</v>
+        <v>3692.6000000000004</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3718,11 +3718,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3738,11 +3738,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>227541.71999999991</v>
+        <v>242302.11999999994</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>97458.280000000086</v>
+        <v>82697.880000000063</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3757,11 +3757,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4445.28</v>
+        <v>6971.079999999999</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5394.72</v>
+        <v>2868.920000000001</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>267282.20000000083</v>
+        <v>267282.20000000024</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-97282.200000000827</v>
+        <v>-97282.200000000244</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3834,11 +3834,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2622.35</v>
+        <v>2791.9200000000005</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2227.65</v>
+        <v>2058.0799999999995</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3872,11 +3872,11 @@
       </c>
       <c r="V17" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="W17" s="19">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3911,11 +3911,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1030.8499999999999</v>
+        <v>1709.3500000000001</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5809.15</v>
+        <v>5130.6499999999996</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3936,11 +3936,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3975,11 +3975,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>553.65</v>
+        <v>2753.39</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6566.35</v>
+        <v>4366.6100000000006</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -4035,11 +4035,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7772.1999999999989</v>
+        <v>11574.8</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7227.8000000000011</v>
+        <v>3425.2000000000007</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4088,11 +4088,11 @@
       </c>
       <c r="D21" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>281906.1999999999</v>
+        <v>287660.6999999999</v>
       </c>
       <c r="E21" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>133093.8000000001</v>
+        <v>127339.3000000001</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="21" t="s">
@@ -4107,11 +4107,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>509.6</v>
+        <v>1261.6000000000001</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4590.3999999999996</v>
+        <v>3838.3999999999996</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4163,11 +4163,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>73495.229999999981</v>
+        <v>74173.729999999981</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>48504.770000000019</v>
+        <v>47826.270000000019</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4218,11 +4218,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4238,11 +4238,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>134433.21499999968</v>
+        <v>136632.95499999967</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>60566.785000000324</v>
+        <v>58367.045000000333</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4293,11 +4293,11 @@
       </c>
       <c r="V23" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W23" s="19">
         <f t="shared" si="2"/>
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -4349,11 +4349,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>606766.99999999977</v>
+        <v>629008.51999999967</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>12551.181818182115</v>
+        <v>-9690.3381818177877</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4388,11 +4388,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>85485.779999999824</v>
+        <v>86181.329999999798</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>57014.220000000176</v>
+        <v>56318.670000000202</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4407,11 +4407,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2136.54</v>
+        <v>2448.94</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>553.46</v>
+        <v>241.05999999999995</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4443,11 +4443,11 @@
       </c>
       <c r="V25" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="W25" s="19">
         <f t="shared" si="2"/>
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -4463,11 +4463,11 @@
       </c>
       <c r="D26" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51458.900000000111</v>
+        <v>51628.47000000011</v>
       </c>
       <c r="E26" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>38541.099999999889</v>
+        <v>38371.52999999989</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="21" t="s">
@@ -4482,11 +4482,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1072.3</v>
+        <v>1615.8200000000004</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2457.6999999999998</v>
+        <v>1914.1799999999996</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4507,11 +4507,11 @@
       </c>
       <c r="V26" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="W26" s="19">
         <f t="shared" si="2"/>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
@@ -4527,11 +4527,11 @@
       </c>
       <c r="D27" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>174036.50999999969</v>
+        <v>177256.26999999961</v>
       </c>
       <c r="E27" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>63463.490000000311</v>
+        <v>60243.730000000389</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="21" t="s">
@@ -4546,11 +4546,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>457.9</v>
+        <v>2020.05</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2212.1</v>
+        <v>649.95000000000005</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4573,11 +4573,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>242282.50999999946</v>
+        <v>244351.82999999938</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>76217.490000000544</v>
+        <v>74148.170000000624</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4606,11 +4606,11 @@
       </c>
       <c r="D29" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>104009.45999999996</v>
+        <v>105736.07999999996</v>
       </c>
       <c r="E29" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>70990.540000000037</v>
+        <v>69263.920000000042</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -4652,11 +4652,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>94354.929999999935</v>
+        <v>95643.829999999944</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>40145.070000000065</v>
+        <v>38856.170000000056</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4709,11 +4709,11 @@
       </c>
       <c r="D31" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>120766.18999999997</v>
+        <v>123291.98999999996</v>
       </c>
       <c r="E31" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>46233.810000000027</v>
+        <v>43708.010000000038</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -4769,11 +4769,11 @@
       </c>
       <c r="D32" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>183158.83999999976</v>
+        <v>185314.89999999973</v>
       </c>
       <c r="E32" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>76841.160000000236</v>
+        <v>74685.100000000268</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -4829,11 +4829,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>60477.930000000088</v>
+        <v>60790.330000000104</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>39522.069999999912</v>
+        <v>39209.669999999896</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4869,11 +4869,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>-39.727272727272748</v>
+        <v>-55.727272727272748</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4889,11 +4889,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>30740.140000000014</v>
+        <v>31283.660000000022</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>24259.859999999986</v>
+        <v>23716.339999999978</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4906,11 +4906,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>485580.64500000241</v>
+        <v>512178.16500000301</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>165669.35499999759</v>
+        <v>139071.83499999699</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -5217,11 +5217,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1092601.5350000008</v>
+        <v>1141440.5750000011</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-441351.53500000085</v>
+        <v>-490190.57500000112</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 23/07/2026 14:02
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38BAB39-E347-47E9-892C-61C0AAB0B2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3AA7503-AEC8-416E-B77C-B4F6B1BF2F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1730,13 +1730,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>41266.429999999978</v>
+            <v>41352.389999999978</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>2020.05</v>
+            <v>2106.0099999999998</v>
           </cell>
         </row>
         <row r="6">
@@ -1744,13 +1744,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>272023.67999999953</v>
+            <v>272788.47999999952</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>11307.4</v>
+            <v>12072.2</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1767,7 +1767,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>602.70000000000005</v>
+            <v>1257.3499999999999</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -1787,7 +1787,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>11574.8</v>
+            <v>11655.55</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
@@ -1801,7 +1801,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>51909.51</v>
+            <v>52564.160000000003</v>
           </cell>
           <cell r="H9" t="str">
             <v>JUNDIAI</v>
@@ -1821,19 +1821,19 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>186373.18999999983</v>
+            <v>186453.93999999983</v>
           </cell>
           <cell r="H10" t="str">
             <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>30672.1</v>
+            <v>47946.1</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="N10">
-            <v>34</v>
+            <v>35</v>
           </cell>
         </row>
         <row r="11">
@@ -1861,7 +1861,7 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>242302.11999999994</v>
+            <v>259576.11999999994</v>
           </cell>
           <cell r="H12" t="str">
             <v>KEY PIRACICABA</v>
@@ -1927,7 +1927,7 @@
             <v>LESTE</v>
           </cell>
           <cell r="I15">
-            <v>1709.3500000000001</v>
+            <v>1714.3500000000001</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
@@ -1947,7 +1947,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I16">
-            <v>2753.39</v>
+            <v>4774.07</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -1967,7 +1967,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I17">
-            <v>966.94999999999993</v>
+            <v>1483.75</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
@@ -1987,7 +1987,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I18">
-            <v>1628.2500000000002</v>
+            <v>1758.1500000000003</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
@@ -2001,7 +2001,7 @@
             <v>LESTE</v>
           </cell>
           <cell r="F19">
-            <v>74173.729999999981</v>
+            <v>74178.729999999981</v>
           </cell>
           <cell r="H19" t="str">
             <v>MOGI</v>
@@ -2021,7 +2021,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>136632.95499999967</v>
+            <v>138653.63499999963</v>
           </cell>
           <cell r="H20" t="str">
             <v>NORTE</v>
@@ -2041,13 +2041,13 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>97046.740000000093</v>
+            <v>97563.540000000081</v>
           </cell>
           <cell r="H21" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I21">
-            <v>8158.1999999999971</v>
+            <v>8678.7999999999975</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
@@ -2061,13 +2061,13 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F22">
-            <v>86181.329999999798</v>
+            <v>86311.229999999792</v>
           </cell>
           <cell r="H22" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I22">
-            <v>2935.4000000000005</v>
+            <v>5626.22</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
@@ -2121,7 +2121,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>244351.82999999938</v>
+            <v>244872.42999999938</v>
           </cell>
           <cell r="H25" t="str">
             <v>SJC</v>
@@ -2133,7 +2133,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>598</v>
+            <v>599</v>
           </cell>
         </row>
         <row r="26">
@@ -2141,13 +2141,13 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F26">
-            <v>95643.829999999944</v>
+            <v>98334.649999999921</v>
           </cell>
           <cell r="H26" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I26">
-            <v>1615.8200000000004</v>
+            <v>1620.8200000000004</v>
           </cell>
         </row>
         <row r="27">
@@ -2161,7 +2161,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I27">
-            <v>521.16000000000008</v>
+            <v>839.7600000000001</v>
           </cell>
         </row>
         <row r="28">
@@ -2175,7 +2175,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="I28">
-            <v>158489.38</v>
+            <v>183556.93999999994</v>
           </cell>
         </row>
         <row r="29">
@@ -2191,7 +2191,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>31283.660000000022</v>
+            <v>31288.660000000022</v>
           </cell>
         </row>
         <row r="31">
@@ -2199,7 +2199,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>53366.01</v>
+            <v>53684.61</v>
           </cell>
         </row>
         <row r="32">
@@ -2207,7 +2207,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4174905.4949999442</v>
+            <v>4199973.0549999438</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4174905.4949999982</v>
+        <v>4199973.0549999978</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>79162.070000000007</v>
+        <v>86955.63</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>61074.490000000005</v>
+        <v>78348.490000000005</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1417594.5050000018</v>
+        <v>1392526.9450000022</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>50837.929999999993</v>
+        <v>43044.369999999995</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-61074.490000000005</v>
+        <v>-78348.490000000005</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.74651864014304836</v>
+        <v>0.75100099329459058</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.60893900000000012</v>
+        <v>0.66888946153846152</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.78891820580474936</v>
+        <v>0.79023746701846964</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3280,11 +3280,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>41266.429999999978</v>
+        <v>41352.389999999978</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>23233.570000000022</v>
+        <v>23147.610000000022</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3299,11 +3299,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8158.1999999999971</v>
+        <v>8678.7999999999975</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3931.8000000000029</v>
+        <v>3411.2000000000025</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3354,11 +3354,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>272023.67999999953</v>
+        <v>272788.47999999952</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>52976.320000000473</v>
+        <v>52211.520000000484</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3392,11 +3392,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>30672.1</v>
+        <v>47946.1</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>-30672.1</v>
+        <v>-47946.1</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3449,11 +3449,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2935.4000000000005</v>
+        <v>5626.22</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2464.5999999999995</v>
+        <v>-226.22000000000025</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3487,11 +3487,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3507,11 +3507,11 @@
       </c>
       <c r="D13" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51909.51</v>
+        <v>52564.160000000003</v>
       </c>
       <c r="E13" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>38090.49</v>
+        <v>37435.839999999997</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="21" t="s">
@@ -3584,11 +3584,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>186373.18999999983</v>
+        <v>186453.93999999983</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>86626.810000000172</v>
+        <v>86546.060000000172</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3603,11 +3603,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1628.2500000000002</v>
+        <v>1758.1500000000003</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2211.75</v>
+        <v>2081.8499999999995</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11307.4</v>
+        <v>12072.2</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3692.6000000000004</v>
+        <v>2927.7999999999993</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3738,11 +3738,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>242302.11999999994</v>
+        <v>259576.11999999994</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>82697.880000000063</v>
+        <v>65423.880000000063</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3911,11 +3911,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1709.3500000000001</v>
+        <v>1714.3500000000001</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5130.6499999999996</v>
+        <v>5125.6499999999996</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3975,11 +3975,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2753.39</v>
+        <v>4774.07</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4366.6100000000006</v>
+        <v>2345.9300000000003</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -4035,11 +4035,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11574.8</v>
+        <v>11655.55</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3425.2000000000007</v>
+        <v>3344.4500000000007</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4163,11 +4163,11 @@
       </c>
       <c r="D22" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>74173.729999999981</v>
+        <v>74178.729999999981</v>
       </c>
       <c r="E22" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>47826.270000000019</v>
+        <v>47821.270000000019</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="21" t="s">
@@ -4182,11 +4182,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>966.94999999999993</v>
+        <v>1483.75</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2353.0500000000002</v>
+        <v>1836.25</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4238,11 +4238,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>136632.95499999967</v>
+        <v>138653.63499999963</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>58367.045000000333</v>
+        <v>56346.365000000369</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4257,11 +4257,11 @@
       </c>
       <c r="J23" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>602.70000000000005</v>
+        <v>1257.3499999999999</v>
       </c>
       <c r="K23" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3407.3</v>
+        <v>2752.65</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -4313,11 +4313,11 @@
       </c>
       <c r="D24" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>97046.740000000093</v>
+        <v>97563.540000000081</v>
       </c>
       <c r="E24" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>42953.259999999907</v>
+        <v>42436.459999999919</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="21" t="s">
@@ -4332,11 +4332,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>521.16000000000008</v>
+        <v>839.7600000000001</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4178.84</v>
+        <v>3860.24</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4349,11 +4349,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>629008.51999999967</v>
+        <v>646282.51999999967</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>-9690.3381818177877</v>
+        <v>-26964.338181817788</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4388,11 +4388,11 @@
       </c>
       <c r="D25" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>86181.329999999798</v>
+        <v>86311.229999999792</v>
       </c>
       <c r="E25" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>56318.670000000202</v>
+        <v>56188.770000000208</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="21" t="s">
@@ -4482,11 +4482,11 @@
       </c>
       <c r="J26" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1615.8200000000004</v>
+        <v>1620.8200000000004</v>
       </c>
       <c r="K26" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1914.1799999999996</v>
+        <v>1909.1799999999996</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -4546,11 +4546,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2020.05</v>
+        <v>2106.0099999999998</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>649.95000000000005</v>
+        <v>563.99000000000024</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4573,11 +4573,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>244351.82999999938</v>
+        <v>244872.42999999938</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>74148.170000000624</v>
+        <v>73627.570000000618</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4652,11 +4652,11 @@
       </c>
       <c r="D30" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>95643.829999999944</v>
+        <v>98334.649999999921</v>
       </c>
       <c r="E30" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>38856.170000000056</v>
+        <v>36165.350000000079</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -4869,11 +4869,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>-55.727272727272748</v>
+        <v>-60.727272727272748</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4889,11 +4889,11 @@
       </c>
       <c r="D34" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>31283.660000000022</v>
+        <v>31288.660000000022</v>
       </c>
       <c r="E34" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>23716.339999999978</v>
+        <v>23711.339999999978</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -4906,11 +4906,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>512178.16500000301</v>
+        <v>519971.72500000335</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>139071.83499999699</v>
+        <v>131278.27499999665</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4949,11 +4949,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>53366.01</v>
+        <v>53684.61</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>19633.989999999998</v>
+        <v>19315.39</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5217,11 +5217,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1141440.5750000011</v>
+        <v>1166508.1350000007</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-490190.57500000112</v>
+        <v>-515258.13500000071</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 23/07/2026 15:04
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3AA7503-AEC8-416E-B77C-B4F6B1BF2F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B2FB21-2DFC-4CC1-AAD4-23D64724828D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -1730,13 +1730,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>41352.389999999978</v>
+            <v>42019.389999999978</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>2106.0099999999998</v>
+            <v>2773.0099999999998</v>
           </cell>
         </row>
         <row r="6">
@@ -1744,7 +1744,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>272788.47999999952</v>
+            <v>272788.47999999957</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
@@ -1793,7 +1793,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="N8">
-            <v>25</v>
+            <v>26</v>
           </cell>
         </row>
         <row r="9">
@@ -1827,7 +1827,7 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>47946.1</v>
+            <v>47346.099999999991</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
@@ -1847,7 +1847,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="I11">
-            <v>4507.2</v>
+            <v>8325.48</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
@@ -1861,7 +1861,7 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>259576.11999999994</v>
+            <v>258976.11999999994</v>
           </cell>
           <cell r="H12" t="str">
             <v>KEY PIRACICABA</v>
@@ -1881,7 +1881,7 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>267282.20000000024</v>
+            <v>271100.4800000001</v>
           </cell>
           <cell r="H13" t="str">
             <v>KEY SP</v>
@@ -1947,7 +1947,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I16">
-            <v>4774.07</v>
+            <v>5167.5699999999988</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -2021,7 +2021,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>138653.63499999963</v>
+            <v>139047.13499999966</v>
           </cell>
           <cell r="H20" t="str">
             <v>NORTE</v>
@@ -2121,19 +2121,19 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>244872.42999999938</v>
+            <v>244872.42999999935</v>
           </cell>
           <cell r="H25" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I25">
-            <v>2448.94</v>
+            <v>3393.64</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="N25">
-            <v>599</v>
+            <v>600</v>
           </cell>
         </row>
         <row r="26">
@@ -2161,7 +2161,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I27">
-            <v>839.7600000000001</v>
+            <v>1007.7600000000001</v>
           </cell>
         </row>
         <row r="28">
@@ -2175,7 +2175,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="I28">
-            <v>183556.93999999994</v>
+            <v>188948.41999999993</v>
           </cell>
         </row>
         <row r="29">
@@ -2183,7 +2183,7 @@
             <v>SJC</v>
           </cell>
           <cell r="F29">
-            <v>60790.330000000104</v>
+            <v>61735.030000000093</v>
           </cell>
         </row>
         <row r="30">
@@ -2199,7 +2199,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F31">
-            <v>53684.61</v>
+            <v>53852.61</v>
           </cell>
         </row>
         <row r="32">
@@ -2207,7 +2207,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4199973.0549999438</v>
+            <v>4205364.5349999433</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4199973.0549999978</v>
+        <v>4205364.5349999983</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>86955.63</v>
+        <v>89128.83</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>78348.490000000005</v>
+        <v>81566.76999999999</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1392526.9450000022</v>
+        <v>1387135.4650000017</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>43044.369999999995</v>
+        <v>40871.17</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-78348.490000000005</v>
+        <v>-81566.76999999999</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.75100099329459058</v>
+        <v>0.75196504872597192</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.66888946153846152</v>
+        <v>0.68560638461538459</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.79023746701846964</v>
+        <v>0.79155672823219003</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3280,11 +3280,11 @@
       </c>
       <c r="D10" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>41352.389999999978</v>
+        <v>42019.389999999978</v>
       </c>
       <c r="E10" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>23147.610000000022</v>
+        <v>22480.610000000022</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="21" t="s">
@@ -3334,11 +3334,11 @@
       </c>
       <c r="V10" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="W10" s="19">
         <f>U10-V10</f>
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -3354,11 +3354,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>272788.47999999952</v>
+        <v>272788.47999999957</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>52211.520000000484</v>
+        <v>52211.520000000426</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3392,11 +3392,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>47946.1</v>
+        <v>47346.099999999991</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>-47946.1</v>
+        <v>-47346.099999999991</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3738,11 +3738,11 @@
       </c>
       <c r="D16" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>259576.11999999994</v>
+        <v>258976.11999999994</v>
       </c>
       <c r="E16" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65423.880000000063</v>
+        <v>66023.880000000063</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="21" t="s">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>267282.20000000024</v>
+        <v>271100.4800000001</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-97282.200000000244</v>
+        <v>-101100.4800000001</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3853,11 +3853,11 @@
       </c>
       <c r="P17" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4507.2</v>
+        <v>8325.48</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="1"/>
-        <v>-4507.2</v>
+        <v>-8325.48</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="19" t="s">
@@ -3975,11 +3975,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4774.07</v>
+        <v>5167.5699999999988</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2345.9300000000003</v>
+        <v>1952.4300000000012</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -4238,11 +4238,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>138653.63499999963</v>
+        <v>139047.13499999966</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>56346.365000000369</v>
+        <v>55952.86500000034</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4332,11 +4332,11 @@
       </c>
       <c r="J24" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>839.7600000000001</v>
+        <v>1007.7600000000001</v>
       </c>
       <c r="K24" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3860.24</v>
+        <v>3692.24</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -4349,11 +4349,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>646282.51999999967</v>
+        <v>649500.79999999981</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>-26964.338181817788</v>
+        <v>-30182.618181817932</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="19" t="s">
@@ -4407,11 +4407,11 @@
       </c>
       <c r="J25" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2448.94</v>
+        <v>3393.64</v>
       </c>
       <c r="K25" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>241.05999999999995</v>
+        <v>-703.63999999999987</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -4546,11 +4546,11 @@
       </c>
       <c r="J27" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2106.0099999999998</v>
+        <v>2773.0099999999998</v>
       </c>
       <c r="K27" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>563.99000000000024</v>
+        <v>-103.00999999999976</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -4573,11 +4573,11 @@
       </c>
       <c r="D28" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>244872.42999999938</v>
+        <v>244872.42999999935</v>
       </c>
       <c r="E28" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>73627.570000000618</v>
+        <v>73627.570000000647</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -4829,11 +4829,11 @@
       </c>
       <c r="D33" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>60790.330000000104</v>
+        <v>61735.030000000093</v>
       </c>
       <c r="E33" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>39209.669999999896</v>
+        <v>38264.969999999907</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -4869,11 +4869,11 @@
       </c>
       <c r="V33" s="6">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE]",'[1]BASE PYTHON'!$P$85,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="3"/>
-        <v>-60.727272727272748</v>
+        <v>-61.727272727272748</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -4906,11 +4906,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>519971.72500000335</v>
+        <v>522144.92500000342</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="4"/>
-        <v>131278.27499999665</v>
+        <v>129105.07499999658</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -4949,11 +4949,11 @@
       </c>
       <c r="D35" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>53684.61</v>
+        <v>53852.61</v>
       </c>
       <c r="E35" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>19315.39</v>
+        <v>19147.39</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -5217,11 +5217,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>1166508.1350000007</v>
+        <v>1171899.6150000005</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="5"/>
-        <v>-515258.13500000071</v>
+        <v>-520649.61500000046</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 24/07/2026 07:10
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B2FB21-2DFC-4CC1-AAD4-23D64724828D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF28961-6D00-4A4B-A4EE-E25DF7D606CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
   <metadataStrings count="3">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-07-23T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;}"/>
   </metadataStrings>
   <mdxMetadata count="2">
     <mdx n="0" f="s">
@@ -1694,7 +1694,7 @@
             <v>DATA</v>
           </cell>
           <cell r="I2" t="str" vm="2">
-            <v>23/07/2026</v>
+            <v/>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -1732,25 +1732,13 @@
           <cell r="F5">
             <v>42019.389999999978</v>
           </cell>
-          <cell r="H5" t="str">
-            <v>CAMPINAS</v>
-          </cell>
-          <cell r="I5">
-            <v>2773.0099999999998</v>
-          </cell>
         </row>
         <row r="6">
           <cell r="E6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>272788.47999999957</v>
-          </cell>
-          <cell r="H6" t="str">
-            <v>CENTRO</v>
-          </cell>
-          <cell r="I6">
-            <v>12072.2</v>
+            <v>274081.17999999953</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -1763,17 +1751,8 @@
           <cell r="F7">
             <v>1082.83</v>
           </cell>
-          <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
-          </cell>
-          <cell r="I7">
-            <v>1257.3499999999999</v>
-          </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
-          </cell>
-          <cell r="N7" t="str">
-            <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
@@ -1783,17 +1762,8 @@
           <cell r="F8">
             <v>151.09</v>
           </cell>
-          <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
-          </cell>
-          <cell r="I8">
-            <v>11655.55</v>
-          </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
-          </cell>
-          <cell r="N8">
-            <v>26</v>
           </cell>
         </row>
         <row r="9">
@@ -1803,17 +1773,8 @@
           <cell r="F9">
             <v>52564.160000000003</v>
           </cell>
-          <cell r="H9" t="str">
-            <v>JUNDIAI</v>
-          </cell>
-          <cell r="I9">
-            <v>1261.6000000000001</v>
-          </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
-          </cell>
-          <cell r="N9">
-            <v>45</v>
           </cell>
         </row>
         <row r="10">
@@ -1821,19 +1782,10 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>186453.93999999983</v>
-          </cell>
-          <cell r="H10" t="str">
-            <v>KEY ABC</v>
-          </cell>
-          <cell r="I10">
-            <v>47346.099999999991</v>
+            <v>187939.73999999982</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
-          </cell>
-          <cell r="N10">
-            <v>35</v>
           </cell>
         </row>
         <row r="11">
@@ -1843,17 +1795,8 @@
           <cell r="F11">
             <v>53021.480000000069</v>
           </cell>
-          <cell r="H11" t="str">
-            <v>KEY CASA</v>
-          </cell>
-          <cell r="I11">
-            <v>8325.48</v>
-          </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
-          </cell>
-          <cell r="N11">
-            <v>52</v>
           </cell>
         </row>
         <row r="12">
@@ -1863,17 +1806,8 @@
           <cell r="F12">
             <v>258976.11999999994</v>
           </cell>
-          <cell r="H12" t="str">
-            <v>KEY PIRACICABA</v>
-          </cell>
-          <cell r="I12">
-            <v>18252.82</v>
-          </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
-          </cell>
-          <cell r="N12">
-            <v>21</v>
           </cell>
         </row>
         <row r="13">
@@ -1881,19 +1815,10 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>271100.4800000001</v>
-          </cell>
-          <cell r="H13" t="str">
-            <v>KEY SP</v>
-          </cell>
-          <cell r="I13">
-            <v>16606.490000000002</v>
+            <v>266593.28000000014</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
-          </cell>
-          <cell r="N13">
-            <v>31</v>
           </cell>
         </row>
         <row r="14">
@@ -1901,19 +1826,10 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>851393.40000000026</v>
-          </cell>
-          <cell r="H14" t="str">
-            <v>KEY ZL</v>
-          </cell>
-          <cell r="I14">
-            <v>9288.7000000000007</v>
+            <v>851393.40000000037</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
-          </cell>
-          <cell r="N14">
-            <v>50</v>
           </cell>
         </row>
         <row r="15">
@@ -1923,17 +1839,8 @@
           <cell r="F15">
             <v>105736.07999999996</v>
           </cell>
-          <cell r="H15" t="str">
-            <v>LESTE</v>
-          </cell>
-          <cell r="I15">
-            <v>1714.3500000000001</v>
-          </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
-          </cell>
-          <cell r="N15">
-            <v>25</v>
           </cell>
         </row>
         <row r="16">
@@ -1943,17 +1850,8 @@
           <cell r="F16">
             <v>114220.90000000004</v>
           </cell>
-          <cell r="H16" t="str">
-            <v>LESTE MOOCA</v>
-          </cell>
-          <cell r="I16">
-            <v>5167.5699999999988</v>
-          </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="N16">
-            <v>38</v>
           </cell>
         </row>
         <row r="17">
@@ -1961,19 +1859,10 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>283519.83999999997</v>
-          </cell>
-          <cell r="H17" t="str">
-            <v>LESTE PENHA</v>
-          </cell>
-          <cell r="I17">
-            <v>1483.75</v>
+            <v>288608.1399999999</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
-          </cell>
-          <cell r="N17">
-            <v>36</v>
           </cell>
         </row>
         <row r="18">
@@ -1983,17 +1872,8 @@
           <cell r="F18">
             <v>287660.6999999999</v>
           </cell>
-          <cell r="H18" t="str">
-            <v>LESTE TATUAPE</v>
-          </cell>
-          <cell r="I18">
-            <v>1758.1500000000003</v>
-          </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
-          </cell>
-          <cell r="N18">
-            <v>43</v>
           </cell>
         </row>
         <row r="19">
@@ -2003,17 +1883,8 @@
           <cell r="F19">
             <v>74178.729999999981</v>
           </cell>
-          <cell r="H19" t="str">
-            <v>MOGI</v>
-          </cell>
-          <cell r="I19">
-            <v>2791.9200000000005</v>
-          </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
-          </cell>
-          <cell r="N19">
-            <v>60</v>
           </cell>
         </row>
         <row r="20">
@@ -2021,19 +1892,10 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F20">
-            <v>139047.13499999966</v>
-          </cell>
-          <cell r="H20" t="str">
-            <v>NORTE</v>
-          </cell>
-          <cell r="I20">
-            <v>14091.089999999997</v>
+            <v>139594.11499999967</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
-          </cell>
-          <cell r="N20">
-            <v>27</v>
           </cell>
         </row>
         <row r="21">
@@ -2041,19 +1903,10 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F21">
-            <v>97563.540000000081</v>
-          </cell>
-          <cell r="H21" t="str">
-            <v>OSASCO</v>
-          </cell>
-          <cell r="I21">
-            <v>8678.7999999999975</v>
+            <v>97563.540000000095</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="N21">
-            <v>28</v>
           </cell>
         </row>
         <row r="22">
@@ -2063,17 +1916,8 @@
           <cell r="F22">
             <v>86311.229999999792</v>
           </cell>
-          <cell r="H22" t="str">
-            <v>PIRITUBA</v>
-          </cell>
-          <cell r="I22">
-            <v>5626.22</v>
-          </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
-          </cell>
-          <cell r="N22">
-            <v>36</v>
           </cell>
         </row>
         <row r="23">
@@ -2083,17 +1927,8 @@
           <cell r="F23">
             <v>51628.47000000011</v>
           </cell>
-          <cell r="H23" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
-          <cell r="I23">
-            <v>6971.079999999999</v>
-          </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
-          </cell>
-          <cell r="N23">
-            <v>22</v>
           </cell>
         </row>
         <row r="24">
@@ -2103,17 +1938,8 @@
           <cell r="F24">
             <v>177256.26999999961</v>
           </cell>
-          <cell r="H24" t="str">
-            <v>SBC</v>
-          </cell>
-          <cell r="I24">
-            <v>5803.97</v>
-          </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
-          </cell>
-          <cell r="N24">
-            <v>25</v>
           </cell>
         </row>
         <row r="25">
@@ -2121,19 +1947,10 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F25">
-            <v>244872.42999999935</v>
-          </cell>
-          <cell r="H25" t="str">
-            <v>SJC</v>
-          </cell>
-          <cell r="I25">
-            <v>3393.64</v>
+            <v>244872.4299999995</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
-          </cell>
-          <cell r="N25">
-            <v>600</v>
           </cell>
         </row>
         <row r="26">
@@ -2143,25 +1960,13 @@
           <cell r="F26">
             <v>98334.649999999921</v>
           </cell>
-          <cell r="H26" t="str">
-            <v>SJC/VALE</v>
-          </cell>
-          <cell r="I26">
-            <v>1620.8200000000004</v>
-          </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F27">
-            <v>123291.98999999996</v>
-          </cell>
-          <cell r="H27" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
-          <cell r="I27">
-            <v>1007.7600000000001</v>
+            <v>123291.98999999998</v>
           </cell>
         </row>
         <row r="28">
@@ -2171,12 +1976,6 @@
           <cell r="F28">
             <v>185314.89999999973</v>
           </cell>
-          <cell r="H28" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I28">
-            <v>188948.41999999993</v>
-          </cell>
         </row>
         <row r="29">
           <cell r="E29" t="str">
@@ -2191,7 +1990,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F30">
-            <v>31288.660000000022</v>
+            <v>31876.060000000023</v>
           </cell>
         </row>
         <row r="31">
@@ -2207,7 +2006,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F32">
-            <v>4205364.5349999433</v>
+            <v>4209858.5149999438</v>
           </cell>
           <cell r="P32" t="str">
             <v>Soma de TOTAL</v>
@@ -3058,7 +2857,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>4205364.5349999983</v>
+        <v>4209858.5149999987</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -3069,7 +2868,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>89128.83</v>
+        <v>0</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -3080,7 +2879,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>81566.76999999999</v>
+        <v>0</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3091,7 +2890,7 @@
       </c>
       <c r="U5" s="4">
         <f>SUM(V10:V26)</f>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -3103,7 +2902,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>1387135.4650000017</v>
+        <v>1382641.4850000013</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -3114,7 +2913,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>40871.17</v>
+        <v>130000</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -3125,7 +2924,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-81566.76999999999</v>
+        <v>0</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -3136,7 +2935,7 @@
       </c>
       <c r="U6" s="4">
         <f>U4-U5</f>
-        <v>158</v>
+        <v>758</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -3148,7 +2947,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.75196504872597192</v>
+        <v>0.75276862136790323</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -3159,7 +2958,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.68560638461538459</v>
+        <v>0</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -3181,7 +2980,7 @@
       </c>
       <c r="U7" s="3">
         <f>1-(U6/U4)</f>
-        <v>0.79155672823219003</v>
+        <v>0</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -3299,11 +3098,11 @@
       </c>
       <c r="J10" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8678.7999999999975</v>
+        <v>0</v>
       </c>
       <c r="K10" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3411.2000000000025</v>
+        <v>12090</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -3334,11 +3133,11 @@
       </c>
       <c r="V10" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="W10" s="19">
         <f>U10-V10</f>
-        <v>10</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
@@ -3354,11 +3153,11 @@
       </c>
       <c r="D11" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>272788.47999999957</v>
+        <v>274081.17999999953</v>
       </c>
       <c r="E11" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>52211.520000000426</v>
+        <v>50918.820000000473</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="21" t="s">
@@ -3373,11 +3172,11 @@
       </c>
       <c r="J11" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14091.089999999997</v>
+        <v>0</v>
       </c>
       <c r="K11" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-3091.0899999999965</v>
+        <v>11000</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -3392,11 +3191,11 @@
       </c>
       <c r="P11" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>47346.099999999991</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="2">
         <f>O11-P11</f>
-        <v>-47346.099999999991</v>
+        <v>0</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="19" t="s">
@@ -3411,11 +3210,11 @@
       </c>
       <c r="V11" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="W11" s="19">
         <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>7</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -3449,11 +3248,11 @@
       </c>
       <c r="J12" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5626.22</v>
+        <v>0</v>
       </c>
       <c r="K12" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-226.22000000000025</v>
+        <v>5400</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -3487,11 +3286,11 @@
       </c>
       <c r="V12" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="W12" s="19">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -3526,11 +3325,11 @@
       </c>
       <c r="J13" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5803.97</v>
+        <v>0</v>
       </c>
       <c r="K13" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7196.03</v>
+        <v>13000</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -3545,11 +3344,11 @@
       </c>
       <c r="P13" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9288.7000000000007</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ref="Q13:Q17" si="1">O13-P13</f>
-        <v>-9288.7000000000007</v>
+        <v>0</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="19" t="s">
@@ -3564,11 +3363,11 @@
       </c>
       <c r="V13" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="W13" s="19">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
@@ -3584,11 +3383,11 @@
       </c>
       <c r="D14" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>186453.93999999983</v>
+        <v>187939.73999999982</v>
       </c>
       <c r="E14" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>86546.060000000172</v>
+        <v>85060.260000000184</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="21" t="s">
@@ -3603,11 +3402,11 @@
       </c>
       <c r="J14" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1758.1500000000003</v>
+        <v>0</v>
       </c>
       <c r="K14" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2081.8499999999995</v>
+        <v>3840</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -3641,11 +3440,11 @@
       </c>
       <c r="V14" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="W14" s="19">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3680,11 +3479,11 @@
       </c>
       <c r="J15" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>12072.2</v>
+        <v>0</v>
       </c>
       <c r="K15" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2927.7999999999993</v>
+        <v>15000</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -3699,11 +3498,11 @@
       </c>
       <c r="P15" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>16606.490000000002</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="1"/>
-        <v>-16606.490000000002</v>
+        <v>0</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="19" t="s">
@@ -3718,11 +3517,11 @@
       </c>
       <c r="V15" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="W15" s="19">
         <f>U15-V15</f>
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
@@ -3757,11 +3556,11 @@
       </c>
       <c r="J16" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6971.079999999999</v>
+        <v>0</v>
       </c>
       <c r="K16" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2868.920000000001</v>
+        <v>9840</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -3795,11 +3594,11 @@
       </c>
       <c r="V16" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="W16" s="19">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
@@ -3815,11 +3614,11 @@
       </c>
       <c r="D17" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>271100.4800000001</v>
+        <v>266593.28000000014</v>
       </c>
       <c r="E17" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-101100.4800000001</v>
+        <v>-96593.280000000144</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="21" t="s">
@@ -3834,11 +3633,11 @@
       </c>
       <c r="J17" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2791.9200000000005</v>
+        <v>0</v>
       </c>
       <c r="K17" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2058.0799999999995</v>
+        <v>4850</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -3853,11 +3652,11 @@
       </c>
       <c r="P17" s="2">
         <f>_xlfn.XLOOKUP(Tabela8[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8325.48</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="1"/>
-        <v>-8325.48</v>
+        <v>0</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="19" t="s">
@@ -3872,11 +3671,11 @@
       </c>
       <c r="V17" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="W17" s="19">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
@@ -3892,11 +3691,11 @@
       </c>
       <c r="D18" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>851393.40000000026</v>
+        <v>851393.40000000037</v>
       </c>
       <c r="E18" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>98606.599999999744</v>
+        <v>98606.599999999627</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="21" t="s">
@@ -3911,11 +3710,11 @@
       </c>
       <c r="J18" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1714.3500000000001</v>
+        <v>0</v>
       </c>
       <c r="K18" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5125.6499999999996</v>
+        <v>6840</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -3936,11 +3735,11 @@
       </c>
       <c r="V18" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="W18" s="19">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
@@ -3975,11 +3774,11 @@
       </c>
       <c r="J19" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5167.5699999999988</v>
+        <v>0</v>
       </c>
       <c r="K19" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1952.4300000000012</v>
+        <v>7120</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -3996,11 +3795,11 @@
       </c>
       <c r="V19" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="W19" s="19">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
@@ -4016,11 +3815,11 @@
       </c>
       <c r="D20" s="26">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>283519.83999999997</v>
+        <v>288608.1399999999</v>
       </c>
       <c r="E20" s="27">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>276480.16000000003</v>
+        <v>271391.8600000001</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="21" t="s">
@@ -4035,11 +3834,11 @@
       </c>
       <c r="J20" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11655.55</v>
+        <v>0</v>
       </c>
       <c r="K20" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3344.4500000000007</v>
+        <v>15000</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -4068,11 +3867,11 @@
       </c>
       <c r="V20" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="W20" s="19">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
@@ -4107,11 +3906,11 @@
       </c>
       <c r="J21" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1261.6000000000001</v>
+        <v>0</v>
       </c>
       <c r="K21" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3838.3999999999996</v>
+        <v>5100</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -4143,11 +3942,11 @@
       </c>
       <c r="V21" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="W21" s="19">
         <f t="shared" ref="W21:W26" si="2">U21-V21</f>
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
@@ -4182,11 +3981,11 @@
       </c>
       <c r="J22" s="22">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1483.75</v>
+        <v>0</v>
       </c>
       <c r="K22" s="23">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1836.25</v>
+        <v>3320</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -4218,11 +4017,11 @@
       </c>
       <c r="V22" s="19">
         <f>_xlfn.XLOOKUP(Tabela2[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0)</f>
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="W22" s="19">
         <f t="shared" si="2"/>
-        <v>12</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
@@ -4238,11 +4037,11 @@
       </c>
       <c r="D23" s="17">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[VENDEDOR]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>139047.13499999966</v>
+        <v>139594.11499999967</v>
       </c>
       <c r="E23" s="24">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>55952.86500000034</v>
+        <v>55405.885000000329</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="21" t="s">
@@ -4257,11 +4056,11 @@
       </c>
       <c r="J23" s="22">
       